<commit_message>
Actualiza portafolio 2026-06-22 15:07 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -473,6 +473,9 @@
   </si>
   <si>
     <t xml:space="preserve">OT 4353 - Reparacion VDF Danfoss 110 KW </t>
+  </si>
+  <si>
+    <t>Finalizados</t>
   </si>
   <si>
     <t>TABL3-277</t>
@@ -925,9 +928,6 @@
   </si>
   <si>
     <t>OT 4249 - RODETE S/PLANO 1991.10.30.D48</t>
-  </si>
-  <si>
-    <t>Finalizados</t>
   </si>
   <si>
     <t>TABL3-209</t>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="10">
-        <v>46185.62463690972</v>
+        <v>46195.566871620365</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>55</v>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="C39" s="11"/>
       <c r="D39" s="10">
-        <v>46188.63100862269</v>
+        <v>46195.60458381944</v>
       </c>
       <c r="E39" s="11" t="s">
         <v>145</v>
@@ -4117,15 +4117,17 @@
       <c r="B41" s="10">
         <v>46188.630276365744</v>
       </c>
-      <c r="C41" s="11"/>
+      <c r="C41" s="10">
+        <v>46195.60462475695</v>
+      </c>
       <c r="D41" s="10">
-        <v>46188.63049422453</v>
+        <v>46195.60464252315</v>
       </c>
       <c r="E41" s="11" t="s">
         <v>151</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>28</v>
+        <v>152</v>
       </c>
       <c r="G41" s="11" t="s">
         <v>28</v>
@@ -4142,7 +4144,7 @@
         <v>28</v>
       </c>
       <c r="M41" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N41" s="11" t="s">
         <v>145</v>
@@ -4154,7 +4156,7 @@
         <v>28</v>
       </c>
       <c r="Q41" s="11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="R41" s="11"/>
       <c r="S41" s="11"/>
@@ -4163,7 +4165,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B42" s="5">
         <v>46133.79734877315</v>
@@ -4173,10 +4175,10 @@
         <v>46141.74131788194</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>56</v>
@@ -4207,7 +4209,7 @@
         <v>28</v>
       </c>
       <c r="Q42" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="R42" s="6"/>
       <c r="S42" s="12" t="s">
@@ -4220,7 +4222,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B43" s="10">
         <v>46133.79847596065</v>
@@ -4230,7 +4232,7 @@
         <v>46134.65975528935</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F43" s="11" t="s">
         <v>28</v>
@@ -4251,7 +4253,7 @@
         <v>28</v>
       </c>
       <c r="N43" s="11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O43" s="11" t="s">
         <v>28</v>
@@ -4260,7 +4262,7 @@
         <v>28</v>
       </c>
       <c r="Q43" s="11" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R43" s="11"/>
       <c r="S43" s="11"/>
@@ -4269,7 +4271,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B44" s="5">
         <v>46133.800000937495</v>
@@ -4279,10 +4281,10 @@
         <v>46141.74254248843</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G44" s="6" t="s">
         <v>56</v>
@@ -4313,7 +4315,7 @@
         <v>28</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="R44" s="6"/>
       <c r="S44" s="7" t="s">
@@ -4326,7 +4328,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B45" s="10">
         <v>46133.800366041665</v>
@@ -4336,7 +4338,7 @@
         <v>46133.800594699074</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F45" s="11" t="s">
         <v>28</v>
@@ -4357,7 +4359,7 @@
         <v>28</v>
       </c>
       <c r="N45" s="11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="O45" s="11" t="s">
         <v>28</v>
@@ -4366,7 +4368,7 @@
         <v>28</v>
       </c>
       <c r="Q45" s="11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R45" s="11"/>
       <c r="S45" s="11"/>
@@ -4375,20 +4377,20 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B46" s="5">
         <v>46093.55797671297</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46193.570451481486</v>
+        <v>46195.57757945602</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G46" s="6" t="s">
         <v>56</v>
@@ -4421,7 +4423,7 @@
         <v>28</v>
       </c>
       <c r="Q46" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R46" s="6"/>
       <c r="S46" s="12" t="s">
@@ -4434,7 +4436,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B47" s="10">
         <v>46094.639967870375</v>
@@ -4444,7 +4446,7 @@
         <v>46130.18563101852</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F47" s="11" t="s">
         <v>28</v>
@@ -4467,7 +4469,7 @@
         <v>28</v>
       </c>
       <c r="N47" s="11" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O47" s="11" t="s">
         <v>28</v>
@@ -4476,7 +4478,7 @@
         <v>28</v>
       </c>
       <c r="Q47" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="R47" s="11"/>
       <c r="S47" s="12" t="s">
@@ -4487,7 +4489,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B48" s="5">
         <v>46094.64022527778</v>
@@ -4497,7 +4499,7 @@
         <v>46101.15093898148</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>28</v>
@@ -4520,7 +4522,7 @@
         <v>28</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>28</v>
@@ -4529,7 +4531,7 @@
         <v>28</v>
       </c>
       <c r="Q48" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="R48" s="6"/>
       <c r="S48" s="12" t="s">
@@ -4540,7 +4542,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B49" s="10">
         <v>46133.81046972222</v>
@@ -4550,10 +4552,10 @@
         <v>46162.79059445602</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G49" s="11" t="s">
         <v>56</v>
@@ -4584,7 +4586,7 @@
         <v>28</v>
       </c>
       <c r="Q49" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="R49" s="11"/>
       <c r="S49" s="7" t="s">
@@ -4597,7 +4599,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B50" s="5">
         <v>46133.8107147338</v>
@@ -4607,7 +4609,7 @@
         <v>46133.81087918981</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>28</v>
@@ -4628,7 +4630,7 @@
         <v>28</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>28</v>
@@ -4637,7 +4639,7 @@
         <v>28</v>
       </c>
       <c r="Q50" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R50" s="6"/>
       <c r="S50" s="6"/>
@@ -4646,7 +4648,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B51" s="10">
         <v>46133.80470612268</v>
@@ -4656,10 +4658,10 @@
         <v>46185.60141636574</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G51" s="11" t="s">
         <v>56</v>
@@ -4690,7 +4692,7 @@
         <v>28</v>
       </c>
       <c r="Q51" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="R51" s="11"/>
       <c r="S51" s="12" t="s">
@@ -4703,7 +4705,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B52" s="5">
         <v>46133.80545771991</v>
@@ -4713,7 +4715,7 @@
         <v>46133.80564510416</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>28</v>
@@ -4734,7 +4736,7 @@
         <v>28</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>28</v>
@@ -4743,7 +4745,7 @@
         <v>28</v>
       </c>
       <c r="Q52" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="R52" s="6"/>
       <c r="S52" s="6"/>
@@ -4752,7 +4754,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B53" s="10">
         <v>46133.80570512731</v>
@@ -4762,7 +4764,7 @@
         <v>46133.80583366899</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F53" s="11" t="s">
         <v>28</v>
@@ -4783,7 +4785,7 @@
         <v>28</v>
       </c>
       <c r="N53" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O53" s="11" t="s">
         <v>28</v>
@@ -4792,7 +4794,7 @@
         <v>28</v>
       </c>
       <c r="Q53" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="R53" s="11"/>
       <c r="S53" s="11"/>
@@ -4801,7 +4803,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B54" s="5">
         <v>46133.8058850463</v>
@@ -4811,7 +4813,7 @@
         <v>46133.80636234954</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>28</v>
@@ -4832,7 +4834,7 @@
         <v>28</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>28</v>
@@ -4841,7 +4843,7 @@
         <v>28</v>
       </c>
       <c r="Q54" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="R54" s="6"/>
       <c r="S54" s="6"/>
@@ -4850,7 +4852,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B55" s="10">
         <v>46133.80664880787</v>
@@ -4860,7 +4862,7 @@
         <v>46133.80681135417</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F55" s="11" t="s">
         <v>28</v>
@@ -4881,7 +4883,7 @@
         <v>28</v>
       </c>
       <c r="N55" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O55" s="11" t="s">
         <v>28</v>
@@ -4890,7 +4892,7 @@
         <v>28</v>
       </c>
       <c r="Q55" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="R55" s="11"/>
       <c r="S55" s="11"/>
@@ -4899,7 +4901,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B56" s="5">
         <v>46133.80701400463</v>
@@ -4909,10 +4911,10 @@
         <v>46162.79057355324</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G56" s="6" t="s">
         <v>56</v>
@@ -4928,7 +4930,7 @@
         <v>28</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M56" s="6" t="s">
         <v>0</v>
@@ -4943,7 +4945,7 @@
         <v>28</v>
       </c>
       <c r="Q56" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="R56" s="6"/>
       <c r="S56" s="12" t="s">
@@ -4954,7 +4956,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B57" s="10">
         <v>46133.80727017361</v>
@@ -4964,7 +4966,7 @@
         <v>46133.80736961805</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F57" s="11" t="s">
         <v>28</v>
@@ -4985,7 +4987,7 @@
         <v>28</v>
       </c>
       <c r="N57" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O57" s="11" t="s">
         <v>28</v>
@@ -4994,7 +4996,7 @@
         <v>28</v>
       </c>
       <c r="Q57" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="R57" s="11"/>
       <c r="S57" s="11"/>
@@ -5003,7 +5005,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B58" s="5">
         <v>46133.79901350694</v>
@@ -5013,10 +5015,10 @@
         <v>46162.79056252315</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G58" s="6" t="s">
         <v>56</v>
@@ -5047,7 +5049,7 @@
         <v>28</v>
       </c>
       <c r="Q58" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="R58" s="6"/>
       <c r="S58" s="12" t="s">
@@ -5060,7 +5062,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B59" s="10">
         <v>46133.79961443287</v>
@@ -5070,7 +5072,7 @@
         <v>46133.79989851852</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F59" s="11" t="s">
         <v>28</v>
@@ -5091,7 +5093,7 @@
         <v>28</v>
       </c>
       <c r="N59" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="O59" s="11" t="s">
         <v>28</v>
@@ -5100,7 +5102,7 @@
         <v>28</v>
       </c>
       <c r="Q59" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="R59" s="11"/>
       <c r="S59" s="11"/>
@@ -5109,7 +5111,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B60" s="5">
         <v>46093.557977812496</v>
@@ -5119,10 +5121,10 @@
         <v>46162.79054756944</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G60" s="6" t="s">
         <v>56</v>
@@ -5153,7 +5155,7 @@
         <v>28</v>
       </c>
       <c r="Q60" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="R60" s="6"/>
       <c r="S60" s="12" t="s">
@@ -5166,7 +5168,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B61" s="10">
         <v>46094.64358574074</v>
@@ -5176,7 +5178,7 @@
         <v>46094.643782430554</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F61" s="11" t="s">
         <v>28</v>
@@ -5197,7 +5199,7 @@
         <v>28</v>
       </c>
       <c r="N61" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="O61" s="11" t="s">
         <v>28</v>
@@ -5206,7 +5208,7 @@
         <v>28</v>
       </c>
       <c r="Q61" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="R61" s="11"/>
       <c r="S61" s="11"/>
@@ -5215,7 +5217,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B62" s="5">
         <v>46133.80890888889</v>
@@ -5225,10 +5227,10 @@
         <v>46162.7905368287</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G62" s="6" t="s">
         <v>56</v>
@@ -5244,7 +5246,7 @@
         <v>28</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="M62" s="6" t="s">
         <v>0</v>
@@ -5259,7 +5261,7 @@
         <v>28</v>
       </c>
       <c r="Q62" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="R62" s="6"/>
       <c r="S62" s="15" t="s">
@@ -5272,7 +5274,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B63" s="10">
         <v>46133.809437812495</v>
@@ -5282,7 +5284,7 @@
         <v>46133.80958457176</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F63" s="11" t="s">
         <v>28</v>
@@ -5303,7 +5305,7 @@
         <v>28</v>
       </c>
       <c r="N63" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="O63" s="11" t="s">
         <v>28</v>
@@ -5312,7 +5314,7 @@
         <v>28</v>
       </c>
       <c r="Q63" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="R63" s="11"/>
       <c r="S63" s="11"/>
@@ -5321,7 +5323,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B64" s="5">
         <v>46093.55797666666</v>
@@ -5331,10 +5333,10 @@
         <v>46162.790523668984</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G64" s="6" t="s">
         <v>56</v>
@@ -5365,7 +5367,7 @@
         <v>28</v>
       </c>
       <c r="Q64" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="R64" s="6"/>
       <c r="S64" s="12" t="s">
@@ -5378,7 +5380,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B65" s="10">
         <v>46094.64611630787</v>
@@ -5388,7 +5390,7 @@
         <v>46094.64631732639</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F65" s="11" t="s">
         <v>28</v>
@@ -5409,7 +5411,7 @@
         <v>28</v>
       </c>
       <c r="N65" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O65" s="11" t="s">
         <v>28</v>
@@ -5418,7 +5420,7 @@
         <v>28</v>
       </c>
       <c r="Q65" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="R65" s="11"/>
       <c r="S65" s="11"/>
@@ -5427,7 +5429,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B66" s="5">
         <v>46094.64632454861</v>
@@ -5437,7 +5439,7 @@
         <v>46094.64655788195</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>28</v>
@@ -5458,7 +5460,7 @@
         <v>28</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O66" s="6" t="s">
         <v>28</v>
@@ -5467,7 +5469,7 @@
         <v>28</v>
       </c>
       <c r="Q66" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="R66" s="6"/>
       <c r="S66" s="6"/>
@@ -5476,7 +5478,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B67" s="10">
         <v>46093.55797637731</v>
@@ -5486,10 +5488,10 @@
         <v>46162.79050667824</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G67" s="11" t="s">
         <v>56</v>
@@ -5520,7 +5522,7 @@
         <v>28</v>
       </c>
       <c r="Q67" s="11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="R67" s="11"/>
       <c r="S67" s="12" t="s">
@@ -5533,7 +5535,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B68" s="5">
         <v>46094.645434618054</v>
@@ -5543,7 +5545,7 @@
         <v>46094.645602916666</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>28</v>
@@ -5564,7 +5566,7 @@
         <v>28</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O68" s="6" t="s">
         <v>28</v>
@@ -5573,7 +5575,7 @@
         <v>28</v>
       </c>
       <c r="Q68" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="R68" s="6"/>
       <c r="S68" s="6"/>
@@ -5582,7 +5584,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B69" s="10">
         <v>46093.55797821759</v>
@@ -5592,10 +5594,10 @@
         <v>46162.79049341435</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G69" s="11" t="s">
         <v>56</v>
@@ -5626,7 +5628,7 @@
         <v>28</v>
       </c>
       <c r="Q69" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="R69" s="11"/>
       <c r="S69" s="12" t="s">
@@ -5639,7 +5641,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B70" s="5">
         <v>46094.65140127315</v>
@@ -5649,7 +5651,7 @@
         <v>46094.65150827546</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>28</v>
@@ -5670,7 +5672,7 @@
         <v>28</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="O70" s="6" t="s">
         <v>28</v>
@@ -5679,7 +5681,7 @@
         <v>28</v>
       </c>
       <c r="Q70" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="R70" s="6"/>
       <c r="S70" s="6"/>
@@ -5688,7 +5690,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B71" s="10">
         <v>46093.557976192125</v>
@@ -5698,10 +5700,10 @@
         <v>46142.16936487269</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G71" s="11" t="s">
         <v>56</v>
@@ -5732,20 +5734,20 @@
         <v>28</v>
       </c>
       <c r="Q71" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="R71" s="11"/>
       <c r="S71" s="15" t="s">
         <v>96</v>
       </c>
       <c r="T71" s="17" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="U71" s="11"/>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B72" s="5">
         <v>46094.63540701389</v>
@@ -5755,7 +5757,7 @@
         <v>46094.63563651621</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>28</v>
@@ -5776,7 +5778,7 @@
         <v>28</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="O72" s="6" t="s">
         <v>28</v>
@@ -5785,7 +5787,7 @@
         <v>28</v>
       </c>
       <c r="Q72" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="R72" s="6"/>
       <c r="S72" s="6"/>
@@ -5794,7 +5796,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="9" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B73" s="10">
         <v>46093.55797792824</v>
@@ -5804,10 +5806,10 @@
         <v>46134.689549421295</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G73" s="11" t="s">
         <v>26</v>
@@ -5838,7 +5840,7 @@
         <v>28</v>
       </c>
       <c r="Q73" s="11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="R73" s="11"/>
       <c r="S73" s="12" t="s">
@@ -5851,7 +5853,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B74" s="5">
         <v>46094.64988140046</v>
@@ -5861,7 +5863,7 @@
         <v>46094.64998811342</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>28</v>
@@ -5882,7 +5884,7 @@
         <v>28</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="O74" s="6" t="s">
         <v>28</v>
@@ -5891,7 +5893,7 @@
         <v>28</v>
       </c>
       <c r="Q74" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="R74" s="6"/>
       <c r="S74" s="6"/>
@@ -5900,7 +5902,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="9" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B75" s="10">
         <v>46093.55797513889</v>
@@ -5910,10 +5912,10 @@
         <v>46098.62589137732</v>
       </c>
       <c r="E75" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F75" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G75" s="11" t="s">
         <v>26</v>
@@ -5946,20 +5948,20 @@
         <v>28</v>
       </c>
       <c r="Q75" s="11" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="R75" s="11"/>
       <c r="S75" s="12" t="s">
         <v>43</v>
       </c>
       <c r="T75" s="17" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="U75" s="11"/>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B76" s="5">
         <v>46094.566601597224</v>
@@ -5969,7 +5971,7 @@
         <v>46094.56736538194</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>28</v>
@@ -5990,7 +5992,7 @@
         <v>28</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O76" s="6" t="s">
         <v>28</v>
@@ -5999,7 +6001,7 @@
         <v>28</v>
       </c>
       <c r="Q76" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R76" s="6"/>
       <c r="S76" s="6"/>
@@ -6008,7 +6010,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B77" s="10">
         <v>46094.566937951386</v>
@@ -6018,7 +6020,7 @@
         <v>46094.56773407407</v>
       </c>
       <c r="E77" s="11" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F77" s="11" t="s">
         <v>28</v>
@@ -6039,7 +6041,7 @@
         <v>28</v>
       </c>
       <c r="N77" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O77" s="11" t="s">
         <v>28</v>
@@ -6048,7 +6050,7 @@
         <v>28</v>
       </c>
       <c r="Q77" s="11" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R77" s="11"/>
       <c r="S77" s="11"/>
@@ -6057,7 +6059,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B78" s="5">
         <v>46094.56748170139</v>
@@ -6067,7 +6069,7 @@
         <v>46094.56795886574</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>28</v>
@@ -6088,7 +6090,7 @@
         <v>28</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O78" s="6" t="s">
         <v>28</v>
@@ -6097,7 +6099,7 @@
         <v>28</v>
       </c>
       <c r="Q78" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="R78" s="6"/>
       <c r="S78" s="6"/>
@@ -6106,7 +6108,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="9" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B79" s="10">
         <v>46094.56796667824</v>
@@ -6116,7 +6118,7 @@
         <v>46094.56820407408</v>
       </c>
       <c r="E79" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F79" s="11" t="s">
         <v>28</v>
@@ -6137,7 +6139,7 @@
         <v>28</v>
       </c>
       <c r="N79" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="O79" s="11" t="s">
         <v>28</v>
@@ -6146,7 +6148,7 @@
         <v>28</v>
       </c>
       <c r="Q79" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="R79" s="11"/>
       <c r="S79" s="11"/>
@@ -6155,7 +6157,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B80" s="5">
         <v>46093.557975625</v>
@@ -6165,10 +6167,10 @@
         <v>46112.84178105324</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G80" s="6" t="s">
         <v>26</v>
@@ -6201,20 +6203,20 @@
         <v>28</v>
       </c>
       <c r="Q80" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="R80" s="6"/>
       <c r="S80" s="12" t="s">
         <v>43</v>
       </c>
       <c r="T80" s="17" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="U80" s="6"/>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="9" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B81" s="10">
         <v>46094.57064802083</v>
@@ -6224,7 +6226,7 @@
         <v>46094.59020585648</v>
       </c>
       <c r="E81" s="11" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F81" s="11" t="s">
         <v>28</v>
@@ -6245,7 +6247,7 @@
         <v>28</v>
       </c>
       <c r="N81" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="O81" s="11" t="s">
         <v>28</v>
@@ -6254,7 +6256,7 @@
         <v>28</v>
       </c>
       <c r="Q81" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="R81" s="11"/>
       <c r="S81" s="11"/>
@@ -6263,7 +6265,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B82" s="5">
         <v>46094.57343428241</v>
@@ -6273,7 +6275,7 @@
         <v>46094.59023394676</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>28</v>
@@ -6294,7 +6296,7 @@
         <v>28</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="O82" s="6" t="s">
         <v>28</v>
@@ -6303,7 +6305,7 @@
         <v>28</v>
       </c>
       <c r="Q82" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="R82" s="6"/>
       <c r="S82" s="6"/>
@@ -6312,7 +6314,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B83" s="10">
         <v>46094.573594710644</v>
@@ -6322,7 +6324,7 @@
         <v>46094.59026199074</v>
       </c>
       <c r="E83" s="11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F83" s="11" t="s">
         <v>28</v>
@@ -6343,7 +6345,7 @@
         <v>28</v>
       </c>
       <c r="N83" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="O83" s="11" t="s">
         <v>28</v>
@@ -6352,7 +6354,7 @@
         <v>28</v>
       </c>
       <c r="Q83" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="R83" s="11"/>
       <c r="S83" s="11"/>
@@ -6361,7 +6363,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B84" s="5">
         <v>46094.57373981482</v>
@@ -6371,7 +6373,7 @@
         <v>46094.59030239584</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>28</v>
@@ -6392,7 +6394,7 @@
         <v>28</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="O84" s="6" t="s">
         <v>28</v>
@@ -6401,7 +6403,7 @@
         <v>28</v>
       </c>
       <c r="Q84" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R84" s="6"/>
       <c r="S84" s="6"/>
@@ -6410,7 +6412,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="9" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B85" s="10">
         <v>46094.573880254626</v>
@@ -6420,7 +6422,7 @@
         <v>46094.59033287037</v>
       </c>
       <c r="E85" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F85" s="11" t="s">
         <v>28</v>
@@ -6441,7 +6443,7 @@
         <v>28</v>
       </c>
       <c r="N85" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="O85" s="11" t="s">
         <v>28</v>
@@ -6450,7 +6452,7 @@
         <v>28</v>
       </c>
       <c r="Q85" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R85" s="11"/>
       <c r="S85" s="11"/>
@@ -6459,7 +6461,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B86" s="5">
         <v>46093.55797761574</v>
@@ -6469,10 +6471,10 @@
         <v>46099.63241893519</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F86" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G86" s="6" t="s">
         <v>26</v>
@@ -6503,20 +6505,20 @@
         <v>28</v>
       </c>
       <c r="Q86" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="R86" s="6"/>
       <c r="S86" s="12" t="s">
         <v>43</v>
       </c>
       <c r="T86" s="17" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="U86" s="6"/>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="9" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B87" s="10">
         <v>46094.65047047454</v>
@@ -6526,10 +6528,10 @@
         <v>46111.83610230324</v>
       </c>
       <c r="E87" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F87" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G87" s="11" t="s">
         <v>28</v>
@@ -6547,7 +6549,7 @@
         <v>0</v>
       </c>
       <c r="N87" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O87" s="11" t="s">
         <v>28</v>
@@ -6596,7 +6598,7 @@
         <v>28</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O88" s="6" t="s">
         <v>28</v>
@@ -6645,7 +6647,7 @@
         <v>28</v>
       </c>
       <c r="N89" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O89" s="11" t="s">
         <v>28</v>
@@ -6694,7 +6696,7 @@
         <v>28</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="O90" s="6" t="s">
         <v>28</v>
@@ -6725,7 +6727,7 @@
         <v>307</v>
       </c>
       <c r="F91" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G91" s="11" t="s">
         <v>56</v>
@@ -6831,7 +6833,7 @@
         <v>313</v>
       </c>
       <c r="F93" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G93" s="11" t="s">
         <v>26</v>
@@ -6869,7 +6871,7 @@
         <v>43</v>
       </c>
       <c r="T93" s="17" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="U93" s="11"/>
     </row>
@@ -6937,7 +6939,7 @@
         <v>319</v>
       </c>
       <c r="F95" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G95" s="11" t="s">
         <v>56</v>
@@ -7035,13 +7037,13 @@
       </c>
       <c r="C97" s="11"/>
       <c r="D97" s="10">
-        <v>46185.62184413194</v>
+        <v>46195.5664856713</v>
       </c>
       <c r="E97" s="11" t="s">
         <v>325</v>
       </c>
       <c r="F97" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G97" s="11" t="s">
         <v>56</v>
@@ -7249,7 +7251,7 @@
         <v>337</v>
       </c>
       <c r="F101" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G101" s="11" t="s">
         <v>56</v>
@@ -7404,7 +7406,7 @@
         <v>346</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G104" s="6" t="s">
         <v>56</v>
@@ -7610,7 +7612,7 @@
         <v>358</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G108" s="6" t="s">
         <v>56</v>
@@ -7669,7 +7671,7 @@
         <v>361</v>
       </c>
       <c r="F109" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G109" s="11" t="s">
         <v>28</v>
@@ -7724,7 +7726,7 @@
         <v>364</v>
       </c>
       <c r="F110" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G110" s="6" t="s">
         <v>28</v>
@@ -7779,7 +7781,7 @@
         <v>367</v>
       </c>
       <c r="F111" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G111" s="11" t="s">
         <v>28</v>
@@ -7834,7 +7836,7 @@
         <v>370</v>
       </c>
       <c r="F112" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G112" s="6" t="s">
         <v>28</v>
@@ -7885,7 +7887,7 @@
         <v>371</v>
       </c>
       <c r="F113" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G113" s="11" t="s">
         <v>26</v>
@@ -7944,7 +7946,7 @@
         <v>376</v>
       </c>
       <c r="F114" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G114" s="6" t="s">
         <v>28</v>
@@ -7995,7 +7997,7 @@
         <v>377</v>
       </c>
       <c r="F115" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G115" s="11" t="s">
         <v>26</v>
@@ -8054,7 +8056,7 @@
         <v>382</v>
       </c>
       <c r="F116" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G116" s="6" t="s">
         <v>28</v>
@@ -8105,7 +8107,7 @@
         <v>385</v>
       </c>
       <c r="F117" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G117" s="11" t="s">
         <v>28</v>
@@ -8160,7 +8162,7 @@
         <v>386</v>
       </c>
       <c r="F118" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G118" s="6" t="s">
         <v>26</v>
@@ -8219,7 +8221,7 @@
         <v>391</v>
       </c>
       <c r="F119" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G119" s="11" t="s">
         <v>56</v>
@@ -8272,7 +8274,7 @@
         <v>395</v>
       </c>
       <c r="F120" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G120" s="6" t="s">
         <v>56</v>
@@ -8325,7 +8327,7 @@
         <v>392</v>
       </c>
       <c r="F121" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G121" s="11" t="s">
         <v>56</v>
@@ -8384,7 +8386,7 @@
         <v>400</v>
       </c>
       <c r="F122" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G122" s="6" t="s">
         <v>56</v>
@@ -8437,7 +8439,7 @@
         <v>403</v>
       </c>
       <c r="F123" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G123" s="11" t="s">
         <v>56</v>
@@ -8490,7 +8492,7 @@
         <v>406</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G124" s="6" t="s">
         <v>56</v>
@@ -8543,7 +8545,7 @@
         <v>409</v>
       </c>
       <c r="F125" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G125" s="11" t="s">
         <v>56</v>
@@ -8596,7 +8598,7 @@
         <v>412</v>
       </c>
       <c r="F126" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G126" s="6" t="s">
         <v>56</v>
@@ -8649,7 +8651,7 @@
         <v>415</v>
       </c>
       <c r="F127" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G127" s="11" t="s">
         <v>56</v>
@@ -8702,7 +8704,7 @@
         <v>418</v>
       </c>
       <c r="F128" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G128" s="6" t="s">
         <v>56</v>
@@ -8755,7 +8757,7 @@
         <v>421</v>
       </c>
       <c r="F129" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G129" s="11" t="s">
         <v>56</v>
@@ -8808,7 +8810,7 @@
         <v>424</v>
       </c>
       <c r="F130" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G130" s="6" t="s">
         <v>56</v>
@@ -8916,7 +8918,7 @@
         <v>432</v>
       </c>
       <c r="F132" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G132" s="6" t="s">
         <v>56</v>
@@ -9367,7 +9369,7 @@
         <v>459</v>
       </c>
       <c r="F141" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G141" s="11" t="s">
         <v>56</v>
@@ -9420,7 +9422,7 @@
         <v>462</v>
       </c>
       <c r="F142" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G142" s="6" t="s">
         <v>56</v>
@@ -9473,7 +9475,7 @@
         <v>465</v>
       </c>
       <c r="F143" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G143" s="11" t="s">
         <v>56</v>
@@ -9534,7 +9536,7 @@
         <v>468</v>
       </c>
       <c r="F144" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G144" s="6" t="s">
         <v>28</v>
@@ -9585,7 +9587,7 @@
         <v>471</v>
       </c>
       <c r="F145" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G145" s="11" t="s">
         <v>28</v>
@@ -9636,7 +9638,7 @@
         <v>474</v>
       </c>
       <c r="F146" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G146" s="6" t="s">
         <v>28</v>
@@ -9687,7 +9689,7 @@
         <v>477</v>
       </c>
       <c r="F147" s="11" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G147" s="11" t="s">
         <v>40</v>
@@ -9746,7 +9748,7 @@
         <v>480</v>
       </c>
       <c r="F148" s="6" t="s">
-        <v>295</v>
+        <v>152</v>
       </c>
       <c r="G148" s="6" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-26 13:13 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -2144,11 +2144,11 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46164.530937407406</v>
+        <v>46164.69760407407</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="5">
-        <v>46196.002313715275</v>
+        <v>46196.168980381946</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -2203,11 +2203,11 @@
         <v>32</v>
       </c>
       <c r="B5" s="10">
-        <v>46164.53118508102</v>
+        <v>46164.69785174768</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="10">
-        <v>46164.531429236114</v>
+        <v>46164.69809590278</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>33</v>
@@ -2252,11 +2252,11 @@
         <v>35</v>
       </c>
       <c r="B6" s="5">
-        <v>46164.53126233796</v>
+        <v>46164.69792900463</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="5">
-        <v>46164.53159351852</v>
+        <v>46164.698260185185</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>36</v>
@@ -2301,11 +2301,11 @@
         <v>38</v>
       </c>
       <c r="B7" s="10">
-        <v>46155.63600853009</v>
+        <v>46155.802675196755</v>
       </c>
       <c r="C7" s="11"/>
       <c r="D7" s="10">
-        <v>46155.63846498843</v>
+        <v>46155.80513165509</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>39</v>
@@ -2358,11 +2358,11 @@
         <v>45</v>
       </c>
       <c r="B8" s="5">
-        <v>46155.63648939815</v>
+        <v>46155.803156064816</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="5">
-        <v>46155.63809114583</v>
+        <v>46155.8047578125</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>46</v>
@@ -2411,11 +2411,11 @@
         <v>48</v>
       </c>
       <c r="B9" s="10">
-        <v>46188.464606747686</v>
+        <v>46188.63127341435</v>
       </c>
       <c r="C9" s="11"/>
       <c r="D9" s="10">
-        <v>46188.46520918982</v>
+        <v>46188.63187585648</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>49</v>
@@ -2466,11 +2466,11 @@
         <v>52</v>
       </c>
       <c r="B10" s="5">
-        <v>46188.46489559028</v>
+        <v>46188.631562256945</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46188.46504497685</v>
+        <v>46188.631711643524</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>53</v>
@@ -2515,11 +2515,11 @@
         <v>55</v>
       </c>
       <c r="B11" s="10">
-        <v>46093.39130898148</v>
+        <v>46093.557975648146</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="10">
-        <v>46196.40792715277</v>
+        <v>46196.574593819445</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>56</v>
@@ -2568,11 +2568,11 @@
         <v>60</v>
       </c>
       <c r="B12" s="5">
-        <v>46094.46779931713</v>
+        <v>46094.63446598379</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46094.46797046297</v>
+        <v>46094.63463712963</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>61</v>
@@ -2617,11 +2617,11 @@
         <v>63</v>
       </c>
       <c r="B13" s="10">
-        <v>46188.46551144676</v>
+        <v>46188.632178113425</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="10">
-        <v>46188.46600372685</v>
+        <v>46188.63267039352</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>64</v>
@@ -2672,11 +2672,11 @@
         <v>66</v>
       </c>
       <c r="B14" s="5">
-        <v>46188.46571405092</v>
+        <v>46188.632380717594</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46188.46590284722</v>
+        <v>46188.63256951389</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>67</v>
@@ -2721,11 +2721,11 @@
         <v>69</v>
       </c>
       <c r="B15" s="10">
-        <v>46093.39131063657</v>
+        <v>46093.55797730324</v>
       </c>
       <c r="C15" s="11"/>
       <c r="D15" s="10">
-        <v>46134.49523165509</v>
+        <v>46134.66189832176</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>70</v>
@@ -2778,11 +2778,11 @@
         <v>73</v>
       </c>
       <c r="B16" s="5">
-        <v>46094.480701736116</v>
+        <v>46094.64736840277</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="5">
-        <v>46094.482618090275</v>
+        <v>46094.649284756946</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>74</v>
@@ -2829,11 +2829,11 @@
         <v>76</v>
       </c>
       <c r="B17" s="10">
-        <v>46094.480831469904</v>
+        <v>46094.647498136575</v>
       </c>
       <c r="C17" s="11"/>
       <c r="D17" s="10">
-        <v>46094.48267085648</v>
+        <v>46094.64933752315</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>77</v>
@@ -2880,11 +2880,11 @@
         <v>79</v>
       </c>
       <c r="B18" s="5">
-        <v>46094.48094486111</v>
+        <v>46094.64761152778</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46094.48273704862</v>
+        <v>46094.64940371527</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>80</v>
@@ -2931,11 +2931,11 @@
         <v>82</v>
       </c>
       <c r="B19" s="10">
-        <v>46094.48106497685</v>
+        <v>46094.64773164352</v>
       </c>
       <c r="C19" s="11"/>
       <c r="D19" s="10">
-        <v>46094.48279043981</v>
+        <v>46094.64945710648</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>83</v>
@@ -2982,11 +2982,11 @@
         <v>85</v>
       </c>
       <c r="B20" s="5">
-        <v>46094.481176643516</v>
+        <v>46094.64784331019</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="5">
-        <v>46094.48295435186</v>
+        <v>46094.649621018514</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>86</v>
@@ -3033,11 +3033,11 @@
         <v>88</v>
       </c>
       <c r="B21" s="10">
-        <v>46093.39131086806</v>
+        <v>46093.55797753472</v>
       </c>
       <c r="C21" s="11"/>
       <c r="D21" s="10">
-        <v>46134.495340671296</v>
+        <v>46134.66200733796</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>89</v>
@@ -3090,11 +3090,11 @@
         <v>91</v>
       </c>
       <c r="B22" s="5">
-        <v>46094.47638525463</v>
+        <v>46094.643051921295</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46094.47650232639</v>
+        <v>46094.643168993054</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>92</v>
@@ -3139,11 +3139,11 @@
         <v>94</v>
       </c>
       <c r="B23" s="10">
-        <v>46133.64463065972</v>
+        <v>46133.81129732639</v>
       </c>
       <c r="C23" s="11"/>
       <c r="D23" s="10">
-        <v>46139.00650162037</v>
+        <v>46139.17316828704</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>95</v>
@@ -3196,11 +3196,11 @@
         <v>97</v>
       </c>
       <c r="B24" s="5">
-        <v>46133.645201956024</v>
+        <v>46133.81186862268</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="5">
-        <v>46133.64537636574</v>
+        <v>46133.812043032405</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>98</v>
@@ -3245,11 +3245,11 @@
         <v>100</v>
       </c>
       <c r="B25" s="10">
-        <v>46148.99289465278</v>
+        <v>46149.159561319444</v>
       </c>
       <c r="C25" s="11"/>
       <c r="D25" s="10">
-        <v>46170.0010299537</v>
+        <v>46170.16769662037</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>101</v>
@@ -3302,11 +3302,11 @@
         <v>103</v>
       </c>
       <c r="B26" s="5">
-        <v>46148.99377987269</v>
+        <v>46149.16044653935</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="5">
-        <v>46148.99748721065</v>
+        <v>46149.16415387731</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>104</v>
@@ -3351,11 +3351,11 @@
         <v>106</v>
       </c>
       <c r="B27" s="10">
-        <v>46148.99753195602</v>
+        <v>46149.16419862269</v>
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="10">
-        <v>46148.99788972222</v>
+        <v>46149.16455638889</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>107</v>
@@ -3400,11 +3400,11 @@
         <v>109</v>
       </c>
       <c r="B28" s="5">
-        <v>46148.99789677083</v>
+        <v>46149.1645634375</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46148.99824690972</v>
+        <v>46149.16491357639</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>110</v>
@@ -3449,11 +3449,11 @@
         <v>112</v>
       </c>
       <c r="B29" s="10">
-        <v>46155.63856789352</v>
+        <v>46155.80523456019</v>
       </c>
       <c r="C29" s="11"/>
       <c r="D29" s="10">
-        <v>46163.02779288194</v>
+        <v>46163.19445954861</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>113</v>
@@ -3506,11 +3506,11 @@
         <v>115</v>
       </c>
       <c r="B30" s="5">
-        <v>46155.63897260417</v>
+        <v>46155.80563927084</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46163.02779289352</v>
+        <v>46163.19445956018</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>116</v>
@@ -3561,11 +3561,11 @@
         <v>118</v>
       </c>
       <c r="B31" s="10">
-        <v>46155.63913358796</v>
+        <v>46155.80580025463</v>
       </c>
       <c r="C31" s="11"/>
       <c r="D31" s="10">
-        <v>46163.02779299769</v>
+        <v>46163.19445966435</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>119</v>
@@ -3616,11 +3616,11 @@
         <v>121</v>
       </c>
       <c r="B32" s="5">
-        <v>46155.63985895833</v>
+        <v>46155.806525625</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="5">
-        <v>46163.027794525464</v>
+        <v>46163.19446119213</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>122</v>
@@ -3673,11 +3673,11 @@
         <v>125</v>
       </c>
       <c r="B33" s="10">
-        <v>46155.64006034722</v>
+        <v>46155.806727013885</v>
       </c>
       <c r="C33" s="11"/>
       <c r="D33" s="10">
-        <v>46163.02779371528</v>
+        <v>46163.19446038194</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>126</v>
@@ -3728,11 +3728,11 @@
         <v>128</v>
       </c>
       <c r="B34" s="5">
-        <v>46155.64067324074</v>
+        <v>46155.807339907406</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="5">
-        <v>46197.627945520835</v>
+        <v>46197.7946121875</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>129</v>
@@ -3785,11 +3785,11 @@
         <v>131</v>
       </c>
       <c r="B35" s="10">
-        <v>46155.64121944444</v>
+        <v>46155.80788611111</v>
       </c>
       <c r="C35" s="11"/>
       <c r="D35" s="10">
-        <v>46170.001030451385</v>
+        <v>46170.16769711806</v>
       </c>
       <c r="E35" s="11" t="s">
         <v>132</v>
@@ -3840,11 +3840,11 @@
         <v>134</v>
       </c>
       <c r="B36" s="5">
-        <v>46156.62160987269</v>
+        <v>46156.78827653935</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46169.00965846065</v>
+        <v>46169.176325127315</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>135</v>
@@ -3897,11 +3897,11 @@
         <v>138</v>
       </c>
       <c r="B37" s="10">
-        <v>46156.622255243055</v>
+        <v>46156.78892190973</v>
       </c>
       <c r="C37" s="11"/>
       <c r="D37" s="10">
-        <v>46169.00965871528</v>
+        <v>46169.176325381944</v>
       </c>
       <c r="E37" s="11" t="s">
         <v>139</v>
@@ -3952,11 +3952,11 @@
         <v>141</v>
       </c>
       <c r="B38" s="5">
-        <v>46156.6225257176</v>
+        <v>46156.789192384254</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46169.00965869213</v>
+        <v>46169.1763253588</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>142</v>
@@ -4007,11 +4007,11 @@
         <v>144</v>
       </c>
       <c r="B39" s="10">
-        <v>46188.46295746528</v>
+        <v>46188.62962413194</v>
       </c>
       <c r="C39" s="11"/>
       <c r="D39" s="10">
-        <v>46196.4505393287</v>
+        <v>46196.61720599537</v>
       </c>
       <c r="E39" s="11" t="s">
         <v>145</v>
@@ -4062,11 +4062,11 @@
         <v>147</v>
       </c>
       <c r="B40" s="5">
-        <v>46188.463355879634</v>
+        <v>46188.63002254629</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46196.03406662037</v>
+        <v>46196.20073328704</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>148</v>
@@ -4117,13 +4117,13 @@
         <v>150</v>
       </c>
       <c r="B41" s="10">
-        <v>46188.46360969907</v>
+        <v>46188.630276365744</v>
       </c>
       <c r="C41" s="10">
-        <v>46195.437958090275</v>
+        <v>46195.60462475695</v>
       </c>
       <c r="D41" s="10">
-        <v>46195.43797585648</v>
+        <v>46195.60464252315</v>
       </c>
       <c r="E41" s="11" t="s">
         <v>151</v>
@@ -4170,11 +4170,11 @@
         <v>154</v>
       </c>
       <c r="B42" s="5">
-        <v>46133.63068210648</v>
+        <v>46133.79734877315</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46141.57465121528</v>
+        <v>46141.74131788194</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>155</v>
@@ -4227,11 +4227,11 @@
         <v>158</v>
       </c>
       <c r="B43" s="10">
-        <v>46133.63180929398</v>
+        <v>46133.79847596065</v>
       </c>
       <c r="C43" s="11"/>
       <c r="D43" s="10">
-        <v>46134.49308862269</v>
+        <v>46134.65975528935</v>
       </c>
       <c r="E43" s="11" t="s">
         <v>159</v>
@@ -4276,11 +4276,11 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46133.63333427084</v>
+        <v>46133.800000937495</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46141.575875821756</v>
+        <v>46141.74254248843</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4333,11 +4333,11 @@
         <v>164</v>
       </c>
       <c r="B45" s="10">
-        <v>46133.633699375</v>
+        <v>46133.800366041665</v>
       </c>
       <c r="C45" s="11"/>
       <c r="D45" s="10">
-        <v>46133.6339280324</v>
+        <v>46133.800594699074</v>
       </c>
       <c r="E45" s="11" t="s">
         <v>165</v>
@@ -4382,11 +4382,11 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46093.391310046296</v>
+        <v>46093.55797671297</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46195.41091278935</v>
+        <v>46195.57757945602</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4441,11 +4441,11 @@
         <v>171</v>
       </c>
       <c r="B47" s="10">
-        <v>46094.4733012037</v>
+        <v>46094.639967870375</v>
       </c>
       <c r="C47" s="11"/>
       <c r="D47" s="10">
-        <v>46130.01896435185</v>
+        <v>46130.18563101852</v>
       </c>
       <c r="E47" s="11" t="s">
         <v>172</v>
@@ -4494,11 +4494,11 @@
         <v>174</v>
       </c>
       <c r="B48" s="5">
-        <v>46094.47355861111</v>
+        <v>46094.64022527778</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46100.98427231482</v>
+        <v>46101.15093898148</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>175</v>
@@ -4547,11 +4547,11 @@
         <v>177</v>
       </c>
       <c r="B49" s="10">
-        <v>46133.64380305556</v>
+        <v>46133.81046972222</v>
       </c>
       <c r="C49" s="11"/>
       <c r="D49" s="10">
-        <v>46162.62392778935</v>
+        <v>46162.79059445602</v>
       </c>
       <c r="E49" s="11" t="s">
         <v>178</v>
@@ -4604,11 +4604,11 @@
         <v>180</v>
       </c>
       <c r="B50" s="5">
-        <v>46133.64404806713</v>
+        <v>46133.8107147338</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46133.64421252315</v>
+        <v>46133.81087918981</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>181</v>
@@ -4653,11 +4653,11 @@
         <v>183</v>
       </c>
       <c r="B51" s="10">
-        <v>46133.63803945602</v>
+        <v>46133.80470612268</v>
       </c>
       <c r="C51" s="11"/>
       <c r="D51" s="10">
-        <v>46196.74914542824</v>
+        <v>46196.91581209491</v>
       </c>
       <c r="E51" s="11" t="s">
         <v>184</v>
@@ -4710,11 +4710,11 @@
         <v>186</v>
       </c>
       <c r="B52" s="5">
-        <v>46133.638791053236</v>
+        <v>46133.80545771991</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46133.6389784375</v>
+        <v>46133.80564510416</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>187</v>
@@ -4759,11 +4759,11 @@
         <v>189</v>
       </c>
       <c r="B53" s="10">
-        <v>46133.63903846065</v>
+        <v>46133.80570512731</v>
       </c>
       <c r="C53" s="11"/>
       <c r="D53" s="10">
-        <v>46133.639167002315</v>
+        <v>46133.80583366899</v>
       </c>
       <c r="E53" s="11" t="s">
         <v>190</v>
@@ -4808,11 +4808,11 @@
         <v>192</v>
       </c>
       <c r="B54" s="5">
-        <v>46133.63921837963</v>
+        <v>46133.8058850463</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46133.63969568287</v>
+        <v>46133.80636234954</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>193</v>
@@ -4857,11 +4857,11 @@
         <v>195</v>
       </c>
       <c r="B55" s="10">
-        <v>46133.639982141205</v>
+        <v>46133.80664880787</v>
       </c>
       <c r="C55" s="11"/>
       <c r="D55" s="10">
-        <v>46133.640144687495</v>
+        <v>46133.80681135417</v>
       </c>
       <c r="E55" s="11" t="s">
         <v>196</v>
@@ -4906,11 +4906,11 @@
         <v>198</v>
       </c>
       <c r="B56" s="5">
-        <v>46133.64034733796</v>
+        <v>46133.80701400463</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46162.62390688657</v>
+        <v>46162.79057355324</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>199</v>
@@ -4961,11 +4961,11 @@
         <v>202</v>
       </c>
       <c r="B57" s="10">
-        <v>46133.640603506945</v>
+        <v>46133.80727017361</v>
       </c>
       <c r="C57" s="11"/>
       <c r="D57" s="10">
-        <v>46133.640702951394</v>
+        <v>46133.80736961805</v>
       </c>
       <c r="E57" s="11" t="s">
         <v>203</v>
@@ -5010,11 +5010,11 @@
         <v>205</v>
       </c>
       <c r="B58" s="5">
-        <v>46133.63234684028</v>
+        <v>46133.79901350694</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46162.62389585648</v>
+        <v>46162.79056252315</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>206</v>
@@ -5067,11 +5067,11 @@
         <v>208</v>
       </c>
       <c r="B59" s="10">
-        <v>46133.63294776621</v>
+        <v>46133.79961443287</v>
       </c>
       <c r="C59" s="11"/>
       <c r="D59" s="10">
-        <v>46133.633231851854</v>
+        <v>46133.79989851852</v>
       </c>
       <c r="E59" s="11" t="s">
         <v>209</v>
@@ -5116,11 +5116,11 @@
         <v>211</v>
       </c>
       <c r="B60" s="5">
-        <v>46093.39131114584</v>
+        <v>46093.557977812496</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46162.62388090278</v>
+        <v>46162.79054756944</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>212</v>
@@ -5173,11 +5173,11 @@
         <v>214</v>
       </c>
       <c r="B61" s="10">
-        <v>46094.47691907408</v>
+        <v>46094.64358574074</v>
       </c>
       <c r="C61" s="11"/>
       <c r="D61" s="10">
-        <v>46094.47711576389</v>
+        <v>46094.643782430554</v>
       </c>
       <c r="E61" s="11" t="s">
         <v>215</v>
@@ -5222,11 +5222,11 @@
         <v>217</v>
       </c>
       <c r="B62" s="5">
-        <v>46133.642242222224</v>
+        <v>46133.80890888889</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46162.62387016204</v>
+        <v>46162.7905368287</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>218</v>
@@ -5279,11 +5279,11 @@
         <v>221</v>
       </c>
       <c r="B63" s="10">
-        <v>46133.64277114584</v>
+        <v>46133.809437812495</v>
       </c>
       <c r="C63" s="11"/>
       <c r="D63" s="10">
-        <v>46133.64291790509</v>
+        <v>46133.80958457176</v>
       </c>
       <c r="E63" s="11" t="s">
         <v>222</v>
@@ -5328,11 +5328,11 @@
         <v>224</v>
       </c>
       <c r="B64" s="5">
-        <v>46093.39131</v>
+        <v>46093.55797666666</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46162.62385700231</v>
+        <v>46162.790523668984</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>225</v>
@@ -5385,11 +5385,11 @@
         <v>227</v>
       </c>
       <c r="B65" s="10">
-        <v>46094.47944964121</v>
+        <v>46094.64611630787</v>
       </c>
       <c r="C65" s="11"/>
       <c r="D65" s="10">
-        <v>46094.47965065972</v>
+        <v>46094.64631732639</v>
       </c>
       <c r="E65" s="11" t="s">
         <v>228</v>
@@ -5434,11 +5434,11 @@
         <v>230</v>
       </c>
       <c r="B66" s="5">
-        <v>46094.479657881944</v>
+        <v>46094.64632454861</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46094.47989121528</v>
+        <v>46094.64655788195</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>231</v>
@@ -5483,11 +5483,11 @@
         <v>233</v>
       </c>
       <c r="B67" s="10">
-        <v>46093.39130971065</v>
+        <v>46093.55797637731</v>
       </c>
       <c r="C67" s="11"/>
       <c r="D67" s="10">
-        <v>46162.62384001157</v>
+        <v>46162.79050667824</v>
       </c>
       <c r="E67" s="11" t="s">
         <v>234</v>
@@ -5540,11 +5540,11 @@
         <v>236</v>
       </c>
       <c r="B68" s="5">
-        <v>46094.47876795139</v>
+        <v>46094.645434618054</v>
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46094.47893625</v>
+        <v>46094.645602916666</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>237</v>
@@ -5589,11 +5589,11 @@
         <v>239</v>
       </c>
       <c r="B69" s="10">
-        <v>46093.39131155093</v>
+        <v>46093.55797821759</v>
       </c>
       <c r="C69" s="11"/>
       <c r="D69" s="10">
-        <v>46162.62382674769</v>
+        <v>46162.79049341435</v>
       </c>
       <c r="E69" s="11" t="s">
         <v>240</v>
@@ -5646,11 +5646,11 @@
         <v>242</v>
       </c>
       <c r="B70" s="5">
-        <v>46094.48473460648</v>
+        <v>46094.65140127315</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46094.48484160879</v>
+        <v>46094.65150827546</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>243</v>
@@ -5695,11 +5695,11 @@
         <v>245</v>
       </c>
       <c r="B71" s="10">
-        <v>46093.39130952547</v>
+        <v>46093.557976192125</v>
       </c>
       <c r="C71" s="11"/>
       <c r="D71" s="10">
-        <v>46142.00269820602</v>
+        <v>46142.16936487269</v>
       </c>
       <c r="E71" s="11" t="s">
         <v>246</v>
@@ -5752,11 +5752,11 @@
         <v>249</v>
       </c>
       <c r="B72" s="5">
-        <v>46094.46874034722</v>
+        <v>46094.63540701389</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46094.468969849535</v>
+        <v>46094.63563651621</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>250</v>
@@ -5801,11 +5801,11 @@
         <v>252</v>
       </c>
       <c r="B73" s="10">
-        <v>46093.39131126157</v>
+        <v>46093.55797792824</v>
       </c>
       <c r="C73" s="11"/>
       <c r="D73" s="10">
-        <v>46134.52288275463</v>
+        <v>46134.689549421295</v>
       </c>
       <c r="E73" s="11" t="s">
         <v>253</v>
@@ -5858,11 +5858,11 @@
         <v>255</v>
       </c>
       <c r="B74" s="5">
-        <v>46094.483214733795</v>
+        <v>46094.64988140046</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46094.48332144676</v>
+        <v>46094.64998811342</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>256</v>
@@ -5907,11 +5907,11 @@
         <v>258</v>
       </c>
       <c r="B75" s="10">
-        <v>46093.39130847222</v>
+        <v>46093.55797513889</v>
       </c>
       <c r="C75" s="11"/>
       <c r="D75" s="10">
-        <v>46098.45922471065</v>
+        <v>46098.62589137732</v>
       </c>
       <c r="E75" s="11" t="s">
         <v>259</v>
@@ -5966,11 +5966,11 @@
         <v>261</v>
       </c>
       <c r="B76" s="5">
-        <v>46094.39993493055</v>
+        <v>46094.566601597224</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46094.40069871528</v>
+        <v>46094.56736538194</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>262</v>
@@ -6015,11 +6015,11 @@
         <v>264</v>
       </c>
       <c r="B77" s="10">
-        <v>46094.40027128472</v>
+        <v>46094.566937951386</v>
       </c>
       <c r="C77" s="11"/>
       <c r="D77" s="10">
-        <v>46094.40106740741</v>
+        <v>46094.56773407407</v>
       </c>
       <c r="E77" s="11" t="s">
         <v>265</v>
@@ -6064,11 +6064,11 @@
         <v>267</v>
       </c>
       <c r="B78" s="5">
-        <v>46094.40081503472</v>
+        <v>46094.56748170139</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46094.40129219907</v>
+        <v>46094.56795886574</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>268</v>
@@ -6113,11 +6113,11 @@
         <v>270</v>
       </c>
       <c r="B79" s="10">
-        <v>46094.401300011574</v>
+        <v>46094.56796667824</v>
       </c>
       <c r="C79" s="11"/>
       <c r="D79" s="10">
-        <v>46094.40153740741</v>
+        <v>46094.56820407408</v>
       </c>
       <c r="E79" s="11" t="s">
         <v>271</v>
@@ -6162,11 +6162,11 @@
         <v>273</v>
       </c>
       <c r="B80" s="5">
-        <v>46093.39130895834</v>
+        <v>46093.557975625</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46112.67511438657</v>
+        <v>46112.84178105324</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>274</v>
@@ -6221,11 +6221,11 @@
         <v>276</v>
       </c>
       <c r="B81" s="10">
-        <v>46094.40398135417</v>
+        <v>46094.57064802083</v>
       </c>
       <c r="C81" s="11"/>
       <c r="D81" s="10">
-        <v>46094.42353918981</v>
+        <v>46094.59020585648</v>
       </c>
       <c r="E81" s="11" t="s">
         <v>277</v>
@@ -6270,11 +6270,11 @@
         <v>279</v>
       </c>
       <c r="B82" s="5">
-        <v>46094.40676761574</v>
+        <v>46094.57343428241</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46094.42356728009</v>
+        <v>46094.59023394676</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>280</v>
@@ -6319,11 +6319,11 @@
         <v>282</v>
       </c>
       <c r="B83" s="10">
-        <v>46094.40692804398</v>
+        <v>46094.573594710644</v>
       </c>
       <c r="C83" s="11"/>
       <c r="D83" s="10">
-        <v>46094.42359532407</v>
+        <v>46094.59026199074</v>
       </c>
       <c r="E83" s="11" t="s">
         <v>283</v>
@@ -6368,11 +6368,11 @@
         <v>285</v>
       </c>
       <c r="B84" s="5">
-        <v>46094.40707314815</v>
+        <v>46094.57373981482</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46094.42363572917</v>
+        <v>46094.59030239584</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>286</v>
@@ -6417,11 +6417,11 @@
         <v>288</v>
       </c>
       <c r="B85" s="10">
-        <v>46094.40721358796</v>
+        <v>46094.573880254626</v>
       </c>
       <c r="C85" s="11"/>
       <c r="D85" s="10">
-        <v>46094.4236662037</v>
+        <v>46094.59033287037</v>
       </c>
       <c r="E85" s="11" t="s">
         <v>289</v>
@@ -6466,11 +6466,11 @@
         <v>291</v>
       </c>
       <c r="B86" s="5">
-        <v>46093.391310949075</v>
+        <v>46093.55797761574</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46099.465752268516</v>
+        <v>46099.63241893519</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>292</v>
@@ -6523,11 +6523,11 @@
         <v>294</v>
       </c>
       <c r="B87" s="10">
-        <v>46094.483803807874</v>
+        <v>46094.65047047454</v>
       </c>
       <c r="C87" s="11"/>
       <c r="D87" s="10">
-        <v>46111.66943563658</v>
+        <v>46111.83610230324</v>
       </c>
       <c r="E87" s="11" t="s">
         <v>295</v>
@@ -6572,11 +6572,11 @@
         <v>297</v>
       </c>
       <c r="B88" s="5">
-        <v>46094.48406188657</v>
+        <v>46094.65072855324</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46094.48416918982</v>
+        <v>46094.65083585648</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>298</v>
@@ -6621,11 +6621,11 @@
         <v>300</v>
       </c>
       <c r="B89" s="10">
-        <v>46094.48417696759</v>
+        <v>46094.650843634256</v>
       </c>
       <c r="C89" s="11"/>
       <c r="D89" s="10">
-        <v>46094.484524722226</v>
+        <v>46094.65119138889</v>
       </c>
       <c r="E89" s="11" t="s">
         <v>301</v>
@@ -6670,11 +6670,11 @@
         <v>303</v>
       </c>
       <c r="B90" s="5">
-        <v>46094.484286990744</v>
+        <v>46094.65095365741</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46094.48455228009</v>
+        <v>46094.65121894676</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>304</v>
@@ -6719,11 +6719,11 @@
         <v>306</v>
       </c>
       <c r="B91" s="10">
-        <v>46093.39131060185</v>
+        <v>46093.557977268516</v>
       </c>
       <c r="C91" s="11"/>
       <c r="D91" s="10">
-        <v>46099.47254487268</v>
+        <v>46099.639211539354</v>
       </c>
       <c r="E91" s="11" t="s">
         <v>307</v>
@@ -6776,11 +6776,11 @@
         <v>309</v>
       </c>
       <c r="B92" s="5">
-        <v>46094.475925590275</v>
+        <v>46094.64259225695</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46094.476118402774</v>
+        <v>46094.642785069445</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>310</v>
@@ -6825,11 +6825,11 @@
         <v>312</v>
       </c>
       <c r="B93" s="10">
-        <v>46093.39131184028</v>
+        <v>46093.55797850694</v>
       </c>
       <c r="C93" s="11"/>
       <c r="D93" s="10">
-        <v>46099.45819986111</v>
+        <v>46099.62486652778</v>
       </c>
       <c r="E93" s="11" t="s">
         <v>313</v>
@@ -6882,11 +6882,11 @@
         <v>315</v>
       </c>
       <c r="B94" s="5">
-        <v>46094.485353125</v>
+        <v>46094.65201979167</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46094.48547309027</v>
+        <v>46094.652139756945</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>316</v>
@@ -6931,11 +6931,11 @@
         <v>318</v>
       </c>
       <c r="B95" s="10">
-        <v>46093.39131032408</v>
+        <v>46093.55797699074</v>
       </c>
       <c r="C95" s="11"/>
       <c r="D95" s="10">
-        <v>46134.495801909725</v>
+        <v>46134.66246857639</v>
       </c>
       <c r="E95" s="11" t="s">
         <v>319</v>
@@ -6986,11 +6986,11 @@
         <v>321</v>
       </c>
       <c r="B96" s="5">
-        <v>46094.480051342594</v>
+        <v>46094.64671800926</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46094.48015737269</v>
+        <v>46094.64682403935</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>322</v>
@@ -7035,11 +7035,11 @@
         <v>324</v>
       </c>
       <c r="B97" s="10">
-        <v>46093.39131074074</v>
+        <v>46093.55797740741</v>
       </c>
       <c r="C97" s="11"/>
       <c r="D97" s="10">
-        <v>46196.40619525463</v>
+        <v>46196.5728619213</v>
       </c>
       <c r="E97" s="11" t="s">
         <v>325</v>
@@ -7094,11 +7094,11 @@
         <v>327</v>
       </c>
       <c r="B98" s="5">
-        <v>46094.41762021991</v>
+        <v>46094.58428688657</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46094.41827144676</v>
+        <v>46094.584938113425</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>328</v>
@@ -7143,11 +7143,11 @@
         <v>330</v>
       </c>
       <c r="B99" s="10">
-        <v>46094.41780956018</v>
+        <v>46094.58447622685</v>
       </c>
       <c r="C99" s="11"/>
       <c r="D99" s="10">
-        <v>46094.41829931713</v>
+        <v>46094.5849659838</v>
       </c>
       <c r="E99" s="11" t="s">
         <v>331</v>
@@ -7192,11 +7192,11 @@
         <v>333</v>
       </c>
       <c r="B100" s="5">
-        <v>46094.41804420139</v>
+        <v>46094.58471086806</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46094.41832512731</v>
+        <v>46094.58499179398</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>334</v>
@@ -7241,13 +7241,13 @@
         <v>336</v>
       </c>
       <c r="B101" s="10">
-        <v>46093.39130938657</v>
+        <v>46093.55797605324</v>
       </c>
       <c r="C101" s="10">
-        <v>46140.56400518518</v>
+        <v>46140.73067185185</v>
       </c>
       <c r="D101" s="10">
-        <v>46140.56400658565</v>
+        <v>46140.730673252314</v>
       </c>
       <c r="E101" s="11" t="s">
         <v>337</v>
@@ -7300,11 +7300,11 @@
         <v>339</v>
       </c>
       <c r="B102" s="5">
-        <v>46094.47807909722</v>
+        <v>46094.644745763886</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46094.47822538194</v>
+        <v>46094.644892048615</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>340</v>
@@ -7349,11 +7349,11 @@
         <v>342</v>
       </c>
       <c r="B103" s="10">
-        <v>46094.47823179398</v>
+        <v>46094.64489846065</v>
       </c>
       <c r="C103" s="11"/>
       <c r="D103" s="10">
-        <v>46094.47837561343</v>
+        <v>46094.64504228009</v>
       </c>
       <c r="E103" s="11" t="s">
         <v>343</v>
@@ -7398,11 +7398,11 @@
         <v>345</v>
       </c>
       <c r="B104" s="5">
-        <v>46133.635163240746</v>
+        <v>46133.8018299074</v>
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="5">
-        <v>46185.42787950231</v>
+        <v>46185.594546168984</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>346</v>
@@ -7455,11 +7455,11 @@
         <v>348</v>
       </c>
       <c r="B105" s="10">
-        <v>46133.635545428246</v>
+        <v>46133.8022120949</v>
       </c>
       <c r="C105" s="11"/>
       <c r="D105" s="10">
-        <v>46133.635998391204</v>
+        <v>46133.80266505787</v>
       </c>
       <c r="E105" s="11" t="s">
         <v>349</v>
@@ -7504,11 +7504,11 @@
         <v>351</v>
       </c>
       <c r="B106" s="5">
-        <v>46133.63569149305</v>
+        <v>46133.80235815972</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46133.636034270836</v>
+        <v>46133.8027009375</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>352</v>
@@ -7553,11 +7553,11 @@
         <v>354</v>
       </c>
       <c r="B107" s="10">
-        <v>46133.63582138889</v>
+        <v>46133.80248805556</v>
       </c>
       <c r="C107" s="11"/>
       <c r="D107" s="10">
-        <v>46133.63607395833</v>
+        <v>46133.802740625004</v>
       </c>
       <c r="E107" s="11" t="s">
         <v>355</v>
@@ -7602,13 +7602,13 @@
         <v>357</v>
       </c>
       <c r="B108" s="5">
-        <v>46093.39130979167</v>
+        <v>46093.55797645834</v>
       </c>
       <c r="C108" s="5">
-        <v>46162.68825068287</v>
+        <v>46162.85491734954</v>
       </c>
       <c r="D108" s="5">
-        <v>46162.688266620375</v>
+        <v>46162.85493328703</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>358</v>
@@ -7661,13 +7661,13 @@
         <v>360</v>
       </c>
       <c r="B109" s="10">
-        <v>46094.471592835645</v>
+        <v>46094.63825950232</v>
       </c>
       <c r="C109" s="10">
-        <v>46135.86566570602</v>
+        <v>46136.032332372684</v>
       </c>
       <c r="D109" s="10">
-        <v>46135.865686018515</v>
+        <v>46136.032352685186</v>
       </c>
       <c r="E109" s="11" t="s">
         <v>361</v>
@@ -7716,13 +7716,13 @@
         <v>363</v>
       </c>
       <c r="B110" s="5">
-        <v>46094.471750902776</v>
+        <v>46094.63841756944</v>
       </c>
       <c r="C110" s="5">
-        <v>46135.865679166665</v>
+        <v>46136.03234583333</v>
       </c>
       <c r="D110" s="5">
-        <v>46135.86569502315</v>
+        <v>46136.03236168981</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>364</v>
@@ -7771,13 +7771,13 @@
         <v>366</v>
       </c>
       <c r="B111" s="10">
-        <v>46094.471949687504</v>
+        <v>46094.63861635417</v>
       </c>
       <c r="C111" s="10">
-        <v>46135.865691921295</v>
+        <v>46136.03235858797</v>
       </c>
       <c r="D111" s="10">
-        <v>46135.86570789352</v>
+        <v>46136.032374560185</v>
       </c>
       <c r="E111" s="11" t="s">
         <v>367</v>
@@ -7826,13 +7826,13 @@
         <v>369</v>
       </c>
       <c r="B112" s="5">
-        <v>46133.64361054398</v>
+        <v>46133.81027721065</v>
       </c>
       <c r="C112" s="5">
-        <v>46161.746328078705</v>
+        <v>46161.91299474537</v>
       </c>
       <c r="D112" s="5">
-        <v>46161.74634914352</v>
+        <v>46161.91301581018</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>370</v>
@@ -7877,13 +7877,13 @@
         <v>373</v>
       </c>
       <c r="B113" s="10">
-        <v>46133.642986527775</v>
+        <v>46133.80965319445</v>
       </c>
       <c r="C113" s="10">
-        <v>46161.74627729166</v>
+        <v>46161.912943958334</v>
       </c>
       <c r="D113" s="10">
-        <v>46161.74629459491</v>
+        <v>46161.91296126157</v>
       </c>
       <c r="E113" s="11" t="s">
         <v>371</v>
@@ -7936,13 +7936,13 @@
         <v>375</v>
       </c>
       <c r="B114" s="5">
-        <v>46133.62895975694</v>
+        <v>46133.79562642361</v>
       </c>
       <c r="C114" s="5">
-        <v>46161.74608435185</v>
+        <v>46161.91275101852</v>
       </c>
       <c r="D114" s="5">
-        <v>46161.74610462963</v>
+        <v>46161.912771296295</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>376</v>
@@ -7987,13 +7987,13 @@
         <v>379</v>
       </c>
       <c r="B115" s="10">
-        <v>46133.628206203706</v>
+        <v>46133.79487287037</v>
       </c>
       <c r="C115" s="10">
-        <v>46161.746088252316</v>
+        <v>46161.91275491898</v>
       </c>
       <c r="D115" s="10">
-        <v>46161.74610438658</v>
+        <v>46161.91277105324</v>
       </c>
       <c r="E115" s="11" t="s">
         <v>377</v>
@@ -8046,13 +8046,13 @@
         <v>381</v>
       </c>
       <c r="B116" s="5">
-        <v>46133.629160324075</v>
+        <v>46133.79582699074</v>
       </c>
       <c r="C116" s="5">
-        <v>46161.746091180554</v>
+        <v>46161.912757847225</v>
       </c>
       <c r="D116" s="5">
-        <v>46161.74610591435</v>
+        <v>46161.91277258102</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>382</v>
@@ -8097,13 +8097,13 @@
         <v>384</v>
       </c>
       <c r="B117" s="10">
-        <v>46094.47474982639</v>
+        <v>46094.641416493054</v>
       </c>
       <c r="C117" s="10">
-        <v>46161.74575371528</v>
+        <v>46161.912420381945</v>
       </c>
       <c r="D117" s="10">
-        <v>46161.74577292824</v>
+        <v>46161.912439594904</v>
       </c>
       <c r="E117" s="11" t="s">
         <v>385</v>
@@ -8152,13 +8152,13 @@
         <v>388</v>
       </c>
       <c r="B118" s="5">
-        <v>46093.39131034722</v>
+        <v>46093.55797701389</v>
       </c>
       <c r="C118" s="5">
-        <v>46161.745760011574</v>
+        <v>46161.912426678246</v>
       </c>
       <c r="D118" s="5">
-        <v>46161.74577501157</v>
+        <v>46161.91244167824</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>386</v>
@@ -8211,13 +8211,13 @@
         <v>390</v>
       </c>
       <c r="B119" s="10">
-        <v>46094.41602628472</v>
+        <v>46094.582692951386</v>
       </c>
       <c r="C119" s="10">
-        <v>46134.50651302084</v>
+        <v>46134.673179687496</v>
       </c>
       <c r="D119" s="10">
-        <v>46134.50652981481</v>
+        <v>46134.67319648148</v>
       </c>
       <c r="E119" s="11" t="s">
         <v>391</v>
@@ -8264,13 +8264,13 @@
         <v>394</v>
       </c>
       <c r="B120" s="5">
-        <v>46093.39130895834</v>
+        <v>46093.557975625</v>
       </c>
       <c r="C120" s="5">
-        <v>46134.47554357639</v>
+        <v>46134.64221024305</v>
       </c>
       <c r="D120" s="5">
-        <v>46134.49599736111</v>
+        <v>46134.66266402778</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>395</v>
@@ -8317,13 +8317,13 @@
         <v>397</v>
       </c>
       <c r="B121" s="10">
-        <v>46093.39131046296</v>
+        <v>46093.55797712963</v>
       </c>
       <c r="C121" s="10">
-        <v>46134.473207511575</v>
+        <v>46134.63987417824</v>
       </c>
       <c r="D121" s="10">
-        <v>46134.47322237269</v>
+        <v>46134.63988903935</v>
       </c>
       <c r="E121" s="11" t="s">
         <v>392</v>
@@ -8376,13 +8376,13 @@
         <v>399</v>
       </c>
       <c r="B122" s="5">
-        <v>46094.41527780093</v>
+        <v>46094.58194446759</v>
       </c>
       <c r="C122" s="5">
-        <v>46134.47254018519</v>
+        <v>46134.63920685185</v>
       </c>
       <c r="D122" s="5">
-        <v>46134.49657511574</v>
+        <v>46134.66324178241</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>400</v>
@@ -8429,13 +8429,13 @@
         <v>402</v>
       </c>
       <c r="B123" s="10">
-        <v>46094.415486909726</v>
+        <v>46094.58215357639</v>
       </c>
       <c r="C123" s="10">
-        <v>46134.47256253472</v>
+        <v>46134.63922920139</v>
       </c>
       <c r="D123" s="10">
-        <v>46134.49639373843</v>
+        <v>46134.66306040509</v>
       </c>
       <c r="E123" s="11" t="s">
         <v>403</v>
@@ -8482,13 +8482,13 @@
         <v>405</v>
       </c>
       <c r="B124" s="5">
-        <v>46094.41564641204</v>
+        <v>46094.5823130787</v>
       </c>
       <c r="C124" s="5">
-        <v>46134.47256783565</v>
+        <v>46134.63923450232</v>
       </c>
       <c r="D124" s="5">
-        <v>46134.496473101855</v>
+        <v>46134.66313976852</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>406</v>
@@ -8535,13 +8535,13 @@
         <v>408</v>
       </c>
       <c r="B125" s="10">
-        <v>46094.41574372685</v>
+        <v>46094.582410393516</v>
       </c>
       <c r="C125" s="10">
-        <v>46134.47257288195</v>
+        <v>46134.63923954861</v>
       </c>
       <c r="D125" s="10">
-        <v>46134.49632251158</v>
+        <v>46134.662989178236</v>
       </c>
       <c r="E125" s="11" t="s">
         <v>409</v>
@@ -8588,13 +8588,13 @@
         <v>411</v>
       </c>
       <c r="B126" s="5">
-        <v>46094.41587055556</v>
+        <v>46094.58253722222</v>
       </c>
       <c r="C126" s="5">
-        <v>46134.47257902777</v>
+        <v>46134.639245694445</v>
       </c>
       <c r="D126" s="5">
-        <v>46134.4962590162</v>
+        <v>46134.662925682875</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>412</v>
@@ -8641,13 +8641,13 @@
         <v>414</v>
       </c>
       <c r="B127" s="10">
-        <v>46094.41613084491</v>
+        <v>46094.582797511575</v>
       </c>
       <c r="C127" s="10">
-        <v>46134.47258864583</v>
+        <v>46134.639255312504</v>
       </c>
       <c r="D127" s="10">
-        <v>46155.4116539699</v>
+        <v>46155.578320636574</v>
       </c>
       <c r="E127" s="11" t="s">
         <v>415</v>
@@ -8694,13 +8694,13 @@
         <v>417</v>
       </c>
       <c r="B128" s="5">
-        <v>46094.416218425926</v>
+        <v>46094.58288509259</v>
       </c>
       <c r="C128" s="5">
-        <v>46134.47259387732</v>
+        <v>46134.63926054398</v>
       </c>
       <c r="D128" s="5">
-        <v>46134.49612207176</v>
+        <v>46134.662788738424</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>418</v>
@@ -8747,13 +8747,13 @@
         <v>420</v>
       </c>
       <c r="B129" s="10">
-        <v>46094.41639663195</v>
+        <v>46094.58306329861</v>
       </c>
       <c r="C129" s="10">
-        <v>46134.47259942129</v>
+        <v>46134.639266087965</v>
       </c>
       <c r="D129" s="10">
-        <v>46134.49606914352</v>
+        <v>46134.66273581018</v>
       </c>
       <c r="E129" s="11" t="s">
         <v>421</v>
@@ -8800,13 +8800,13 @@
         <v>423</v>
       </c>
       <c r="B130" s="5">
-        <v>46133.62551017361</v>
+        <v>46133.792176840274</v>
       </c>
       <c r="C130" s="5">
-        <v>46134.46938997685</v>
+        <v>46134.63605664352</v>
       </c>
       <c r="D130" s="5">
-        <v>46134.469526307876</v>
+        <v>46134.63619297453</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>424</v>
@@ -8859,11 +8859,11 @@
         <v>428</v>
       </c>
       <c r="B131" s="10">
-        <v>46133.62596824074</v>
+        <v>46133.79263490741</v>
       </c>
       <c r="C131" s="11"/>
       <c r="D131" s="10">
-        <v>46133.62684295139</v>
+        <v>46133.79350961806</v>
       </c>
       <c r="E131" s="11" t="s">
         <v>429</v>
@@ -8908,13 +8908,13 @@
         <v>431</v>
       </c>
       <c r="B132" s="5">
-        <v>46091.42727399306</v>
+        <v>46091.59394065972</v>
       </c>
       <c r="C132" s="5">
-        <v>46133.53927418981</v>
+        <v>46133.70594085648</v>
       </c>
       <c r="D132" s="5">
-        <v>46133.53928864583</v>
+        <v>46133.7059553125</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>432</v>
@@ -8967,11 +8967,11 @@
         <v>434</v>
       </c>
       <c r="B133" s="10">
-        <v>46094.45867290509</v>
+        <v>46094.62533957176</v>
       </c>
       <c r="C133" s="11"/>
       <c r="D133" s="10">
-        <v>46133.53927112269</v>
+        <v>46133.70593778935</v>
       </c>
       <c r="E133" s="11" t="s">
         <v>435</v>
@@ -9016,11 +9016,11 @@
         <v>437</v>
       </c>
       <c r="B134" s="5">
-        <v>46094.45876127315</v>
+        <v>46094.62542793981</v>
       </c>
       <c r="C134" s="6"/>
       <c r="D134" s="5">
-        <v>46133.53927171296</v>
+        <v>46133.70593837963</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>438</v>
@@ -9065,11 +9065,11 @@
         <v>440</v>
       </c>
       <c r="B135" s="10">
-        <v>46094.45947127315</v>
+        <v>46094.62613793982</v>
       </c>
       <c r="C135" s="11"/>
       <c r="D135" s="10">
-        <v>46133.539272106485</v>
+        <v>46133.70593877315</v>
       </c>
       <c r="E135" s="11" t="s">
         <v>441</v>
@@ -9114,11 +9114,11 @@
         <v>443</v>
       </c>
       <c r="B136" s="5">
-        <v>46094.45974203704</v>
+        <v>46094.626408703705</v>
       </c>
       <c r="C136" s="6"/>
       <c r="D136" s="5">
-        <v>46133.53927252315</v>
+        <v>46133.705939189815</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>444</v>
@@ -9163,11 +9163,11 @@
         <v>446</v>
       </c>
       <c r="B137" s="10">
-        <v>46094.45982255787</v>
+        <v>46094.62648922454</v>
       </c>
       <c r="C137" s="11"/>
       <c r="D137" s="10">
-        <v>46133.539272951384</v>
+        <v>46133.705939618056</v>
       </c>
       <c r="E137" s="11" t="s">
         <v>447</v>
@@ -9212,11 +9212,11 @@
         <v>449</v>
       </c>
       <c r="B138" s="5">
-        <v>46094.45994241898</v>
+        <v>46094.62660908565</v>
       </c>
       <c r="C138" s="6"/>
       <c r="D138" s="5">
-        <v>46133.53927328704</v>
+        <v>46133.7059399537</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>450</v>
@@ -9261,11 +9261,11 @@
         <v>452</v>
       </c>
       <c r="B139" s="10">
-        <v>46094.46004679398</v>
+        <v>46094.626713460646</v>
       </c>
       <c r="C139" s="11"/>
       <c r="D139" s="10">
-        <v>46133.53927363426</v>
+        <v>46133.705940300926</v>
       </c>
       <c r="E139" s="11" t="s">
         <v>453</v>
@@ -9310,11 +9310,11 @@
         <v>455</v>
       </c>
       <c r="B140" s="5">
-        <v>46094.46014135417</v>
+        <v>46094.62680802083</v>
       </c>
       <c r="C140" s="6"/>
       <c r="D140" s="5">
-        <v>46133.539273981485</v>
+        <v>46133.70594064815</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>456</v>
@@ -9359,13 +9359,13 @@
         <v>458</v>
       </c>
       <c r="B141" s="10">
-        <v>46093.391309259256</v>
+        <v>46093.55797592593</v>
       </c>
       <c r="C141" s="10">
-        <v>46127.708363391204</v>
+        <v>46127.87503005787</v>
       </c>
       <c r="D141" s="10">
-        <v>46134.49664273148</v>
+        <v>46134.66330939815</v>
       </c>
       <c r="E141" s="11" t="s">
         <v>459</v>
@@ -9412,13 +9412,13 @@
         <v>461</v>
       </c>
       <c r="B142" s="5">
-        <v>46094.46808032408</v>
+        <v>46094.63474699074</v>
       </c>
       <c r="C142" s="5">
-        <v>46127.70834715277</v>
+        <v>46127.875013819445</v>
       </c>
       <c r="D142" s="5">
-        <v>46134.496786250005</v>
+        <v>46134.66345291666</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>462</v>
@@ -9465,13 +9465,13 @@
         <v>464</v>
       </c>
       <c r="B143" s="10">
-        <v>46093.39130944444</v>
+        <v>46093.557976111115</v>
       </c>
       <c r="C143" s="10">
-        <v>46111.66991109954</v>
+        <v>46111.836577766204</v>
       </c>
       <c r="D143" s="10">
-        <v>46111.66992547453</v>
+        <v>46111.836592141204</v>
       </c>
       <c r="E143" s="11" t="s">
         <v>465</v>
@@ -9526,13 +9526,13 @@
         <v>467</v>
       </c>
       <c r="B144" s="5">
-        <v>46094.40905268519</v>
+        <v>46094.57571935185</v>
       </c>
       <c r="C144" s="5">
-        <v>46111.66987857639</v>
+        <v>46111.83654524306</v>
       </c>
       <c r="D144" s="5">
-        <v>46111.66989445602</v>
+        <v>46111.83656112268</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>468</v>
@@ -9577,13 +9577,13 @@
         <v>470</v>
       </c>
       <c r="B145" s="10">
-        <v>46094.4093472338</v>
+        <v>46094.57601390046</v>
       </c>
       <c r="C145" s="10">
-        <v>46111.66989234954</v>
+        <v>46111.8365590162</v>
       </c>
       <c r="D145" s="10">
-        <v>46111.66991091435</v>
+        <v>46111.83657758102</v>
       </c>
       <c r="E145" s="11" t="s">
         <v>471</v>
@@ -9628,13 +9628,13 @@
         <v>473</v>
       </c>
       <c r="B146" s="5">
-        <v>46094.40953752315</v>
+        <v>46094.57620418981</v>
       </c>
       <c r="C146" s="5">
-        <v>46111.6699066088</v>
+        <v>46111.83657327546</v>
       </c>
       <c r="D146" s="5">
-        <v>46111.66992586806</v>
+        <v>46111.83659253472</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>474</v>
@@ -9679,13 +9679,13 @@
         <v>476</v>
       </c>
       <c r="B147" s="10">
-        <v>46093.39130920139</v>
+        <v>46093.557975868054</v>
       </c>
       <c r="C147" s="10">
-        <v>46097.61039002315</v>
+        <v>46097.77705668981</v>
       </c>
       <c r="D147" s="10">
-        <v>46097.61040666667</v>
+        <v>46097.77707333333</v>
       </c>
       <c r="E147" s="11" t="s">
         <v>477</v>
@@ -9738,13 +9738,13 @@
         <v>479</v>
       </c>
       <c r="B148" s="5">
-        <v>46094.40786840278</v>
+        <v>46094.57453506945</v>
       </c>
       <c r="C148" s="5">
-        <v>46097.61037094907</v>
+        <v>46097.77703761574</v>
       </c>
       <c r="D148" s="5">
-        <v>46097.61038972222</v>
+        <v>46097.77705638889</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>480</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-26 13:15 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -2144,11 +2144,11 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46164.69760407407</v>
+        <v>46164.530937407406</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="5">
-        <v>46196.168980381946</v>
+        <v>46196.002313715275</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -2203,11 +2203,11 @@
         <v>32</v>
       </c>
       <c r="B5" s="10">
-        <v>46164.69785174768</v>
+        <v>46164.53118508102</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="10">
-        <v>46164.69809590278</v>
+        <v>46164.531429236114</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>33</v>
@@ -2252,11 +2252,11 @@
         <v>35</v>
       </c>
       <c r="B6" s="5">
-        <v>46164.69792900463</v>
+        <v>46164.53126233796</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="5">
-        <v>46164.698260185185</v>
+        <v>46164.53159351852</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>36</v>
@@ -2301,11 +2301,11 @@
         <v>38</v>
       </c>
       <c r="B7" s="10">
-        <v>46155.802675196755</v>
+        <v>46155.63600853009</v>
       </c>
       <c r="C7" s="11"/>
       <c r="D7" s="10">
-        <v>46155.80513165509</v>
+        <v>46155.63846498843</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>39</v>
@@ -2358,11 +2358,11 @@
         <v>45</v>
       </c>
       <c r="B8" s="5">
-        <v>46155.803156064816</v>
+        <v>46155.63648939815</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="5">
-        <v>46155.8047578125</v>
+        <v>46155.63809114583</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>46</v>
@@ -2411,11 +2411,11 @@
         <v>48</v>
       </c>
       <c r="B9" s="10">
-        <v>46188.63127341435</v>
+        <v>46188.464606747686</v>
       </c>
       <c r="C9" s="11"/>
       <c r="D9" s="10">
-        <v>46188.63187585648</v>
+        <v>46188.46520918982</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>49</v>
@@ -2466,11 +2466,11 @@
         <v>52</v>
       </c>
       <c r="B10" s="5">
-        <v>46188.631562256945</v>
+        <v>46188.46489559028</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46188.631711643524</v>
+        <v>46188.46504497685</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>53</v>
@@ -2515,11 +2515,11 @@
         <v>55</v>
       </c>
       <c r="B11" s="10">
-        <v>46093.557975648146</v>
+        <v>46093.39130898148</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="10">
-        <v>46196.574593819445</v>
+        <v>46196.40792715277</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>56</v>
@@ -2568,11 +2568,11 @@
         <v>60</v>
       </c>
       <c r="B12" s="5">
-        <v>46094.63446598379</v>
+        <v>46094.46779931713</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46094.63463712963</v>
+        <v>46094.46797046297</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>61</v>
@@ -2617,11 +2617,11 @@
         <v>63</v>
       </c>
       <c r="B13" s="10">
-        <v>46188.632178113425</v>
+        <v>46188.46551144676</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="10">
-        <v>46188.63267039352</v>
+        <v>46188.46600372685</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>64</v>
@@ -2672,11 +2672,11 @@
         <v>66</v>
       </c>
       <c r="B14" s="5">
-        <v>46188.632380717594</v>
+        <v>46188.46571405092</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46188.63256951389</v>
+        <v>46188.46590284722</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>67</v>
@@ -2721,11 +2721,11 @@
         <v>69</v>
       </c>
       <c r="B15" s="10">
-        <v>46093.55797730324</v>
+        <v>46093.39131063657</v>
       </c>
       <c r="C15" s="11"/>
       <c r="D15" s="10">
-        <v>46134.66189832176</v>
+        <v>46134.49523165509</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>70</v>
@@ -2778,11 +2778,11 @@
         <v>73</v>
       </c>
       <c r="B16" s="5">
-        <v>46094.64736840277</v>
+        <v>46094.480701736116</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="5">
-        <v>46094.649284756946</v>
+        <v>46094.482618090275</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>74</v>
@@ -2829,11 +2829,11 @@
         <v>76</v>
       </c>
       <c r="B17" s="10">
-        <v>46094.647498136575</v>
+        <v>46094.480831469904</v>
       </c>
       <c r="C17" s="11"/>
       <c r="D17" s="10">
-        <v>46094.64933752315</v>
+        <v>46094.48267085648</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>77</v>
@@ -2880,11 +2880,11 @@
         <v>79</v>
       </c>
       <c r="B18" s="5">
-        <v>46094.64761152778</v>
+        <v>46094.48094486111</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46094.64940371527</v>
+        <v>46094.48273704862</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>80</v>
@@ -2931,11 +2931,11 @@
         <v>82</v>
       </c>
       <c r="B19" s="10">
-        <v>46094.64773164352</v>
+        <v>46094.48106497685</v>
       </c>
       <c r="C19" s="11"/>
       <c r="D19" s="10">
-        <v>46094.64945710648</v>
+        <v>46094.48279043981</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>83</v>
@@ -2982,11 +2982,11 @@
         <v>85</v>
       </c>
       <c r="B20" s="5">
-        <v>46094.64784331019</v>
+        <v>46094.481176643516</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="5">
-        <v>46094.649621018514</v>
+        <v>46094.48295435186</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>86</v>
@@ -3033,11 +3033,11 @@
         <v>88</v>
       </c>
       <c r="B21" s="10">
-        <v>46093.55797753472</v>
+        <v>46093.39131086806</v>
       </c>
       <c r="C21" s="11"/>
       <c r="D21" s="10">
-        <v>46134.66200733796</v>
+        <v>46134.495340671296</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>89</v>
@@ -3090,11 +3090,11 @@
         <v>91</v>
       </c>
       <c r="B22" s="5">
-        <v>46094.643051921295</v>
+        <v>46094.47638525463</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46094.643168993054</v>
+        <v>46094.47650232639</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>92</v>
@@ -3139,11 +3139,11 @@
         <v>94</v>
       </c>
       <c r="B23" s="10">
-        <v>46133.81129732639</v>
+        <v>46133.64463065972</v>
       </c>
       <c r="C23" s="11"/>
       <c r="D23" s="10">
-        <v>46139.17316828704</v>
+        <v>46139.00650162037</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>95</v>
@@ -3196,11 +3196,11 @@
         <v>97</v>
       </c>
       <c r="B24" s="5">
-        <v>46133.81186862268</v>
+        <v>46133.645201956024</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="5">
-        <v>46133.812043032405</v>
+        <v>46133.64537636574</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>98</v>
@@ -3245,11 +3245,11 @@
         <v>100</v>
       </c>
       <c r="B25" s="10">
-        <v>46149.159561319444</v>
+        <v>46148.99289465278</v>
       </c>
       <c r="C25" s="11"/>
       <c r="D25" s="10">
-        <v>46170.16769662037</v>
+        <v>46170.0010299537</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>101</v>
@@ -3302,11 +3302,11 @@
         <v>103</v>
       </c>
       <c r="B26" s="5">
-        <v>46149.16044653935</v>
+        <v>46148.99377987269</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="5">
-        <v>46149.16415387731</v>
+        <v>46148.99748721065</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>104</v>
@@ -3351,11 +3351,11 @@
         <v>106</v>
       </c>
       <c r="B27" s="10">
-        <v>46149.16419862269</v>
+        <v>46148.99753195602</v>
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="10">
-        <v>46149.16455638889</v>
+        <v>46148.99788972222</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>107</v>
@@ -3400,11 +3400,11 @@
         <v>109</v>
       </c>
       <c r="B28" s="5">
-        <v>46149.1645634375</v>
+        <v>46148.99789677083</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46149.16491357639</v>
+        <v>46148.99824690972</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>110</v>
@@ -3449,11 +3449,11 @@
         <v>112</v>
       </c>
       <c r="B29" s="10">
-        <v>46155.80523456019</v>
+        <v>46155.63856789352</v>
       </c>
       <c r="C29" s="11"/>
       <c r="D29" s="10">
-        <v>46163.19445954861</v>
+        <v>46163.02779288194</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>113</v>
@@ -3506,11 +3506,11 @@
         <v>115</v>
       </c>
       <c r="B30" s="5">
-        <v>46155.80563927084</v>
+        <v>46155.63897260417</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46163.19445956018</v>
+        <v>46163.02779289352</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>116</v>
@@ -3561,11 +3561,11 @@
         <v>118</v>
       </c>
       <c r="B31" s="10">
-        <v>46155.80580025463</v>
+        <v>46155.63913358796</v>
       </c>
       <c r="C31" s="11"/>
       <c r="D31" s="10">
-        <v>46163.19445966435</v>
+        <v>46163.02779299769</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>119</v>
@@ -3616,11 +3616,11 @@
         <v>121</v>
       </c>
       <c r="B32" s="5">
-        <v>46155.806525625</v>
+        <v>46155.63985895833</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="5">
-        <v>46163.19446119213</v>
+        <v>46163.027794525464</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>122</v>
@@ -3673,11 +3673,11 @@
         <v>125</v>
       </c>
       <c r="B33" s="10">
-        <v>46155.806727013885</v>
+        <v>46155.64006034722</v>
       </c>
       <c r="C33" s="11"/>
       <c r="D33" s="10">
-        <v>46163.19446038194</v>
+        <v>46163.02779371528</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>126</v>
@@ -3728,11 +3728,11 @@
         <v>128</v>
       </c>
       <c r="B34" s="5">
-        <v>46155.807339907406</v>
+        <v>46155.64067324074</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="5">
-        <v>46197.7946121875</v>
+        <v>46197.627945520835</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>129</v>
@@ -3785,11 +3785,11 @@
         <v>131</v>
       </c>
       <c r="B35" s="10">
-        <v>46155.80788611111</v>
+        <v>46155.64121944444</v>
       </c>
       <c r="C35" s="11"/>
       <c r="D35" s="10">
-        <v>46170.16769711806</v>
+        <v>46170.001030451385</v>
       </c>
       <c r="E35" s="11" t="s">
         <v>132</v>
@@ -3840,11 +3840,11 @@
         <v>134</v>
       </c>
       <c r="B36" s="5">
-        <v>46156.78827653935</v>
+        <v>46156.62160987269</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46169.176325127315</v>
+        <v>46169.00965846065</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>135</v>
@@ -3897,11 +3897,11 @@
         <v>138</v>
       </c>
       <c r="B37" s="10">
-        <v>46156.78892190973</v>
+        <v>46156.622255243055</v>
       </c>
       <c r="C37" s="11"/>
       <c r="D37" s="10">
-        <v>46169.176325381944</v>
+        <v>46169.00965871528</v>
       </c>
       <c r="E37" s="11" t="s">
         <v>139</v>
@@ -3952,11 +3952,11 @@
         <v>141</v>
       </c>
       <c r="B38" s="5">
-        <v>46156.789192384254</v>
+        <v>46156.6225257176</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46169.1763253588</v>
+        <v>46169.00965869213</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>142</v>
@@ -4007,11 +4007,11 @@
         <v>144</v>
       </c>
       <c r="B39" s="10">
-        <v>46188.62962413194</v>
+        <v>46188.46295746528</v>
       </c>
       <c r="C39" s="11"/>
       <c r="D39" s="10">
-        <v>46196.61720599537</v>
+        <v>46196.4505393287</v>
       </c>
       <c r="E39" s="11" t="s">
         <v>145</v>
@@ -4062,11 +4062,11 @@
         <v>147</v>
       </c>
       <c r="B40" s="5">
-        <v>46188.63002254629</v>
+        <v>46188.463355879634</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46196.20073328704</v>
+        <v>46196.03406662037</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>148</v>
@@ -4117,13 +4117,13 @@
         <v>150</v>
       </c>
       <c r="B41" s="10">
-        <v>46188.630276365744</v>
+        <v>46188.46360969907</v>
       </c>
       <c r="C41" s="10">
-        <v>46195.60462475695</v>
+        <v>46195.437958090275</v>
       </c>
       <c r="D41" s="10">
-        <v>46195.60464252315</v>
+        <v>46195.43797585648</v>
       </c>
       <c r="E41" s="11" t="s">
         <v>151</v>
@@ -4170,11 +4170,11 @@
         <v>154</v>
       </c>
       <c r="B42" s="5">
-        <v>46133.79734877315</v>
+        <v>46133.63068210648</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46141.74131788194</v>
+        <v>46141.57465121528</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>155</v>
@@ -4227,11 +4227,11 @@
         <v>158</v>
       </c>
       <c r="B43" s="10">
-        <v>46133.79847596065</v>
+        <v>46133.63180929398</v>
       </c>
       <c r="C43" s="11"/>
       <c r="D43" s="10">
-        <v>46134.65975528935</v>
+        <v>46134.49308862269</v>
       </c>
       <c r="E43" s="11" t="s">
         <v>159</v>
@@ -4276,11 +4276,11 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46133.800000937495</v>
+        <v>46133.63333427084</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46141.74254248843</v>
+        <v>46141.575875821756</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4333,11 +4333,11 @@
         <v>164</v>
       </c>
       <c r="B45" s="10">
-        <v>46133.800366041665</v>
+        <v>46133.633699375</v>
       </c>
       <c r="C45" s="11"/>
       <c r="D45" s="10">
-        <v>46133.800594699074</v>
+        <v>46133.6339280324</v>
       </c>
       <c r="E45" s="11" t="s">
         <v>165</v>
@@ -4382,11 +4382,11 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46093.55797671297</v>
+        <v>46093.391310046296</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46195.57757945602</v>
+        <v>46195.41091278935</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4441,11 +4441,11 @@
         <v>171</v>
       </c>
       <c r="B47" s="10">
-        <v>46094.639967870375</v>
+        <v>46094.4733012037</v>
       </c>
       <c r="C47" s="11"/>
       <c r="D47" s="10">
-        <v>46130.18563101852</v>
+        <v>46130.01896435185</v>
       </c>
       <c r="E47" s="11" t="s">
         <v>172</v>
@@ -4494,11 +4494,11 @@
         <v>174</v>
       </c>
       <c r="B48" s="5">
-        <v>46094.64022527778</v>
+        <v>46094.47355861111</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46101.15093898148</v>
+        <v>46100.98427231482</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>175</v>
@@ -4547,11 +4547,11 @@
         <v>177</v>
       </c>
       <c r="B49" s="10">
-        <v>46133.81046972222</v>
+        <v>46133.64380305556</v>
       </c>
       <c r="C49" s="11"/>
       <c r="D49" s="10">
-        <v>46162.79059445602</v>
+        <v>46162.62392778935</v>
       </c>
       <c r="E49" s="11" t="s">
         <v>178</v>
@@ -4604,11 +4604,11 @@
         <v>180</v>
       </c>
       <c r="B50" s="5">
-        <v>46133.8107147338</v>
+        <v>46133.64404806713</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46133.81087918981</v>
+        <v>46133.64421252315</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>181</v>
@@ -4653,11 +4653,11 @@
         <v>183</v>
       </c>
       <c r="B51" s="10">
-        <v>46133.80470612268</v>
+        <v>46133.63803945602</v>
       </c>
       <c r="C51" s="11"/>
       <c r="D51" s="10">
-        <v>46196.91581209491</v>
+        <v>46196.74914542824</v>
       </c>
       <c r="E51" s="11" t="s">
         <v>184</v>
@@ -4710,11 +4710,11 @@
         <v>186</v>
       </c>
       <c r="B52" s="5">
-        <v>46133.80545771991</v>
+        <v>46133.638791053236</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46133.80564510416</v>
+        <v>46133.6389784375</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>187</v>
@@ -4759,11 +4759,11 @@
         <v>189</v>
       </c>
       <c r="B53" s="10">
-        <v>46133.80570512731</v>
+        <v>46133.63903846065</v>
       </c>
       <c r="C53" s="11"/>
       <c r="D53" s="10">
-        <v>46133.80583366899</v>
+        <v>46133.639167002315</v>
       </c>
       <c r="E53" s="11" t="s">
         <v>190</v>
@@ -4808,11 +4808,11 @@
         <v>192</v>
       </c>
       <c r="B54" s="5">
-        <v>46133.8058850463</v>
+        <v>46133.63921837963</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46133.80636234954</v>
+        <v>46133.63969568287</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>193</v>
@@ -4857,11 +4857,11 @@
         <v>195</v>
       </c>
       <c r="B55" s="10">
-        <v>46133.80664880787</v>
+        <v>46133.639982141205</v>
       </c>
       <c r="C55" s="11"/>
       <c r="D55" s="10">
-        <v>46133.80681135417</v>
+        <v>46133.640144687495</v>
       </c>
       <c r="E55" s="11" t="s">
         <v>196</v>
@@ -4906,11 +4906,11 @@
         <v>198</v>
       </c>
       <c r="B56" s="5">
-        <v>46133.80701400463</v>
+        <v>46133.64034733796</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46162.79057355324</v>
+        <v>46162.62390688657</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>199</v>
@@ -4961,11 +4961,11 @@
         <v>202</v>
       </c>
       <c r="B57" s="10">
-        <v>46133.80727017361</v>
+        <v>46133.640603506945</v>
       </c>
       <c r="C57" s="11"/>
       <c r="D57" s="10">
-        <v>46133.80736961805</v>
+        <v>46133.640702951394</v>
       </c>
       <c r="E57" s="11" t="s">
         <v>203</v>
@@ -5010,11 +5010,11 @@
         <v>205</v>
       </c>
       <c r="B58" s="5">
-        <v>46133.79901350694</v>
+        <v>46133.63234684028</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46162.79056252315</v>
+        <v>46162.62389585648</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>206</v>
@@ -5067,11 +5067,11 @@
         <v>208</v>
       </c>
       <c r="B59" s="10">
-        <v>46133.79961443287</v>
+        <v>46133.63294776621</v>
       </c>
       <c r="C59" s="11"/>
       <c r="D59" s="10">
-        <v>46133.79989851852</v>
+        <v>46133.633231851854</v>
       </c>
       <c r="E59" s="11" t="s">
         <v>209</v>
@@ -5116,11 +5116,11 @@
         <v>211</v>
       </c>
       <c r="B60" s="5">
-        <v>46093.557977812496</v>
+        <v>46093.39131114584</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46162.79054756944</v>
+        <v>46162.62388090278</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>212</v>
@@ -5173,11 +5173,11 @@
         <v>214</v>
       </c>
       <c r="B61" s="10">
-        <v>46094.64358574074</v>
+        <v>46094.47691907408</v>
       </c>
       <c r="C61" s="11"/>
       <c r="D61" s="10">
-        <v>46094.643782430554</v>
+        <v>46094.47711576389</v>
       </c>
       <c r="E61" s="11" t="s">
         <v>215</v>
@@ -5222,11 +5222,11 @@
         <v>217</v>
       </c>
       <c r="B62" s="5">
-        <v>46133.80890888889</v>
+        <v>46133.642242222224</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46162.7905368287</v>
+        <v>46162.62387016204</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>218</v>
@@ -5279,11 +5279,11 @@
         <v>221</v>
       </c>
       <c r="B63" s="10">
-        <v>46133.809437812495</v>
+        <v>46133.64277114584</v>
       </c>
       <c r="C63" s="11"/>
       <c r="D63" s="10">
-        <v>46133.80958457176</v>
+        <v>46133.64291790509</v>
       </c>
       <c r="E63" s="11" t="s">
         <v>222</v>
@@ -5328,11 +5328,11 @@
         <v>224</v>
       </c>
       <c r="B64" s="5">
-        <v>46093.55797666666</v>
+        <v>46093.39131</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46162.790523668984</v>
+        <v>46162.62385700231</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>225</v>
@@ -5385,11 +5385,11 @@
         <v>227</v>
       </c>
       <c r="B65" s="10">
-        <v>46094.64611630787</v>
+        <v>46094.47944964121</v>
       </c>
       <c r="C65" s="11"/>
       <c r="D65" s="10">
-        <v>46094.64631732639</v>
+        <v>46094.47965065972</v>
       </c>
       <c r="E65" s="11" t="s">
         <v>228</v>
@@ -5434,11 +5434,11 @@
         <v>230</v>
       </c>
       <c r="B66" s="5">
-        <v>46094.64632454861</v>
+        <v>46094.479657881944</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46094.64655788195</v>
+        <v>46094.47989121528</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>231</v>
@@ -5483,11 +5483,11 @@
         <v>233</v>
       </c>
       <c r="B67" s="10">
-        <v>46093.55797637731</v>
+        <v>46093.39130971065</v>
       </c>
       <c r="C67" s="11"/>
       <c r="D67" s="10">
-        <v>46162.79050667824</v>
+        <v>46162.62384001157</v>
       </c>
       <c r="E67" s="11" t="s">
         <v>234</v>
@@ -5540,11 +5540,11 @@
         <v>236</v>
       </c>
       <c r="B68" s="5">
-        <v>46094.645434618054</v>
+        <v>46094.47876795139</v>
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46094.645602916666</v>
+        <v>46094.47893625</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>237</v>
@@ -5589,11 +5589,11 @@
         <v>239</v>
       </c>
       <c r="B69" s="10">
-        <v>46093.55797821759</v>
+        <v>46093.39131155093</v>
       </c>
       <c r="C69" s="11"/>
       <c r="D69" s="10">
-        <v>46162.79049341435</v>
+        <v>46162.62382674769</v>
       </c>
       <c r="E69" s="11" t="s">
         <v>240</v>
@@ -5646,11 +5646,11 @@
         <v>242</v>
       </c>
       <c r="B70" s="5">
-        <v>46094.65140127315</v>
+        <v>46094.48473460648</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46094.65150827546</v>
+        <v>46094.48484160879</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>243</v>
@@ -5695,11 +5695,11 @@
         <v>245</v>
       </c>
       <c r="B71" s="10">
-        <v>46093.557976192125</v>
+        <v>46093.39130952547</v>
       </c>
       <c r="C71" s="11"/>
       <c r="D71" s="10">
-        <v>46142.16936487269</v>
+        <v>46142.00269820602</v>
       </c>
       <c r="E71" s="11" t="s">
         <v>246</v>
@@ -5752,11 +5752,11 @@
         <v>249</v>
       </c>
       <c r="B72" s="5">
-        <v>46094.63540701389</v>
+        <v>46094.46874034722</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46094.63563651621</v>
+        <v>46094.468969849535</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>250</v>
@@ -5801,11 +5801,11 @@
         <v>252</v>
       </c>
       <c r="B73" s="10">
-        <v>46093.55797792824</v>
+        <v>46093.39131126157</v>
       </c>
       <c r="C73" s="11"/>
       <c r="D73" s="10">
-        <v>46134.689549421295</v>
+        <v>46134.52288275463</v>
       </c>
       <c r="E73" s="11" t="s">
         <v>253</v>
@@ -5858,11 +5858,11 @@
         <v>255</v>
       </c>
       <c r="B74" s="5">
-        <v>46094.64988140046</v>
+        <v>46094.483214733795</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46094.64998811342</v>
+        <v>46094.48332144676</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>256</v>
@@ -5907,11 +5907,11 @@
         <v>258</v>
       </c>
       <c r="B75" s="10">
-        <v>46093.55797513889</v>
+        <v>46093.39130847222</v>
       </c>
       <c r="C75" s="11"/>
       <c r="D75" s="10">
-        <v>46098.62589137732</v>
+        <v>46098.45922471065</v>
       </c>
       <c r="E75" s="11" t="s">
         <v>259</v>
@@ -5966,11 +5966,11 @@
         <v>261</v>
       </c>
       <c r="B76" s="5">
-        <v>46094.566601597224</v>
+        <v>46094.39993493055</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46094.56736538194</v>
+        <v>46094.40069871528</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>262</v>
@@ -6015,11 +6015,11 @@
         <v>264</v>
       </c>
       <c r="B77" s="10">
-        <v>46094.566937951386</v>
+        <v>46094.40027128472</v>
       </c>
       <c r="C77" s="11"/>
       <c r="D77" s="10">
-        <v>46094.56773407407</v>
+        <v>46094.40106740741</v>
       </c>
       <c r="E77" s="11" t="s">
         <v>265</v>
@@ -6064,11 +6064,11 @@
         <v>267</v>
       </c>
       <c r="B78" s="5">
-        <v>46094.56748170139</v>
+        <v>46094.40081503472</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46094.56795886574</v>
+        <v>46094.40129219907</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>268</v>
@@ -6113,11 +6113,11 @@
         <v>270</v>
       </c>
       <c r="B79" s="10">
-        <v>46094.56796667824</v>
+        <v>46094.401300011574</v>
       </c>
       <c r="C79" s="11"/>
       <c r="D79" s="10">
-        <v>46094.56820407408</v>
+        <v>46094.40153740741</v>
       </c>
       <c r="E79" s="11" t="s">
         <v>271</v>
@@ -6162,11 +6162,11 @@
         <v>273</v>
       </c>
       <c r="B80" s="5">
-        <v>46093.557975625</v>
+        <v>46093.39130895834</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46112.84178105324</v>
+        <v>46112.67511438657</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>274</v>
@@ -6221,11 +6221,11 @@
         <v>276</v>
       </c>
       <c r="B81" s="10">
-        <v>46094.57064802083</v>
+        <v>46094.40398135417</v>
       </c>
       <c r="C81" s="11"/>
       <c r="D81" s="10">
-        <v>46094.59020585648</v>
+        <v>46094.42353918981</v>
       </c>
       <c r="E81" s="11" t="s">
         <v>277</v>
@@ -6270,11 +6270,11 @@
         <v>279</v>
       </c>
       <c r="B82" s="5">
-        <v>46094.57343428241</v>
+        <v>46094.40676761574</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46094.59023394676</v>
+        <v>46094.42356728009</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>280</v>
@@ -6319,11 +6319,11 @@
         <v>282</v>
       </c>
       <c r="B83" s="10">
-        <v>46094.573594710644</v>
+        <v>46094.40692804398</v>
       </c>
       <c r="C83" s="11"/>
       <c r="D83" s="10">
-        <v>46094.59026199074</v>
+        <v>46094.42359532407</v>
       </c>
       <c r="E83" s="11" t="s">
         <v>283</v>
@@ -6368,11 +6368,11 @@
         <v>285</v>
       </c>
       <c r="B84" s="5">
-        <v>46094.57373981482</v>
+        <v>46094.40707314815</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46094.59030239584</v>
+        <v>46094.42363572917</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>286</v>
@@ -6417,11 +6417,11 @@
         <v>288</v>
       </c>
       <c r="B85" s="10">
-        <v>46094.573880254626</v>
+        <v>46094.40721358796</v>
       </c>
       <c r="C85" s="11"/>
       <c r="D85" s="10">
-        <v>46094.59033287037</v>
+        <v>46094.4236662037</v>
       </c>
       <c r="E85" s="11" t="s">
         <v>289</v>
@@ -6466,11 +6466,11 @@
         <v>291</v>
       </c>
       <c r="B86" s="5">
-        <v>46093.55797761574</v>
+        <v>46093.391310949075</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46099.63241893519</v>
+        <v>46099.465752268516</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>292</v>
@@ -6523,11 +6523,11 @@
         <v>294</v>
       </c>
       <c r="B87" s="10">
-        <v>46094.65047047454</v>
+        <v>46094.483803807874</v>
       </c>
       <c r="C87" s="11"/>
       <c r="D87" s="10">
-        <v>46111.83610230324</v>
+        <v>46111.66943563658</v>
       </c>
       <c r="E87" s="11" t="s">
         <v>295</v>
@@ -6572,11 +6572,11 @@
         <v>297</v>
       </c>
       <c r="B88" s="5">
-        <v>46094.65072855324</v>
+        <v>46094.48406188657</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46094.65083585648</v>
+        <v>46094.48416918982</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>298</v>
@@ -6621,11 +6621,11 @@
         <v>300</v>
       </c>
       <c r="B89" s="10">
-        <v>46094.650843634256</v>
+        <v>46094.48417696759</v>
       </c>
       <c r="C89" s="11"/>
       <c r="D89" s="10">
-        <v>46094.65119138889</v>
+        <v>46094.484524722226</v>
       </c>
       <c r="E89" s="11" t="s">
         <v>301</v>
@@ -6670,11 +6670,11 @@
         <v>303</v>
       </c>
       <c r="B90" s="5">
-        <v>46094.65095365741</v>
+        <v>46094.484286990744</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46094.65121894676</v>
+        <v>46094.48455228009</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>304</v>
@@ -6719,11 +6719,11 @@
         <v>306</v>
       </c>
       <c r="B91" s="10">
-        <v>46093.557977268516</v>
+        <v>46093.39131060185</v>
       </c>
       <c r="C91" s="11"/>
       <c r="D91" s="10">
-        <v>46099.639211539354</v>
+        <v>46099.47254487268</v>
       </c>
       <c r="E91" s="11" t="s">
         <v>307</v>
@@ -6776,11 +6776,11 @@
         <v>309</v>
       </c>
       <c r="B92" s="5">
-        <v>46094.64259225695</v>
+        <v>46094.475925590275</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46094.642785069445</v>
+        <v>46094.476118402774</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>310</v>
@@ -6825,11 +6825,11 @@
         <v>312</v>
       </c>
       <c r="B93" s="10">
-        <v>46093.55797850694</v>
+        <v>46093.39131184028</v>
       </c>
       <c r="C93" s="11"/>
       <c r="D93" s="10">
-        <v>46099.62486652778</v>
+        <v>46099.45819986111</v>
       </c>
       <c r="E93" s="11" t="s">
         <v>313</v>
@@ -6882,11 +6882,11 @@
         <v>315</v>
       </c>
       <c r="B94" s="5">
-        <v>46094.65201979167</v>
+        <v>46094.485353125</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46094.652139756945</v>
+        <v>46094.48547309027</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>316</v>
@@ -6931,11 +6931,11 @@
         <v>318</v>
       </c>
       <c r="B95" s="10">
-        <v>46093.55797699074</v>
+        <v>46093.39131032408</v>
       </c>
       <c r="C95" s="11"/>
       <c r="D95" s="10">
-        <v>46134.66246857639</v>
+        <v>46134.495801909725</v>
       </c>
       <c r="E95" s="11" t="s">
         <v>319</v>
@@ -6986,11 +6986,11 @@
         <v>321</v>
       </c>
       <c r="B96" s="5">
-        <v>46094.64671800926</v>
+        <v>46094.480051342594</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46094.64682403935</v>
+        <v>46094.48015737269</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>322</v>
@@ -7035,11 +7035,11 @@
         <v>324</v>
       </c>
       <c r="B97" s="10">
-        <v>46093.55797740741</v>
+        <v>46093.39131074074</v>
       </c>
       <c r="C97" s="11"/>
       <c r="D97" s="10">
-        <v>46196.5728619213</v>
+        <v>46196.40619525463</v>
       </c>
       <c r="E97" s="11" t="s">
         <v>325</v>
@@ -7094,11 +7094,11 @@
         <v>327</v>
       </c>
       <c r="B98" s="5">
-        <v>46094.58428688657</v>
+        <v>46094.41762021991</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46094.584938113425</v>
+        <v>46094.41827144676</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>328</v>
@@ -7143,11 +7143,11 @@
         <v>330</v>
       </c>
       <c r="B99" s="10">
-        <v>46094.58447622685</v>
+        <v>46094.41780956018</v>
       </c>
       <c r="C99" s="11"/>
       <c r="D99" s="10">
-        <v>46094.5849659838</v>
+        <v>46094.41829931713</v>
       </c>
       <c r="E99" s="11" t="s">
         <v>331</v>
@@ -7192,11 +7192,11 @@
         <v>333</v>
       </c>
       <c r="B100" s="5">
-        <v>46094.58471086806</v>
+        <v>46094.41804420139</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46094.58499179398</v>
+        <v>46094.41832512731</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>334</v>
@@ -7241,13 +7241,13 @@
         <v>336</v>
       </c>
       <c r="B101" s="10">
-        <v>46093.55797605324</v>
+        <v>46093.39130938657</v>
       </c>
       <c r="C101" s="10">
-        <v>46140.73067185185</v>
+        <v>46140.56400518518</v>
       </c>
       <c r="D101" s="10">
-        <v>46140.730673252314</v>
+        <v>46140.56400658565</v>
       </c>
       <c r="E101" s="11" t="s">
         <v>337</v>
@@ -7300,11 +7300,11 @@
         <v>339</v>
       </c>
       <c r="B102" s="5">
-        <v>46094.644745763886</v>
+        <v>46094.47807909722</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46094.644892048615</v>
+        <v>46094.47822538194</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>340</v>
@@ -7349,11 +7349,11 @@
         <v>342</v>
       </c>
       <c r="B103" s="10">
-        <v>46094.64489846065</v>
+        <v>46094.47823179398</v>
       </c>
       <c r="C103" s="11"/>
       <c r="D103" s="10">
-        <v>46094.64504228009</v>
+        <v>46094.47837561343</v>
       </c>
       <c r="E103" s="11" t="s">
         <v>343</v>
@@ -7398,11 +7398,11 @@
         <v>345</v>
       </c>
       <c r="B104" s="5">
-        <v>46133.8018299074</v>
+        <v>46133.635163240746</v>
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="5">
-        <v>46185.594546168984</v>
+        <v>46185.42787950231</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>346</v>
@@ -7455,11 +7455,11 @@
         <v>348</v>
       </c>
       <c r="B105" s="10">
-        <v>46133.8022120949</v>
+        <v>46133.635545428246</v>
       </c>
       <c r="C105" s="11"/>
       <c r="D105" s="10">
-        <v>46133.80266505787</v>
+        <v>46133.635998391204</v>
       </c>
       <c r="E105" s="11" t="s">
         <v>349</v>
@@ -7504,11 +7504,11 @@
         <v>351</v>
       </c>
       <c r="B106" s="5">
-        <v>46133.80235815972</v>
+        <v>46133.63569149305</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46133.8027009375</v>
+        <v>46133.636034270836</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>352</v>
@@ -7553,11 +7553,11 @@
         <v>354</v>
       </c>
       <c r="B107" s="10">
-        <v>46133.80248805556</v>
+        <v>46133.63582138889</v>
       </c>
       <c r="C107" s="11"/>
       <c r="D107" s="10">
-        <v>46133.802740625004</v>
+        <v>46133.63607395833</v>
       </c>
       <c r="E107" s="11" t="s">
         <v>355</v>
@@ -7602,13 +7602,13 @@
         <v>357</v>
       </c>
       <c r="B108" s="5">
-        <v>46093.55797645834</v>
+        <v>46093.39130979167</v>
       </c>
       <c r="C108" s="5">
-        <v>46162.85491734954</v>
+        <v>46162.68825068287</v>
       </c>
       <c r="D108" s="5">
-        <v>46162.85493328703</v>
+        <v>46162.688266620375</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>358</v>
@@ -7661,13 +7661,13 @@
         <v>360</v>
       </c>
       <c r="B109" s="10">
-        <v>46094.63825950232</v>
+        <v>46094.471592835645</v>
       </c>
       <c r="C109" s="10">
-        <v>46136.032332372684</v>
+        <v>46135.86566570602</v>
       </c>
       <c r="D109" s="10">
-        <v>46136.032352685186</v>
+        <v>46135.865686018515</v>
       </c>
       <c r="E109" s="11" t="s">
         <v>361</v>
@@ -7716,13 +7716,13 @@
         <v>363</v>
       </c>
       <c r="B110" s="5">
-        <v>46094.63841756944</v>
+        <v>46094.471750902776</v>
       </c>
       <c r="C110" s="5">
-        <v>46136.03234583333</v>
+        <v>46135.865679166665</v>
       </c>
       <c r="D110" s="5">
-        <v>46136.03236168981</v>
+        <v>46135.86569502315</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>364</v>
@@ -7771,13 +7771,13 @@
         <v>366</v>
       </c>
       <c r="B111" s="10">
-        <v>46094.63861635417</v>
+        <v>46094.471949687504</v>
       </c>
       <c r="C111" s="10">
-        <v>46136.03235858797</v>
+        <v>46135.865691921295</v>
       </c>
       <c r="D111" s="10">
-        <v>46136.032374560185</v>
+        <v>46135.86570789352</v>
       </c>
       <c r="E111" s="11" t="s">
         <v>367</v>
@@ -7826,13 +7826,13 @@
         <v>369</v>
       </c>
       <c r="B112" s="5">
-        <v>46133.81027721065</v>
+        <v>46133.64361054398</v>
       </c>
       <c r="C112" s="5">
-        <v>46161.91299474537</v>
+        <v>46161.746328078705</v>
       </c>
       <c r="D112" s="5">
-        <v>46161.91301581018</v>
+        <v>46161.74634914352</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>370</v>
@@ -7877,13 +7877,13 @@
         <v>373</v>
       </c>
       <c r="B113" s="10">
-        <v>46133.80965319445</v>
+        <v>46133.642986527775</v>
       </c>
       <c r="C113" s="10">
-        <v>46161.912943958334</v>
+        <v>46161.74627729166</v>
       </c>
       <c r="D113" s="10">
-        <v>46161.91296126157</v>
+        <v>46161.74629459491</v>
       </c>
       <c r="E113" s="11" t="s">
         <v>371</v>
@@ -7936,13 +7936,13 @@
         <v>375</v>
       </c>
       <c r="B114" s="5">
-        <v>46133.79562642361</v>
+        <v>46133.62895975694</v>
       </c>
       <c r="C114" s="5">
-        <v>46161.91275101852</v>
+        <v>46161.74608435185</v>
       </c>
       <c r="D114" s="5">
-        <v>46161.912771296295</v>
+        <v>46161.74610462963</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>376</v>
@@ -7987,13 +7987,13 @@
         <v>379</v>
       </c>
       <c r="B115" s="10">
-        <v>46133.79487287037</v>
+        <v>46133.628206203706</v>
       </c>
       <c r="C115" s="10">
-        <v>46161.91275491898</v>
+        <v>46161.746088252316</v>
       </c>
       <c r="D115" s="10">
-        <v>46161.91277105324</v>
+        <v>46161.74610438658</v>
       </c>
       <c r="E115" s="11" t="s">
         <v>377</v>
@@ -8046,13 +8046,13 @@
         <v>381</v>
       </c>
       <c r="B116" s="5">
-        <v>46133.79582699074</v>
+        <v>46133.629160324075</v>
       </c>
       <c r="C116" s="5">
-        <v>46161.912757847225</v>
+        <v>46161.746091180554</v>
       </c>
       <c r="D116" s="5">
-        <v>46161.91277258102</v>
+        <v>46161.74610591435</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>382</v>
@@ -8097,13 +8097,13 @@
         <v>384</v>
       </c>
       <c r="B117" s="10">
-        <v>46094.641416493054</v>
+        <v>46094.47474982639</v>
       </c>
       <c r="C117" s="10">
-        <v>46161.912420381945</v>
+        <v>46161.74575371528</v>
       </c>
       <c r="D117" s="10">
-        <v>46161.912439594904</v>
+        <v>46161.74577292824</v>
       </c>
       <c r="E117" s="11" t="s">
         <v>385</v>
@@ -8152,13 +8152,13 @@
         <v>388</v>
       </c>
       <c r="B118" s="5">
-        <v>46093.55797701389</v>
+        <v>46093.39131034722</v>
       </c>
       <c r="C118" s="5">
-        <v>46161.912426678246</v>
+        <v>46161.745760011574</v>
       </c>
       <c r="D118" s="5">
-        <v>46161.91244167824</v>
+        <v>46161.74577501157</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>386</v>
@@ -8211,13 +8211,13 @@
         <v>390</v>
       </c>
       <c r="B119" s="10">
-        <v>46094.582692951386</v>
+        <v>46094.41602628472</v>
       </c>
       <c r="C119" s="10">
-        <v>46134.673179687496</v>
+        <v>46134.50651302084</v>
       </c>
       <c r="D119" s="10">
-        <v>46134.67319648148</v>
+        <v>46134.50652981481</v>
       </c>
       <c r="E119" s="11" t="s">
         <v>391</v>
@@ -8264,13 +8264,13 @@
         <v>394</v>
       </c>
       <c r="B120" s="5">
-        <v>46093.557975625</v>
+        <v>46093.39130895834</v>
       </c>
       <c r="C120" s="5">
-        <v>46134.64221024305</v>
+        <v>46134.47554357639</v>
       </c>
       <c r="D120" s="5">
-        <v>46134.66266402778</v>
+        <v>46134.49599736111</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>395</v>
@@ -8317,13 +8317,13 @@
         <v>397</v>
       </c>
       <c r="B121" s="10">
-        <v>46093.55797712963</v>
+        <v>46093.39131046296</v>
       </c>
       <c r="C121" s="10">
-        <v>46134.63987417824</v>
+        <v>46134.473207511575</v>
       </c>
       <c r="D121" s="10">
-        <v>46134.63988903935</v>
+        <v>46134.47322237269</v>
       </c>
       <c r="E121" s="11" t="s">
         <v>392</v>
@@ -8376,13 +8376,13 @@
         <v>399</v>
       </c>
       <c r="B122" s="5">
-        <v>46094.58194446759</v>
+        <v>46094.41527780093</v>
       </c>
       <c r="C122" s="5">
-        <v>46134.63920685185</v>
+        <v>46134.47254018519</v>
       </c>
       <c r="D122" s="5">
-        <v>46134.66324178241</v>
+        <v>46134.49657511574</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>400</v>
@@ -8429,13 +8429,13 @@
         <v>402</v>
       </c>
       <c r="B123" s="10">
-        <v>46094.58215357639</v>
+        <v>46094.415486909726</v>
       </c>
       <c r="C123" s="10">
-        <v>46134.63922920139</v>
+        <v>46134.47256253472</v>
       </c>
       <c r="D123" s="10">
-        <v>46134.66306040509</v>
+        <v>46134.49639373843</v>
       </c>
       <c r="E123" s="11" t="s">
         <v>403</v>
@@ -8482,13 +8482,13 @@
         <v>405</v>
       </c>
       <c r="B124" s="5">
-        <v>46094.5823130787</v>
+        <v>46094.41564641204</v>
       </c>
       <c r="C124" s="5">
-        <v>46134.63923450232</v>
+        <v>46134.47256783565</v>
       </c>
       <c r="D124" s="5">
-        <v>46134.66313976852</v>
+        <v>46134.496473101855</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>406</v>
@@ -8535,13 +8535,13 @@
         <v>408</v>
       </c>
       <c r="B125" s="10">
-        <v>46094.582410393516</v>
+        <v>46094.41574372685</v>
       </c>
       <c r="C125" s="10">
-        <v>46134.63923954861</v>
+        <v>46134.47257288195</v>
       </c>
       <c r="D125" s="10">
-        <v>46134.662989178236</v>
+        <v>46134.49632251158</v>
       </c>
       <c r="E125" s="11" t="s">
         <v>409</v>
@@ -8588,13 +8588,13 @@
         <v>411</v>
       </c>
       <c r="B126" s="5">
-        <v>46094.58253722222</v>
+        <v>46094.41587055556</v>
       </c>
       <c r="C126" s="5">
-        <v>46134.639245694445</v>
+        <v>46134.47257902777</v>
       </c>
       <c r="D126" s="5">
-        <v>46134.662925682875</v>
+        <v>46134.4962590162</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>412</v>
@@ -8641,13 +8641,13 @@
         <v>414</v>
       </c>
       <c r="B127" s="10">
-        <v>46094.582797511575</v>
+        <v>46094.41613084491</v>
       </c>
       <c r="C127" s="10">
-        <v>46134.639255312504</v>
+        <v>46134.47258864583</v>
       </c>
       <c r="D127" s="10">
-        <v>46155.578320636574</v>
+        <v>46155.4116539699</v>
       </c>
       <c r="E127" s="11" t="s">
         <v>415</v>
@@ -8694,13 +8694,13 @@
         <v>417</v>
       </c>
       <c r="B128" s="5">
-        <v>46094.58288509259</v>
+        <v>46094.416218425926</v>
       </c>
       <c r="C128" s="5">
-        <v>46134.63926054398</v>
+        <v>46134.47259387732</v>
       </c>
       <c r="D128" s="5">
-        <v>46134.662788738424</v>
+        <v>46134.49612207176</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>418</v>
@@ -8747,13 +8747,13 @@
         <v>420</v>
       </c>
       <c r="B129" s="10">
-        <v>46094.58306329861</v>
+        <v>46094.41639663195</v>
       </c>
       <c r="C129" s="10">
-        <v>46134.639266087965</v>
+        <v>46134.47259942129</v>
       </c>
       <c r="D129" s="10">
-        <v>46134.66273581018</v>
+        <v>46134.49606914352</v>
       </c>
       <c r="E129" s="11" t="s">
         <v>421</v>
@@ -8800,13 +8800,13 @@
         <v>423</v>
       </c>
       <c r="B130" s="5">
-        <v>46133.792176840274</v>
+        <v>46133.62551017361</v>
       </c>
       <c r="C130" s="5">
-        <v>46134.63605664352</v>
+        <v>46134.46938997685</v>
       </c>
       <c r="D130" s="5">
-        <v>46134.63619297453</v>
+        <v>46134.469526307876</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>424</v>
@@ -8859,11 +8859,11 @@
         <v>428</v>
       </c>
       <c r="B131" s="10">
-        <v>46133.79263490741</v>
+        <v>46133.62596824074</v>
       </c>
       <c r="C131" s="11"/>
       <c r="D131" s="10">
-        <v>46133.79350961806</v>
+        <v>46133.62684295139</v>
       </c>
       <c r="E131" s="11" t="s">
         <v>429</v>
@@ -8908,13 +8908,13 @@
         <v>431</v>
       </c>
       <c r="B132" s="5">
-        <v>46091.59394065972</v>
+        <v>46091.42727399306</v>
       </c>
       <c r="C132" s="5">
-        <v>46133.70594085648</v>
+        <v>46133.53927418981</v>
       </c>
       <c r="D132" s="5">
-        <v>46133.7059553125</v>
+        <v>46133.53928864583</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>432</v>
@@ -8967,11 +8967,11 @@
         <v>434</v>
       </c>
       <c r="B133" s="10">
-        <v>46094.62533957176</v>
+        <v>46094.45867290509</v>
       </c>
       <c r="C133" s="11"/>
       <c r="D133" s="10">
-        <v>46133.70593778935</v>
+        <v>46133.53927112269</v>
       </c>
       <c r="E133" s="11" t="s">
         <v>435</v>
@@ -9016,11 +9016,11 @@
         <v>437</v>
       </c>
       <c r="B134" s="5">
-        <v>46094.62542793981</v>
+        <v>46094.45876127315</v>
       </c>
       <c r="C134" s="6"/>
       <c r="D134" s="5">
-        <v>46133.70593837963</v>
+        <v>46133.53927171296</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>438</v>
@@ -9065,11 +9065,11 @@
         <v>440</v>
       </c>
       <c r="B135" s="10">
-        <v>46094.62613793982</v>
+        <v>46094.45947127315</v>
       </c>
       <c r="C135" s="11"/>
       <c r="D135" s="10">
-        <v>46133.70593877315</v>
+        <v>46133.539272106485</v>
       </c>
       <c r="E135" s="11" t="s">
         <v>441</v>
@@ -9114,11 +9114,11 @@
         <v>443</v>
       </c>
       <c r="B136" s="5">
-        <v>46094.626408703705</v>
+        <v>46094.45974203704</v>
       </c>
       <c r="C136" s="6"/>
       <c r="D136" s="5">
-        <v>46133.705939189815</v>
+        <v>46133.53927252315</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>444</v>
@@ -9163,11 +9163,11 @@
         <v>446</v>
       </c>
       <c r="B137" s="10">
-        <v>46094.62648922454</v>
+        <v>46094.45982255787</v>
       </c>
       <c r="C137" s="11"/>
       <c r="D137" s="10">
-        <v>46133.705939618056</v>
+        <v>46133.539272951384</v>
       </c>
       <c r="E137" s="11" t="s">
         <v>447</v>
@@ -9212,11 +9212,11 @@
         <v>449</v>
       </c>
       <c r="B138" s="5">
-        <v>46094.62660908565</v>
+        <v>46094.45994241898</v>
       </c>
       <c r="C138" s="6"/>
       <c r="D138" s="5">
-        <v>46133.7059399537</v>
+        <v>46133.53927328704</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>450</v>
@@ -9261,11 +9261,11 @@
         <v>452</v>
       </c>
       <c r="B139" s="10">
-        <v>46094.626713460646</v>
+        <v>46094.46004679398</v>
       </c>
       <c r="C139" s="11"/>
       <c r="D139" s="10">
-        <v>46133.705940300926</v>
+        <v>46133.53927363426</v>
       </c>
       <c r="E139" s="11" t="s">
         <v>453</v>
@@ -9310,11 +9310,11 @@
         <v>455</v>
       </c>
       <c r="B140" s="5">
-        <v>46094.62680802083</v>
+        <v>46094.46014135417</v>
       </c>
       <c r="C140" s="6"/>
       <c r="D140" s="5">
-        <v>46133.70594064815</v>
+        <v>46133.539273981485</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>456</v>
@@ -9359,13 +9359,13 @@
         <v>458</v>
       </c>
       <c r="B141" s="10">
-        <v>46093.55797592593</v>
+        <v>46093.391309259256</v>
       </c>
       <c r="C141" s="10">
-        <v>46127.87503005787</v>
+        <v>46127.708363391204</v>
       </c>
       <c r="D141" s="10">
-        <v>46134.66330939815</v>
+        <v>46134.49664273148</v>
       </c>
       <c r="E141" s="11" t="s">
         <v>459</v>
@@ -9412,13 +9412,13 @@
         <v>461</v>
       </c>
       <c r="B142" s="5">
-        <v>46094.63474699074</v>
+        <v>46094.46808032408</v>
       </c>
       <c r="C142" s="5">
-        <v>46127.875013819445</v>
+        <v>46127.70834715277</v>
       </c>
       <c r="D142" s="5">
-        <v>46134.66345291666</v>
+        <v>46134.496786250005</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>462</v>
@@ -9465,13 +9465,13 @@
         <v>464</v>
       </c>
       <c r="B143" s="10">
-        <v>46093.557976111115</v>
+        <v>46093.39130944444</v>
       </c>
       <c r="C143" s="10">
-        <v>46111.836577766204</v>
+        <v>46111.66991109954</v>
       </c>
       <c r="D143" s="10">
-        <v>46111.836592141204</v>
+        <v>46111.66992547453</v>
       </c>
       <c r="E143" s="11" t="s">
         <v>465</v>
@@ -9526,13 +9526,13 @@
         <v>467</v>
       </c>
       <c r="B144" s="5">
-        <v>46094.57571935185</v>
+        <v>46094.40905268519</v>
       </c>
       <c r="C144" s="5">
-        <v>46111.83654524306</v>
+        <v>46111.66987857639</v>
       </c>
       <c r="D144" s="5">
-        <v>46111.83656112268</v>
+        <v>46111.66989445602</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>468</v>
@@ -9577,13 +9577,13 @@
         <v>470</v>
       </c>
       <c r="B145" s="10">
-        <v>46094.57601390046</v>
+        <v>46094.4093472338</v>
       </c>
       <c r="C145" s="10">
-        <v>46111.8365590162</v>
+        <v>46111.66989234954</v>
       </c>
       <c r="D145" s="10">
-        <v>46111.83657758102</v>
+        <v>46111.66991091435</v>
       </c>
       <c r="E145" s="11" t="s">
         <v>471</v>
@@ -9628,13 +9628,13 @@
         <v>473</v>
       </c>
       <c r="B146" s="5">
-        <v>46094.57620418981</v>
+        <v>46094.40953752315</v>
       </c>
       <c r="C146" s="5">
-        <v>46111.83657327546</v>
+        <v>46111.6699066088</v>
       </c>
       <c r="D146" s="5">
-        <v>46111.83659253472</v>
+        <v>46111.66992586806</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>474</v>
@@ -9679,13 +9679,13 @@
         <v>476</v>
       </c>
       <c r="B147" s="10">
-        <v>46093.557975868054</v>
+        <v>46093.39130920139</v>
       </c>
       <c r="C147" s="10">
-        <v>46097.77705668981</v>
+        <v>46097.61039002315</v>
       </c>
       <c r="D147" s="10">
-        <v>46097.77707333333</v>
+        <v>46097.61040666667</v>
       </c>
       <c r="E147" s="11" t="s">
         <v>477</v>
@@ -9738,13 +9738,13 @@
         <v>479</v>
       </c>
       <c r="B148" s="5">
-        <v>46094.57453506945</v>
+        <v>46094.40786840278</v>
       </c>
       <c r="C148" s="5">
-        <v>46097.77703761574</v>
+        <v>46097.61037094907</v>
       </c>
       <c r="D148" s="5">
-        <v>46097.77705638889</v>
+        <v>46097.61038972222</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>480</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-26 15:33 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -2144,11 +2144,11 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46164.530937407406</v>
+        <v>46164.69760407407</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="5">
-        <v>46196.002313715275</v>
+        <v>46196.168980381946</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -2203,11 +2203,11 @@
         <v>32</v>
       </c>
       <c r="B5" s="10">
-        <v>46164.53118508102</v>
+        <v>46164.69785174768</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="10">
-        <v>46164.531429236114</v>
+        <v>46164.69809590278</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>33</v>
@@ -2252,11 +2252,11 @@
         <v>35</v>
       </c>
       <c r="B6" s="5">
-        <v>46164.53126233796</v>
+        <v>46164.69792900463</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="5">
-        <v>46164.53159351852</v>
+        <v>46164.698260185185</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>36</v>
@@ -2301,11 +2301,11 @@
         <v>38</v>
       </c>
       <c r="B7" s="10">
-        <v>46155.63600853009</v>
+        <v>46155.802675196755</v>
       </c>
       <c r="C7" s="11"/>
       <c r="D7" s="10">
-        <v>46155.63846498843</v>
+        <v>46155.80513165509</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>39</v>
@@ -2358,11 +2358,11 @@
         <v>45</v>
       </c>
       <c r="B8" s="5">
-        <v>46155.63648939815</v>
+        <v>46155.803156064816</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="5">
-        <v>46155.63809114583</v>
+        <v>46155.8047578125</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>46</v>
@@ -2411,11 +2411,11 @@
         <v>48</v>
       </c>
       <c r="B9" s="10">
-        <v>46188.464606747686</v>
+        <v>46188.63127341435</v>
       </c>
       <c r="C9" s="11"/>
       <c r="D9" s="10">
-        <v>46188.46520918982</v>
+        <v>46188.63187585648</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>49</v>
@@ -2466,11 +2466,11 @@
         <v>52</v>
       </c>
       <c r="B10" s="5">
-        <v>46188.46489559028</v>
+        <v>46188.631562256945</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46188.46504497685</v>
+        <v>46188.631711643524</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>53</v>
@@ -2515,11 +2515,11 @@
         <v>55</v>
       </c>
       <c r="B11" s="10">
-        <v>46093.39130898148</v>
+        <v>46093.557975648146</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="10">
-        <v>46196.40792715277</v>
+        <v>46196.574593819445</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>56</v>
@@ -2568,11 +2568,11 @@
         <v>60</v>
       </c>
       <c r="B12" s="5">
-        <v>46094.46779931713</v>
+        <v>46094.63446598379</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46094.46797046297</v>
+        <v>46094.63463712963</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>61</v>
@@ -2617,11 +2617,11 @@
         <v>63</v>
       </c>
       <c r="B13" s="10">
-        <v>46188.46551144676</v>
+        <v>46188.632178113425</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="10">
-        <v>46188.46600372685</v>
+        <v>46188.63267039352</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>64</v>
@@ -2672,11 +2672,11 @@
         <v>66</v>
       </c>
       <c r="B14" s="5">
-        <v>46188.46571405092</v>
+        <v>46188.632380717594</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46188.46590284722</v>
+        <v>46188.63256951389</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>67</v>
@@ -2721,11 +2721,11 @@
         <v>69</v>
       </c>
       <c r="B15" s="10">
-        <v>46093.39131063657</v>
+        <v>46093.55797730324</v>
       </c>
       <c r="C15" s="11"/>
       <c r="D15" s="10">
-        <v>46134.49523165509</v>
+        <v>46134.66189832176</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>70</v>
@@ -2778,11 +2778,11 @@
         <v>73</v>
       </c>
       <c r="B16" s="5">
-        <v>46094.480701736116</v>
+        <v>46094.64736840277</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="5">
-        <v>46094.482618090275</v>
+        <v>46094.649284756946</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>74</v>
@@ -2829,11 +2829,11 @@
         <v>76</v>
       </c>
       <c r="B17" s="10">
-        <v>46094.480831469904</v>
+        <v>46094.647498136575</v>
       </c>
       <c r="C17" s="11"/>
       <c r="D17" s="10">
-        <v>46094.48267085648</v>
+        <v>46094.64933752315</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>77</v>
@@ -2880,11 +2880,11 @@
         <v>79</v>
       </c>
       <c r="B18" s="5">
-        <v>46094.48094486111</v>
+        <v>46094.64761152778</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46094.48273704862</v>
+        <v>46094.64940371527</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>80</v>
@@ -2931,11 +2931,11 @@
         <v>82</v>
       </c>
       <c r="B19" s="10">
-        <v>46094.48106497685</v>
+        <v>46094.64773164352</v>
       </c>
       <c r="C19" s="11"/>
       <c r="D19" s="10">
-        <v>46094.48279043981</v>
+        <v>46094.64945710648</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>83</v>
@@ -2982,11 +2982,11 @@
         <v>85</v>
       </c>
       <c r="B20" s="5">
-        <v>46094.481176643516</v>
+        <v>46094.64784331019</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="5">
-        <v>46094.48295435186</v>
+        <v>46094.649621018514</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>86</v>
@@ -3033,11 +3033,11 @@
         <v>88</v>
       </c>
       <c r="B21" s="10">
-        <v>46093.39131086806</v>
+        <v>46093.55797753472</v>
       </c>
       <c r="C21" s="11"/>
       <c r="D21" s="10">
-        <v>46134.495340671296</v>
+        <v>46134.66200733796</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>89</v>
@@ -3090,11 +3090,11 @@
         <v>91</v>
       </c>
       <c r="B22" s="5">
-        <v>46094.47638525463</v>
+        <v>46094.643051921295</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46094.47650232639</v>
+        <v>46094.643168993054</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>92</v>
@@ -3139,11 +3139,11 @@
         <v>94</v>
       </c>
       <c r="B23" s="10">
-        <v>46133.64463065972</v>
+        <v>46133.81129732639</v>
       </c>
       <c r="C23" s="11"/>
       <c r="D23" s="10">
-        <v>46139.00650162037</v>
+        <v>46139.17316828704</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>95</v>
@@ -3196,11 +3196,11 @@
         <v>97</v>
       </c>
       <c r="B24" s="5">
-        <v>46133.645201956024</v>
+        <v>46133.81186862268</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="5">
-        <v>46133.64537636574</v>
+        <v>46133.812043032405</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>98</v>
@@ -3245,11 +3245,11 @@
         <v>100</v>
       </c>
       <c r="B25" s="10">
-        <v>46148.99289465278</v>
+        <v>46149.159561319444</v>
       </c>
       <c r="C25" s="11"/>
       <c r="D25" s="10">
-        <v>46170.0010299537</v>
+        <v>46170.16769662037</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>101</v>
@@ -3302,11 +3302,11 @@
         <v>103</v>
       </c>
       <c r="B26" s="5">
-        <v>46148.99377987269</v>
+        <v>46149.16044653935</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="5">
-        <v>46148.99748721065</v>
+        <v>46149.16415387731</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>104</v>
@@ -3351,11 +3351,11 @@
         <v>106</v>
       </c>
       <c r="B27" s="10">
-        <v>46148.99753195602</v>
+        <v>46149.16419862269</v>
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="10">
-        <v>46148.99788972222</v>
+        <v>46149.16455638889</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>107</v>
@@ -3400,11 +3400,11 @@
         <v>109</v>
       </c>
       <c r="B28" s="5">
-        <v>46148.99789677083</v>
+        <v>46149.1645634375</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46148.99824690972</v>
+        <v>46149.16491357639</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>110</v>
@@ -3449,11 +3449,11 @@
         <v>112</v>
       </c>
       <c r="B29" s="10">
-        <v>46155.63856789352</v>
+        <v>46155.80523456019</v>
       </c>
       <c r="C29" s="11"/>
       <c r="D29" s="10">
-        <v>46163.02779288194</v>
+        <v>46163.19445954861</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>113</v>
@@ -3506,11 +3506,11 @@
         <v>115</v>
       </c>
       <c r="B30" s="5">
-        <v>46155.63897260417</v>
+        <v>46155.80563927084</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46163.02779289352</v>
+        <v>46163.19445956018</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>116</v>
@@ -3561,11 +3561,11 @@
         <v>118</v>
       </c>
       <c r="B31" s="10">
-        <v>46155.63913358796</v>
+        <v>46155.80580025463</v>
       </c>
       <c r="C31" s="11"/>
       <c r="D31" s="10">
-        <v>46163.02779299769</v>
+        <v>46163.19445966435</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>119</v>
@@ -3616,11 +3616,11 @@
         <v>121</v>
       </c>
       <c r="B32" s="5">
-        <v>46155.63985895833</v>
+        <v>46155.806525625</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="5">
-        <v>46163.027794525464</v>
+        <v>46163.19446119213</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>122</v>
@@ -3673,11 +3673,11 @@
         <v>125</v>
       </c>
       <c r="B33" s="10">
-        <v>46155.64006034722</v>
+        <v>46155.806727013885</v>
       </c>
       <c r="C33" s="11"/>
       <c r="D33" s="10">
-        <v>46163.02779371528</v>
+        <v>46163.19446038194</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>126</v>
@@ -3728,11 +3728,11 @@
         <v>128</v>
       </c>
       <c r="B34" s="5">
-        <v>46155.64067324074</v>
+        <v>46155.807339907406</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="5">
-        <v>46197.627945520835</v>
+        <v>46197.7946121875</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>129</v>
@@ -3785,11 +3785,11 @@
         <v>131</v>
       </c>
       <c r="B35" s="10">
-        <v>46155.64121944444</v>
+        <v>46155.80788611111</v>
       </c>
       <c r="C35" s="11"/>
       <c r="D35" s="10">
-        <v>46170.001030451385</v>
+        <v>46170.16769711806</v>
       </c>
       <c r="E35" s="11" t="s">
         <v>132</v>
@@ -3840,11 +3840,11 @@
         <v>134</v>
       </c>
       <c r="B36" s="5">
-        <v>46156.62160987269</v>
+        <v>46156.78827653935</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46169.00965846065</v>
+        <v>46169.176325127315</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>135</v>
@@ -3897,11 +3897,11 @@
         <v>138</v>
       </c>
       <c r="B37" s="10">
-        <v>46156.622255243055</v>
+        <v>46156.78892190973</v>
       </c>
       <c r="C37" s="11"/>
       <c r="D37" s="10">
-        <v>46169.00965871528</v>
+        <v>46169.176325381944</v>
       </c>
       <c r="E37" s="11" t="s">
         <v>139</v>
@@ -3952,11 +3952,11 @@
         <v>141</v>
       </c>
       <c r="B38" s="5">
-        <v>46156.6225257176</v>
+        <v>46156.789192384254</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46169.00965869213</v>
+        <v>46169.1763253588</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>142</v>
@@ -4007,11 +4007,11 @@
         <v>144</v>
       </c>
       <c r="B39" s="10">
-        <v>46188.46295746528</v>
+        <v>46188.62962413194</v>
       </c>
       <c r="C39" s="11"/>
       <c r="D39" s="10">
-        <v>46196.4505393287</v>
+        <v>46196.61720599537</v>
       </c>
       <c r="E39" s="11" t="s">
         <v>145</v>
@@ -4062,11 +4062,11 @@
         <v>147</v>
       </c>
       <c r="B40" s="5">
-        <v>46188.463355879634</v>
+        <v>46188.63002254629</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46196.03406662037</v>
+        <v>46196.20073328704</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>148</v>
@@ -4117,13 +4117,13 @@
         <v>150</v>
       </c>
       <c r="B41" s="10">
-        <v>46188.46360969907</v>
+        <v>46188.630276365744</v>
       </c>
       <c r="C41" s="10">
-        <v>46195.437958090275</v>
+        <v>46195.60462475695</v>
       </c>
       <c r="D41" s="10">
-        <v>46195.43797585648</v>
+        <v>46195.60464252315</v>
       </c>
       <c r="E41" s="11" t="s">
         <v>151</v>
@@ -4170,11 +4170,11 @@
         <v>154</v>
       </c>
       <c r="B42" s="5">
-        <v>46133.63068210648</v>
+        <v>46133.79734877315</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46141.57465121528</v>
+        <v>46141.74131788194</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>155</v>
@@ -4227,11 +4227,11 @@
         <v>158</v>
       </c>
       <c r="B43" s="10">
-        <v>46133.63180929398</v>
+        <v>46133.79847596065</v>
       </c>
       <c r="C43" s="11"/>
       <c r="D43" s="10">
-        <v>46134.49308862269</v>
+        <v>46134.65975528935</v>
       </c>
       <c r="E43" s="11" t="s">
         <v>159</v>
@@ -4276,11 +4276,11 @@
         <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46133.63333427084</v>
+        <v>46133.800000937495</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46141.575875821756</v>
+        <v>46141.74254248843</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>162</v>
@@ -4333,11 +4333,11 @@
         <v>164</v>
       </c>
       <c r="B45" s="10">
-        <v>46133.633699375</v>
+        <v>46133.800366041665</v>
       </c>
       <c r="C45" s="11"/>
       <c r="D45" s="10">
-        <v>46133.6339280324</v>
+        <v>46133.800594699074</v>
       </c>
       <c r="E45" s="11" t="s">
         <v>165</v>
@@ -4382,11 +4382,11 @@
         <v>167</v>
       </c>
       <c r="B46" s="5">
-        <v>46093.391310046296</v>
+        <v>46093.55797671297</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46195.41091278935</v>
+        <v>46195.57757945602</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>168</v>
@@ -4441,11 +4441,11 @@
         <v>171</v>
       </c>
       <c r="B47" s="10">
-        <v>46094.4733012037</v>
+        <v>46094.639967870375</v>
       </c>
       <c r="C47" s="11"/>
       <c r="D47" s="10">
-        <v>46130.01896435185</v>
+        <v>46130.18563101852</v>
       </c>
       <c r="E47" s="11" t="s">
         <v>172</v>
@@ -4494,11 +4494,11 @@
         <v>174</v>
       </c>
       <c r="B48" s="5">
-        <v>46094.47355861111</v>
+        <v>46094.64022527778</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46100.98427231482</v>
+        <v>46101.15093898148</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>175</v>
@@ -4547,11 +4547,11 @@
         <v>177</v>
       </c>
       <c r="B49" s="10">
-        <v>46133.64380305556</v>
+        <v>46133.81046972222</v>
       </c>
       <c r="C49" s="11"/>
       <c r="D49" s="10">
-        <v>46162.62392778935</v>
+        <v>46162.79059445602</v>
       </c>
       <c r="E49" s="11" t="s">
         <v>178</v>
@@ -4604,11 +4604,11 @@
         <v>180</v>
       </c>
       <c r="B50" s="5">
-        <v>46133.64404806713</v>
+        <v>46133.8107147338</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46133.64421252315</v>
+        <v>46133.81087918981</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>181</v>
@@ -4653,11 +4653,11 @@
         <v>183</v>
       </c>
       <c r="B51" s="10">
-        <v>46133.63803945602</v>
+        <v>46133.80470612268</v>
       </c>
       <c r="C51" s="11"/>
       <c r="D51" s="10">
-        <v>46196.74914542824</v>
+        <v>46196.91581209491</v>
       </c>
       <c r="E51" s="11" t="s">
         <v>184</v>
@@ -4710,11 +4710,11 @@
         <v>186</v>
       </c>
       <c r="B52" s="5">
-        <v>46133.638791053236</v>
+        <v>46133.80545771991</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46133.6389784375</v>
+        <v>46133.80564510416</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>187</v>
@@ -4759,11 +4759,11 @@
         <v>189</v>
       </c>
       <c r="B53" s="10">
-        <v>46133.63903846065</v>
+        <v>46133.80570512731</v>
       </c>
       <c r="C53" s="11"/>
       <c r="D53" s="10">
-        <v>46133.639167002315</v>
+        <v>46133.80583366899</v>
       </c>
       <c r="E53" s="11" t="s">
         <v>190</v>
@@ -4808,11 +4808,11 @@
         <v>192</v>
       </c>
       <c r="B54" s="5">
-        <v>46133.63921837963</v>
+        <v>46133.8058850463</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46133.63969568287</v>
+        <v>46133.80636234954</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>193</v>
@@ -4857,11 +4857,11 @@
         <v>195</v>
       </c>
       <c r="B55" s="10">
-        <v>46133.639982141205</v>
+        <v>46133.80664880787</v>
       </c>
       <c r="C55" s="11"/>
       <c r="D55" s="10">
-        <v>46133.640144687495</v>
+        <v>46133.80681135417</v>
       </c>
       <c r="E55" s="11" t="s">
         <v>196</v>
@@ -4906,11 +4906,11 @@
         <v>198</v>
       </c>
       <c r="B56" s="5">
-        <v>46133.64034733796</v>
+        <v>46133.80701400463</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46162.62390688657</v>
+        <v>46162.79057355324</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>199</v>
@@ -4961,11 +4961,11 @@
         <v>202</v>
       </c>
       <c r="B57" s="10">
-        <v>46133.640603506945</v>
+        <v>46133.80727017361</v>
       </c>
       <c r="C57" s="11"/>
       <c r="D57" s="10">
-        <v>46133.640702951394</v>
+        <v>46133.80736961805</v>
       </c>
       <c r="E57" s="11" t="s">
         <v>203</v>
@@ -5010,11 +5010,11 @@
         <v>205</v>
       </c>
       <c r="B58" s="5">
-        <v>46133.63234684028</v>
+        <v>46133.79901350694</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46162.62389585648</v>
+        <v>46162.79056252315</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>206</v>
@@ -5067,11 +5067,11 @@
         <v>208</v>
       </c>
       <c r="B59" s="10">
-        <v>46133.63294776621</v>
+        <v>46133.79961443287</v>
       </c>
       <c r="C59" s="11"/>
       <c r="D59" s="10">
-        <v>46133.633231851854</v>
+        <v>46133.79989851852</v>
       </c>
       <c r="E59" s="11" t="s">
         <v>209</v>
@@ -5116,11 +5116,11 @@
         <v>211</v>
       </c>
       <c r="B60" s="5">
-        <v>46093.39131114584</v>
+        <v>46093.557977812496</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46162.62388090278</v>
+        <v>46162.79054756944</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>212</v>
@@ -5173,11 +5173,11 @@
         <v>214</v>
       </c>
       <c r="B61" s="10">
-        <v>46094.47691907408</v>
+        <v>46094.64358574074</v>
       </c>
       <c r="C61" s="11"/>
       <c r="D61" s="10">
-        <v>46094.47711576389</v>
+        <v>46094.643782430554</v>
       </c>
       <c r="E61" s="11" t="s">
         <v>215</v>
@@ -5222,11 +5222,11 @@
         <v>217</v>
       </c>
       <c r="B62" s="5">
-        <v>46133.642242222224</v>
+        <v>46133.80890888889</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46162.62387016204</v>
+        <v>46162.7905368287</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>218</v>
@@ -5279,11 +5279,11 @@
         <v>221</v>
       </c>
       <c r="B63" s="10">
-        <v>46133.64277114584</v>
+        <v>46133.809437812495</v>
       </c>
       <c r="C63" s="11"/>
       <c r="D63" s="10">
-        <v>46133.64291790509</v>
+        <v>46133.80958457176</v>
       </c>
       <c r="E63" s="11" t="s">
         <v>222</v>
@@ -5328,11 +5328,11 @@
         <v>224</v>
       </c>
       <c r="B64" s="5">
-        <v>46093.39131</v>
+        <v>46093.55797666666</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46162.62385700231</v>
+        <v>46162.790523668984</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>225</v>
@@ -5385,11 +5385,11 @@
         <v>227</v>
       </c>
       <c r="B65" s="10">
-        <v>46094.47944964121</v>
+        <v>46094.64611630787</v>
       </c>
       <c r="C65" s="11"/>
       <c r="D65" s="10">
-        <v>46094.47965065972</v>
+        <v>46094.64631732639</v>
       </c>
       <c r="E65" s="11" t="s">
         <v>228</v>
@@ -5434,11 +5434,11 @@
         <v>230</v>
       </c>
       <c r="B66" s="5">
-        <v>46094.479657881944</v>
+        <v>46094.64632454861</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46094.47989121528</v>
+        <v>46094.64655788195</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>231</v>
@@ -5483,11 +5483,11 @@
         <v>233</v>
       </c>
       <c r="B67" s="10">
-        <v>46093.39130971065</v>
+        <v>46093.55797637731</v>
       </c>
       <c r="C67" s="11"/>
       <c r="D67" s="10">
-        <v>46162.62384001157</v>
+        <v>46162.79050667824</v>
       </c>
       <c r="E67" s="11" t="s">
         <v>234</v>
@@ -5540,11 +5540,11 @@
         <v>236</v>
       </c>
       <c r="B68" s="5">
-        <v>46094.47876795139</v>
+        <v>46094.645434618054</v>
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46094.47893625</v>
+        <v>46094.645602916666</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>237</v>
@@ -5589,11 +5589,11 @@
         <v>239</v>
       </c>
       <c r="B69" s="10">
-        <v>46093.39131155093</v>
+        <v>46093.55797821759</v>
       </c>
       <c r="C69" s="11"/>
       <c r="D69" s="10">
-        <v>46162.62382674769</v>
+        <v>46162.79049341435</v>
       </c>
       <c r="E69" s="11" t="s">
         <v>240</v>
@@ -5646,11 +5646,11 @@
         <v>242</v>
       </c>
       <c r="B70" s="5">
-        <v>46094.48473460648</v>
+        <v>46094.65140127315</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46094.48484160879</v>
+        <v>46094.65150827546</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>243</v>
@@ -5695,11 +5695,11 @@
         <v>245</v>
       </c>
       <c r="B71" s="10">
-        <v>46093.39130952547</v>
+        <v>46093.557976192125</v>
       </c>
       <c r="C71" s="11"/>
       <c r="D71" s="10">
-        <v>46142.00269820602</v>
+        <v>46142.16936487269</v>
       </c>
       <c r="E71" s="11" t="s">
         <v>246</v>
@@ -5752,11 +5752,11 @@
         <v>249</v>
       </c>
       <c r="B72" s="5">
-        <v>46094.46874034722</v>
+        <v>46094.63540701389</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46094.468969849535</v>
+        <v>46094.63563651621</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>250</v>
@@ -5801,11 +5801,11 @@
         <v>252</v>
       </c>
       <c r="B73" s="10">
-        <v>46093.39131126157</v>
+        <v>46093.55797792824</v>
       </c>
       <c r="C73" s="11"/>
       <c r="D73" s="10">
-        <v>46134.52288275463</v>
+        <v>46134.689549421295</v>
       </c>
       <c r="E73" s="11" t="s">
         <v>253</v>
@@ -5858,11 +5858,11 @@
         <v>255</v>
       </c>
       <c r="B74" s="5">
-        <v>46094.483214733795</v>
+        <v>46094.64988140046</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46094.48332144676</v>
+        <v>46094.64998811342</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>256</v>
@@ -5907,11 +5907,11 @@
         <v>258</v>
       </c>
       <c r="B75" s="10">
-        <v>46093.39130847222</v>
+        <v>46093.55797513889</v>
       </c>
       <c r="C75" s="11"/>
       <c r="D75" s="10">
-        <v>46098.45922471065</v>
+        <v>46098.62589137732</v>
       </c>
       <c r="E75" s="11" t="s">
         <v>259</v>
@@ -5966,11 +5966,11 @@
         <v>261</v>
       </c>
       <c r="B76" s="5">
-        <v>46094.39993493055</v>
+        <v>46094.566601597224</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46094.40069871528</v>
+        <v>46094.56736538194</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>262</v>
@@ -6015,11 +6015,11 @@
         <v>264</v>
       </c>
       <c r="B77" s="10">
-        <v>46094.40027128472</v>
+        <v>46094.566937951386</v>
       </c>
       <c r="C77" s="11"/>
       <c r="D77" s="10">
-        <v>46094.40106740741</v>
+        <v>46094.56773407407</v>
       </c>
       <c r="E77" s="11" t="s">
         <v>265</v>
@@ -6064,11 +6064,11 @@
         <v>267</v>
       </c>
       <c r="B78" s="5">
-        <v>46094.40081503472</v>
+        <v>46094.56748170139</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46094.40129219907</v>
+        <v>46094.56795886574</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>268</v>
@@ -6113,11 +6113,11 @@
         <v>270</v>
       </c>
       <c r="B79" s="10">
-        <v>46094.401300011574</v>
+        <v>46094.56796667824</v>
       </c>
       <c r="C79" s="11"/>
       <c r="D79" s="10">
-        <v>46094.40153740741</v>
+        <v>46094.56820407408</v>
       </c>
       <c r="E79" s="11" t="s">
         <v>271</v>
@@ -6162,11 +6162,11 @@
         <v>273</v>
       </c>
       <c r="B80" s="5">
-        <v>46093.39130895834</v>
+        <v>46093.557975625</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46112.67511438657</v>
+        <v>46112.84178105324</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>274</v>
@@ -6221,11 +6221,11 @@
         <v>276</v>
       </c>
       <c r="B81" s="10">
-        <v>46094.40398135417</v>
+        <v>46094.57064802083</v>
       </c>
       <c r="C81" s="11"/>
       <c r="D81" s="10">
-        <v>46094.42353918981</v>
+        <v>46094.59020585648</v>
       </c>
       <c r="E81" s="11" t="s">
         <v>277</v>
@@ -6270,11 +6270,11 @@
         <v>279</v>
       </c>
       <c r="B82" s="5">
-        <v>46094.40676761574</v>
+        <v>46094.57343428241</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46094.42356728009</v>
+        <v>46094.59023394676</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>280</v>
@@ -6319,11 +6319,11 @@
         <v>282</v>
       </c>
       <c r="B83" s="10">
-        <v>46094.40692804398</v>
+        <v>46094.573594710644</v>
       </c>
       <c r="C83" s="11"/>
       <c r="D83" s="10">
-        <v>46094.42359532407</v>
+        <v>46094.59026199074</v>
       </c>
       <c r="E83" s="11" t="s">
         <v>283</v>
@@ -6368,11 +6368,11 @@
         <v>285</v>
       </c>
       <c r="B84" s="5">
-        <v>46094.40707314815</v>
+        <v>46094.57373981482</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46094.42363572917</v>
+        <v>46094.59030239584</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>286</v>
@@ -6417,11 +6417,11 @@
         <v>288</v>
       </c>
       <c r="B85" s="10">
-        <v>46094.40721358796</v>
+        <v>46094.573880254626</v>
       </c>
       <c r="C85" s="11"/>
       <c r="D85" s="10">
-        <v>46094.4236662037</v>
+        <v>46094.59033287037</v>
       </c>
       <c r="E85" s="11" t="s">
         <v>289</v>
@@ -6466,11 +6466,11 @@
         <v>291</v>
       </c>
       <c r="B86" s="5">
-        <v>46093.391310949075</v>
+        <v>46093.55797761574</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46099.465752268516</v>
+        <v>46099.63241893519</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>292</v>
@@ -6523,11 +6523,11 @@
         <v>294</v>
       </c>
       <c r="B87" s="10">
-        <v>46094.483803807874</v>
+        <v>46094.65047047454</v>
       </c>
       <c r="C87" s="11"/>
       <c r="D87" s="10">
-        <v>46111.66943563658</v>
+        <v>46111.83610230324</v>
       </c>
       <c r="E87" s="11" t="s">
         <v>295</v>
@@ -6572,11 +6572,11 @@
         <v>297</v>
       </c>
       <c r="B88" s="5">
-        <v>46094.48406188657</v>
+        <v>46094.65072855324</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46094.48416918982</v>
+        <v>46094.65083585648</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>298</v>
@@ -6621,11 +6621,11 @@
         <v>300</v>
       </c>
       <c r="B89" s="10">
-        <v>46094.48417696759</v>
+        <v>46094.650843634256</v>
       </c>
       <c r="C89" s="11"/>
       <c r="D89" s="10">
-        <v>46094.484524722226</v>
+        <v>46094.65119138889</v>
       </c>
       <c r="E89" s="11" t="s">
         <v>301</v>
@@ -6670,11 +6670,11 @@
         <v>303</v>
       </c>
       <c r="B90" s="5">
-        <v>46094.484286990744</v>
+        <v>46094.65095365741</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46094.48455228009</v>
+        <v>46094.65121894676</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>304</v>
@@ -6719,11 +6719,11 @@
         <v>306</v>
       </c>
       <c r="B91" s="10">
-        <v>46093.39131060185</v>
+        <v>46093.557977268516</v>
       </c>
       <c r="C91" s="11"/>
       <c r="D91" s="10">
-        <v>46099.47254487268</v>
+        <v>46099.639211539354</v>
       </c>
       <c r="E91" s="11" t="s">
         <v>307</v>
@@ -6776,11 +6776,11 @@
         <v>309</v>
       </c>
       <c r="B92" s="5">
-        <v>46094.475925590275</v>
+        <v>46094.64259225695</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46094.476118402774</v>
+        <v>46094.642785069445</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>310</v>
@@ -6825,11 +6825,11 @@
         <v>312</v>
       </c>
       <c r="B93" s="10">
-        <v>46093.39131184028</v>
+        <v>46093.55797850694</v>
       </c>
       <c r="C93" s="11"/>
       <c r="D93" s="10">
-        <v>46099.45819986111</v>
+        <v>46099.62486652778</v>
       </c>
       <c r="E93" s="11" t="s">
         <v>313</v>
@@ -6882,11 +6882,11 @@
         <v>315</v>
       </c>
       <c r="B94" s="5">
-        <v>46094.485353125</v>
+        <v>46094.65201979167</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46094.48547309027</v>
+        <v>46094.652139756945</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>316</v>
@@ -6931,11 +6931,11 @@
         <v>318</v>
       </c>
       <c r="B95" s="10">
-        <v>46093.39131032408</v>
+        <v>46093.55797699074</v>
       </c>
       <c r="C95" s="11"/>
       <c r="D95" s="10">
-        <v>46134.495801909725</v>
+        <v>46134.66246857639</v>
       </c>
       <c r="E95" s="11" t="s">
         <v>319</v>
@@ -6986,11 +6986,11 @@
         <v>321</v>
       </c>
       <c r="B96" s="5">
-        <v>46094.480051342594</v>
+        <v>46094.64671800926</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46094.48015737269</v>
+        <v>46094.64682403935</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>322</v>
@@ -7035,11 +7035,11 @@
         <v>324</v>
       </c>
       <c r="B97" s="10">
-        <v>46093.39131074074</v>
+        <v>46093.55797740741</v>
       </c>
       <c r="C97" s="11"/>
       <c r="D97" s="10">
-        <v>46196.40619525463</v>
+        <v>46196.5728619213</v>
       </c>
       <c r="E97" s="11" t="s">
         <v>325</v>
@@ -7094,11 +7094,11 @@
         <v>327</v>
       </c>
       <c r="B98" s="5">
-        <v>46094.41762021991</v>
+        <v>46094.58428688657</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46094.41827144676</v>
+        <v>46094.584938113425</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>328</v>
@@ -7143,11 +7143,11 @@
         <v>330</v>
       </c>
       <c r="B99" s="10">
-        <v>46094.41780956018</v>
+        <v>46094.58447622685</v>
       </c>
       <c r="C99" s="11"/>
       <c r="D99" s="10">
-        <v>46094.41829931713</v>
+        <v>46094.5849659838</v>
       </c>
       <c r="E99" s="11" t="s">
         <v>331</v>
@@ -7192,11 +7192,11 @@
         <v>333</v>
       </c>
       <c r="B100" s="5">
-        <v>46094.41804420139</v>
+        <v>46094.58471086806</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46094.41832512731</v>
+        <v>46094.58499179398</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>334</v>
@@ -7241,13 +7241,13 @@
         <v>336</v>
       </c>
       <c r="B101" s="10">
-        <v>46093.39130938657</v>
+        <v>46093.55797605324</v>
       </c>
       <c r="C101" s="10">
-        <v>46140.56400518518</v>
+        <v>46140.73067185185</v>
       </c>
       <c r="D101" s="10">
-        <v>46140.56400658565</v>
+        <v>46140.730673252314</v>
       </c>
       <c r="E101" s="11" t="s">
         <v>337</v>
@@ -7300,11 +7300,11 @@
         <v>339</v>
       </c>
       <c r="B102" s="5">
-        <v>46094.47807909722</v>
+        <v>46094.644745763886</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46094.47822538194</v>
+        <v>46094.644892048615</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>340</v>
@@ -7349,11 +7349,11 @@
         <v>342</v>
       </c>
       <c r="B103" s="10">
-        <v>46094.47823179398</v>
+        <v>46094.64489846065</v>
       </c>
       <c r="C103" s="11"/>
       <c r="D103" s="10">
-        <v>46094.47837561343</v>
+        <v>46094.64504228009</v>
       </c>
       <c r="E103" s="11" t="s">
         <v>343</v>
@@ -7398,11 +7398,11 @@
         <v>345</v>
       </c>
       <c r="B104" s="5">
-        <v>46133.635163240746</v>
+        <v>46133.8018299074</v>
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="5">
-        <v>46185.42787950231</v>
+        <v>46185.594546168984</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>346</v>
@@ -7455,11 +7455,11 @@
         <v>348</v>
       </c>
       <c r="B105" s="10">
-        <v>46133.635545428246</v>
+        <v>46133.8022120949</v>
       </c>
       <c r="C105" s="11"/>
       <c r="D105" s="10">
-        <v>46133.635998391204</v>
+        <v>46133.80266505787</v>
       </c>
       <c r="E105" s="11" t="s">
         <v>349</v>
@@ -7504,11 +7504,11 @@
         <v>351</v>
       </c>
       <c r="B106" s="5">
-        <v>46133.63569149305</v>
+        <v>46133.80235815972</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46133.636034270836</v>
+        <v>46133.8027009375</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>352</v>
@@ -7553,11 +7553,11 @@
         <v>354</v>
       </c>
       <c r="B107" s="10">
-        <v>46133.63582138889</v>
+        <v>46133.80248805556</v>
       </c>
       <c r="C107" s="11"/>
       <c r="D107" s="10">
-        <v>46133.63607395833</v>
+        <v>46133.802740625004</v>
       </c>
       <c r="E107" s="11" t="s">
         <v>355</v>
@@ -7602,13 +7602,13 @@
         <v>357</v>
       </c>
       <c r="B108" s="5">
-        <v>46093.39130979167</v>
+        <v>46093.55797645834</v>
       </c>
       <c r="C108" s="5">
-        <v>46162.68825068287</v>
+        <v>46162.85491734954</v>
       </c>
       <c r="D108" s="5">
-        <v>46162.688266620375</v>
+        <v>46162.85493328703</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>358</v>
@@ -7661,13 +7661,13 @@
         <v>360</v>
       </c>
       <c r="B109" s="10">
-        <v>46094.471592835645</v>
+        <v>46094.63825950232</v>
       </c>
       <c r="C109" s="10">
-        <v>46135.86566570602</v>
+        <v>46136.032332372684</v>
       </c>
       <c r="D109" s="10">
-        <v>46135.865686018515</v>
+        <v>46136.032352685186</v>
       </c>
       <c r="E109" s="11" t="s">
         <v>361</v>
@@ -7716,13 +7716,13 @@
         <v>363</v>
       </c>
       <c r="B110" s="5">
-        <v>46094.471750902776</v>
+        <v>46094.63841756944</v>
       </c>
       <c r="C110" s="5">
-        <v>46135.865679166665</v>
+        <v>46136.03234583333</v>
       </c>
       <c r="D110" s="5">
-        <v>46135.86569502315</v>
+        <v>46136.03236168981</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>364</v>
@@ -7771,13 +7771,13 @@
         <v>366</v>
       </c>
       <c r="B111" s="10">
-        <v>46094.471949687504</v>
+        <v>46094.63861635417</v>
       </c>
       <c r="C111" s="10">
-        <v>46135.865691921295</v>
+        <v>46136.03235858797</v>
       </c>
       <c r="D111" s="10">
-        <v>46135.86570789352</v>
+        <v>46136.032374560185</v>
       </c>
       <c r="E111" s="11" t="s">
         <v>367</v>
@@ -7826,13 +7826,13 @@
         <v>369</v>
       </c>
       <c r="B112" s="5">
-        <v>46133.64361054398</v>
+        <v>46133.81027721065</v>
       </c>
       <c r="C112" s="5">
-        <v>46161.746328078705</v>
+        <v>46161.91299474537</v>
       </c>
       <c r="D112" s="5">
-        <v>46161.74634914352</v>
+        <v>46161.91301581018</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>370</v>
@@ -7877,13 +7877,13 @@
         <v>373</v>
       </c>
       <c r="B113" s="10">
-        <v>46133.642986527775</v>
+        <v>46133.80965319445</v>
       </c>
       <c r="C113" s="10">
-        <v>46161.74627729166</v>
+        <v>46161.912943958334</v>
       </c>
       <c r="D113" s="10">
-        <v>46161.74629459491</v>
+        <v>46161.91296126157</v>
       </c>
       <c r="E113" s="11" t="s">
         <v>371</v>
@@ -7936,13 +7936,13 @@
         <v>375</v>
       </c>
       <c r="B114" s="5">
-        <v>46133.62895975694</v>
+        <v>46133.79562642361</v>
       </c>
       <c r="C114" s="5">
-        <v>46161.74608435185</v>
+        <v>46161.91275101852</v>
       </c>
       <c r="D114" s="5">
-        <v>46161.74610462963</v>
+        <v>46161.912771296295</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>376</v>
@@ -7987,13 +7987,13 @@
         <v>379</v>
       </c>
       <c r="B115" s="10">
-        <v>46133.628206203706</v>
+        <v>46133.79487287037</v>
       </c>
       <c r="C115" s="10">
-        <v>46161.746088252316</v>
+        <v>46161.91275491898</v>
       </c>
       <c r="D115" s="10">
-        <v>46161.74610438658</v>
+        <v>46161.91277105324</v>
       </c>
       <c r="E115" s="11" t="s">
         <v>377</v>
@@ -8046,13 +8046,13 @@
         <v>381</v>
       </c>
       <c r="B116" s="5">
-        <v>46133.629160324075</v>
+        <v>46133.79582699074</v>
       </c>
       <c r="C116" s="5">
-        <v>46161.746091180554</v>
+        <v>46161.912757847225</v>
       </c>
       <c r="D116" s="5">
-        <v>46161.74610591435</v>
+        <v>46161.91277258102</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>382</v>
@@ -8097,13 +8097,13 @@
         <v>384</v>
       </c>
       <c r="B117" s="10">
-        <v>46094.47474982639</v>
+        <v>46094.641416493054</v>
       </c>
       <c r="C117" s="10">
-        <v>46161.74575371528</v>
+        <v>46161.912420381945</v>
       </c>
       <c r="D117" s="10">
-        <v>46161.74577292824</v>
+        <v>46161.912439594904</v>
       </c>
       <c r="E117" s="11" t="s">
         <v>385</v>
@@ -8152,13 +8152,13 @@
         <v>388</v>
       </c>
       <c r="B118" s="5">
-        <v>46093.39131034722</v>
+        <v>46093.55797701389</v>
       </c>
       <c r="C118" s="5">
-        <v>46161.745760011574</v>
+        <v>46161.912426678246</v>
       </c>
       <c r="D118" s="5">
-        <v>46161.74577501157</v>
+        <v>46161.91244167824</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>386</v>
@@ -8211,13 +8211,13 @@
         <v>390</v>
       </c>
       <c r="B119" s="10">
-        <v>46094.41602628472</v>
+        <v>46094.582692951386</v>
       </c>
       <c r="C119" s="10">
-        <v>46134.50651302084</v>
+        <v>46134.673179687496</v>
       </c>
       <c r="D119" s="10">
-        <v>46134.50652981481</v>
+        <v>46134.67319648148</v>
       </c>
       <c r="E119" s="11" t="s">
         <v>391</v>
@@ -8264,13 +8264,13 @@
         <v>394</v>
       </c>
       <c r="B120" s="5">
-        <v>46093.39130895834</v>
+        <v>46093.557975625</v>
       </c>
       <c r="C120" s="5">
-        <v>46134.47554357639</v>
+        <v>46134.64221024305</v>
       </c>
       <c r="D120" s="5">
-        <v>46134.49599736111</v>
+        <v>46134.66266402778</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>395</v>
@@ -8317,13 +8317,13 @@
         <v>397</v>
       </c>
       <c r="B121" s="10">
-        <v>46093.39131046296</v>
+        <v>46093.55797712963</v>
       </c>
       <c r="C121" s="10">
-        <v>46134.473207511575</v>
+        <v>46134.63987417824</v>
       </c>
       <c r="D121" s="10">
-        <v>46134.47322237269</v>
+        <v>46134.63988903935</v>
       </c>
       <c r="E121" s="11" t="s">
         <v>392</v>
@@ -8376,13 +8376,13 @@
         <v>399</v>
       </c>
       <c r="B122" s="5">
-        <v>46094.41527780093</v>
+        <v>46094.58194446759</v>
       </c>
       <c r="C122" s="5">
-        <v>46134.47254018519</v>
+        <v>46134.63920685185</v>
       </c>
       <c r="D122" s="5">
-        <v>46134.49657511574</v>
+        <v>46134.66324178241</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>400</v>
@@ -8429,13 +8429,13 @@
         <v>402</v>
       </c>
       <c r="B123" s="10">
-        <v>46094.415486909726</v>
+        <v>46094.58215357639</v>
       </c>
       <c r="C123" s="10">
-        <v>46134.47256253472</v>
+        <v>46134.63922920139</v>
       </c>
       <c r="D123" s="10">
-        <v>46134.49639373843</v>
+        <v>46134.66306040509</v>
       </c>
       <c r="E123" s="11" t="s">
         <v>403</v>
@@ -8482,13 +8482,13 @@
         <v>405</v>
       </c>
       <c r="B124" s="5">
-        <v>46094.41564641204</v>
+        <v>46094.5823130787</v>
       </c>
       <c r="C124" s="5">
-        <v>46134.47256783565</v>
+        <v>46134.63923450232</v>
       </c>
       <c r="D124" s="5">
-        <v>46134.496473101855</v>
+        <v>46134.66313976852</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>406</v>
@@ -8535,13 +8535,13 @@
         <v>408</v>
       </c>
       <c r="B125" s="10">
-        <v>46094.41574372685</v>
+        <v>46094.582410393516</v>
       </c>
       <c r="C125" s="10">
-        <v>46134.47257288195</v>
+        <v>46134.63923954861</v>
       </c>
       <c r="D125" s="10">
-        <v>46134.49632251158</v>
+        <v>46134.662989178236</v>
       </c>
       <c r="E125" s="11" t="s">
         <v>409</v>
@@ -8588,13 +8588,13 @@
         <v>411</v>
       </c>
       <c r="B126" s="5">
-        <v>46094.41587055556</v>
+        <v>46094.58253722222</v>
       </c>
       <c r="C126" s="5">
-        <v>46134.47257902777</v>
+        <v>46134.639245694445</v>
       </c>
       <c r="D126" s="5">
-        <v>46134.4962590162</v>
+        <v>46134.662925682875</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>412</v>
@@ -8641,13 +8641,13 @@
         <v>414</v>
       </c>
       <c r="B127" s="10">
-        <v>46094.41613084491</v>
+        <v>46094.582797511575</v>
       </c>
       <c r="C127" s="10">
-        <v>46134.47258864583</v>
+        <v>46134.639255312504</v>
       </c>
       <c r="D127" s="10">
-        <v>46155.4116539699</v>
+        <v>46155.578320636574</v>
       </c>
       <c r="E127" s="11" t="s">
         <v>415</v>
@@ -8694,13 +8694,13 @@
         <v>417</v>
       </c>
       <c r="B128" s="5">
-        <v>46094.416218425926</v>
+        <v>46094.58288509259</v>
       </c>
       <c r="C128" s="5">
-        <v>46134.47259387732</v>
+        <v>46134.63926054398</v>
       </c>
       <c r="D128" s="5">
-        <v>46134.49612207176</v>
+        <v>46134.662788738424</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>418</v>
@@ -8747,13 +8747,13 @@
         <v>420</v>
       </c>
       <c r="B129" s="10">
-        <v>46094.41639663195</v>
+        <v>46094.58306329861</v>
       </c>
       <c r="C129" s="10">
-        <v>46134.47259942129</v>
+        <v>46134.639266087965</v>
       </c>
       <c r="D129" s="10">
-        <v>46134.49606914352</v>
+        <v>46134.66273581018</v>
       </c>
       <c r="E129" s="11" t="s">
         <v>421</v>
@@ -8800,13 +8800,13 @@
         <v>423</v>
       </c>
       <c r="B130" s="5">
-        <v>46133.62551017361</v>
+        <v>46133.792176840274</v>
       </c>
       <c r="C130" s="5">
-        <v>46134.46938997685</v>
+        <v>46134.63605664352</v>
       </c>
       <c r="D130" s="5">
-        <v>46134.469526307876</v>
+        <v>46134.63619297453</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>424</v>
@@ -8859,11 +8859,11 @@
         <v>428</v>
       </c>
       <c r="B131" s="10">
-        <v>46133.62596824074</v>
+        <v>46133.79263490741</v>
       </c>
       <c r="C131" s="11"/>
       <c r="D131" s="10">
-        <v>46133.62684295139</v>
+        <v>46133.79350961806</v>
       </c>
       <c r="E131" s="11" t="s">
         <v>429</v>
@@ -8908,13 +8908,13 @@
         <v>431</v>
       </c>
       <c r="B132" s="5">
-        <v>46091.42727399306</v>
+        <v>46091.59394065972</v>
       </c>
       <c r="C132" s="5">
-        <v>46133.53927418981</v>
+        <v>46133.70594085648</v>
       </c>
       <c r="D132" s="5">
-        <v>46133.53928864583</v>
+        <v>46133.7059553125</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>432</v>
@@ -8967,11 +8967,11 @@
         <v>434</v>
       </c>
       <c r="B133" s="10">
-        <v>46094.45867290509</v>
+        <v>46094.62533957176</v>
       </c>
       <c r="C133" s="11"/>
       <c r="D133" s="10">
-        <v>46133.53927112269</v>
+        <v>46133.70593778935</v>
       </c>
       <c r="E133" s="11" t="s">
         <v>435</v>
@@ -9016,11 +9016,11 @@
         <v>437</v>
       </c>
       <c r="B134" s="5">
-        <v>46094.45876127315</v>
+        <v>46094.62542793981</v>
       </c>
       <c r="C134" s="6"/>
       <c r="D134" s="5">
-        <v>46133.53927171296</v>
+        <v>46133.70593837963</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>438</v>
@@ -9065,11 +9065,11 @@
         <v>440</v>
       </c>
       <c r="B135" s="10">
-        <v>46094.45947127315</v>
+        <v>46094.62613793982</v>
       </c>
       <c r="C135" s="11"/>
       <c r="D135" s="10">
-        <v>46133.539272106485</v>
+        <v>46133.70593877315</v>
       </c>
       <c r="E135" s="11" t="s">
         <v>441</v>
@@ -9114,11 +9114,11 @@
         <v>443</v>
       </c>
       <c r="B136" s="5">
-        <v>46094.45974203704</v>
+        <v>46094.626408703705</v>
       </c>
       <c r="C136" s="6"/>
       <c r="D136" s="5">
-        <v>46133.53927252315</v>
+        <v>46133.705939189815</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>444</v>
@@ -9163,11 +9163,11 @@
         <v>446</v>
       </c>
       <c r="B137" s="10">
-        <v>46094.45982255787</v>
+        <v>46094.62648922454</v>
       </c>
       <c r="C137" s="11"/>
       <c r="D137" s="10">
-        <v>46133.539272951384</v>
+        <v>46133.705939618056</v>
       </c>
       <c r="E137" s="11" t="s">
         <v>447</v>
@@ -9212,11 +9212,11 @@
         <v>449</v>
       </c>
       <c r="B138" s="5">
-        <v>46094.45994241898</v>
+        <v>46094.62660908565</v>
       </c>
       <c r="C138" s="6"/>
       <c r="D138" s="5">
-        <v>46133.53927328704</v>
+        <v>46133.7059399537</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>450</v>
@@ -9261,11 +9261,11 @@
         <v>452</v>
       </c>
       <c r="B139" s="10">
-        <v>46094.46004679398</v>
+        <v>46094.626713460646</v>
       </c>
       <c r="C139" s="11"/>
       <c r="D139" s="10">
-        <v>46133.53927363426</v>
+        <v>46133.705940300926</v>
       </c>
       <c r="E139" s="11" t="s">
         <v>453</v>
@@ -9310,11 +9310,11 @@
         <v>455</v>
       </c>
       <c r="B140" s="5">
-        <v>46094.46014135417</v>
+        <v>46094.62680802083</v>
       </c>
       <c r="C140" s="6"/>
       <c r="D140" s="5">
-        <v>46133.539273981485</v>
+        <v>46133.70594064815</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>456</v>
@@ -9359,13 +9359,13 @@
         <v>458</v>
       </c>
       <c r="B141" s="10">
-        <v>46093.391309259256</v>
+        <v>46093.55797592593</v>
       </c>
       <c r="C141" s="10">
-        <v>46127.708363391204</v>
+        <v>46127.87503005787</v>
       </c>
       <c r="D141" s="10">
-        <v>46134.49664273148</v>
+        <v>46134.66330939815</v>
       </c>
       <c r="E141" s="11" t="s">
         <v>459</v>
@@ -9412,13 +9412,13 @@
         <v>461</v>
       </c>
       <c r="B142" s="5">
-        <v>46094.46808032408</v>
+        <v>46094.63474699074</v>
       </c>
       <c r="C142" s="5">
-        <v>46127.70834715277</v>
+        <v>46127.875013819445</v>
       </c>
       <c r="D142" s="5">
-        <v>46134.496786250005</v>
+        <v>46134.66345291666</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>462</v>
@@ -9465,13 +9465,13 @@
         <v>464</v>
       </c>
       <c r="B143" s="10">
-        <v>46093.39130944444</v>
+        <v>46093.557976111115</v>
       </c>
       <c r="C143" s="10">
-        <v>46111.66991109954</v>
+        <v>46111.836577766204</v>
       </c>
       <c r="D143" s="10">
-        <v>46111.66992547453</v>
+        <v>46111.836592141204</v>
       </c>
       <c r="E143" s="11" t="s">
         <v>465</v>
@@ -9526,13 +9526,13 @@
         <v>467</v>
       </c>
       <c r="B144" s="5">
-        <v>46094.40905268519</v>
+        <v>46094.57571935185</v>
       </c>
       <c r="C144" s="5">
-        <v>46111.66987857639</v>
+        <v>46111.83654524306</v>
       </c>
       <c r="D144" s="5">
-        <v>46111.66989445602</v>
+        <v>46111.83656112268</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>468</v>
@@ -9577,13 +9577,13 @@
         <v>470</v>
       </c>
       <c r="B145" s="10">
-        <v>46094.4093472338</v>
+        <v>46094.57601390046</v>
       </c>
       <c r="C145" s="10">
-        <v>46111.66989234954</v>
+        <v>46111.8365590162</v>
       </c>
       <c r="D145" s="10">
-        <v>46111.66991091435</v>
+        <v>46111.83657758102</v>
       </c>
       <c r="E145" s="11" t="s">
         <v>471</v>
@@ -9628,13 +9628,13 @@
         <v>473</v>
       </c>
       <c r="B146" s="5">
-        <v>46094.40953752315</v>
+        <v>46094.57620418981</v>
       </c>
       <c r="C146" s="5">
-        <v>46111.6699066088</v>
+        <v>46111.83657327546</v>
       </c>
       <c r="D146" s="5">
-        <v>46111.66992586806</v>
+        <v>46111.83659253472</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>474</v>
@@ -9679,13 +9679,13 @@
         <v>476</v>
       </c>
       <c r="B147" s="10">
-        <v>46093.39130920139</v>
+        <v>46093.557975868054</v>
       </c>
       <c r="C147" s="10">
-        <v>46097.61039002315</v>
+        <v>46097.77705668981</v>
       </c>
       <c r="D147" s="10">
-        <v>46097.61040666667</v>
+        <v>46097.77707333333</v>
       </c>
       <c r="E147" s="11" t="s">
         <v>477</v>
@@ -9738,13 +9738,13 @@
         <v>479</v>
       </c>
       <c r="B148" s="5">
-        <v>46094.40786840278</v>
+        <v>46094.57453506945</v>
       </c>
       <c r="C148" s="5">
-        <v>46097.61037094907</v>
+        <v>46097.77703761574</v>
       </c>
       <c r="D148" s="5">
-        <v>46097.61038972222</v>
+        <v>46097.77705638889</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>480</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-30 15:36 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1779" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1802" uniqueCount="488">
   <si>
     <t>Tablero Servicios y mantención</t>
   </si>
@@ -452,6 +452,24 @@
   </si>
   <si>
     <t>TABL3-277</t>
+  </si>
+  <si>
+    <t>1216153465899953</t>
+  </si>
+  <si>
+    <t>50001568</t>
+  </si>
+  <si>
+    <t>TABL3-282</t>
+  </si>
+  <si>
+    <t>1216153465899956</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4366 -SENSOR DE BOMBEO PREMASGARD DS-205F </t>
+  </si>
+  <si>
+    <t>TABL3-283</t>
   </si>
   <si>
     <t>1214150417415442</t>
@@ -2042,7 +2060,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U148"/>
+  <dimension ref="A1:U150"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -4003,17 +4021,17 @@
         <v>145</v>
       </c>
       <c r="B39" s="10">
-        <v>46133.79734877315</v>
+        <v>46203.64108105324</v>
       </c>
       <c r="C39" s="11"/>
       <c r="D39" s="10">
-        <v>46141.74131788194</v>
+        <v>46203.641200439815</v>
       </c>
       <c r="E39" s="11" t="s">
         <v>146</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>147</v>
+        <v>25</v>
       </c>
       <c r="G39" s="11" t="s">
         <v>57</v>
@@ -4022,9 +4040,7 @@
         <v>58</v>
       </c>
       <c r="I39" s="11"/>
-      <c r="J39" s="10">
-        <v>46120</v>
-      </c>
+      <c r="J39" s="11"/>
       <c r="K39" s="11" t="s">
         <v>28</v>
       </c>
@@ -4044,30 +4060,26 @@
         <v>28</v>
       </c>
       <c r="Q39" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="R39" s="11"/>
-      <c r="S39" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T39" s="17" t="s">
-        <v>128</v>
-      </c>
+      <c r="S39" s="11"/>
+      <c r="T39" s="11"/>
       <c r="U39" s="11"/>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46133.79847596065</v>
+        <v>46203.64119756944</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46134.65975528935</v>
+        <v>46203.641513877315</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>28</v>
@@ -4077,7 +4089,9 @@
       </c>
       <c r="H40" s="6"/>
       <c r="I40" s="6"/>
-      <c r="J40" s="6"/>
+      <c r="J40" s="5">
+        <v>46206</v>
+      </c>
       <c r="K40" s="6" t="s">
         <v>28</v>
       </c>
@@ -4097,7 +4111,7 @@
         <v>28</v>
       </c>
       <c r="Q40" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="R40" s="6"/>
       <c r="S40" s="6"/>
@@ -4106,20 +4120,20 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B41" s="10">
-        <v>46133.800000937495</v>
+        <v>46133.79734877315</v>
       </c>
       <c r="C41" s="11"/>
       <c r="D41" s="10">
-        <v>46141.74254248843</v>
+        <v>46141.74131788194</v>
       </c>
       <c r="E41" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="F41" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="F41" s="11" t="s">
-        <v>147</v>
       </c>
       <c r="G41" s="11" t="s">
         <v>57</v>
@@ -4129,7 +4143,7 @@
       </c>
       <c r="I41" s="11"/>
       <c r="J41" s="10">
-        <v>46234</v>
+        <v>46120</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>28</v>
@@ -4153,8 +4167,8 @@
         <v>154</v>
       </c>
       <c r="R41" s="11"/>
-      <c r="S41" s="14" t="s">
-        <v>51</v>
+      <c r="S41" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="T41" s="17" t="s">
         <v>128</v>
@@ -4166,11 +4180,11 @@
         <v>155</v>
       </c>
       <c r="B42" s="5">
-        <v>46133.800366041665</v>
+        <v>46133.79847596065</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46133.800594699074</v>
+        <v>46134.65975528935</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>156</v>
@@ -4194,7 +4208,7 @@
         <v>28</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>28</v>
@@ -4215,17 +4229,17 @@
         <v>158</v>
       </c>
       <c r="B43" s="10">
-        <v>46093.55797671297</v>
+        <v>46133.800000937495</v>
       </c>
       <c r="C43" s="11"/>
       <c r="D43" s="10">
-        <v>46195.57757945602</v>
+        <v>46141.74254248843</v>
       </c>
       <c r="E43" s="11" t="s">
         <v>159</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="G43" s="11" t="s">
         <v>57</v>
@@ -4233,11 +4247,9 @@
       <c r="H43" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I43" s="10">
-        <v>46129</v>
-      </c>
+      <c r="I43" s="11"/>
       <c r="J43" s="10">
-        <v>46129</v>
+        <v>46234</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>28</v>
@@ -4258,30 +4270,30 @@
         <v>28</v>
       </c>
       <c r="Q43" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R43" s="11"/>
-      <c r="S43" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T43" s="16" t="s">
-        <v>115</v>
+      <c r="S43" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="T43" s="17" t="s">
+        <v>128</v>
       </c>
       <c r="U43" s="11"/>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B44" s="5">
-        <v>46094.639967870375</v>
+        <v>46133.800366041665</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46130.18563101852</v>
+        <v>46133.800594699074</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>28</v>
@@ -4291,9 +4303,7 @@
       </c>
       <c r="H44" s="6"/>
       <c r="I44" s="6"/>
-      <c r="J44" s="5">
-        <v>46129</v>
-      </c>
+      <c r="J44" s="6"/>
       <c r="K44" s="6" t="s">
         <v>28</v>
       </c>
@@ -4313,39 +4323,41 @@
         <v>28</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R44" s="6"/>
-      <c r="S44" s="12" t="s">
-        <v>43</v>
-      </c>
+      <c r="S44" s="6"/>
       <c r="T44" s="6"/>
       <c r="U44" s="6"/>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B45" s="10">
-        <v>46094.64022527778</v>
+        <v>46093.55797671297</v>
       </c>
       <c r="C45" s="11"/>
       <c r="D45" s="10">
-        <v>46101.15093898148</v>
+        <v>46195.57757945602</v>
       </c>
       <c r="E45" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F45" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="F45" s="11" t="s">
-        <v>28</v>
-      </c>
       <c r="G45" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H45" s="11"/>
-      <c r="I45" s="11"/>
+        <v>57</v>
+      </c>
+      <c r="H45" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="I45" s="10">
+        <v>46129</v>
+      </c>
       <c r="J45" s="10">
-        <v>46100</v>
+        <v>46129</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>28</v>
@@ -4354,10 +4366,10 @@
         <v>28</v>
       </c>
       <c r="M45" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N45" s="11" t="s">
-        <v>159</v>
+        <v>28</v>
       </c>
       <c r="O45" s="11" t="s">
         <v>28</v>
@@ -4372,7 +4384,9 @@
       <c r="S45" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T45" s="11"/>
+      <c r="T45" s="16" t="s">
+        <v>115</v>
+      </c>
       <c r="U45" s="11"/>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
@@ -4380,27 +4394,25 @@
         <v>168</v>
       </c>
       <c r="B46" s="5">
-        <v>46133.81046972222</v>
+        <v>46094.639967870375</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46162.79059445602</v>
+        <v>46130.18563101852</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>169</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H46" s="6"/>
       <c r="I46" s="6"/>
       <c r="J46" s="5">
-        <v>46140</v>
+        <v>46129</v>
       </c>
       <c r="K46" s="6" t="s">
         <v>28</v>
@@ -4409,10 +4421,10 @@
         <v>28</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>28</v>
+        <v>165</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>28</v>
@@ -4424,12 +4436,10 @@
         <v>170</v>
       </c>
       <c r="R46" s="6"/>
-      <c r="S46" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="T46" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="S46" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T46" s="6"/>
       <c r="U46" s="6"/>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
@@ -4437,11 +4447,11 @@
         <v>171</v>
       </c>
       <c r="B47" s="10">
-        <v>46133.8107147338</v>
+        <v>46094.64022527778</v>
       </c>
       <c r="C47" s="11"/>
       <c r="D47" s="10">
-        <v>46133.81087918981</v>
+        <v>46101.15093898148</v>
       </c>
       <c r="E47" s="11" t="s">
         <v>172</v>
@@ -4454,7 +4464,9 @@
       </c>
       <c r="H47" s="11"/>
       <c r="I47" s="11"/>
-      <c r="J47" s="11"/>
+      <c r="J47" s="10">
+        <v>46100</v>
+      </c>
       <c r="K47" s="11" t="s">
         <v>28</v>
       </c>
@@ -4465,7 +4477,7 @@
         <v>28</v>
       </c>
       <c r="N47" s="11" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="O47" s="11" t="s">
         <v>28</v>
@@ -4477,7 +4489,9 @@
         <v>173</v>
       </c>
       <c r="R47" s="11"/>
-      <c r="S47" s="11"/>
+      <c r="S47" s="12" t="s">
+        <v>43</v>
+      </c>
       <c r="T47" s="11"/>
       <c r="U47" s="11"/>
     </row>
@@ -4486,17 +4500,17 @@
         <v>174</v>
       </c>
       <c r="B48" s="5">
-        <v>46133.80470612268</v>
+        <v>46133.81046972222</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46196.91581209491</v>
+        <v>46162.79059445602</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>175</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G48" s="6" t="s">
         <v>57</v>
@@ -4506,7 +4520,7 @@
       </c>
       <c r="I48" s="6"/>
       <c r="J48" s="5">
-        <v>46161</v>
+        <v>46140</v>
       </c>
       <c r="K48" s="6" t="s">
         <v>28</v>
@@ -4530,8 +4544,8 @@
         <v>176</v>
       </c>
       <c r="R48" s="6"/>
-      <c r="S48" s="12" t="s">
-        <v>43</v>
+      <c r="S48" s="14" t="s">
+        <v>51</v>
       </c>
       <c r="T48" s="15" t="s">
         <v>72</v>
@@ -4543,11 +4557,11 @@
         <v>177</v>
       </c>
       <c r="B49" s="10">
-        <v>46133.80545771991</v>
+        <v>46133.8107147338</v>
       </c>
       <c r="C49" s="11"/>
       <c r="D49" s="10">
-        <v>46133.80564510416</v>
+        <v>46133.81087918981</v>
       </c>
       <c r="E49" s="11" t="s">
         <v>178</v>
@@ -4592,24 +4606,28 @@
         <v>180</v>
       </c>
       <c r="B50" s="5">
-        <v>46133.80570512731</v>
+        <v>46133.80470612268</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46133.80583366899</v>
+        <v>46196.91581209491</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>181</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>28</v>
+        <v>166</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H50" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I50" s="6"/>
-      <c r="J50" s="6"/>
+      <c r="J50" s="5">
+        <v>46161</v>
+      </c>
       <c r="K50" s="6" t="s">
         <v>28</v>
       </c>
@@ -4617,10 +4635,10 @@
         <v>28</v>
       </c>
       <c r="M50" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>175</v>
+        <v>28</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>28</v>
@@ -4632,8 +4650,12 @@
         <v>182</v>
       </c>
       <c r="R50" s="6"/>
-      <c r="S50" s="6"/>
-      <c r="T50" s="6"/>
+      <c r="S50" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T50" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U50" s="6"/>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4641,11 +4663,11 @@
         <v>183</v>
       </c>
       <c r="B51" s="10">
-        <v>46133.8058850463</v>
+        <v>46133.80545771991</v>
       </c>
       <c r="C51" s="11"/>
       <c r="D51" s="10">
-        <v>46133.80636234954</v>
+        <v>46133.80564510416</v>
       </c>
       <c r="E51" s="11" t="s">
         <v>184</v>
@@ -4669,7 +4691,7 @@
         <v>28</v>
       </c>
       <c r="N51" s="11" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="O51" s="11" t="s">
         <v>28</v>
@@ -4690,11 +4712,11 @@
         <v>186</v>
       </c>
       <c r="B52" s="5">
-        <v>46133.80664880787</v>
+        <v>46133.80570512731</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46133.80681135417</v>
+        <v>46133.80583366899</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>187</v>
@@ -4718,7 +4740,7 @@
         <v>28</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>28</v>
@@ -4739,69 +4761,63 @@
         <v>189</v>
       </c>
       <c r="B53" s="10">
-        <v>46133.80701400463</v>
+        <v>46133.8058850463</v>
       </c>
       <c r="C53" s="11"/>
       <c r="D53" s="10">
-        <v>46162.79057355324</v>
+        <v>46133.80636234954</v>
       </c>
       <c r="E53" s="11" t="s">
         <v>190</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="G53" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H53" s="11" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H53" s="11"/>
       <c r="I53" s="11"/>
-      <c r="J53" s="10">
-        <v>46122</v>
-      </c>
+      <c r="J53" s="11"/>
       <c r="K53" s="11" t="s">
         <v>28</v>
       </c>
       <c r="L53" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="M53" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="N53" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="O53" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="P53" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q53" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="M53" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="N53" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="O53" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="P53" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q53" s="11" t="s">
-        <v>192</v>
-      </c>
       <c r="R53" s="11"/>
-      <c r="S53" s="12" t="s">
-        <v>43</v>
-      </c>
+      <c r="S53" s="11"/>
       <c r="T53" s="11"/>
       <c r="U53" s="11"/>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B54" s="5">
-        <v>46133.80727017361</v>
+        <v>46133.80664880787</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46133.80736961805</v>
+        <v>46133.80681135417</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>28</v>
@@ -4822,7 +4838,7 @@
         <v>28</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>28</v>
@@ -4831,7 +4847,7 @@
         <v>28</v>
       </c>
       <c r="Q54" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="R54" s="6"/>
       <c r="S54" s="6"/>
@@ -4840,20 +4856,20 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B55" s="10">
-        <v>46133.79901350694</v>
+        <v>46133.80701400463</v>
       </c>
       <c r="C55" s="11"/>
       <c r="D55" s="10">
-        <v>46162.79056252315</v>
+        <v>46162.79057355324</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G55" s="11" t="s">
         <v>57</v>
@@ -4863,13 +4879,13 @@
       </c>
       <c r="I55" s="11"/>
       <c r="J55" s="10">
-        <v>46120</v>
+        <v>46122</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>28</v>
       </c>
       <c r="L55" s="11" t="s">
-        <v>28</v>
+        <v>197</v>
       </c>
       <c r="M55" s="11" t="s">
         <v>0</v>
@@ -4890,9 +4906,7 @@
       <c r="S55" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T55" s="17" t="s">
-        <v>128</v>
-      </c>
+      <c r="T55" s="11"/>
       <c r="U55" s="11"/>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
@@ -4900,11 +4914,11 @@
         <v>199</v>
       </c>
       <c r="B56" s="5">
-        <v>46133.79961443287</v>
+        <v>46133.80727017361</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46133.79989851852</v>
+        <v>46133.80736961805</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>200</v>
@@ -4928,7 +4942,7 @@
         <v>28</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>28</v>
@@ -4949,17 +4963,17 @@
         <v>202</v>
       </c>
       <c r="B57" s="10">
-        <v>46093.557977812496</v>
+        <v>46133.79901350694</v>
       </c>
       <c r="C57" s="11"/>
       <c r="D57" s="10">
-        <v>46162.79054756944</v>
+        <v>46162.79056252315</v>
       </c>
       <c r="E57" s="11" t="s">
         <v>203</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G57" s="11" t="s">
         <v>57</v>
@@ -4969,7 +4983,7 @@
       </c>
       <c r="I57" s="11"/>
       <c r="J57" s="10">
-        <v>46039</v>
+        <v>46120</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>28</v>
@@ -4996,8 +5010,8 @@
       <c r="S57" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T57" s="15" t="s">
-        <v>72</v>
+      <c r="T57" s="17" t="s">
+        <v>128</v>
       </c>
       <c r="U57" s="11"/>
     </row>
@@ -5006,11 +5020,11 @@
         <v>205</v>
       </c>
       <c r="B58" s="5">
-        <v>46094.64358574074</v>
+        <v>46133.79961443287</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46094.643782430554</v>
+        <v>46133.79989851852</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>206</v>
@@ -5055,17 +5069,17 @@
         <v>208</v>
       </c>
       <c r="B59" s="10">
-        <v>46093.55797666666</v>
+        <v>46093.557977812496</v>
       </c>
       <c r="C59" s="11"/>
       <c r="D59" s="10">
-        <v>46162.790523668984</v>
+        <v>46162.79054756944</v>
       </c>
       <c r="E59" s="11" t="s">
         <v>209</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G59" s="11" t="s">
         <v>57</v>
@@ -5075,7 +5089,7 @@
       </c>
       <c r="I59" s="11"/>
       <c r="J59" s="10">
-        <v>46083</v>
+        <v>46039</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>28</v>
@@ -5112,11 +5126,11 @@
         <v>211</v>
       </c>
       <c r="B60" s="5">
-        <v>46094.64611630787</v>
+        <v>46094.64358574074</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46094.64631732639</v>
+        <v>46094.643782430554</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>212</v>
@@ -5161,24 +5175,28 @@
         <v>214</v>
       </c>
       <c r="B61" s="10">
-        <v>46094.64632454861</v>
+        <v>46093.55797666666</v>
       </c>
       <c r="C61" s="11"/>
       <c r="D61" s="10">
-        <v>46094.64655788195</v>
+        <v>46162.790523668984</v>
       </c>
       <c r="E61" s="11" t="s">
         <v>215</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>28</v>
+        <v>166</v>
       </c>
       <c r="G61" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H61" s="11"/>
+        <v>57</v>
+      </c>
+      <c r="H61" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="I61" s="11"/>
-      <c r="J61" s="11"/>
+      <c r="J61" s="10">
+        <v>46083</v>
+      </c>
       <c r="K61" s="11" t="s">
         <v>28</v>
       </c>
@@ -5186,10 +5204,10 @@
         <v>28</v>
       </c>
       <c r="M61" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N61" s="11" t="s">
-        <v>209</v>
+        <v>28</v>
       </c>
       <c r="O61" s="11" t="s">
         <v>28</v>
@@ -5201,8 +5219,12 @@
         <v>216</v>
       </c>
       <c r="R61" s="11"/>
-      <c r="S61" s="11"/>
-      <c r="T61" s="11"/>
+      <c r="S61" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T61" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U61" s="11"/>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5210,28 +5232,24 @@
         <v>217</v>
       </c>
       <c r="B62" s="5">
-        <v>46093.55797637731</v>
+        <v>46094.64611630787</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46162.79050667824</v>
+        <v>46094.64631732639</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>218</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H62" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H62" s="6"/>
       <c r="I62" s="6"/>
-      <c r="J62" s="5">
-        <v>46080</v>
-      </c>
+      <c r="J62" s="6"/>
       <c r="K62" s="6" t="s">
         <v>28</v>
       </c>
@@ -5239,10 +5257,10 @@
         <v>28</v>
       </c>
       <c r="M62" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>28</v>
+        <v>215</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>28</v>
@@ -5254,12 +5272,8 @@
         <v>219</v>
       </c>
       <c r="R62" s="6"/>
-      <c r="S62" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T62" s="17" t="s">
-        <v>128</v>
-      </c>
+      <c r="S62" s="6"/>
+      <c r="T62" s="6"/>
       <c r="U62" s="6"/>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -5267,11 +5281,11 @@
         <v>220</v>
       </c>
       <c r="B63" s="10">
-        <v>46094.645434618054</v>
+        <v>46094.64632454861</v>
       </c>
       <c r="C63" s="11"/>
       <c r="D63" s="10">
-        <v>46094.645602916666</v>
+        <v>46094.64655788195</v>
       </c>
       <c r="E63" s="11" t="s">
         <v>221</v>
@@ -5295,7 +5309,7 @@
         <v>28</v>
       </c>
       <c r="N63" s="11" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="O63" s="11" t="s">
         <v>28</v>
@@ -5316,17 +5330,17 @@
         <v>223</v>
       </c>
       <c r="B64" s="5">
-        <v>46093.55797821759</v>
+        <v>46093.55797637731</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46162.79049341435</v>
+        <v>46162.79050667824</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>224</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G64" s="6" t="s">
         <v>57</v>
@@ -5336,7 +5350,7 @@
       </c>
       <c r="I64" s="6"/>
       <c r="J64" s="5">
-        <v>46092</v>
+        <v>46080</v>
       </c>
       <c r="K64" s="6" t="s">
         <v>28</v>
@@ -5363,8 +5377,8 @@
       <c r="S64" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T64" s="15" t="s">
-        <v>72</v>
+      <c r="T64" s="17" t="s">
+        <v>128</v>
       </c>
       <c r="U64" s="6"/>
     </row>
@@ -5373,11 +5387,11 @@
         <v>226</v>
       </c>
       <c r="B65" s="10">
-        <v>46094.65140127315</v>
+        <v>46094.645434618054</v>
       </c>
       <c r="C65" s="11"/>
       <c r="D65" s="10">
-        <v>46094.65150827546</v>
+        <v>46094.645602916666</v>
       </c>
       <c r="E65" s="11" t="s">
         <v>227</v>
@@ -5422,17 +5436,17 @@
         <v>229</v>
       </c>
       <c r="B66" s="5">
-        <v>46093.557976192125</v>
+        <v>46093.55797821759</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46142.16936487269</v>
+        <v>46162.79049341435</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>230</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G66" s="6" t="s">
         <v>57</v>
@@ -5442,7 +5456,7 @@
       </c>
       <c r="I66" s="6"/>
       <c r="J66" s="5">
-        <v>46142</v>
+        <v>46092</v>
       </c>
       <c r="K66" s="6" t="s">
         <v>28</v>
@@ -5466,27 +5480,27 @@
         <v>231</v>
       </c>
       <c r="R66" s="6"/>
-      <c r="S66" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T66" s="17" t="s">
-        <v>232</v>
+      <c r="S66" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T66" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="U66" s="6"/>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B67" s="10">
-        <v>46094.63540701389</v>
+        <v>46094.65140127315</v>
       </c>
       <c r="C67" s="11"/>
       <c r="D67" s="10">
-        <v>46094.63563651621</v>
+        <v>46094.65150827546</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F67" s="11" t="s">
         <v>28</v>
@@ -5516,7 +5530,7 @@
         <v>28</v>
       </c>
       <c r="Q67" s="11" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R67" s="11"/>
       <c r="S67" s="11"/>
@@ -5525,30 +5539,30 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B68" s="5">
-        <v>46093.55797792824</v>
+        <v>46093.557976192125</v>
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46134.689549421295</v>
+        <v>46142.16936487269</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="I68" s="6"/>
       <c r="J68" s="5">
-        <v>46097</v>
+        <v>46142</v>
       </c>
       <c r="K68" s="6" t="s">
         <v>28</v>
@@ -5569,14 +5583,14 @@
         <v>28</v>
       </c>
       <c r="Q68" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="R68" s="6"/>
+      <c r="S68" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T68" s="17" t="s">
         <v>238</v>
-      </c>
-      <c r="R68" s="6"/>
-      <c r="S68" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T68" s="15" t="s">
-        <v>72</v>
       </c>
       <c r="U68" s="6"/>
     </row>
@@ -5585,11 +5599,11 @@
         <v>239</v>
       </c>
       <c r="B69" s="10">
-        <v>46094.64988140046</v>
+        <v>46094.63540701389</v>
       </c>
       <c r="C69" s="11"/>
       <c r="D69" s="10">
-        <v>46094.64998811342</v>
+        <v>46094.63563651621</v>
       </c>
       <c r="E69" s="11" t="s">
         <v>240</v>
@@ -5613,7 +5627,7 @@
         <v>28</v>
       </c>
       <c r="N69" s="11" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="O69" s="11" t="s">
         <v>28</v>
@@ -5634,17 +5648,17 @@
         <v>242</v>
       </c>
       <c r="B70" s="5">
-        <v>46093.55797513889</v>
+        <v>46093.55797792824</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46098.62589137732</v>
+        <v>46134.689549421295</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>243</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G70" s="6" t="s">
         <v>26</v>
@@ -5652,11 +5666,9 @@
       <c r="H70" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="I70" s="5">
-        <v>46041</v>
-      </c>
+      <c r="I70" s="6"/>
       <c r="J70" s="5">
-        <v>46041</v>
+        <v>46097</v>
       </c>
       <c r="K70" s="6" t="s">
         <v>28</v>
@@ -5683,8 +5695,8 @@
       <c r="S70" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T70" s="17" t="s">
-        <v>232</v>
+      <c r="T70" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="U70" s="6"/>
     </row>
@@ -5693,11 +5705,11 @@
         <v>245</v>
       </c>
       <c r="B71" s="10">
-        <v>46094.566601597224</v>
+        <v>46094.64988140046</v>
       </c>
       <c r="C71" s="11"/>
       <c r="D71" s="10">
-        <v>46094.56736538194</v>
+        <v>46094.64998811342</v>
       </c>
       <c r="E71" s="11" t="s">
         <v>246</v>
@@ -5742,24 +5754,30 @@
         <v>248</v>
       </c>
       <c r="B72" s="5">
-        <v>46094.566937951386</v>
+        <v>46093.55797513889</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46094.56773407407</v>
+        <v>46098.62589137732</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>249</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>28</v>
+        <v>166</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H72" s="6"/>
-      <c r="I72" s="6"/>
-      <c r="J72" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I72" s="5">
+        <v>46041</v>
+      </c>
+      <c r="J72" s="5">
+        <v>46041</v>
+      </c>
       <c r="K72" s="6" t="s">
         <v>28</v>
       </c>
@@ -5767,10 +5785,10 @@
         <v>28</v>
       </c>
       <c r="M72" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>243</v>
+        <v>28</v>
       </c>
       <c r="O72" s="6" t="s">
         <v>28</v>
@@ -5782,8 +5800,12 @@
         <v>250</v>
       </c>
       <c r="R72" s="6"/>
-      <c r="S72" s="6"/>
-      <c r="T72" s="6"/>
+      <c r="S72" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T72" s="17" t="s">
+        <v>238</v>
+      </c>
       <c r="U72" s="6"/>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5791,11 +5813,11 @@
         <v>251</v>
       </c>
       <c r="B73" s="10">
-        <v>46094.56748170139</v>
+        <v>46094.566601597224</v>
       </c>
       <c r="C73" s="11"/>
       <c r="D73" s="10">
-        <v>46094.56795886574</v>
+        <v>46094.56736538194</v>
       </c>
       <c r="E73" s="11" t="s">
         <v>252</v>
@@ -5819,7 +5841,7 @@
         <v>28</v>
       </c>
       <c r="N73" s="11" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="O73" s="11" t="s">
         <v>28</v>
@@ -5840,11 +5862,11 @@
         <v>254</v>
       </c>
       <c r="B74" s="5">
-        <v>46094.56796667824</v>
+        <v>46094.566937951386</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46094.56820407408</v>
+        <v>46094.56773407407</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>255</v>
@@ -5868,7 +5890,7 @@
         <v>28</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="O74" s="6" t="s">
         <v>28</v>
@@ -5889,30 +5911,24 @@
         <v>257</v>
       </c>
       <c r="B75" s="10">
-        <v>46093.557975625</v>
+        <v>46094.56748170139</v>
       </c>
       <c r="C75" s="11"/>
       <c r="D75" s="10">
-        <v>46112.84178105324</v>
+        <v>46094.56795886574</v>
       </c>
       <c r="E75" s="11" t="s">
         <v>258</v>
       </c>
       <c r="F75" s="11" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H75" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="I75" s="10">
-        <v>46041</v>
-      </c>
-      <c r="J75" s="10">
-        <v>46041</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H75" s="11"/>
+      <c r="I75" s="11"/>
+      <c r="J75" s="11"/>
       <c r="K75" s="11" t="s">
         <v>28</v>
       </c>
@@ -5920,10 +5936,10 @@
         <v>28</v>
       </c>
       <c r="M75" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N75" s="11" t="s">
-        <v>28</v>
+        <v>249</v>
       </c>
       <c r="O75" s="11" t="s">
         <v>28</v>
@@ -5935,12 +5951,8 @@
         <v>259</v>
       </c>
       <c r="R75" s="11"/>
-      <c r="S75" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T75" s="17" t="s">
-        <v>232</v>
-      </c>
+      <c r="S75" s="11"/>
+      <c r="T75" s="11"/>
       <c r="U75" s="11"/>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -5948,11 +5960,11 @@
         <v>260</v>
       </c>
       <c r="B76" s="5">
-        <v>46094.57064802083</v>
+        <v>46094.56796667824</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46094.59020585648</v>
+        <v>46094.56820407408</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>261</v>
@@ -5976,7 +5988,7 @@
         <v>28</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="O76" s="6" t="s">
         <v>28</v>
@@ -5997,24 +6009,30 @@
         <v>263</v>
       </c>
       <c r="B77" s="10">
-        <v>46094.57343428241</v>
+        <v>46093.557975625</v>
       </c>
       <c r="C77" s="11"/>
       <c r="D77" s="10">
-        <v>46094.59023394676</v>
+        <v>46112.84178105324</v>
       </c>
       <c r="E77" s="11" t="s">
         <v>264</v>
       </c>
       <c r="F77" s="11" t="s">
-        <v>28</v>
+        <v>166</v>
       </c>
       <c r="G77" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H77" s="11"/>
-      <c r="I77" s="11"/>
-      <c r="J77" s="11"/>
+        <v>26</v>
+      </c>
+      <c r="H77" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I77" s="10">
+        <v>46041</v>
+      </c>
+      <c r="J77" s="10">
+        <v>46041</v>
+      </c>
       <c r="K77" s="11" t="s">
         <v>28</v>
       </c>
@@ -6022,10 +6040,10 @@
         <v>28</v>
       </c>
       <c r="M77" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N77" s="11" t="s">
-        <v>258</v>
+        <v>28</v>
       </c>
       <c r="O77" s="11" t="s">
         <v>28</v>
@@ -6037,8 +6055,12 @@
         <v>265</v>
       </c>
       <c r="R77" s="11"/>
-      <c r="S77" s="11"/>
-      <c r="T77" s="11"/>
+      <c r="S77" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T77" s="17" t="s">
+        <v>238</v>
+      </c>
       <c r="U77" s="11"/>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
@@ -6046,11 +6068,11 @@
         <v>266</v>
       </c>
       <c r="B78" s="5">
-        <v>46094.573594710644</v>
+        <v>46094.57064802083</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46094.59026199074</v>
+        <v>46094.59020585648</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>267</v>
@@ -6074,7 +6096,7 @@
         <v>28</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="O78" s="6" t="s">
         <v>28</v>
@@ -6095,11 +6117,11 @@
         <v>269</v>
       </c>
       <c r="B79" s="10">
-        <v>46094.57373981482</v>
+        <v>46094.57343428241</v>
       </c>
       <c r="C79" s="11"/>
       <c r="D79" s="10">
-        <v>46094.59030239584</v>
+        <v>46094.59023394676</v>
       </c>
       <c r="E79" s="11" t="s">
         <v>270</v>
@@ -6123,7 +6145,7 @@
         <v>28</v>
       </c>
       <c r="N79" s="11" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="O79" s="11" t="s">
         <v>28</v>
@@ -6144,11 +6166,11 @@
         <v>272</v>
       </c>
       <c r="B80" s="5">
-        <v>46094.573880254626</v>
+        <v>46094.573594710644</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46094.59033287037</v>
+        <v>46094.59026199074</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>273</v>
@@ -6172,7 +6194,7 @@
         <v>28</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="O80" s="6" t="s">
         <v>28</v>
@@ -6193,28 +6215,24 @@
         <v>275</v>
       </c>
       <c r="B81" s="10">
-        <v>46093.55797761574</v>
+        <v>46094.57373981482</v>
       </c>
       <c r="C81" s="11"/>
       <c r="D81" s="10">
-        <v>46099.63241893519</v>
+        <v>46094.59030239584</v>
       </c>
       <c r="E81" s="11" t="s">
         <v>276</v>
       </c>
       <c r="F81" s="11" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="G81" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H81" s="11" t="s">
-        <v>27</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H81" s="11"/>
       <c r="I81" s="11"/>
-      <c r="J81" s="10">
-        <v>46092</v>
-      </c>
+      <c r="J81" s="11"/>
       <c r="K81" s="11" t="s">
         <v>28</v>
       </c>
@@ -6222,10 +6240,10 @@
         <v>28</v>
       </c>
       <c r="M81" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N81" s="11" t="s">
-        <v>28</v>
+        <v>264</v>
       </c>
       <c r="O81" s="11" t="s">
         <v>28</v>
@@ -6237,12 +6255,8 @@
         <v>277</v>
       </c>
       <c r="R81" s="11"/>
-      <c r="S81" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T81" s="17" t="s">
-        <v>232</v>
-      </c>
+      <c r="S81" s="11"/>
+      <c r="T81" s="11"/>
       <c r="U81" s="11"/>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -6250,17 +6264,17 @@
         <v>278</v>
       </c>
       <c r="B82" s="5">
-        <v>46094.65047047454</v>
+        <v>46094.573880254626</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46111.83610230324</v>
+        <v>46094.59033287037</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>279</v>
       </c>
       <c r="F82" s="6" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G82" s="6" t="s">
         <v>28</v>
@@ -6275,10 +6289,10 @@
         <v>28</v>
       </c>
       <c r="M82" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="O82" s="6" t="s">
         <v>28</v>
@@ -6299,24 +6313,28 @@
         <v>281</v>
       </c>
       <c r="B83" s="10">
-        <v>46094.65072855324</v>
+        <v>46093.55797761574</v>
       </c>
       <c r="C83" s="11"/>
       <c r="D83" s="10">
-        <v>46094.65083585648</v>
+        <v>46099.63241893519</v>
       </c>
       <c r="E83" s="11" t="s">
         <v>282</v>
       </c>
       <c r="F83" s="11" t="s">
-        <v>28</v>
+        <v>166</v>
       </c>
       <c r="G83" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H83" s="11"/>
+        <v>26</v>
+      </c>
+      <c r="H83" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="I83" s="11"/>
-      <c r="J83" s="11"/>
+      <c r="J83" s="10">
+        <v>46092</v>
+      </c>
       <c r="K83" s="11" t="s">
         <v>28</v>
       </c>
@@ -6324,10 +6342,10 @@
         <v>28</v>
       </c>
       <c r="M83" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N83" s="11" t="s">
-        <v>276</v>
+        <v>28</v>
       </c>
       <c r="O83" s="11" t="s">
         <v>28</v>
@@ -6339,8 +6357,12 @@
         <v>283</v>
       </c>
       <c r="R83" s="11"/>
-      <c r="S83" s="11"/>
-      <c r="T83" s="11"/>
+      <c r="S83" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T83" s="17" t="s">
+        <v>238</v>
+      </c>
       <c r="U83" s="11"/>
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
@@ -6348,17 +6370,17 @@
         <v>284</v>
       </c>
       <c r="B84" s="5">
-        <v>46094.650843634256</v>
+        <v>46094.65047047454</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46094.65119138889</v>
+        <v>46111.83610230324</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>285</v>
       </c>
       <c r="F84" s="6" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G84" s="6" t="s">
         <v>28</v>
@@ -6373,10 +6395,10 @@
         <v>28</v>
       </c>
       <c r="M84" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="O84" s="6" t="s">
         <v>28</v>
@@ -6397,11 +6419,11 @@
         <v>287</v>
       </c>
       <c r="B85" s="10">
-        <v>46094.65095365741</v>
+        <v>46094.65072855324</v>
       </c>
       <c r="C85" s="11"/>
       <c r="D85" s="10">
-        <v>46094.65121894676</v>
+        <v>46094.65083585648</v>
       </c>
       <c r="E85" s="11" t="s">
         <v>288</v>
@@ -6425,7 +6447,7 @@
         <v>28</v>
       </c>
       <c r="N85" s="11" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="O85" s="11" t="s">
         <v>28</v>
@@ -6446,28 +6468,24 @@
         <v>290</v>
       </c>
       <c r="B86" s="5">
-        <v>46093.557977268516</v>
+        <v>46094.650843634256</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46099.639211539354</v>
+        <v>46094.65119138889</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>291</v>
       </c>
       <c r="F86" s="6" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H86" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H86" s="6"/>
       <c r="I86" s="6"/>
-      <c r="J86" s="5">
-        <v>46083</v>
-      </c>
+      <c r="J86" s="6"/>
       <c r="K86" s="6" t="s">
         <v>28</v>
       </c>
@@ -6475,10 +6493,10 @@
         <v>28</v>
       </c>
       <c r="M86" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>28</v>
+        <v>282</v>
       </c>
       <c r="O86" s="6" t="s">
         <v>28</v>
@@ -6490,12 +6508,8 @@
         <v>292</v>
       </c>
       <c r="R86" s="6"/>
-      <c r="S86" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T86" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="S86" s="6"/>
+      <c r="T86" s="6"/>
       <c r="U86" s="6"/>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -6503,11 +6517,11 @@
         <v>293</v>
       </c>
       <c r="B87" s="10">
-        <v>46094.64259225695</v>
+        <v>46094.65095365741</v>
       </c>
       <c r="C87" s="11"/>
       <c r="D87" s="10">
-        <v>46094.642785069445</v>
+        <v>46094.65121894676</v>
       </c>
       <c r="E87" s="11" t="s">
         <v>294</v>
@@ -6531,7 +6545,7 @@
         <v>28</v>
       </c>
       <c r="N87" s="11" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="O87" s="11" t="s">
         <v>28</v>
@@ -6552,27 +6566,27 @@
         <v>296</v>
       </c>
       <c r="B88" s="5">
-        <v>46093.55797850694</v>
+        <v>46093.557977268516</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46099.62486652778</v>
+        <v>46099.639211539354</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>297</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="I88" s="6"/>
       <c r="J88" s="5">
-        <v>46092</v>
+        <v>46083</v>
       </c>
       <c r="K88" s="6" t="s">
         <v>28</v>
@@ -6599,8 +6613,8 @@
       <c r="S88" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T88" s="17" t="s">
-        <v>232</v>
+      <c r="T88" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="U88" s="6"/>
     </row>
@@ -6609,11 +6623,11 @@
         <v>299</v>
       </c>
       <c r="B89" s="10">
-        <v>46094.65201979167</v>
+        <v>46094.64259225695</v>
       </c>
       <c r="C89" s="11"/>
       <c r="D89" s="10">
-        <v>46094.652139756945</v>
+        <v>46094.642785069445</v>
       </c>
       <c r="E89" s="11" t="s">
         <v>300</v>
@@ -6658,27 +6672,27 @@
         <v>302</v>
       </c>
       <c r="B90" s="5">
-        <v>46093.55797699074</v>
+        <v>46093.55797850694</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46134.66246857639</v>
+        <v>46099.62486652778</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>303</v>
       </c>
       <c r="F90" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="5">
-        <v>46094</v>
+        <v>46092</v>
       </c>
       <c r="K90" s="6" t="s">
         <v>28</v>
@@ -6705,7 +6719,9 @@
       <c r="S90" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T90" s="6"/>
+      <c r="T90" s="17" t="s">
+        <v>238</v>
+      </c>
       <c r="U90" s="6"/>
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
@@ -6713,11 +6729,11 @@
         <v>305</v>
       </c>
       <c r="B91" s="10">
-        <v>46094.64671800926</v>
+        <v>46094.65201979167</v>
       </c>
       <c r="C91" s="11"/>
       <c r="D91" s="10">
-        <v>46094.64682403935</v>
+        <v>46094.652139756945</v>
       </c>
       <c r="E91" s="11" t="s">
         <v>306</v>
@@ -6762,17 +6778,17 @@
         <v>308</v>
       </c>
       <c r="B92" s="5">
-        <v>46093.55797740741</v>
+        <v>46093.55797699074</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46196.5728619213</v>
+        <v>46134.66246857639</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>309</v>
       </c>
       <c r="F92" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G92" s="6" t="s">
         <v>57</v>
@@ -6780,11 +6796,9 @@
       <c r="H92" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="I92" s="5">
-        <v>46069</v>
-      </c>
+      <c r="I92" s="6"/>
       <c r="J92" s="5">
-        <v>46069</v>
+        <v>46094</v>
       </c>
       <c r="K92" s="6" t="s">
         <v>28</v>
@@ -6811,9 +6825,7 @@
       <c r="S92" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T92" s="17" t="s">
-        <v>128</v>
-      </c>
+      <c r="T92" s="6"/>
       <c r="U92" s="6"/>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
@@ -6821,11 +6833,11 @@
         <v>311</v>
       </c>
       <c r="B93" s="10">
-        <v>46094.58428688657</v>
+        <v>46094.64671800926</v>
       </c>
       <c r="C93" s="11"/>
       <c r="D93" s="10">
-        <v>46094.584938113425</v>
+        <v>46094.64682403935</v>
       </c>
       <c r="E93" s="11" t="s">
         <v>312</v>
@@ -6870,24 +6882,30 @@
         <v>314</v>
       </c>
       <c r="B94" s="5">
-        <v>46094.58447622685</v>
+        <v>46093.55797740741</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46094.5849659838</v>
+        <v>46196.5728619213</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>315</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>28</v>
+        <v>166</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H94" s="6"/>
-      <c r="I94" s="6"/>
-      <c r="J94" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H94" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="I94" s="5">
+        <v>46069</v>
+      </c>
+      <c r="J94" s="5">
+        <v>46069</v>
+      </c>
       <c r="K94" s="6" t="s">
         <v>28</v>
       </c>
@@ -6895,10 +6913,10 @@
         <v>28</v>
       </c>
       <c r="M94" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>309</v>
+        <v>28</v>
       </c>
       <c r="O94" s="6" t="s">
         <v>28</v>
@@ -6910,8 +6928,12 @@
         <v>316</v>
       </c>
       <c r="R94" s="6"/>
-      <c r="S94" s="6"/>
-      <c r="T94" s="6"/>
+      <c r="S94" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T94" s="17" t="s">
+        <v>128</v>
+      </c>
       <c r="U94" s="6"/>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
@@ -6919,11 +6941,11 @@
         <v>317</v>
       </c>
       <c r="B95" s="10">
-        <v>46094.58471086806</v>
+        <v>46094.58428688657</v>
       </c>
       <c r="C95" s="11"/>
       <c r="D95" s="10">
-        <v>46094.58499179398</v>
+        <v>46094.584938113425</v>
       </c>
       <c r="E95" s="11" t="s">
         <v>318</v>
@@ -6947,7 +6969,7 @@
         <v>28</v>
       </c>
       <c r="N95" s="11" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="O95" s="11" t="s">
         <v>28</v>
@@ -6968,30 +6990,24 @@
         <v>320</v>
       </c>
       <c r="B96" s="5">
-        <v>46093.55797605324</v>
-      </c>
-      <c r="C96" s="5">
-        <v>46140.73067185185</v>
-      </c>
+        <v>46094.58447622685</v>
+      </c>
+      <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46140.730673252314</v>
+        <v>46094.5849659838</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>321</v>
       </c>
       <c r="F96" s="6" t="s">
-        <v>160</v>
+        <v>28</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H96" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H96" s="6"/>
       <c r="I96" s="6"/>
-      <c r="J96" s="5">
-        <v>46059</v>
-      </c>
+      <c r="J96" s="6"/>
       <c r="K96" s="6" t="s">
         <v>28</v>
       </c>
@@ -6999,10 +7015,10 @@
         <v>28</v>
       </c>
       <c r="M96" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>28</v>
+        <v>315</v>
       </c>
       <c r="O96" s="6" t="s">
         <v>28</v>
@@ -7014,12 +7030,8 @@
         <v>322</v>
       </c>
       <c r="R96" s="6"/>
-      <c r="S96" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T96" s="17" t="s">
-        <v>128</v>
-      </c>
+      <c r="S96" s="6"/>
+      <c r="T96" s="6"/>
       <c r="U96" s="6"/>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
@@ -7027,11 +7039,11 @@
         <v>323</v>
       </c>
       <c r="B97" s="10">
-        <v>46094.644745763886</v>
+        <v>46094.58471086806</v>
       </c>
       <c r="C97" s="11"/>
       <c r="D97" s="10">
-        <v>46094.644892048615</v>
+        <v>46094.58499179398</v>
       </c>
       <c r="E97" s="11" t="s">
         <v>324</v>
@@ -7055,7 +7067,7 @@
         <v>28</v>
       </c>
       <c r="N97" s="11" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="O97" s="11" t="s">
         <v>28</v>
@@ -7076,24 +7088,30 @@
         <v>326</v>
       </c>
       <c r="B98" s="5">
-        <v>46094.64489846065</v>
-      </c>
-      <c r="C98" s="6"/>
+        <v>46093.55797605324</v>
+      </c>
+      <c r="C98" s="5">
+        <v>46140.73067185185</v>
+      </c>
       <c r="D98" s="5">
-        <v>46094.64504228009</v>
+        <v>46140.730673252314</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>327</v>
       </c>
       <c r="F98" s="6" t="s">
-        <v>28</v>
+        <v>166</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H98" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H98" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I98" s="6"/>
-      <c r="J98" s="6"/>
+      <c r="J98" s="5">
+        <v>46059</v>
+      </c>
       <c r="K98" s="6" t="s">
         <v>28</v>
       </c>
@@ -7101,10 +7119,10 @@
         <v>28</v>
       </c>
       <c r="M98" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>321</v>
+        <v>28</v>
       </c>
       <c r="O98" s="6" t="s">
         <v>28</v>
@@ -7116,8 +7134,12 @@
         <v>328</v>
       </c>
       <c r="R98" s="6"/>
-      <c r="S98" s="6"/>
-      <c r="T98" s="6"/>
+      <c r="S98" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T98" s="17" t="s">
+        <v>128</v>
+      </c>
       <c r="U98" s="6"/>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -7125,78 +7147,66 @@
         <v>329</v>
       </c>
       <c r="B99" s="10">
-        <v>46133.80890888889</v>
-      </c>
-      <c r="C99" s="10">
-        <v>46203.59473923611</v>
-      </c>
+        <v>46094.644745763886</v>
+      </c>
+      <c r="C99" s="11"/>
       <c r="D99" s="10">
-        <v>46203.59475351852</v>
+        <v>46094.644892048615</v>
       </c>
       <c r="E99" s="11" t="s">
         <v>330</v>
       </c>
       <c r="F99" s="11" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G99" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H99" s="11" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H99" s="11"/>
       <c r="I99" s="11"/>
-      <c r="J99" s="10">
-        <v>46142</v>
-      </c>
+      <c r="J99" s="11"/>
       <c r="K99" s="11" t="s">
         <v>28</v>
       </c>
       <c r="L99" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="M99" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="N99" s="11" t="s">
+        <v>327</v>
+      </c>
+      <c r="O99" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="P99" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q99" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="M99" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="N99" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="O99" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="P99" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q99" s="11" t="s">
-        <v>332</v>
-      </c>
       <c r="R99" s="11"/>
-      <c r="S99" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T99" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="S99" s="11"/>
+      <c r="T99" s="11"/>
       <c r="U99" s="11"/>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="B100" s="5">
+        <v>46094.64489846065</v>
+      </c>
+      <c r="C100" s="6"/>
+      <c r="D100" s="5">
+        <v>46094.64504228009</v>
+      </c>
+      <c r="E100" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="B100" s="5">
-        <v>46133.809437812495</v>
-      </c>
-      <c r="C100" s="5">
-        <v>46203.594679999995</v>
-      </c>
-      <c r="D100" s="5">
-        <v>46203.59469834491</v>
-      </c>
-      <c r="E100" s="6" t="s">
-        <v>334</v>
-      </c>
       <c r="F100" s="6" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G100" s="6" t="s">
         <v>28</v>
@@ -7211,10 +7221,10 @@
         <v>28</v>
       </c>
       <c r="M100" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N100" s="6" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="O100" s="6" t="s">
         <v>28</v>
@@ -7223,7 +7233,7 @@
         <v>28</v>
       </c>
       <c r="Q100" s="6" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="R100" s="6"/>
       <c r="S100" s="6"/>
@@ -7232,19 +7242,19 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="B101" s="10">
+        <v>46133.80890888889</v>
+      </c>
+      <c r="C101" s="10">
+        <v>46203.59473923611</v>
+      </c>
+      <c r="D101" s="10">
+        <v>46203.59475351852</v>
+      </c>
+      <c r="E101" s="11" t="s">
         <v>336</v>
-      </c>
-      <c r="B101" s="10">
-        <v>46155.80580025463</v>
-      </c>
-      <c r="C101" s="10">
-        <v>46203.58947402777</v>
-      </c>
-      <c r="D101" s="10">
-        <v>46203.5894903588</v>
-      </c>
-      <c r="E101" s="11" t="s">
-        <v>337</v>
       </c>
       <c r="F101" s="11" t="s">
         <v>143</v>
@@ -7257,65 +7267,63 @@
       </c>
       <c r="I101" s="11"/>
       <c r="J101" s="10">
-        <v>46162</v>
+        <v>46142</v>
       </c>
       <c r="K101" s="11" t="s">
         <v>28</v>
       </c>
       <c r="L101" s="11" t="s">
-        <v>28</v>
+        <v>337</v>
       </c>
       <c r="M101" s="11" t="s">
         <v>0</v>
       </c>
       <c r="N101" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="O101" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="P101" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q101" s="11" t="s">
         <v>338</v>
       </c>
-      <c r="O101" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="P101" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q101" s="11" t="s">
-        <v>339</v>
-      </c>
       <c r="R101" s="11"/>
-      <c r="S101" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T101" s="11"/>
+      <c r="S101" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T101" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U101" s="11"/>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="B102" s="5">
+        <v>46133.809437812495</v>
+      </c>
+      <c r="C102" s="5">
+        <v>46203.594679999995</v>
+      </c>
+      <c r="D102" s="5">
+        <v>46203.59469834491</v>
+      </c>
+      <c r="E102" s="6" t="s">
         <v>340</v>
-      </c>
-      <c r="B102" s="5">
-        <v>46155.80563927084</v>
-      </c>
-      <c r="C102" s="5">
-        <v>46203.58946413195</v>
-      </c>
-      <c r="D102" s="5">
-        <v>46203.58948405093</v>
-      </c>
-      <c r="E102" s="6" t="s">
-        <v>341</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>143</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H102" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H102" s="6"/>
       <c r="I102" s="6"/>
-      <c r="J102" s="5">
-        <v>46162</v>
-      </c>
+      <c r="J102" s="6"/>
       <c r="K102" s="6" t="s">
         <v>28</v>
       </c>
@@ -7326,7 +7334,7 @@
         <v>0</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="O102" s="6" t="s">
         <v>28</v>
@@ -7335,30 +7343,28 @@
         <v>28</v>
       </c>
       <c r="Q102" s="6" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="R102" s="6"/>
-      <c r="S102" s="12" t="s">
-        <v>43</v>
-      </c>
+      <c r="S102" s="6"/>
       <c r="T102" s="6"/>
       <c r="U102" s="6"/>
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="9" t="s">
+        <v>342</v>
+      </c>
+      <c r="B103" s="10">
+        <v>46155.80580025463</v>
+      </c>
+      <c r="C103" s="10">
+        <v>46203.58947402777</v>
+      </c>
+      <c r="D103" s="10">
+        <v>46203.5894903588</v>
+      </c>
+      <c r="E103" s="11" t="s">
         <v>343</v>
-      </c>
-      <c r="B103" s="10">
-        <v>46155.80523456019</v>
-      </c>
-      <c r="C103" s="10">
-        <v>46203.589470266204</v>
-      </c>
-      <c r="D103" s="10">
-        <v>46203.589486400466</v>
-      </c>
-      <c r="E103" s="11" t="s">
-        <v>338</v>
       </c>
       <c r="F103" s="11" t="s">
         <v>143</v>
@@ -7383,7 +7389,7 @@
         <v>0</v>
       </c>
       <c r="N103" s="11" t="s">
-        <v>28</v>
+        <v>344</v>
       </c>
       <c r="O103" s="11" t="s">
         <v>28</v>
@@ -7392,30 +7398,30 @@
         <v>28</v>
       </c>
       <c r="Q103" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="R103" s="11"/>
       <c r="S103" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T103" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="T103" s="11"/>
       <c r="U103" s="11"/>
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B104" s="5">
-        <v>46133.8018299074</v>
-      </c>
-      <c r="C104" s="6"/>
+        <v>46155.80563927084</v>
+      </c>
+      <c r="C104" s="5">
+        <v>46203.58946413195</v>
+      </c>
       <c r="D104" s="5">
-        <v>46185.594546168984</v>
+        <v>46203.58948405093</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>143</v>
@@ -7428,7 +7434,7 @@
       </c>
       <c r="I104" s="6"/>
       <c r="J104" s="5">
-        <v>46157</v>
+        <v>46162</v>
       </c>
       <c r="K104" s="6" t="s">
         <v>28</v>
@@ -7440,7 +7446,7 @@
         <v>0</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>28</v>
+        <v>344</v>
       </c>
       <c r="O104" s="6" t="s">
         <v>28</v>
@@ -7449,40 +7455,44 @@
         <v>28</v>
       </c>
       <c r="Q104" s="6" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R104" s="6"/>
       <c r="S104" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T104" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="T104" s="6"/>
       <c r="U104" s="6"/>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="9" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B105" s="10">
-        <v>46133.8022120949</v>
-      </c>
-      <c r="C105" s="11"/>
+        <v>46155.80523456019</v>
+      </c>
+      <c r="C105" s="10">
+        <v>46203.589470266204</v>
+      </c>
       <c r="D105" s="10">
-        <v>46133.80266505787</v>
+        <v>46203.589486400466</v>
       </c>
       <c r="E105" s="11" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="F105" s="11" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G105" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H105" s="11"/>
+        <v>57</v>
+      </c>
+      <c r="H105" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="I105" s="11"/>
-      <c r="J105" s="11"/>
+      <c r="J105" s="10">
+        <v>46162</v>
+      </c>
       <c r="K105" s="11" t="s">
         <v>28</v>
       </c>
@@ -7490,10 +7500,10 @@
         <v>28</v>
       </c>
       <c r="M105" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N105" s="11" t="s">
-        <v>346</v>
+        <v>28</v>
       </c>
       <c r="O105" s="11" t="s">
         <v>28</v>
@@ -7505,8 +7515,12 @@
         <v>350</v>
       </c>
       <c r="R105" s="11"/>
-      <c r="S105" s="11"/>
-      <c r="T105" s="11"/>
+      <c r="S105" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T105" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U105" s="11"/>
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
@@ -7514,24 +7528,28 @@
         <v>351</v>
       </c>
       <c r="B106" s="5">
-        <v>46133.80235815972</v>
+        <v>46133.8018299074</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46133.8027009375</v>
+        <v>46185.594546168984</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>352</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G106" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H106" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H106" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I106" s="6"/>
-      <c r="J106" s="6"/>
+      <c r="J106" s="5">
+        <v>46157</v>
+      </c>
       <c r="K106" s="6" t="s">
         <v>28</v>
       </c>
@@ -7539,10 +7557,10 @@
         <v>28</v>
       </c>
       <c r="M106" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>346</v>
+        <v>28</v>
       </c>
       <c r="O106" s="6" t="s">
         <v>28</v>
@@ -7554,8 +7572,12 @@
         <v>353</v>
       </c>
       <c r="R106" s="6"/>
-      <c r="S106" s="6"/>
-      <c r="T106" s="6"/>
+      <c r="S106" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T106" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U106" s="6"/>
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
@@ -7563,11 +7585,11 @@
         <v>354</v>
       </c>
       <c r="B107" s="10">
-        <v>46133.80248805556</v>
+        <v>46133.8022120949</v>
       </c>
       <c r="C107" s="11"/>
       <c r="D107" s="10">
-        <v>46133.802740625004</v>
+        <v>46133.80266505787</v>
       </c>
       <c r="E107" s="11" t="s">
         <v>355</v>
@@ -7591,7 +7613,7 @@
         <v>28</v>
       </c>
       <c r="N107" s="11" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="O107" s="11" t="s">
         <v>28</v>
@@ -7612,30 +7634,24 @@
         <v>357</v>
       </c>
       <c r="B108" s="5">
-        <v>46093.55797645834</v>
-      </c>
-      <c r="C108" s="5">
-        <v>46162.85491734954</v>
-      </c>
+        <v>46133.80235815972</v>
+      </c>
+      <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46162.85493328703</v>
+        <v>46133.8027009375</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>358</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H108" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H108" s="6"/>
       <c r="I108" s="6"/>
-      <c r="J108" s="5">
-        <v>46063</v>
-      </c>
+      <c r="J108" s="6"/>
       <c r="K108" s="6" t="s">
         <v>28</v>
       </c>
@@ -7643,10 +7659,10 @@
         <v>28</v>
       </c>
       <c r="M108" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>28</v>
+        <v>352</v>
       </c>
       <c r="O108" s="6" t="s">
         <v>28</v>
@@ -7658,12 +7674,8 @@
         <v>359</v>
       </c>
       <c r="R108" s="6"/>
-      <c r="S108" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T108" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="S108" s="6"/>
+      <c r="T108" s="6"/>
       <c r="U108" s="6"/>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
@@ -7671,30 +7683,24 @@
         <v>360</v>
       </c>
       <c r="B109" s="10">
-        <v>46094.63825950232</v>
-      </c>
-      <c r="C109" s="10">
-        <v>46136.032332372684</v>
-      </c>
+        <v>46133.80248805556</v>
+      </c>
+      <c r="C109" s="11"/>
       <c r="D109" s="10">
-        <v>46136.032352685186</v>
+        <v>46133.802740625004</v>
       </c>
       <c r="E109" s="11" t="s">
         <v>361</v>
       </c>
       <c r="F109" s="11" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G109" s="11" t="s">
         <v>28</v>
       </c>
       <c r="H109" s="11"/>
-      <c r="I109" s="10">
-        <v>45988</v>
-      </c>
-      <c r="J109" s="10">
-        <v>45988</v>
-      </c>
+      <c r="I109" s="11"/>
+      <c r="J109" s="11"/>
       <c r="K109" s="11" t="s">
         <v>28</v>
       </c>
@@ -7702,10 +7708,10 @@
         <v>28</v>
       </c>
       <c r="M109" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N109" s="11" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="O109" s="11" t="s">
         <v>28</v>
@@ -7726,13 +7732,13 @@
         <v>363</v>
       </c>
       <c r="B110" s="5">
-        <v>46094.63841756944</v>
+        <v>46093.55797645834</v>
       </c>
       <c r="C110" s="5">
-        <v>46136.03234583333</v>
+        <v>46162.85491734954</v>
       </c>
       <c r="D110" s="5">
-        <v>46136.03236168981</v>
+        <v>46162.85493328703</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>364</v>
@@ -7741,14 +7747,14 @@
         <v>143</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H110" s="6"/>
-      <c r="I110" s="5">
-        <v>45988</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="H110" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="I110" s="6"/>
       <c r="J110" s="5">
-        <v>45988</v>
+        <v>46063</v>
       </c>
       <c r="K110" s="6" t="s">
         <v>28</v>
@@ -7760,7 +7766,7 @@
         <v>0</v>
       </c>
       <c r="N110" s="6" t="s">
-        <v>358</v>
+        <v>28</v>
       </c>
       <c r="O110" s="6" t="s">
         <v>28</v>
@@ -7772,8 +7778,12 @@
         <v>365</v>
       </c>
       <c r="R110" s="6"/>
-      <c r="S110" s="6"/>
-      <c r="T110" s="6"/>
+      <c r="S110" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T110" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U110" s="6"/>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
@@ -7781,13 +7791,13 @@
         <v>366</v>
       </c>
       <c r="B111" s="10">
-        <v>46094.63861635417</v>
+        <v>46094.63825950232</v>
       </c>
       <c r="C111" s="10">
-        <v>46136.03235858797</v>
+        <v>46136.032332372684</v>
       </c>
       <c r="D111" s="10">
-        <v>46136.032374560185</v>
+        <v>46136.032352685186</v>
       </c>
       <c r="E111" s="11" t="s">
         <v>367</v>
@@ -7800,10 +7810,10 @@
       </c>
       <c r="H111" s="11"/>
       <c r="I111" s="10">
-        <v>46063</v>
+        <v>45988</v>
       </c>
       <c r="J111" s="10">
-        <v>46063</v>
+        <v>45988</v>
       </c>
       <c r="K111" s="11" t="s">
         <v>28</v>
@@ -7815,7 +7825,7 @@
         <v>0</v>
       </c>
       <c r="N111" s="11" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="O111" s="11" t="s">
         <v>28</v>
@@ -7836,13 +7846,13 @@
         <v>369</v>
       </c>
       <c r="B112" s="5">
-        <v>46133.81027721065</v>
+        <v>46094.63841756944</v>
       </c>
       <c r="C112" s="5">
-        <v>46161.91299474537</v>
+        <v>46136.03234583333</v>
       </c>
       <c r="D112" s="5">
-        <v>46161.91301581018</v>
+        <v>46136.03236168981</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>370</v>
@@ -7854,8 +7864,12 @@
         <v>28</v>
       </c>
       <c r="H112" s="6"/>
-      <c r="I112" s="6"/>
-      <c r="J112" s="6"/>
+      <c r="I112" s="5">
+        <v>45988</v>
+      </c>
+      <c r="J112" s="5">
+        <v>45988</v>
+      </c>
       <c r="K112" s="6" t="s">
         <v>28</v>
       </c>
@@ -7866,16 +7880,16 @@
         <v>0</v>
       </c>
       <c r="N112" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="O112" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P112" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q112" s="6" t="s">
         <v>371</v>
-      </c>
-      <c r="O112" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="P112" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q112" s="6" t="s">
-        <v>372</v>
       </c>
       <c r="R112" s="6"/>
       <c r="S112" s="6"/>
@@ -7884,32 +7898,32 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B113" s="10">
+        <v>46094.63861635417</v>
+      </c>
+      <c r="C113" s="10">
+        <v>46136.03235858797</v>
+      </c>
+      <c r="D113" s="10">
+        <v>46136.032374560185</v>
+      </c>
+      <c r="E113" s="11" t="s">
         <v>373</v>
-      </c>
-      <c r="B113" s="10">
-        <v>46133.80965319445</v>
-      </c>
-      <c r="C113" s="10">
-        <v>46161.912943958334</v>
-      </c>
-      <c r="D113" s="10">
-        <v>46161.91296126157</v>
-      </c>
-      <c r="E113" s="11" t="s">
-        <v>371</v>
       </c>
       <c r="F113" s="11" t="s">
         <v>143</v>
       </c>
       <c r="G113" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H113" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="I113" s="11"/>
+        <v>28</v>
+      </c>
+      <c r="H113" s="11"/>
+      <c r="I113" s="10">
+        <v>46063</v>
+      </c>
       <c r="J113" s="10">
-        <v>46140</v>
+        <v>46063</v>
       </c>
       <c r="K113" s="11" t="s">
         <v>28</v>
@@ -7921,7 +7935,7 @@
         <v>0</v>
       </c>
       <c r="N113" s="11" t="s">
-        <v>28</v>
+        <v>364</v>
       </c>
       <c r="O113" s="11" t="s">
         <v>28</v>
@@ -7933,12 +7947,8 @@
         <v>374</v>
       </c>
       <c r="R113" s="11"/>
-      <c r="S113" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="T113" s="8" t="s">
-        <v>31</v>
-      </c>
+      <c r="S113" s="11"/>
+      <c r="T113" s="11"/>
       <c r="U113" s="11"/>
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
@@ -7946,13 +7956,13 @@
         <v>375</v>
       </c>
       <c r="B114" s="5">
-        <v>46133.79562642361</v>
+        <v>46133.81027721065</v>
       </c>
       <c r="C114" s="5">
-        <v>46161.91275101852</v>
+        <v>46161.91299474537</v>
       </c>
       <c r="D114" s="5">
-        <v>46161.912771296295</v>
+        <v>46161.91301581018</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>376</v>
@@ -7997,13 +8007,13 @@
         <v>379</v>
       </c>
       <c r="B115" s="10">
-        <v>46133.79487287037</v>
+        <v>46133.80965319445</v>
       </c>
       <c r="C115" s="10">
-        <v>46161.91275491898</v>
+        <v>46161.912943958334</v>
       </c>
       <c r="D115" s="10">
-        <v>46161.91277105324</v>
+        <v>46161.91296126157</v>
       </c>
       <c r="E115" s="11" t="s">
         <v>377</v>
@@ -8019,7 +8029,7 @@
       </c>
       <c r="I115" s="11"/>
       <c r="J115" s="10">
-        <v>46118</v>
+        <v>46140</v>
       </c>
       <c r="K115" s="11" t="s">
         <v>28</v>
@@ -8043,8 +8053,8 @@
         <v>380</v>
       </c>
       <c r="R115" s="11"/>
-      <c r="S115" s="12" t="s">
-        <v>43</v>
+      <c r="S115" s="14" t="s">
+        <v>51</v>
       </c>
       <c r="T115" s="8" t="s">
         <v>31</v>
@@ -8056,13 +8066,13 @@
         <v>381</v>
       </c>
       <c r="B116" s="5">
-        <v>46133.79582699074</v>
+        <v>46133.79562642361</v>
       </c>
       <c r="C116" s="5">
-        <v>46161.912757847225</v>
+        <v>46161.91275101852</v>
       </c>
       <c r="D116" s="5">
-        <v>46161.91277258102</v>
+        <v>46161.912771296295</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>382</v>
@@ -8086,7 +8096,7 @@
         <v>0</v>
       </c>
       <c r="N116" s="6" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="O116" s="6" t="s">
         <v>28</v>
@@ -8095,7 +8105,7 @@
         <v>28</v>
       </c>
       <c r="Q116" s="6" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="R116" s="6"/>
       <c r="S116" s="6"/>
@@ -8104,32 +8114,32 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="9" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B117" s="10">
-        <v>46094.641416493054</v>
+        <v>46133.79487287037</v>
       </c>
       <c r="C117" s="10">
-        <v>46161.912420381945</v>
+        <v>46161.91275491898</v>
       </c>
       <c r="D117" s="10">
-        <v>46161.912439594904</v>
+        <v>46161.91277105324</v>
       </c>
       <c r="E117" s="11" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="F117" s="11" t="s">
         <v>143</v>
       </c>
       <c r="G117" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H117" s="11"/>
-      <c r="I117" s="10">
-        <v>45986</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H117" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I117" s="11"/>
       <c r="J117" s="10">
-        <v>45986</v>
+        <v>46118</v>
       </c>
       <c r="K117" s="11" t="s">
         <v>28</v>
@@ -8141,51 +8151,51 @@
         <v>0</v>
       </c>
       <c r="N117" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="O117" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="P117" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q117" s="11" t="s">
         <v>386</v>
       </c>
-      <c r="O117" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="P117" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q117" s="11" t="s">
-        <v>387</v>
-      </c>
       <c r="R117" s="11"/>
-      <c r="S117" s="11"/>
-      <c r="T117" s="11"/>
+      <c r="S117" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T117" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="U117" s="11"/>
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="B118" s="5">
+        <v>46133.79582699074</v>
+      </c>
+      <c r="C118" s="5">
+        <v>46161.912757847225</v>
+      </c>
+      <c r="D118" s="5">
+        <v>46161.91277258102</v>
+      </c>
+      <c r="E118" s="6" t="s">
         <v>388</v>
-      </c>
-      <c r="B118" s="5">
-        <v>46093.55797701389</v>
-      </c>
-      <c r="C118" s="5">
-        <v>46161.912426678246</v>
-      </c>
-      <c r="D118" s="5">
-        <v>46161.91244167824</v>
-      </c>
-      <c r="E118" s="6" t="s">
-        <v>386</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>143</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H118" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H118" s="6"/>
       <c r="I118" s="6"/>
-      <c r="J118" s="5">
-        <v>45986</v>
-      </c>
+      <c r="J118" s="6"/>
       <c r="K118" s="6" t="s">
         <v>28</v>
       </c>
@@ -8196,7 +8206,7 @@
         <v>0</v>
       </c>
       <c r="N118" s="6" t="s">
-        <v>28</v>
+        <v>383</v>
       </c>
       <c r="O118" s="6" t="s">
         <v>28</v>
@@ -8208,12 +8218,8 @@
         <v>389</v>
       </c>
       <c r="R118" s="6"/>
-      <c r="S118" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T118" s="8" t="s">
-        <v>31</v>
-      </c>
+      <c r="S118" s="6"/>
+      <c r="T118" s="6"/>
       <c r="U118" s="6"/>
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
@@ -8221,13 +8227,13 @@
         <v>390</v>
       </c>
       <c r="B119" s="10">
-        <v>46094.582692951386</v>
+        <v>46094.641416493054</v>
       </c>
       <c r="C119" s="10">
-        <v>46134.673179687496</v>
+        <v>46161.912420381945</v>
       </c>
       <c r="D119" s="10">
-        <v>46134.67319648148</v>
+        <v>46161.912439594904</v>
       </c>
       <c r="E119" s="11" t="s">
         <v>391</v>
@@ -8236,13 +8242,15 @@
         <v>143</v>
       </c>
       <c r="G119" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H119" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="I119" s="11"/>
-      <c r="J119" s="11"/>
+        <v>28</v>
+      </c>
+      <c r="H119" s="11"/>
+      <c r="I119" s="10">
+        <v>45986</v>
+      </c>
+      <c r="J119" s="10">
+        <v>45986</v>
+      </c>
       <c r="K119" s="11" t="s">
         <v>28</v>
       </c>
@@ -8274,28 +8282,30 @@
         <v>394</v>
       </c>
       <c r="B120" s="5">
-        <v>46093.557975625</v>
+        <v>46093.55797701389</v>
       </c>
       <c r="C120" s="5">
-        <v>46134.64221024305</v>
+        <v>46161.912426678246</v>
       </c>
       <c r="D120" s="5">
-        <v>46134.66266402778</v>
+        <v>46161.91244167824</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="F120" s="6" t="s">
         <v>143</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="H120" s="6" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="I120" s="6"/>
-      <c r="J120" s="6"/>
+      <c r="J120" s="5">
+        <v>45986</v>
+      </c>
       <c r="K120" s="6" t="s">
         <v>28</v>
       </c>
@@ -8315,28 +8325,32 @@
         <v>28</v>
       </c>
       <c r="Q120" s="6" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="R120" s="6"/>
-      <c r="S120" s="6"/>
-      <c r="T120" s="6"/>
+      <c r="S120" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T120" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="U120" s="6"/>
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A121" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="B121" s="10">
+        <v>46094.582692951386</v>
+      </c>
+      <c r="C121" s="10">
+        <v>46134.673179687496</v>
+      </c>
+      <c r="D121" s="10">
+        <v>46134.67319648148</v>
+      </c>
+      <c r="E121" s="11" t="s">
         <v>397</v>
-      </c>
-      <c r="B121" s="10">
-        <v>46093.55797712963</v>
-      </c>
-      <c r="C121" s="10">
-        <v>46134.63987417824</v>
-      </c>
-      <c r="D121" s="10">
-        <v>46134.63988903935</v>
-      </c>
-      <c r="E121" s="11" t="s">
-        <v>392</v>
       </c>
       <c r="F121" s="11" t="s">
         <v>143</v>
@@ -8347,12 +8361,8 @@
       <c r="H121" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I121" s="10">
-        <v>46039</v>
-      </c>
-      <c r="J121" s="10">
-        <v>46039</v>
-      </c>
+      <c r="I121" s="11"/>
+      <c r="J121" s="11"/>
       <c r="K121" s="11" t="s">
         <v>28</v>
       </c>
@@ -8363,7 +8373,7 @@
         <v>0</v>
       </c>
       <c r="N121" s="11" t="s">
-        <v>28</v>
+        <v>398</v>
       </c>
       <c r="O121" s="11" t="s">
         <v>28</v>
@@ -8372,30 +8382,28 @@
         <v>28</v>
       </c>
       <c r="Q121" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="R121" s="11"/>
       <c r="S121" s="11"/>
-      <c r="T121" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="T121" s="11"/>
       <c r="U121" s="11"/>
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B122" s="5">
-        <v>46094.58194446759</v>
+        <v>46093.557975625</v>
       </c>
       <c r="C122" s="5">
-        <v>46134.63920685185</v>
+        <v>46134.64221024305</v>
       </c>
       <c r="D122" s="5">
-        <v>46134.66324178241</v>
+        <v>46134.66266402778</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F122" s="6" t="s">
         <v>143</v>
@@ -8418,7 +8426,7 @@
         <v>0</v>
       </c>
       <c r="N122" s="6" t="s">
-        <v>392</v>
+        <v>28</v>
       </c>
       <c r="O122" s="6" t="s">
         <v>28</v>
@@ -8427,7 +8435,7 @@
         <v>28</v>
       </c>
       <c r="Q122" s="6" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="R122" s="6"/>
       <c r="S122" s="6"/>
@@ -8436,19 +8444,19 @@
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A123" s="9" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B123" s="10">
-        <v>46094.58215357639</v>
+        <v>46093.55797712963</v>
       </c>
       <c r="C123" s="10">
-        <v>46134.63922920139</v>
+        <v>46134.63987417824</v>
       </c>
       <c r="D123" s="10">
-        <v>46134.66306040509</v>
+        <v>46134.63988903935</v>
       </c>
       <c r="E123" s="11" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="F123" s="11" t="s">
         <v>143</v>
@@ -8459,8 +8467,12 @@
       <c r="H123" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I123" s="11"/>
-      <c r="J123" s="11"/>
+      <c r="I123" s="10">
+        <v>46039</v>
+      </c>
+      <c r="J123" s="10">
+        <v>46039</v>
+      </c>
       <c r="K123" s="11" t="s">
         <v>28</v>
       </c>
@@ -8471,7 +8483,7 @@
         <v>0</v>
       </c>
       <c r="N123" s="11" t="s">
-        <v>392</v>
+        <v>28</v>
       </c>
       <c r="O123" s="11" t="s">
         <v>28</v>
@@ -8484,7 +8496,9 @@
       </c>
       <c r="R123" s="11"/>
       <c r="S123" s="11"/>
-      <c r="T123" s="11"/>
+      <c r="T123" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U123" s="11"/>
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
@@ -8492,13 +8506,13 @@
         <v>405</v>
       </c>
       <c r="B124" s="5">
-        <v>46094.5823130787</v>
+        <v>46094.58194446759</v>
       </c>
       <c r="C124" s="5">
-        <v>46134.63923450232</v>
+        <v>46134.63920685185</v>
       </c>
       <c r="D124" s="5">
-        <v>46134.66313976852</v>
+        <v>46134.66324178241</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>406</v>
@@ -8524,7 +8538,7 @@
         <v>0</v>
       </c>
       <c r="N124" s="6" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="O124" s="6" t="s">
         <v>28</v>
@@ -8545,13 +8559,13 @@
         <v>408</v>
       </c>
       <c r="B125" s="10">
-        <v>46094.582410393516</v>
+        <v>46094.58215357639</v>
       </c>
       <c r="C125" s="10">
-        <v>46134.63923954861</v>
+        <v>46134.63922920139</v>
       </c>
       <c r="D125" s="10">
-        <v>46134.662989178236</v>
+        <v>46134.66306040509</v>
       </c>
       <c r="E125" s="11" t="s">
         <v>409</v>
@@ -8577,7 +8591,7 @@
         <v>0</v>
       </c>
       <c r="N125" s="11" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="O125" s="11" t="s">
         <v>28</v>
@@ -8598,13 +8612,13 @@
         <v>411</v>
       </c>
       <c r="B126" s="5">
-        <v>46094.58253722222</v>
+        <v>46094.5823130787</v>
       </c>
       <c r="C126" s="5">
-        <v>46134.639245694445</v>
+        <v>46134.63923450232</v>
       </c>
       <c r="D126" s="5">
-        <v>46134.662925682875</v>
+        <v>46134.66313976852</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>412</v>
@@ -8630,7 +8644,7 @@
         <v>0</v>
       </c>
       <c r="N126" s="6" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="O126" s="6" t="s">
         <v>28</v>
@@ -8651,13 +8665,13 @@
         <v>414</v>
       </c>
       <c r="B127" s="10">
-        <v>46094.582797511575</v>
+        <v>46094.582410393516</v>
       </c>
       <c r="C127" s="10">
-        <v>46134.639255312504</v>
+        <v>46134.63923954861</v>
       </c>
       <c r="D127" s="10">
-        <v>46155.578320636574</v>
+        <v>46134.662989178236</v>
       </c>
       <c r="E127" s="11" t="s">
         <v>415</v>
@@ -8683,7 +8697,7 @@
         <v>0</v>
       </c>
       <c r="N127" s="11" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="O127" s="11" t="s">
         <v>28</v>
@@ -8704,13 +8718,13 @@
         <v>417</v>
       </c>
       <c r="B128" s="5">
-        <v>46094.58288509259</v>
+        <v>46094.58253722222</v>
       </c>
       <c r="C128" s="5">
-        <v>46134.63926054398</v>
+        <v>46134.639245694445</v>
       </c>
       <c r="D128" s="5">
-        <v>46134.662788738424</v>
+        <v>46134.662925682875</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>418</v>
@@ -8736,7 +8750,7 @@
         <v>0</v>
       </c>
       <c r="N128" s="6" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="O128" s="6" t="s">
         <v>28</v>
@@ -8757,13 +8771,13 @@
         <v>420</v>
       </c>
       <c r="B129" s="10">
-        <v>46094.58306329861</v>
+        <v>46094.582797511575</v>
       </c>
       <c r="C129" s="10">
-        <v>46134.639266087965</v>
+        <v>46134.639255312504</v>
       </c>
       <c r="D129" s="10">
-        <v>46134.66273581018</v>
+        <v>46155.578320636574</v>
       </c>
       <c r="E129" s="11" t="s">
         <v>421</v>
@@ -8789,7 +8803,7 @@
         <v>0</v>
       </c>
       <c r="N129" s="11" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="O129" s="11" t="s">
         <v>28</v>
@@ -8810,13 +8824,13 @@
         <v>423</v>
       </c>
       <c r="B130" s="5">
-        <v>46133.792176840274</v>
+        <v>46094.58288509259</v>
       </c>
       <c r="C130" s="5">
-        <v>46134.63605664352</v>
+        <v>46134.63926054398</v>
       </c>
       <c r="D130" s="5">
-        <v>46134.63619297453</v>
+        <v>46134.662788738424</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>424</v>
@@ -8831,20 +8845,18 @@
         <v>58</v>
       </c>
       <c r="I130" s="6"/>
-      <c r="J130" s="5">
-        <v>46112</v>
-      </c>
+      <c r="J130" s="6"/>
       <c r="K130" s="6" t="s">
         <v>28</v>
       </c>
       <c r="L130" s="6" t="s">
-        <v>425</v>
+        <v>28</v>
       </c>
       <c r="M130" s="6" t="s">
         <v>0</v>
       </c>
       <c r="N130" s="6" t="s">
-        <v>28</v>
+        <v>398</v>
       </c>
       <c r="O130" s="6" t="s">
         <v>28</v>
@@ -8853,38 +8865,38 @@
         <v>28</v>
       </c>
       <c r="Q130" s="6" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="R130" s="6"/>
-      <c r="S130" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T130" s="12" t="s">
-        <v>427</v>
-      </c>
+      <c r="S130" s="6"/>
+      <c r="T130" s="6"/>
       <c r="U130" s="6"/>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A131" s="9" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B131" s="10">
-        <v>46133.79263490741</v>
-      </c>
-      <c r="C131" s="11"/>
+        <v>46094.58306329861</v>
+      </c>
+      <c r="C131" s="10">
+        <v>46134.639266087965</v>
+      </c>
       <c r="D131" s="10">
-        <v>46133.79350961806</v>
+        <v>46134.66273581018</v>
       </c>
       <c r="E131" s="11" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="F131" s="11" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G131" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H131" s="11"/>
+        <v>57</v>
+      </c>
+      <c r="H131" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="I131" s="11"/>
       <c r="J131" s="11"/>
       <c r="K131" s="11" t="s">
@@ -8894,10 +8906,10 @@
         <v>28</v>
       </c>
       <c r="M131" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N131" s="11" t="s">
-        <v>424</v>
+        <v>398</v>
       </c>
       <c r="O131" s="11" t="s">
         <v>28</v>
@@ -8906,7 +8918,7 @@
         <v>28</v>
       </c>
       <c r="Q131" s="11" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="R131" s="11"/>
       <c r="S131" s="11"/>
@@ -8915,19 +8927,19 @@
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B132" s="5">
-        <v>46091.59394065972</v>
+        <v>46133.792176840274</v>
       </c>
       <c r="C132" s="5">
-        <v>46133.70594085648</v>
+        <v>46134.63605664352</v>
       </c>
       <c r="D132" s="5">
-        <v>46133.7059553125</v>
+        <v>46134.63619297453</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="F132" s="6" t="s">
         <v>143</v>
@@ -8940,13 +8952,13 @@
       </c>
       <c r="I132" s="6"/>
       <c r="J132" s="5">
-        <v>46083</v>
+        <v>46112</v>
       </c>
       <c r="K132" s="6" t="s">
         <v>28</v>
       </c>
       <c r="L132" s="6" t="s">
-        <v>28</v>
+        <v>431</v>
       </c>
       <c r="M132" s="6" t="s">
         <v>0</v>
@@ -8961,14 +8973,14 @@
         <v>28</v>
       </c>
       <c r="Q132" s="6" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="R132" s="6"/>
       <c r="S132" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T132" s="16" t="s">
-        <v>115</v>
+      <c r="T132" s="12" t="s">
+        <v>433</v>
       </c>
       <c r="U132" s="6"/>
     </row>
@@ -8977,11 +8989,11 @@
         <v>434</v>
       </c>
       <c r="B133" s="10">
-        <v>46094.62533957176</v>
+        <v>46133.79263490741</v>
       </c>
       <c r="C133" s="11"/>
       <c r="D133" s="10">
-        <v>46133.70593778935</v>
+        <v>46133.79350961806</v>
       </c>
       <c r="E133" s="11" t="s">
         <v>435</v>
@@ -9005,7 +9017,7 @@
         <v>28</v>
       </c>
       <c r="N133" s="11" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="O133" s="11" t="s">
         <v>28</v>
@@ -9026,24 +9038,30 @@
         <v>437</v>
       </c>
       <c r="B134" s="5">
-        <v>46094.62542793981</v>
-      </c>
-      <c r="C134" s="6"/>
+        <v>46091.59394065972</v>
+      </c>
+      <c r="C134" s="5">
+        <v>46133.70594085648</v>
+      </c>
       <c r="D134" s="5">
-        <v>46133.70593837963</v>
+        <v>46133.7059553125</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>438</v>
       </c>
       <c r="F134" s="6" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G134" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H134" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H134" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I134" s="6"/>
-      <c r="J134" s="6"/>
+      <c r="J134" s="5">
+        <v>46083</v>
+      </c>
       <c r="K134" s="6" t="s">
         <v>28</v>
       </c>
@@ -9051,10 +9069,10 @@
         <v>28</v>
       </c>
       <c r="M134" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N134" s="6" t="s">
-        <v>432</v>
+        <v>28</v>
       </c>
       <c r="O134" s="6" t="s">
         <v>28</v>
@@ -9066,8 +9084,12 @@
         <v>439</v>
       </c>
       <c r="R134" s="6"/>
-      <c r="S134" s="6"/>
-      <c r="T134" s="6"/>
+      <c r="S134" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T134" s="16" t="s">
+        <v>115</v>
+      </c>
       <c r="U134" s="6"/>
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.25">
@@ -9075,11 +9097,11 @@
         <v>440</v>
       </c>
       <c r="B135" s="10">
-        <v>46094.62613793982</v>
+        <v>46094.62533957176</v>
       </c>
       <c r="C135" s="11"/>
       <c r="D135" s="10">
-        <v>46133.70593877315</v>
+        <v>46133.70593778935</v>
       </c>
       <c r="E135" s="11" t="s">
         <v>441</v>
@@ -9103,7 +9125,7 @@
         <v>28</v>
       </c>
       <c r="N135" s="11" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="O135" s="11" t="s">
         <v>28</v>
@@ -9124,11 +9146,11 @@
         <v>443</v>
       </c>
       <c r="B136" s="5">
-        <v>46094.626408703705</v>
+        <v>46094.62542793981</v>
       </c>
       <c r="C136" s="6"/>
       <c r="D136" s="5">
-        <v>46133.705939189815</v>
+        <v>46133.70593837963</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>444</v>
@@ -9152,7 +9174,7 @@
         <v>28</v>
       </c>
       <c r="N136" s="6" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="O136" s="6" t="s">
         <v>28</v>
@@ -9173,11 +9195,11 @@
         <v>446</v>
       </c>
       <c r="B137" s="10">
-        <v>46094.62648922454</v>
+        <v>46094.62613793982</v>
       </c>
       <c r="C137" s="11"/>
       <c r="D137" s="10">
-        <v>46133.705939618056</v>
+        <v>46133.70593877315</v>
       </c>
       <c r="E137" s="11" t="s">
         <v>447</v>
@@ -9201,7 +9223,7 @@
         <v>28</v>
       </c>
       <c r="N137" s="11" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="O137" s="11" t="s">
         <v>28</v>
@@ -9222,11 +9244,11 @@
         <v>449</v>
       </c>
       <c r="B138" s="5">
-        <v>46094.62660908565</v>
+        <v>46094.626408703705</v>
       </c>
       <c r="C138" s="6"/>
       <c r="D138" s="5">
-        <v>46133.7059399537</v>
+        <v>46133.705939189815</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>450</v>
@@ -9250,7 +9272,7 @@
         <v>28</v>
       </c>
       <c r="N138" s="6" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="O138" s="6" t="s">
         <v>28</v>
@@ -9271,11 +9293,11 @@
         <v>452</v>
       </c>
       <c r="B139" s="10">
-        <v>46094.626713460646</v>
+        <v>46094.62648922454</v>
       </c>
       <c r="C139" s="11"/>
       <c r="D139" s="10">
-        <v>46133.705940300926</v>
+        <v>46133.705939618056</v>
       </c>
       <c r="E139" s="11" t="s">
         <v>453</v>
@@ -9299,7 +9321,7 @@
         <v>28</v>
       </c>
       <c r="N139" s="11" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="O139" s="11" t="s">
         <v>28</v>
@@ -9320,11 +9342,11 @@
         <v>455</v>
       </c>
       <c r="B140" s="5">
-        <v>46094.62680802083</v>
+        <v>46094.62660908565</v>
       </c>
       <c r="C140" s="6"/>
       <c r="D140" s="5">
-        <v>46133.70594064815</v>
+        <v>46133.7059399537</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>456</v>
@@ -9348,7 +9370,7 @@
         <v>28</v>
       </c>
       <c r="N140" s="6" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="O140" s="6" t="s">
         <v>28</v>
@@ -9369,26 +9391,22 @@
         <v>458</v>
       </c>
       <c r="B141" s="10">
-        <v>46093.55797592593</v>
-      </c>
-      <c r="C141" s="10">
-        <v>46127.87503005787</v>
-      </c>
+        <v>46094.626713460646</v>
+      </c>
+      <c r="C141" s="11"/>
       <c r="D141" s="10">
-        <v>46134.66330939815</v>
+        <v>46133.705940300926</v>
       </c>
       <c r="E141" s="11" t="s">
         <v>459</v>
       </c>
       <c r="F141" s="11" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G141" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H141" s="11" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H141" s="11"/>
       <c r="I141" s="11"/>
       <c r="J141" s="11"/>
       <c r="K141" s="11" t="s">
@@ -9398,10 +9416,10 @@
         <v>28</v>
       </c>
       <c r="M141" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N141" s="11" t="s">
-        <v>28</v>
+        <v>438</v>
       </c>
       <c r="O141" s="11" t="s">
         <v>28</v>
@@ -9422,26 +9440,22 @@
         <v>461</v>
       </c>
       <c r="B142" s="5">
-        <v>46094.63474699074</v>
-      </c>
-      <c r="C142" s="5">
-        <v>46127.875013819445</v>
-      </c>
+        <v>46094.62680802083</v>
+      </c>
+      <c r="C142" s="6"/>
       <c r="D142" s="5">
-        <v>46134.66345291666</v>
+        <v>46133.70594064815</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>462</v>
       </c>
       <c r="F142" s="6" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G142" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H142" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H142" s="6"/>
       <c r="I142" s="6"/>
       <c r="J142" s="6"/>
       <c r="K142" s="6" t="s">
@@ -9451,10 +9465,10 @@
         <v>28</v>
       </c>
       <c r="M142" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N142" s="6" t="s">
-        <v>459</v>
+        <v>438</v>
       </c>
       <c r="O142" s="6" t="s">
         <v>28</v>
@@ -9475,13 +9489,13 @@
         <v>464</v>
       </c>
       <c r="B143" s="10">
-        <v>46093.557976111115</v>
+        <v>46093.55797592593</v>
       </c>
       <c r="C143" s="10">
-        <v>46111.836577766204</v>
+        <v>46127.87503005787</v>
       </c>
       <c r="D143" s="10">
-        <v>46111.836592141204</v>
+        <v>46134.66330939815</v>
       </c>
       <c r="E143" s="11" t="s">
         <v>465</v>
@@ -9495,12 +9509,8 @@
       <c r="H143" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I143" s="10">
-        <v>46003</v>
-      </c>
-      <c r="J143" s="10">
-        <v>46003</v>
-      </c>
+      <c r="I143" s="11"/>
+      <c r="J143" s="11"/>
       <c r="K143" s="11" t="s">
         <v>28</v>
       </c>
@@ -9523,12 +9533,8 @@
         <v>466</v>
       </c>
       <c r="R143" s="11"/>
-      <c r="S143" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T143" s="17" t="s">
-        <v>128</v>
-      </c>
+      <c r="S143" s="11"/>
+      <c r="T143" s="11"/>
       <c r="U143" s="11"/>
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.25">
@@ -9536,13 +9542,13 @@
         <v>467</v>
       </c>
       <c r="B144" s="5">
-        <v>46094.57571935185</v>
+        <v>46094.63474699074</v>
       </c>
       <c r="C144" s="5">
-        <v>46111.83654524306</v>
+        <v>46127.875013819445</v>
       </c>
       <c r="D144" s="5">
-        <v>46111.83656112268</v>
+        <v>46134.66345291666</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>468</v>
@@ -9551,9 +9557,11 @@
         <v>143</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H144" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H144" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I144" s="6"/>
       <c r="J144" s="6"/>
       <c r="K144" s="6" t="s">
@@ -9587,13 +9595,13 @@
         <v>470</v>
       </c>
       <c r="B145" s="10">
-        <v>46094.57601390046</v>
+        <v>46093.557976111115</v>
       </c>
       <c r="C145" s="10">
-        <v>46111.8365590162</v>
+        <v>46111.836577766204</v>
       </c>
       <c r="D145" s="10">
-        <v>46111.83657758102</v>
+        <v>46111.836592141204</v>
       </c>
       <c r="E145" s="11" t="s">
         <v>471</v>
@@ -9602,11 +9610,17 @@
         <v>143</v>
       </c>
       <c r="G145" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H145" s="11"/>
-      <c r="I145" s="11"/>
-      <c r="J145" s="11"/>
+        <v>57</v>
+      </c>
+      <c r="H145" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="I145" s="10">
+        <v>46003</v>
+      </c>
+      <c r="J145" s="10">
+        <v>46003</v>
+      </c>
       <c r="K145" s="11" t="s">
         <v>28</v>
       </c>
@@ -9617,7 +9631,7 @@
         <v>0</v>
       </c>
       <c r="N145" s="11" t="s">
-        <v>465</v>
+        <v>28</v>
       </c>
       <c r="O145" s="11" t="s">
         <v>28</v>
@@ -9629,8 +9643,12 @@
         <v>472</v>
       </c>
       <c r="R145" s="11"/>
-      <c r="S145" s="11"/>
-      <c r="T145" s="11"/>
+      <c r="S145" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T145" s="17" t="s">
+        <v>128</v>
+      </c>
       <c r="U145" s="11"/>
     </row>
     <row r="146" spans="1:21" x14ac:dyDescent="0.25">
@@ -9638,13 +9656,13 @@
         <v>473</v>
       </c>
       <c r="B146" s="5">
-        <v>46094.57620418981</v>
+        <v>46094.57571935185</v>
       </c>
       <c r="C146" s="5">
-        <v>46111.83657327546</v>
+        <v>46111.83654524306</v>
       </c>
       <c r="D146" s="5">
-        <v>46111.83659253472</v>
+        <v>46111.83656112268</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>474</v>
@@ -9668,7 +9686,7 @@
         <v>0</v>
       </c>
       <c r="N146" s="6" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="O146" s="6" t="s">
         <v>28</v>
@@ -9689,13 +9707,13 @@
         <v>476</v>
       </c>
       <c r="B147" s="10">
-        <v>46093.557975868054</v>
+        <v>46094.57601390046</v>
       </c>
       <c r="C147" s="10">
-        <v>46097.77705668981</v>
+        <v>46111.8365590162</v>
       </c>
       <c r="D147" s="10">
-        <v>46097.77707333333</v>
+        <v>46111.83657758102</v>
       </c>
       <c r="E147" s="11" t="s">
         <v>477</v>
@@ -9704,15 +9722,11 @@
         <v>143</v>
       </c>
       <c r="G147" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="H147" s="11" t="s">
-        <v>41</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H147" s="11"/>
       <c r="I147" s="11"/>
-      <c r="J147" s="10">
-        <v>46031</v>
-      </c>
+      <c r="J147" s="11"/>
       <c r="K147" s="11" t="s">
         <v>28</v>
       </c>
@@ -9723,7 +9737,7 @@
         <v>0</v>
       </c>
       <c r="N147" s="11" t="s">
-        <v>28</v>
+        <v>471</v>
       </c>
       <c r="O147" s="11" t="s">
         <v>28</v>
@@ -9735,12 +9749,8 @@
         <v>478</v>
       </c>
       <c r="R147" s="11"/>
-      <c r="S147" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T147" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="S147" s="11"/>
+      <c r="T147" s="11"/>
       <c r="U147" s="11"/>
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.25">
@@ -9748,13 +9758,13 @@
         <v>479</v>
       </c>
       <c r="B148" s="5">
-        <v>46094.57453506945</v>
+        <v>46094.57620418981</v>
       </c>
       <c r="C148" s="5">
-        <v>46097.77703761574</v>
+        <v>46111.83657327546</v>
       </c>
       <c r="D148" s="5">
-        <v>46097.77705638889</v>
+        <v>46111.83659253472</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>480</v>
@@ -9778,7 +9788,7 @@
         <v>0</v>
       </c>
       <c r="N148" s="6" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="O148" s="6" t="s">
         <v>28</v>
@@ -9793,6 +9803,116 @@
       <c r="S148" s="6"/>
       <c r="T148" s="6"/>
       <c r="U148" s="6"/>
+    </row>
+    <row r="149" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A149" s="9" t="s">
+        <v>482</v>
+      </c>
+      <c r="B149" s="10">
+        <v>46093.557975868054</v>
+      </c>
+      <c r="C149" s="10">
+        <v>46097.77705668981</v>
+      </c>
+      <c r="D149" s="10">
+        <v>46097.77707333333</v>
+      </c>
+      <c r="E149" s="11" t="s">
+        <v>483</v>
+      </c>
+      <c r="F149" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="G149" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H149" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="I149" s="11"/>
+      <c r="J149" s="10">
+        <v>46031</v>
+      </c>
+      <c r="K149" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="L149" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="M149" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="N149" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="O149" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="P149" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q149" s="11" t="s">
+        <v>484</v>
+      </c>
+      <c r="R149" s="11"/>
+      <c r="S149" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T149" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="U149" s="11"/>
+    </row>
+    <row r="150" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A150" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="B150" s="5">
+        <v>46094.57453506945</v>
+      </c>
+      <c r="C150" s="5">
+        <v>46097.77703761574</v>
+      </c>
+      <c r="D150" s="5">
+        <v>46097.77705638889</v>
+      </c>
+      <c r="E150" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="F150" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G150" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H150" s="6"/>
+      <c r="I150" s="6"/>
+      <c r="J150" s="6"/>
+      <c r="K150" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L150" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M150" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N150" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="O150" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P150" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q150" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="R150" s="6"/>
+      <c r="S150" s="6"/>
+      <c r="T150" s="6"/>
+      <c r="U150" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-30 15:39 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1802" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1779" uniqueCount="482">
   <si>
     <t>Tablero Servicios y mantención</t>
   </si>
@@ -452,24 +452,6 @@
   </si>
   <si>
     <t>TABL3-277</t>
-  </si>
-  <si>
-    <t>1216153465899953</t>
-  </si>
-  <si>
-    <t>50001568</t>
-  </si>
-  <si>
-    <t>TABL3-282</t>
-  </si>
-  <si>
-    <t>1216153465899956</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4366 -SENSOR DE BOMBEO PREMASGARD DS-205F </t>
-  </si>
-  <si>
-    <t>TABL3-283</t>
   </si>
   <si>
     <t>1214150417415442</t>
@@ -2060,7 +2042,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U150"/>
+  <dimension ref="A1:U148"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -4021,17 +4003,17 @@
         <v>145</v>
       </c>
       <c r="B39" s="10">
-        <v>46203.64108105324</v>
+        <v>46133.79734877315</v>
       </c>
       <c r="C39" s="11"/>
       <c r="D39" s="10">
-        <v>46203.641200439815</v>
+        <v>46141.74131788194</v>
       </c>
       <c r="E39" s="11" t="s">
         <v>146</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>25</v>
+        <v>147</v>
       </c>
       <c r="G39" s="11" t="s">
         <v>57</v>
@@ -4040,7 +4022,9 @@
         <v>58</v>
       </c>
       <c r="I39" s="11"/>
-      <c r="J39" s="11"/>
+      <c r="J39" s="10">
+        <v>46120</v>
+      </c>
       <c r="K39" s="11" t="s">
         <v>28</v>
       </c>
@@ -4060,26 +4044,30 @@
         <v>28</v>
       </c>
       <c r="Q39" s="11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="R39" s="11"/>
-      <c r="S39" s="11"/>
-      <c r="T39" s="11"/>
+      <c r="S39" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T39" s="17" t="s">
+        <v>128</v>
+      </c>
       <c r="U39" s="11"/>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B40" s="5">
-        <v>46203.64119756944</v>
+        <v>46133.79847596065</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46203.641513877315</v>
+        <v>46134.65975528935</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>28</v>
@@ -4089,9 +4077,7 @@
       </c>
       <c r="H40" s="6"/>
       <c r="I40" s="6"/>
-      <c r="J40" s="5">
-        <v>46206</v>
-      </c>
+      <c r="J40" s="6"/>
       <c r="K40" s="6" t="s">
         <v>28</v>
       </c>
@@ -4111,7 +4097,7 @@
         <v>28</v>
       </c>
       <c r="Q40" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="R40" s="6"/>
       <c r="S40" s="6"/>
@@ -4120,20 +4106,20 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B41" s="10">
-        <v>46133.79734877315</v>
+        <v>46133.800000937495</v>
       </c>
       <c r="C41" s="11"/>
       <c r="D41" s="10">
-        <v>46141.74131788194</v>
+        <v>46141.74254248843</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G41" s="11" t="s">
         <v>57</v>
@@ -4143,7 +4129,7 @@
       </c>
       <c r="I41" s="11"/>
       <c r="J41" s="10">
-        <v>46120</v>
+        <v>46234</v>
       </c>
       <c r="K41" s="11" t="s">
         <v>28</v>
@@ -4167,8 +4153,8 @@
         <v>154</v>
       </c>
       <c r="R41" s="11"/>
-      <c r="S41" s="12" t="s">
-        <v>43</v>
+      <c r="S41" s="14" t="s">
+        <v>51</v>
       </c>
       <c r="T41" s="17" t="s">
         <v>128</v>
@@ -4180,11 +4166,11 @@
         <v>155</v>
       </c>
       <c r="B42" s="5">
-        <v>46133.79847596065</v>
+        <v>46133.800366041665</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46134.65975528935</v>
+        <v>46133.800594699074</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>156</v>
@@ -4208,7 +4194,7 @@
         <v>28</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>28</v>
@@ -4229,17 +4215,17 @@
         <v>158</v>
       </c>
       <c r="B43" s="10">
-        <v>46133.800000937495</v>
+        <v>46093.55797671297</v>
       </c>
       <c r="C43" s="11"/>
       <c r="D43" s="10">
-        <v>46141.74254248843</v>
+        <v>46195.57757945602</v>
       </c>
       <c r="E43" s="11" t="s">
         <v>159</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="G43" s="11" t="s">
         <v>57</v>
@@ -4247,9 +4233,11 @@
       <c r="H43" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I43" s="11"/>
+      <c r="I43" s="10">
+        <v>46129</v>
+      </c>
       <c r="J43" s="10">
-        <v>46234</v>
+        <v>46129</v>
       </c>
       <c r="K43" s="11" t="s">
         <v>28</v>
@@ -4270,30 +4258,30 @@
         <v>28</v>
       </c>
       <c r="Q43" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R43" s="11"/>
-      <c r="S43" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="T43" s="17" t="s">
-        <v>128</v>
+      <c r="S43" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T43" s="16" t="s">
+        <v>115</v>
       </c>
       <c r="U43" s="11"/>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B44" s="5">
-        <v>46133.800366041665</v>
+        <v>46094.639967870375</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46133.800594699074</v>
+        <v>46130.18563101852</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>28</v>
@@ -4303,7 +4291,9 @@
       </c>
       <c r="H44" s="6"/>
       <c r="I44" s="6"/>
-      <c r="J44" s="6"/>
+      <c r="J44" s="5">
+        <v>46129</v>
+      </c>
       <c r="K44" s="6" t="s">
         <v>28</v>
       </c>
@@ -4323,41 +4313,39 @@
         <v>28</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R44" s="6"/>
-      <c r="S44" s="6"/>
+      <c r="S44" s="12" t="s">
+        <v>43</v>
+      </c>
       <c r="T44" s="6"/>
       <c r="U44" s="6"/>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B45" s="10">
-        <v>46093.55797671297</v>
+        <v>46094.64022527778</v>
       </c>
       <c r="C45" s="11"/>
       <c r="D45" s="10">
-        <v>46195.57757945602</v>
+        <v>46101.15093898148</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>166</v>
+        <v>28</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H45" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="I45" s="10">
-        <v>46129</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H45" s="11"/>
+      <c r="I45" s="11"/>
       <c r="J45" s="10">
-        <v>46129</v>
+        <v>46100</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>28</v>
@@ -4366,10 +4354,10 @@
         <v>28</v>
       </c>
       <c r="M45" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N45" s="11" t="s">
-        <v>28</v>
+        <v>159</v>
       </c>
       <c r="O45" s="11" t="s">
         <v>28</v>
@@ -4384,9 +4372,7 @@
       <c r="S45" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T45" s="16" t="s">
-        <v>115</v>
-      </c>
+      <c r="T45" s="11"/>
       <c r="U45" s="11"/>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
@@ -4394,25 +4380,27 @@
         <v>168</v>
       </c>
       <c r="B46" s="5">
-        <v>46094.639967870375</v>
+        <v>46133.81046972222</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46130.18563101852</v>
+        <v>46162.79059445602</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>169</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>28</v>
+        <v>160</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H46" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I46" s="6"/>
       <c r="J46" s="5">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="K46" s="6" t="s">
         <v>28</v>
@@ -4421,10 +4409,10 @@
         <v>28</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>165</v>
+        <v>28</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>28</v>
@@ -4436,10 +4424,12 @@
         <v>170</v>
       </c>
       <c r="R46" s="6"/>
-      <c r="S46" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T46" s="6"/>
+      <c r="S46" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="T46" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U46" s="6"/>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
@@ -4447,11 +4437,11 @@
         <v>171</v>
       </c>
       <c r="B47" s="10">
-        <v>46094.64022527778</v>
+        <v>46133.8107147338</v>
       </c>
       <c r="C47" s="11"/>
       <c r="D47" s="10">
-        <v>46101.15093898148</v>
+        <v>46133.81087918981</v>
       </c>
       <c r="E47" s="11" t="s">
         <v>172</v>
@@ -4464,9 +4454,7 @@
       </c>
       <c r="H47" s="11"/>
       <c r="I47" s="11"/>
-      <c r="J47" s="10">
-        <v>46100</v>
-      </c>
+      <c r="J47" s="11"/>
       <c r="K47" s="11" t="s">
         <v>28</v>
       </c>
@@ -4477,7 +4465,7 @@
         <v>28</v>
       </c>
       <c r="N47" s="11" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="O47" s="11" t="s">
         <v>28</v>
@@ -4489,9 +4477,7 @@
         <v>173</v>
       </c>
       <c r="R47" s="11"/>
-      <c r="S47" s="12" t="s">
-        <v>43</v>
-      </c>
+      <c r="S47" s="11"/>
       <c r="T47" s="11"/>
       <c r="U47" s="11"/>
     </row>
@@ -4500,17 +4486,17 @@
         <v>174</v>
       </c>
       <c r="B48" s="5">
-        <v>46133.81046972222</v>
+        <v>46133.80470612268</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46162.79059445602</v>
+        <v>46196.91581209491</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>175</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G48" s="6" t="s">
         <v>57</v>
@@ -4520,7 +4506,7 @@
       </c>
       <c r="I48" s="6"/>
       <c r="J48" s="5">
-        <v>46140</v>
+        <v>46161</v>
       </c>
       <c r="K48" s="6" t="s">
         <v>28</v>
@@ -4544,8 +4530,8 @@
         <v>176</v>
       </c>
       <c r="R48" s="6"/>
-      <c r="S48" s="14" t="s">
-        <v>51</v>
+      <c r="S48" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="T48" s="15" t="s">
         <v>72</v>
@@ -4557,11 +4543,11 @@
         <v>177</v>
       </c>
       <c r="B49" s="10">
-        <v>46133.8107147338</v>
+        <v>46133.80545771991</v>
       </c>
       <c r="C49" s="11"/>
       <c r="D49" s="10">
-        <v>46133.81087918981</v>
+        <v>46133.80564510416</v>
       </c>
       <c r="E49" s="11" t="s">
         <v>178</v>
@@ -4606,28 +4592,24 @@
         <v>180</v>
       </c>
       <c r="B50" s="5">
-        <v>46133.80470612268</v>
+        <v>46133.80570512731</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46196.91581209491</v>
+        <v>46133.80583366899</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>181</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>166</v>
+        <v>28</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H50" s="6"/>
       <c r="I50" s="6"/>
-      <c r="J50" s="5">
-        <v>46161</v>
-      </c>
+      <c r="J50" s="6"/>
       <c r="K50" s="6" t="s">
         <v>28</v>
       </c>
@@ -4635,10 +4617,10 @@
         <v>28</v>
       </c>
       <c r="M50" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>28</v>
+        <v>175</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>28</v>
@@ -4650,12 +4632,8 @@
         <v>182</v>
       </c>
       <c r="R50" s="6"/>
-      <c r="S50" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T50" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="S50" s="6"/>
+      <c r="T50" s="6"/>
       <c r="U50" s="6"/>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4663,11 +4641,11 @@
         <v>183</v>
       </c>
       <c r="B51" s="10">
-        <v>46133.80545771991</v>
+        <v>46133.8058850463</v>
       </c>
       <c r="C51" s="11"/>
       <c r="D51" s="10">
-        <v>46133.80564510416</v>
+        <v>46133.80636234954</v>
       </c>
       <c r="E51" s="11" t="s">
         <v>184</v>
@@ -4691,7 +4669,7 @@
         <v>28</v>
       </c>
       <c r="N51" s="11" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="O51" s="11" t="s">
         <v>28</v>
@@ -4712,11 +4690,11 @@
         <v>186</v>
       </c>
       <c r="B52" s="5">
-        <v>46133.80570512731</v>
+        <v>46133.80664880787</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46133.80583366899</v>
+        <v>46133.80681135417</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>187</v>
@@ -4740,7 +4718,7 @@
         <v>28</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>28</v>
@@ -4761,35 +4739,39 @@
         <v>189</v>
       </c>
       <c r="B53" s="10">
-        <v>46133.8058850463</v>
+        <v>46133.80701400463</v>
       </c>
       <c r="C53" s="11"/>
       <c r="D53" s="10">
-        <v>46133.80636234954</v>
+        <v>46162.79057355324</v>
       </c>
       <c r="E53" s="11" t="s">
         <v>190</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>28</v>
+        <v>160</v>
       </c>
       <c r="G53" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H53" s="11"/>
+        <v>57</v>
+      </c>
+      <c r="H53" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="I53" s="11"/>
-      <c r="J53" s="11"/>
+      <c r="J53" s="10">
+        <v>46122</v>
+      </c>
       <c r="K53" s="11" t="s">
         <v>28</v>
       </c>
       <c r="L53" s="11" t="s">
-        <v>28</v>
+        <v>191</v>
       </c>
       <c r="M53" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N53" s="11" t="s">
-        <v>181</v>
+        <v>28</v>
       </c>
       <c r="O53" s="11" t="s">
         <v>28</v>
@@ -4798,26 +4780,28 @@
         <v>28</v>
       </c>
       <c r="Q53" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="R53" s="11"/>
-      <c r="S53" s="11"/>
+      <c r="S53" s="12" t="s">
+        <v>43</v>
+      </c>
       <c r="T53" s="11"/>
       <c r="U53" s="11"/>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B54" s="5">
-        <v>46133.80664880787</v>
+        <v>46133.80727017361</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46133.80681135417</v>
+        <v>46133.80736961805</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>28</v>
@@ -4838,7 +4822,7 @@
         <v>28</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>28</v>
@@ -4847,7 +4831,7 @@
         <v>28</v>
       </c>
       <c r="Q54" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="R54" s="6"/>
       <c r="S54" s="6"/>
@@ -4856,20 +4840,20 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B55" s="10">
-        <v>46133.80701400463</v>
+        <v>46133.79901350694</v>
       </c>
       <c r="C55" s="11"/>
       <c r="D55" s="10">
-        <v>46162.79057355324</v>
+        <v>46162.79056252315</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G55" s="11" t="s">
         <v>57</v>
@@ -4879,13 +4863,13 @@
       </c>
       <c r="I55" s="11"/>
       <c r="J55" s="10">
-        <v>46122</v>
+        <v>46120</v>
       </c>
       <c r="K55" s="11" t="s">
         <v>28</v>
       </c>
       <c r="L55" s="11" t="s">
-        <v>197</v>
+        <v>28</v>
       </c>
       <c r="M55" s="11" t="s">
         <v>0</v>
@@ -4906,7 +4890,9 @@
       <c r="S55" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T55" s="11"/>
+      <c r="T55" s="17" t="s">
+        <v>128</v>
+      </c>
       <c r="U55" s="11"/>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
@@ -4914,11 +4900,11 @@
         <v>199</v>
       </c>
       <c r="B56" s="5">
-        <v>46133.80727017361</v>
+        <v>46133.79961443287</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46133.80736961805</v>
+        <v>46133.79989851852</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>200</v>
@@ -4942,7 +4928,7 @@
         <v>28</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>28</v>
@@ -4963,17 +4949,17 @@
         <v>202</v>
       </c>
       <c r="B57" s="10">
-        <v>46133.79901350694</v>
+        <v>46093.557977812496</v>
       </c>
       <c r="C57" s="11"/>
       <c r="D57" s="10">
-        <v>46162.79056252315</v>
+        <v>46162.79054756944</v>
       </c>
       <c r="E57" s="11" t="s">
         <v>203</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G57" s="11" t="s">
         <v>57</v>
@@ -4983,7 +4969,7 @@
       </c>
       <c r="I57" s="11"/>
       <c r="J57" s="10">
-        <v>46120</v>
+        <v>46039</v>
       </c>
       <c r="K57" s="11" t="s">
         <v>28</v>
@@ -5010,8 +4996,8 @@
       <c r="S57" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T57" s="17" t="s">
-        <v>128</v>
+      <c r="T57" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="U57" s="11"/>
     </row>
@@ -5020,11 +5006,11 @@
         <v>205</v>
       </c>
       <c r="B58" s="5">
-        <v>46133.79961443287</v>
+        <v>46094.64358574074</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46133.79989851852</v>
+        <v>46094.643782430554</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>206</v>
@@ -5069,17 +5055,17 @@
         <v>208</v>
       </c>
       <c r="B59" s="10">
-        <v>46093.557977812496</v>
+        <v>46093.55797666666</v>
       </c>
       <c r="C59" s="11"/>
       <c r="D59" s="10">
-        <v>46162.79054756944</v>
+        <v>46162.790523668984</v>
       </c>
       <c r="E59" s="11" t="s">
         <v>209</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G59" s="11" t="s">
         <v>57</v>
@@ -5089,7 +5075,7 @@
       </c>
       <c r="I59" s="11"/>
       <c r="J59" s="10">
-        <v>46039</v>
+        <v>46083</v>
       </c>
       <c r="K59" s="11" t="s">
         <v>28</v>
@@ -5126,11 +5112,11 @@
         <v>211</v>
       </c>
       <c r="B60" s="5">
-        <v>46094.64358574074</v>
+        <v>46094.64611630787</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46094.643782430554</v>
+        <v>46094.64631732639</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>212</v>
@@ -5175,28 +5161,24 @@
         <v>214</v>
       </c>
       <c r="B61" s="10">
-        <v>46093.55797666666</v>
+        <v>46094.64632454861</v>
       </c>
       <c r="C61" s="11"/>
       <c r="D61" s="10">
-        <v>46162.790523668984</v>
+        <v>46094.64655788195</v>
       </c>
       <c r="E61" s="11" t="s">
         <v>215</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>166</v>
+        <v>28</v>
       </c>
       <c r="G61" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H61" s="11" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H61" s="11"/>
       <c r="I61" s="11"/>
-      <c r="J61" s="10">
-        <v>46083</v>
-      </c>
+      <c r="J61" s="11"/>
       <c r="K61" s="11" t="s">
         <v>28</v>
       </c>
@@ -5204,10 +5186,10 @@
         <v>28</v>
       </c>
       <c r="M61" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N61" s="11" t="s">
-        <v>28</v>
+        <v>209</v>
       </c>
       <c r="O61" s="11" t="s">
         <v>28</v>
@@ -5219,12 +5201,8 @@
         <v>216</v>
       </c>
       <c r="R61" s="11"/>
-      <c r="S61" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T61" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="S61" s="11"/>
+      <c r="T61" s="11"/>
       <c r="U61" s="11"/>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5232,24 +5210,28 @@
         <v>217</v>
       </c>
       <c r="B62" s="5">
-        <v>46094.64611630787</v>
+        <v>46093.55797637731</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46094.64631732639</v>
+        <v>46162.79050667824</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>218</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>28</v>
+        <v>160</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H62" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H62" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I62" s="6"/>
-      <c r="J62" s="6"/>
+      <c r="J62" s="5">
+        <v>46080</v>
+      </c>
       <c r="K62" s="6" t="s">
         <v>28</v>
       </c>
@@ -5257,10 +5239,10 @@
         <v>28</v>
       </c>
       <c r="M62" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>215</v>
+        <v>28</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>28</v>
@@ -5272,8 +5254,12 @@
         <v>219</v>
       </c>
       <c r="R62" s="6"/>
-      <c r="S62" s="6"/>
-      <c r="T62" s="6"/>
+      <c r="S62" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T62" s="17" t="s">
+        <v>128</v>
+      </c>
       <c r="U62" s="6"/>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -5281,11 +5267,11 @@
         <v>220</v>
       </c>
       <c r="B63" s="10">
-        <v>46094.64632454861</v>
+        <v>46094.645434618054</v>
       </c>
       <c r="C63" s="11"/>
       <c r="D63" s="10">
-        <v>46094.64655788195</v>
+        <v>46094.645602916666</v>
       </c>
       <c r="E63" s="11" t="s">
         <v>221</v>
@@ -5309,7 +5295,7 @@
         <v>28</v>
       </c>
       <c r="N63" s="11" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="O63" s="11" t="s">
         <v>28</v>
@@ -5330,17 +5316,17 @@
         <v>223</v>
       </c>
       <c r="B64" s="5">
-        <v>46093.55797637731</v>
+        <v>46093.55797821759</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46162.79050667824</v>
+        <v>46162.79049341435</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>224</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G64" s="6" t="s">
         <v>57</v>
@@ -5350,7 +5336,7 @@
       </c>
       <c r="I64" s="6"/>
       <c r="J64" s="5">
-        <v>46080</v>
+        <v>46092</v>
       </c>
       <c r="K64" s="6" t="s">
         <v>28</v>
@@ -5377,8 +5363,8 @@
       <c r="S64" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T64" s="17" t="s">
-        <v>128</v>
+      <c r="T64" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="U64" s="6"/>
     </row>
@@ -5387,11 +5373,11 @@
         <v>226</v>
       </c>
       <c r="B65" s="10">
-        <v>46094.645434618054</v>
+        <v>46094.65140127315</v>
       </c>
       <c r="C65" s="11"/>
       <c r="D65" s="10">
-        <v>46094.645602916666</v>
+        <v>46094.65150827546</v>
       </c>
       <c r="E65" s="11" t="s">
         <v>227</v>
@@ -5436,17 +5422,17 @@
         <v>229</v>
       </c>
       <c r="B66" s="5">
-        <v>46093.55797821759</v>
+        <v>46093.557976192125</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46162.79049341435</v>
+        <v>46142.16936487269</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>230</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G66" s="6" t="s">
         <v>57</v>
@@ -5456,7 +5442,7 @@
       </c>
       <c r="I66" s="6"/>
       <c r="J66" s="5">
-        <v>46092</v>
+        <v>46142</v>
       </c>
       <c r="K66" s="6" t="s">
         <v>28</v>
@@ -5480,27 +5466,27 @@
         <v>231</v>
       </c>
       <c r="R66" s="6"/>
-      <c r="S66" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T66" s="15" t="s">
-        <v>72</v>
+      <c r="S66" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T66" s="17" t="s">
+        <v>232</v>
       </c>
       <c r="U66" s="6"/>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B67" s="10">
-        <v>46094.65140127315</v>
+        <v>46094.63540701389</v>
       </c>
       <c r="C67" s="11"/>
       <c r="D67" s="10">
-        <v>46094.65150827546</v>
+        <v>46094.63563651621</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F67" s="11" t="s">
         <v>28</v>
@@ -5530,7 +5516,7 @@
         <v>28</v>
       </c>
       <c r="Q67" s="11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="R67" s="11"/>
       <c r="S67" s="11"/>
@@ -5539,30 +5525,30 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B68" s="5">
-        <v>46093.557976192125</v>
+        <v>46093.55797792824</v>
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46142.16936487269</v>
+        <v>46134.689549421295</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="I68" s="6"/>
       <c r="J68" s="5">
-        <v>46142</v>
+        <v>46097</v>
       </c>
       <c r="K68" s="6" t="s">
         <v>28</v>
@@ -5583,14 +5569,14 @@
         <v>28</v>
       </c>
       <c r="Q68" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="R68" s="6"/>
-      <c r="S68" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T68" s="17" t="s">
-        <v>238</v>
+      <c r="S68" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T68" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="U68" s="6"/>
     </row>
@@ -5599,11 +5585,11 @@
         <v>239</v>
       </c>
       <c r="B69" s="10">
-        <v>46094.63540701389</v>
+        <v>46094.64988140046</v>
       </c>
       <c r="C69" s="11"/>
       <c r="D69" s="10">
-        <v>46094.63563651621</v>
+        <v>46094.64998811342</v>
       </c>
       <c r="E69" s="11" t="s">
         <v>240</v>
@@ -5627,7 +5613,7 @@
         <v>28</v>
       </c>
       <c r="N69" s="11" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="O69" s="11" t="s">
         <v>28</v>
@@ -5648,17 +5634,17 @@
         <v>242</v>
       </c>
       <c r="B70" s="5">
-        <v>46093.55797792824</v>
+        <v>46093.55797513889</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46134.689549421295</v>
+        <v>46098.62589137732</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>243</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G70" s="6" t="s">
         <v>26</v>
@@ -5666,9 +5652,11 @@
       <c r="H70" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="I70" s="6"/>
+      <c r="I70" s="5">
+        <v>46041</v>
+      </c>
       <c r="J70" s="5">
-        <v>46097</v>
+        <v>46041</v>
       </c>
       <c r="K70" s="6" t="s">
         <v>28</v>
@@ -5695,8 +5683,8 @@
       <c r="S70" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T70" s="15" t="s">
-        <v>72</v>
+      <c r="T70" s="17" t="s">
+        <v>232</v>
       </c>
       <c r="U70" s="6"/>
     </row>
@@ -5705,11 +5693,11 @@
         <v>245</v>
       </c>
       <c r="B71" s="10">
-        <v>46094.64988140046</v>
+        <v>46094.566601597224</v>
       </c>
       <c r="C71" s="11"/>
       <c r="D71" s="10">
-        <v>46094.64998811342</v>
+        <v>46094.56736538194</v>
       </c>
       <c r="E71" s="11" t="s">
         <v>246</v>
@@ -5754,30 +5742,24 @@
         <v>248</v>
       </c>
       <c r="B72" s="5">
-        <v>46093.55797513889</v>
+        <v>46094.566937951386</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46098.62589137732</v>
+        <v>46094.56773407407</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>249</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>166</v>
+        <v>28</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="I72" s="5">
-        <v>46041</v>
-      </c>
-      <c r="J72" s="5">
-        <v>46041</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H72" s="6"/>
+      <c r="I72" s="6"/>
+      <c r="J72" s="6"/>
       <c r="K72" s="6" t="s">
         <v>28</v>
       </c>
@@ -5785,10 +5767,10 @@
         <v>28</v>
       </c>
       <c r="M72" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>28</v>
+        <v>243</v>
       </c>
       <c r="O72" s="6" t="s">
         <v>28</v>
@@ -5800,12 +5782,8 @@
         <v>250</v>
       </c>
       <c r="R72" s="6"/>
-      <c r="S72" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T72" s="17" t="s">
-        <v>238</v>
-      </c>
+      <c r="S72" s="6"/>
+      <c r="T72" s="6"/>
       <c r="U72" s="6"/>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5813,11 +5791,11 @@
         <v>251</v>
       </c>
       <c r="B73" s="10">
-        <v>46094.566601597224</v>
+        <v>46094.56748170139</v>
       </c>
       <c r="C73" s="11"/>
       <c r="D73" s="10">
-        <v>46094.56736538194</v>
+        <v>46094.56795886574</v>
       </c>
       <c r="E73" s="11" t="s">
         <v>252</v>
@@ -5841,7 +5819,7 @@
         <v>28</v>
       </c>
       <c r="N73" s="11" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="O73" s="11" t="s">
         <v>28</v>
@@ -5862,11 +5840,11 @@
         <v>254</v>
       </c>
       <c r="B74" s="5">
-        <v>46094.566937951386</v>
+        <v>46094.56796667824</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46094.56773407407</v>
+        <v>46094.56820407408</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>255</v>
@@ -5890,7 +5868,7 @@
         <v>28</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="O74" s="6" t="s">
         <v>28</v>
@@ -5911,24 +5889,30 @@
         <v>257</v>
       </c>
       <c r="B75" s="10">
-        <v>46094.56748170139</v>
+        <v>46093.557975625</v>
       </c>
       <c r="C75" s="11"/>
       <c r="D75" s="10">
-        <v>46094.56795886574</v>
+        <v>46112.84178105324</v>
       </c>
       <c r="E75" s="11" t="s">
         <v>258</v>
       </c>
       <c r="F75" s="11" t="s">
-        <v>28</v>
+        <v>160</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H75" s="11"/>
-      <c r="I75" s="11"/>
-      <c r="J75" s="11"/>
+        <v>26</v>
+      </c>
+      <c r="H75" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I75" s="10">
+        <v>46041</v>
+      </c>
+      <c r="J75" s="10">
+        <v>46041</v>
+      </c>
       <c r="K75" s="11" t="s">
         <v>28</v>
       </c>
@@ -5936,10 +5920,10 @@
         <v>28</v>
       </c>
       <c r="M75" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N75" s="11" t="s">
-        <v>249</v>
+        <v>28</v>
       </c>
       <c r="O75" s="11" t="s">
         <v>28</v>
@@ -5951,8 +5935,12 @@
         <v>259</v>
       </c>
       <c r="R75" s="11"/>
-      <c r="S75" s="11"/>
-      <c r="T75" s="11"/>
+      <c r="S75" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T75" s="17" t="s">
+        <v>232</v>
+      </c>
       <c r="U75" s="11"/>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -5960,11 +5948,11 @@
         <v>260</v>
       </c>
       <c r="B76" s="5">
-        <v>46094.56796667824</v>
+        <v>46094.57064802083</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46094.56820407408</v>
+        <v>46094.59020585648</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>261</v>
@@ -5988,7 +5976,7 @@
         <v>28</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="O76" s="6" t="s">
         <v>28</v>
@@ -6009,30 +5997,24 @@
         <v>263</v>
       </c>
       <c r="B77" s="10">
-        <v>46093.557975625</v>
+        <v>46094.57343428241</v>
       </c>
       <c r="C77" s="11"/>
       <c r="D77" s="10">
-        <v>46112.84178105324</v>
+        <v>46094.59023394676</v>
       </c>
       <c r="E77" s="11" t="s">
         <v>264</v>
       </c>
       <c r="F77" s="11" t="s">
-        <v>166</v>
+        <v>28</v>
       </c>
       <c r="G77" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H77" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="I77" s="10">
-        <v>46041</v>
-      </c>
-      <c r="J77" s="10">
-        <v>46041</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H77" s="11"/>
+      <c r="I77" s="11"/>
+      <c r="J77" s="11"/>
       <c r="K77" s="11" t="s">
         <v>28</v>
       </c>
@@ -6040,10 +6022,10 @@
         <v>28</v>
       </c>
       <c r="M77" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N77" s="11" t="s">
-        <v>28</v>
+        <v>258</v>
       </c>
       <c r="O77" s="11" t="s">
         <v>28</v>
@@ -6055,12 +6037,8 @@
         <v>265</v>
       </c>
       <c r="R77" s="11"/>
-      <c r="S77" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T77" s="17" t="s">
-        <v>238</v>
-      </c>
+      <c r="S77" s="11"/>
+      <c r="T77" s="11"/>
       <c r="U77" s="11"/>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
@@ -6068,11 +6046,11 @@
         <v>266</v>
       </c>
       <c r="B78" s="5">
-        <v>46094.57064802083</v>
+        <v>46094.573594710644</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46094.59020585648</v>
+        <v>46094.59026199074</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>267</v>
@@ -6096,7 +6074,7 @@
         <v>28</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="O78" s="6" t="s">
         <v>28</v>
@@ -6117,11 +6095,11 @@
         <v>269</v>
       </c>
       <c r="B79" s="10">
-        <v>46094.57343428241</v>
+        <v>46094.57373981482</v>
       </c>
       <c r="C79" s="11"/>
       <c r="D79" s="10">
-        <v>46094.59023394676</v>
+        <v>46094.59030239584</v>
       </c>
       <c r="E79" s="11" t="s">
         <v>270</v>
@@ -6145,7 +6123,7 @@
         <v>28</v>
       </c>
       <c r="N79" s="11" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="O79" s="11" t="s">
         <v>28</v>
@@ -6166,11 +6144,11 @@
         <v>272</v>
       </c>
       <c r="B80" s="5">
-        <v>46094.573594710644</v>
+        <v>46094.573880254626</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46094.59026199074</v>
+        <v>46094.59033287037</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>273</v>
@@ -6194,7 +6172,7 @@
         <v>28</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="O80" s="6" t="s">
         <v>28</v>
@@ -6215,24 +6193,28 @@
         <v>275</v>
       </c>
       <c r="B81" s="10">
-        <v>46094.57373981482</v>
+        <v>46093.55797761574</v>
       </c>
       <c r="C81" s="11"/>
       <c r="D81" s="10">
-        <v>46094.59030239584</v>
+        <v>46099.63241893519</v>
       </c>
       <c r="E81" s="11" t="s">
         <v>276</v>
       </c>
       <c r="F81" s="11" t="s">
-        <v>28</v>
+        <v>160</v>
       </c>
       <c r="G81" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H81" s="11"/>
+        <v>26</v>
+      </c>
+      <c r="H81" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="I81" s="11"/>
-      <c r="J81" s="11"/>
+      <c r="J81" s="10">
+        <v>46092</v>
+      </c>
       <c r="K81" s="11" t="s">
         <v>28</v>
       </c>
@@ -6240,10 +6222,10 @@
         <v>28</v>
       </c>
       <c r="M81" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N81" s="11" t="s">
-        <v>264</v>
+        <v>28</v>
       </c>
       <c r="O81" s="11" t="s">
         <v>28</v>
@@ -6255,8 +6237,12 @@
         <v>277</v>
       </c>
       <c r="R81" s="11"/>
-      <c r="S81" s="11"/>
-      <c r="T81" s="11"/>
+      <c r="S81" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T81" s="17" t="s">
+        <v>232</v>
+      </c>
       <c r="U81" s="11"/>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -6264,17 +6250,17 @@
         <v>278</v>
       </c>
       <c r="B82" s="5">
-        <v>46094.573880254626</v>
+        <v>46094.65047047454</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46094.59033287037</v>
+        <v>46111.83610230324</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>279</v>
       </c>
       <c r="F82" s="6" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G82" s="6" t="s">
         <v>28</v>
@@ -6289,10 +6275,10 @@
         <v>28</v>
       </c>
       <c r="M82" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="O82" s="6" t="s">
         <v>28</v>
@@ -6313,28 +6299,24 @@
         <v>281</v>
       </c>
       <c r="B83" s="10">
-        <v>46093.55797761574</v>
+        <v>46094.65072855324</v>
       </c>
       <c r="C83" s="11"/>
       <c r="D83" s="10">
-        <v>46099.63241893519</v>
+        <v>46094.65083585648</v>
       </c>
       <c r="E83" s="11" t="s">
         <v>282</v>
       </c>
       <c r="F83" s="11" t="s">
-        <v>166</v>
+        <v>28</v>
       </c>
       <c r="G83" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H83" s="11" t="s">
-        <v>27</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H83" s="11"/>
       <c r="I83" s="11"/>
-      <c r="J83" s="10">
-        <v>46092</v>
-      </c>
+      <c r="J83" s="11"/>
       <c r="K83" s="11" t="s">
         <v>28</v>
       </c>
@@ -6342,10 +6324,10 @@
         <v>28</v>
       </c>
       <c r="M83" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N83" s="11" t="s">
-        <v>28</v>
+        <v>276</v>
       </c>
       <c r="O83" s="11" t="s">
         <v>28</v>
@@ -6357,12 +6339,8 @@
         <v>283</v>
       </c>
       <c r="R83" s="11"/>
-      <c r="S83" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T83" s="17" t="s">
-        <v>238</v>
-      </c>
+      <c r="S83" s="11"/>
+      <c r="T83" s="11"/>
       <c r="U83" s="11"/>
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
@@ -6370,17 +6348,17 @@
         <v>284</v>
       </c>
       <c r="B84" s="5">
-        <v>46094.65047047454</v>
+        <v>46094.650843634256</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46111.83610230324</v>
+        <v>46094.65119138889</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>285</v>
       </c>
       <c r="F84" s="6" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G84" s="6" t="s">
         <v>28</v>
@@ -6395,10 +6373,10 @@
         <v>28</v>
       </c>
       <c r="M84" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="O84" s="6" t="s">
         <v>28</v>
@@ -6419,11 +6397,11 @@
         <v>287</v>
       </c>
       <c r="B85" s="10">
-        <v>46094.65072855324</v>
+        <v>46094.65095365741</v>
       </c>
       <c r="C85" s="11"/>
       <c r="D85" s="10">
-        <v>46094.65083585648</v>
+        <v>46094.65121894676</v>
       </c>
       <c r="E85" s="11" t="s">
         <v>288</v>
@@ -6447,7 +6425,7 @@
         <v>28</v>
       </c>
       <c r="N85" s="11" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="O85" s="11" t="s">
         <v>28</v>
@@ -6468,24 +6446,28 @@
         <v>290</v>
       </c>
       <c r="B86" s="5">
-        <v>46094.650843634256</v>
+        <v>46093.557977268516</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46094.65119138889</v>
+        <v>46099.639211539354</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>291</v>
       </c>
       <c r="F86" s="6" t="s">
-        <v>28</v>
+        <v>160</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H86" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H86" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I86" s="6"/>
-      <c r="J86" s="6"/>
+      <c r="J86" s="5">
+        <v>46083</v>
+      </c>
       <c r="K86" s="6" t="s">
         <v>28</v>
       </c>
@@ -6493,10 +6475,10 @@
         <v>28</v>
       </c>
       <c r="M86" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>282</v>
+        <v>28</v>
       </c>
       <c r="O86" s="6" t="s">
         <v>28</v>
@@ -6508,8 +6490,12 @@
         <v>292</v>
       </c>
       <c r="R86" s="6"/>
-      <c r="S86" s="6"/>
-      <c r="T86" s="6"/>
+      <c r="S86" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T86" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U86" s="6"/>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -6517,11 +6503,11 @@
         <v>293</v>
       </c>
       <c r="B87" s="10">
-        <v>46094.65095365741</v>
+        <v>46094.64259225695</v>
       </c>
       <c r="C87" s="11"/>
       <c r="D87" s="10">
-        <v>46094.65121894676</v>
+        <v>46094.642785069445</v>
       </c>
       <c r="E87" s="11" t="s">
         <v>294</v>
@@ -6545,7 +6531,7 @@
         <v>28</v>
       </c>
       <c r="N87" s="11" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="O87" s="11" t="s">
         <v>28</v>
@@ -6566,27 +6552,27 @@
         <v>296</v>
       </c>
       <c r="B88" s="5">
-        <v>46093.557977268516</v>
+        <v>46093.55797850694</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46099.639211539354</v>
+        <v>46099.62486652778</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>297</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="I88" s="6"/>
       <c r="J88" s="5">
-        <v>46083</v>
+        <v>46092</v>
       </c>
       <c r="K88" s="6" t="s">
         <v>28</v>
@@ -6613,8 +6599,8 @@
       <c r="S88" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T88" s="15" t="s">
-        <v>72</v>
+      <c r="T88" s="17" t="s">
+        <v>232</v>
       </c>
       <c r="U88" s="6"/>
     </row>
@@ -6623,11 +6609,11 @@
         <v>299</v>
       </c>
       <c r="B89" s="10">
-        <v>46094.64259225695</v>
+        <v>46094.65201979167</v>
       </c>
       <c r="C89" s="11"/>
       <c r="D89" s="10">
-        <v>46094.642785069445</v>
+        <v>46094.652139756945</v>
       </c>
       <c r="E89" s="11" t="s">
         <v>300</v>
@@ -6672,27 +6658,27 @@
         <v>302</v>
       </c>
       <c r="B90" s="5">
-        <v>46093.55797850694</v>
+        <v>46093.55797699074</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46099.62486652778</v>
+        <v>46134.66246857639</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>303</v>
       </c>
       <c r="F90" s="6" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="5">
-        <v>46092</v>
+        <v>46094</v>
       </c>
       <c r="K90" s="6" t="s">
         <v>28</v>
@@ -6719,9 +6705,7 @@
       <c r="S90" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T90" s="17" t="s">
-        <v>238</v>
-      </c>
+      <c r="T90" s="6"/>
       <c r="U90" s="6"/>
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
@@ -6729,11 +6713,11 @@
         <v>305</v>
       </c>
       <c r="B91" s="10">
-        <v>46094.65201979167</v>
+        <v>46094.64671800926</v>
       </c>
       <c r="C91" s="11"/>
       <c r="D91" s="10">
-        <v>46094.652139756945</v>
+        <v>46094.64682403935</v>
       </c>
       <c r="E91" s="11" t="s">
         <v>306</v>
@@ -6778,17 +6762,17 @@
         <v>308</v>
       </c>
       <c r="B92" s="5">
-        <v>46093.55797699074</v>
+        <v>46093.55797740741</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46134.66246857639</v>
+        <v>46196.5728619213</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>309</v>
       </c>
       <c r="F92" s="6" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G92" s="6" t="s">
         <v>57</v>
@@ -6796,9 +6780,11 @@
       <c r="H92" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="I92" s="6"/>
+      <c r="I92" s="5">
+        <v>46069</v>
+      </c>
       <c r="J92" s="5">
-        <v>46094</v>
+        <v>46069</v>
       </c>
       <c r="K92" s="6" t="s">
         <v>28</v>
@@ -6825,7 +6811,9 @@
       <c r="S92" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T92" s="6"/>
+      <c r="T92" s="17" t="s">
+        <v>128</v>
+      </c>
       <c r="U92" s="6"/>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
@@ -6833,11 +6821,11 @@
         <v>311</v>
       </c>
       <c r="B93" s="10">
-        <v>46094.64671800926</v>
+        <v>46094.58428688657</v>
       </c>
       <c r="C93" s="11"/>
       <c r="D93" s="10">
-        <v>46094.64682403935</v>
+        <v>46094.584938113425</v>
       </c>
       <c r="E93" s="11" t="s">
         <v>312</v>
@@ -6882,30 +6870,24 @@
         <v>314</v>
       </c>
       <c r="B94" s="5">
-        <v>46093.55797740741</v>
+        <v>46094.58447622685</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46196.5728619213</v>
+        <v>46094.5849659838</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>315</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>166</v>
+        <v>28</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H94" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="I94" s="5">
-        <v>46069</v>
-      </c>
-      <c r="J94" s="5">
-        <v>46069</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H94" s="6"/>
+      <c r="I94" s="6"/>
+      <c r="J94" s="6"/>
       <c r="K94" s="6" t="s">
         <v>28</v>
       </c>
@@ -6913,10 +6895,10 @@
         <v>28</v>
       </c>
       <c r="M94" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>28</v>
+        <v>309</v>
       </c>
       <c r="O94" s="6" t="s">
         <v>28</v>
@@ -6928,12 +6910,8 @@
         <v>316</v>
       </c>
       <c r="R94" s="6"/>
-      <c r="S94" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T94" s="17" t="s">
-        <v>128</v>
-      </c>
+      <c r="S94" s="6"/>
+      <c r="T94" s="6"/>
       <c r="U94" s="6"/>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
@@ -6941,11 +6919,11 @@
         <v>317</v>
       </c>
       <c r="B95" s="10">
-        <v>46094.58428688657</v>
+        <v>46094.58471086806</v>
       </c>
       <c r="C95" s="11"/>
       <c r="D95" s="10">
-        <v>46094.584938113425</v>
+        <v>46094.58499179398</v>
       </c>
       <c r="E95" s="11" t="s">
         <v>318</v>
@@ -6969,7 +6947,7 @@
         <v>28</v>
       </c>
       <c r="N95" s="11" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="O95" s="11" t="s">
         <v>28</v>
@@ -6990,24 +6968,30 @@
         <v>320</v>
       </c>
       <c r="B96" s="5">
-        <v>46094.58447622685</v>
-      </c>
-      <c r="C96" s="6"/>
+        <v>46093.55797605324</v>
+      </c>
+      <c r="C96" s="5">
+        <v>46140.73067185185</v>
+      </c>
       <c r="D96" s="5">
-        <v>46094.5849659838</v>
+        <v>46140.730673252314</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>321</v>
       </c>
       <c r="F96" s="6" t="s">
-        <v>28</v>
+        <v>160</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H96" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H96" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I96" s="6"/>
-      <c r="J96" s="6"/>
+      <c r="J96" s="5">
+        <v>46059</v>
+      </c>
       <c r="K96" s="6" t="s">
         <v>28</v>
       </c>
@@ -7015,10 +6999,10 @@
         <v>28</v>
       </c>
       <c r="M96" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>315</v>
+        <v>28</v>
       </c>
       <c r="O96" s="6" t="s">
         <v>28</v>
@@ -7030,8 +7014,12 @@
         <v>322</v>
       </c>
       <c r="R96" s="6"/>
-      <c r="S96" s="6"/>
-      <c r="T96" s="6"/>
+      <c r="S96" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T96" s="17" t="s">
+        <v>128</v>
+      </c>
       <c r="U96" s="6"/>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
@@ -7039,11 +7027,11 @@
         <v>323</v>
       </c>
       <c r="B97" s="10">
-        <v>46094.58471086806</v>
+        <v>46094.644745763886</v>
       </c>
       <c r="C97" s="11"/>
       <c r="D97" s="10">
-        <v>46094.58499179398</v>
+        <v>46094.644892048615</v>
       </c>
       <c r="E97" s="11" t="s">
         <v>324</v>
@@ -7067,7 +7055,7 @@
         <v>28</v>
       </c>
       <c r="N97" s="11" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="O97" s="11" t="s">
         <v>28</v>
@@ -7088,30 +7076,24 @@
         <v>326</v>
       </c>
       <c r="B98" s="5">
-        <v>46093.55797605324</v>
-      </c>
-      <c r="C98" s="5">
-        <v>46140.73067185185</v>
-      </c>
+        <v>46094.64489846065</v>
+      </c>
+      <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46140.730673252314</v>
+        <v>46094.64504228009</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>327</v>
       </c>
       <c r="F98" s="6" t="s">
-        <v>166</v>
+        <v>28</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H98" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H98" s="6"/>
       <c r="I98" s="6"/>
-      <c r="J98" s="5">
-        <v>46059</v>
-      </c>
+      <c r="J98" s="6"/>
       <c r="K98" s="6" t="s">
         <v>28</v>
       </c>
@@ -7119,10 +7101,10 @@
         <v>28</v>
       </c>
       <c r="M98" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>28</v>
+        <v>321</v>
       </c>
       <c r="O98" s="6" t="s">
         <v>28</v>
@@ -7134,12 +7116,8 @@
         <v>328</v>
       </c>
       <c r="R98" s="6"/>
-      <c r="S98" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T98" s="17" t="s">
-        <v>128</v>
-      </c>
+      <c r="S98" s="6"/>
+      <c r="T98" s="6"/>
       <c r="U98" s="6"/>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -7147,35 +7125,41 @@
         <v>329</v>
       </c>
       <c r="B99" s="10">
-        <v>46094.644745763886</v>
-      </c>
-      <c r="C99" s="11"/>
+        <v>46133.80890888889</v>
+      </c>
+      <c r="C99" s="10">
+        <v>46203.59473923611</v>
+      </c>
       <c r="D99" s="10">
-        <v>46094.644892048615</v>
+        <v>46203.59475351852</v>
       </c>
       <c r="E99" s="11" t="s">
         <v>330</v>
       </c>
       <c r="F99" s="11" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G99" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H99" s="11"/>
+        <v>57</v>
+      </c>
+      <c r="H99" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="I99" s="11"/>
-      <c r="J99" s="11"/>
+      <c r="J99" s="10">
+        <v>46142</v>
+      </c>
       <c r="K99" s="11" t="s">
         <v>28</v>
       </c>
       <c r="L99" s="11" t="s">
-        <v>28</v>
+        <v>331</v>
       </c>
       <c r="M99" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N99" s="11" t="s">
-        <v>327</v>
+        <v>28</v>
       </c>
       <c r="O99" s="11" t="s">
         <v>28</v>
@@ -7184,29 +7168,35 @@
         <v>28</v>
       </c>
       <c r="Q99" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="R99" s="11"/>
-      <c r="S99" s="11"/>
-      <c r="T99" s="11"/>
+      <c r="S99" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T99" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U99" s="11"/>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B100" s="5">
-        <v>46094.64489846065</v>
-      </c>
-      <c r="C100" s="6"/>
+        <v>46133.809437812495</v>
+      </c>
+      <c r="C100" s="5">
+        <v>46203.594679999995</v>
+      </c>
       <c r="D100" s="5">
-        <v>46094.64504228009</v>
+        <v>46203.59469834491</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F100" s="6" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G100" s="6" t="s">
         <v>28</v>
@@ -7221,10 +7211,10 @@
         <v>28</v>
       </c>
       <c r="M100" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N100" s="6" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="O100" s="6" t="s">
         <v>28</v>
@@ -7233,7 +7223,7 @@
         <v>28</v>
       </c>
       <c r="Q100" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="R100" s="6"/>
       <c r="S100" s="6"/>
@@ -7242,19 +7232,19 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B101" s="10">
-        <v>46133.80890888889</v>
+        <v>46155.80580025463</v>
       </c>
       <c r="C101" s="10">
-        <v>46203.59473923611</v>
+        <v>46203.58947402777</v>
       </c>
       <c r="D101" s="10">
-        <v>46203.59475351852</v>
+        <v>46203.5894903588</v>
       </c>
       <c r="E101" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F101" s="11" t="s">
         <v>143</v>
@@ -7267,19 +7257,19 @@
       </c>
       <c r="I101" s="11"/>
       <c r="J101" s="10">
-        <v>46142</v>
+        <v>46162</v>
       </c>
       <c r="K101" s="11" t="s">
         <v>28</v>
       </c>
       <c r="L101" s="11" t="s">
-        <v>337</v>
+        <v>28</v>
       </c>
       <c r="M101" s="11" t="s">
         <v>0</v>
       </c>
       <c r="N101" s="11" t="s">
-        <v>28</v>
+        <v>338</v>
       </c>
       <c r="O101" s="11" t="s">
         <v>28</v>
@@ -7288,42 +7278,44 @@
         <v>28</v>
       </c>
       <c r="Q101" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="R101" s="11"/>
-      <c r="S101" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T101" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="S101" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T101" s="11"/>
       <c r="U101" s="11"/>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B102" s="5">
-        <v>46133.809437812495</v>
+        <v>46155.80563927084</v>
       </c>
       <c r="C102" s="5">
-        <v>46203.594679999995</v>
+        <v>46203.58946413195</v>
       </c>
       <c r="D102" s="5">
-        <v>46203.59469834491</v>
+        <v>46203.58948405093</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>143</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H102" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H102" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I102" s="6"/>
-      <c r="J102" s="6"/>
+      <c r="J102" s="5">
+        <v>46162</v>
+      </c>
       <c r="K102" s="6" t="s">
         <v>28</v>
       </c>
@@ -7334,7 +7326,7 @@
         <v>0</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="O102" s="6" t="s">
         <v>28</v>
@@ -7343,28 +7335,30 @@
         <v>28</v>
       </c>
       <c r="Q102" s="6" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="R102" s="6"/>
-      <c r="S102" s="6"/>
+      <c r="S102" s="12" t="s">
+        <v>43</v>
+      </c>
       <c r="T102" s="6"/>
       <c r="U102" s="6"/>
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="9" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B103" s="10">
-        <v>46155.80580025463</v>
+        <v>46155.80523456019</v>
       </c>
       <c r="C103" s="10">
-        <v>46203.58947402777</v>
+        <v>46203.589470266204</v>
       </c>
       <c r="D103" s="10">
-        <v>46203.5894903588</v>
+        <v>46203.589486400466</v>
       </c>
       <c r="E103" s="11" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="F103" s="11" t="s">
         <v>143</v>
@@ -7389,39 +7383,39 @@
         <v>0</v>
       </c>
       <c r="N103" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="O103" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="P103" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q103" s="11" t="s">
         <v>344</v>
-      </c>
-      <c r="O103" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="P103" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q103" s="11" t="s">
-        <v>345</v>
       </c>
       <c r="R103" s="11"/>
       <c r="S103" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T103" s="11"/>
+      <c r="T103" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U103" s="11"/>
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="B104" s="5">
+        <v>46133.8018299074</v>
+      </c>
+      <c r="C104" s="6"/>
+      <c r="D104" s="5">
+        <v>46185.594546168984</v>
+      </c>
+      <c r="E104" s="6" t="s">
         <v>346</v>
-      </c>
-      <c r="B104" s="5">
-        <v>46155.80563927084</v>
-      </c>
-      <c r="C104" s="5">
-        <v>46203.58946413195</v>
-      </c>
-      <c r="D104" s="5">
-        <v>46203.58948405093</v>
-      </c>
-      <c r="E104" s="6" t="s">
-        <v>347</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>143</v>
@@ -7434,7 +7428,7 @@
       </c>
       <c r="I104" s="6"/>
       <c r="J104" s="5">
-        <v>46162</v>
+        <v>46157</v>
       </c>
       <c r="K104" s="6" t="s">
         <v>28</v>
@@ -7446,7 +7440,7 @@
         <v>0</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>344</v>
+        <v>28</v>
       </c>
       <c r="O104" s="6" t="s">
         <v>28</v>
@@ -7455,44 +7449,40 @@
         <v>28</v>
       </c>
       <c r="Q104" s="6" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R104" s="6"/>
       <c r="S104" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T104" s="6"/>
+      <c r="T104" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U104" s="6"/>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="B105" s="10">
+        <v>46133.8022120949</v>
+      </c>
+      <c r="C105" s="11"/>
+      <c r="D105" s="10">
+        <v>46133.80266505787</v>
+      </c>
+      <c r="E105" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="B105" s="10">
-        <v>46155.80523456019</v>
-      </c>
-      <c r="C105" s="10">
-        <v>46203.589470266204</v>
-      </c>
-      <c r="D105" s="10">
-        <v>46203.589486400466</v>
-      </c>
-      <c r="E105" s="11" t="s">
-        <v>344</v>
-      </c>
       <c r="F105" s="11" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G105" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H105" s="11" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H105" s="11"/>
       <c r="I105" s="11"/>
-      <c r="J105" s="10">
-        <v>46162</v>
-      </c>
+      <c r="J105" s="11"/>
       <c r="K105" s="11" t="s">
         <v>28</v>
       </c>
@@ -7500,10 +7490,10 @@
         <v>28</v>
       </c>
       <c r="M105" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N105" s="11" t="s">
-        <v>28</v>
+        <v>346</v>
       </c>
       <c r="O105" s="11" t="s">
         <v>28</v>
@@ -7515,12 +7505,8 @@
         <v>350</v>
       </c>
       <c r="R105" s="11"/>
-      <c r="S105" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T105" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="S105" s="11"/>
+      <c r="T105" s="11"/>
       <c r="U105" s="11"/>
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
@@ -7528,28 +7514,24 @@
         <v>351</v>
       </c>
       <c r="B106" s="5">
-        <v>46133.8018299074</v>
+        <v>46133.80235815972</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46185.594546168984</v>
+        <v>46133.8027009375</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>352</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G106" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H106" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H106" s="6"/>
       <c r="I106" s="6"/>
-      <c r="J106" s="5">
-        <v>46157</v>
-      </c>
+      <c r="J106" s="6"/>
       <c r="K106" s="6" t="s">
         <v>28</v>
       </c>
@@ -7557,10 +7539,10 @@
         <v>28</v>
       </c>
       <c r="M106" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>28</v>
+        <v>346</v>
       </c>
       <c r="O106" s="6" t="s">
         <v>28</v>
@@ -7572,12 +7554,8 @@
         <v>353</v>
       </c>
       <c r="R106" s="6"/>
-      <c r="S106" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T106" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="S106" s="6"/>
+      <c r="T106" s="6"/>
       <c r="U106" s="6"/>
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
@@ -7585,11 +7563,11 @@
         <v>354</v>
       </c>
       <c r="B107" s="10">
-        <v>46133.8022120949</v>
+        <v>46133.80248805556</v>
       </c>
       <c r="C107" s="11"/>
       <c r="D107" s="10">
-        <v>46133.80266505787</v>
+        <v>46133.802740625004</v>
       </c>
       <c r="E107" s="11" t="s">
         <v>355</v>
@@ -7613,7 +7591,7 @@
         <v>28</v>
       </c>
       <c r="N107" s="11" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="O107" s="11" t="s">
         <v>28</v>
@@ -7634,24 +7612,30 @@
         <v>357</v>
       </c>
       <c r="B108" s="5">
-        <v>46133.80235815972</v>
-      </c>
-      <c r="C108" s="6"/>
+        <v>46093.55797645834</v>
+      </c>
+      <c r="C108" s="5">
+        <v>46162.85491734954</v>
+      </c>
       <c r="D108" s="5">
-        <v>46133.8027009375</v>
+        <v>46162.85493328703</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>358</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H108" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H108" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I108" s="6"/>
-      <c r="J108" s="6"/>
+      <c r="J108" s="5">
+        <v>46063</v>
+      </c>
       <c r="K108" s="6" t="s">
         <v>28</v>
       </c>
@@ -7659,10 +7643,10 @@
         <v>28</v>
       </c>
       <c r="M108" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>352</v>
+        <v>28</v>
       </c>
       <c r="O108" s="6" t="s">
         <v>28</v>
@@ -7674,8 +7658,12 @@
         <v>359</v>
       </c>
       <c r="R108" s="6"/>
-      <c r="S108" s="6"/>
-      <c r="T108" s="6"/>
+      <c r="S108" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T108" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U108" s="6"/>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
@@ -7683,24 +7671,30 @@
         <v>360</v>
       </c>
       <c r="B109" s="10">
-        <v>46133.80248805556</v>
-      </c>
-      <c r="C109" s="11"/>
+        <v>46094.63825950232</v>
+      </c>
+      <c r="C109" s="10">
+        <v>46136.032332372684</v>
+      </c>
       <c r="D109" s="10">
-        <v>46133.802740625004</v>
+        <v>46136.032352685186</v>
       </c>
       <c r="E109" s="11" t="s">
         <v>361</v>
       </c>
       <c r="F109" s="11" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G109" s="11" t="s">
         <v>28</v>
       </c>
       <c r="H109" s="11"/>
-      <c r="I109" s="11"/>
-      <c r="J109" s="11"/>
+      <c r="I109" s="10">
+        <v>45988</v>
+      </c>
+      <c r="J109" s="10">
+        <v>45988</v>
+      </c>
       <c r="K109" s="11" t="s">
         <v>28</v>
       </c>
@@ -7708,10 +7702,10 @@
         <v>28</v>
       </c>
       <c r="M109" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N109" s="11" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="O109" s="11" t="s">
         <v>28</v>
@@ -7732,13 +7726,13 @@
         <v>363</v>
       </c>
       <c r="B110" s="5">
-        <v>46093.55797645834</v>
+        <v>46094.63841756944</v>
       </c>
       <c r="C110" s="5">
-        <v>46162.85491734954</v>
+        <v>46136.03234583333</v>
       </c>
       <c r="D110" s="5">
-        <v>46162.85493328703</v>
+        <v>46136.03236168981</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>364</v>
@@ -7747,14 +7741,14 @@
         <v>143</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H110" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="I110" s="6"/>
+        <v>28</v>
+      </c>
+      <c r="H110" s="6"/>
+      <c r="I110" s="5">
+        <v>45988</v>
+      </c>
       <c r="J110" s="5">
-        <v>46063</v>
+        <v>45988</v>
       </c>
       <c r="K110" s="6" t="s">
         <v>28</v>
@@ -7766,7 +7760,7 @@
         <v>0</v>
       </c>
       <c r="N110" s="6" t="s">
-        <v>28</v>
+        <v>358</v>
       </c>
       <c r="O110" s="6" t="s">
         <v>28</v>
@@ -7778,12 +7772,8 @@
         <v>365</v>
       </c>
       <c r="R110" s="6"/>
-      <c r="S110" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T110" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="S110" s="6"/>
+      <c r="T110" s="6"/>
       <c r="U110" s="6"/>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
@@ -7791,13 +7781,13 @@
         <v>366</v>
       </c>
       <c r="B111" s="10">
-        <v>46094.63825950232</v>
+        <v>46094.63861635417</v>
       </c>
       <c r="C111" s="10">
-        <v>46136.032332372684</v>
+        <v>46136.03235858797</v>
       </c>
       <c r="D111" s="10">
-        <v>46136.032352685186</v>
+        <v>46136.032374560185</v>
       </c>
       <c r="E111" s="11" t="s">
         <v>367</v>
@@ -7810,10 +7800,10 @@
       </c>
       <c r="H111" s="11"/>
       <c r="I111" s="10">
-        <v>45988</v>
+        <v>46063</v>
       </c>
       <c r="J111" s="10">
-        <v>45988</v>
+        <v>46063</v>
       </c>
       <c r="K111" s="11" t="s">
         <v>28</v>
@@ -7825,7 +7815,7 @@
         <v>0</v>
       </c>
       <c r="N111" s="11" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="O111" s="11" t="s">
         <v>28</v>
@@ -7846,13 +7836,13 @@
         <v>369</v>
       </c>
       <c r="B112" s="5">
-        <v>46094.63841756944</v>
+        <v>46133.81027721065</v>
       </c>
       <c r="C112" s="5">
-        <v>46136.03234583333</v>
+        <v>46161.91299474537</v>
       </c>
       <c r="D112" s="5">
-        <v>46136.03236168981</v>
+        <v>46161.91301581018</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>370</v>
@@ -7864,12 +7854,8 @@
         <v>28</v>
       </c>
       <c r="H112" s="6"/>
-      <c r="I112" s="5">
-        <v>45988</v>
-      </c>
-      <c r="J112" s="5">
-        <v>45988</v>
-      </c>
+      <c r="I112" s="6"/>
+      <c r="J112" s="6"/>
       <c r="K112" s="6" t="s">
         <v>28</v>
       </c>
@@ -7880,7 +7866,7 @@
         <v>0</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="O112" s="6" t="s">
         <v>28</v>
@@ -7889,7 +7875,7 @@
         <v>28</v>
       </c>
       <c r="Q112" s="6" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="R112" s="6"/>
       <c r="S112" s="6"/>
@@ -7898,32 +7884,32 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="9" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B113" s="10">
-        <v>46094.63861635417</v>
+        <v>46133.80965319445</v>
       </c>
       <c r="C113" s="10">
-        <v>46136.03235858797</v>
+        <v>46161.912943958334</v>
       </c>
       <c r="D113" s="10">
-        <v>46136.032374560185</v>
+        <v>46161.91296126157</v>
       </c>
       <c r="E113" s="11" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="F113" s="11" t="s">
         <v>143</v>
       </c>
       <c r="G113" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H113" s="11"/>
-      <c r="I113" s="10">
-        <v>46063</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="H113" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I113" s="11"/>
       <c r="J113" s="10">
-        <v>46063</v>
+        <v>46140</v>
       </c>
       <c r="K113" s="11" t="s">
         <v>28</v>
@@ -7935,7 +7921,7 @@
         <v>0</v>
       </c>
       <c r="N113" s="11" t="s">
-        <v>364</v>
+        <v>28</v>
       </c>
       <c r="O113" s="11" t="s">
         <v>28</v>
@@ -7947,8 +7933,12 @@
         <v>374</v>
       </c>
       <c r="R113" s="11"/>
-      <c r="S113" s="11"/>
-      <c r="T113" s="11"/>
+      <c r="S113" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="T113" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="U113" s="11"/>
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
@@ -7956,13 +7946,13 @@
         <v>375</v>
       </c>
       <c r="B114" s="5">
-        <v>46133.81027721065</v>
+        <v>46133.79562642361</v>
       </c>
       <c r="C114" s="5">
-        <v>46161.91299474537</v>
+        <v>46161.91275101852</v>
       </c>
       <c r="D114" s="5">
-        <v>46161.91301581018</v>
+        <v>46161.912771296295</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>376</v>
@@ -8007,13 +7997,13 @@
         <v>379</v>
       </c>
       <c r="B115" s="10">
-        <v>46133.80965319445</v>
+        <v>46133.79487287037</v>
       </c>
       <c r="C115" s="10">
-        <v>46161.912943958334</v>
+        <v>46161.91275491898</v>
       </c>
       <c r="D115" s="10">
-        <v>46161.91296126157</v>
+        <v>46161.91277105324</v>
       </c>
       <c r="E115" s="11" t="s">
         <v>377</v>
@@ -8029,7 +8019,7 @@
       </c>
       <c r="I115" s="11"/>
       <c r="J115" s="10">
-        <v>46140</v>
+        <v>46118</v>
       </c>
       <c r="K115" s="11" t="s">
         <v>28</v>
@@ -8053,8 +8043,8 @@
         <v>380</v>
       </c>
       <c r="R115" s="11"/>
-      <c r="S115" s="14" t="s">
-        <v>51</v>
+      <c r="S115" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="T115" s="8" t="s">
         <v>31</v>
@@ -8066,13 +8056,13 @@
         <v>381</v>
       </c>
       <c r="B116" s="5">
-        <v>46133.79562642361</v>
+        <v>46133.79582699074</v>
       </c>
       <c r="C116" s="5">
-        <v>46161.91275101852</v>
+        <v>46161.912757847225</v>
       </c>
       <c r="D116" s="5">
-        <v>46161.912771296295</v>
+        <v>46161.91277258102</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>382</v>
@@ -8096,16 +8086,16 @@
         <v>0</v>
       </c>
       <c r="N116" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="O116" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P116" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q116" s="6" t="s">
         <v>383</v>
-      </c>
-      <c r="O116" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="P116" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q116" s="6" t="s">
-        <v>384</v>
       </c>
       <c r="R116" s="6"/>
       <c r="S116" s="6"/>
@@ -8114,32 +8104,32 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="9" t="s">
+        <v>384</v>
+      </c>
+      <c r="B117" s="10">
+        <v>46094.641416493054</v>
+      </c>
+      <c r="C117" s="10">
+        <v>46161.912420381945</v>
+      </c>
+      <c r="D117" s="10">
+        <v>46161.912439594904</v>
+      </c>
+      <c r="E117" s="11" t="s">
         <v>385</v>
-      </c>
-      <c r="B117" s="10">
-        <v>46133.79487287037</v>
-      </c>
-      <c r="C117" s="10">
-        <v>46161.91275491898</v>
-      </c>
-      <c r="D117" s="10">
-        <v>46161.91277105324</v>
-      </c>
-      <c r="E117" s="11" t="s">
-        <v>383</v>
       </c>
       <c r="F117" s="11" t="s">
         <v>143</v>
       </c>
       <c r="G117" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H117" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="I117" s="11"/>
+        <v>28</v>
+      </c>
+      <c r="H117" s="11"/>
+      <c r="I117" s="10">
+        <v>45986</v>
+      </c>
       <c r="J117" s="10">
-        <v>46118</v>
+        <v>45986</v>
       </c>
       <c r="K117" s="11" t="s">
         <v>28</v>
@@ -8151,7 +8141,7 @@
         <v>0</v>
       </c>
       <c r="N117" s="11" t="s">
-        <v>28</v>
+        <v>386</v>
       </c>
       <c r="O117" s="11" t="s">
         <v>28</v>
@@ -8160,42 +8150,42 @@
         <v>28</v>
       </c>
       <c r="Q117" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="R117" s="11"/>
-      <c r="S117" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T117" s="8" t="s">
-        <v>31</v>
-      </c>
+      <c r="S117" s="11"/>
+      <c r="T117" s="11"/>
       <c r="U117" s="11"/>
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B118" s="5">
-        <v>46133.79582699074</v>
+        <v>46093.55797701389</v>
       </c>
       <c r="C118" s="5">
-        <v>46161.912757847225</v>
+        <v>46161.912426678246</v>
       </c>
       <c r="D118" s="5">
-        <v>46161.91277258102</v>
+        <v>46161.91244167824</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>143</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H118" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="H118" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="I118" s="6"/>
-      <c r="J118" s="6"/>
+      <c r="J118" s="5">
+        <v>45986</v>
+      </c>
       <c r="K118" s="6" t="s">
         <v>28</v>
       </c>
@@ -8206,7 +8196,7 @@
         <v>0</v>
       </c>
       <c r="N118" s="6" t="s">
-        <v>383</v>
+        <v>28</v>
       </c>
       <c r="O118" s="6" t="s">
         <v>28</v>
@@ -8218,8 +8208,12 @@
         <v>389</v>
       </c>
       <c r="R118" s="6"/>
-      <c r="S118" s="6"/>
-      <c r="T118" s="6"/>
+      <c r="S118" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T118" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="U118" s="6"/>
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
@@ -8227,13 +8221,13 @@
         <v>390</v>
       </c>
       <c r="B119" s="10">
-        <v>46094.641416493054</v>
+        <v>46094.582692951386</v>
       </c>
       <c r="C119" s="10">
-        <v>46161.912420381945</v>
+        <v>46134.673179687496</v>
       </c>
       <c r="D119" s="10">
-        <v>46161.912439594904</v>
+        <v>46134.67319648148</v>
       </c>
       <c r="E119" s="11" t="s">
         <v>391</v>
@@ -8242,15 +8236,13 @@
         <v>143</v>
       </c>
       <c r="G119" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H119" s="11"/>
-      <c r="I119" s="10">
-        <v>45986</v>
-      </c>
-      <c r="J119" s="10">
-        <v>45986</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="H119" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="I119" s="11"/>
+      <c r="J119" s="11"/>
       <c r="K119" s="11" t="s">
         <v>28</v>
       </c>
@@ -8282,30 +8274,28 @@
         <v>394</v>
       </c>
       <c r="B120" s="5">
-        <v>46093.55797701389</v>
+        <v>46093.557975625</v>
       </c>
       <c r="C120" s="5">
-        <v>46161.912426678246</v>
+        <v>46134.64221024305</v>
       </c>
       <c r="D120" s="5">
-        <v>46161.91244167824</v>
+        <v>46134.66266402778</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="F120" s="6" t="s">
         <v>143</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="H120" s="6" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="I120" s="6"/>
-      <c r="J120" s="5">
-        <v>45986</v>
-      </c>
+      <c r="J120" s="6"/>
       <c r="K120" s="6" t="s">
         <v>28</v>
       </c>
@@ -8325,32 +8315,28 @@
         <v>28</v>
       </c>
       <c r="Q120" s="6" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="R120" s="6"/>
-      <c r="S120" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T120" s="8" t="s">
-        <v>31</v>
-      </c>
+      <c r="S120" s="6"/>
+      <c r="T120" s="6"/>
       <c r="U120" s="6"/>
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A121" s="9" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B121" s="10">
-        <v>46094.582692951386</v>
+        <v>46093.55797712963</v>
       </c>
       <c r="C121" s="10">
-        <v>46134.673179687496</v>
+        <v>46134.63987417824</v>
       </c>
       <c r="D121" s="10">
-        <v>46134.67319648148</v>
+        <v>46134.63988903935</v>
       </c>
       <c r="E121" s="11" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="F121" s="11" t="s">
         <v>143</v>
@@ -8361,8 +8347,12 @@
       <c r="H121" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I121" s="11"/>
-      <c r="J121" s="11"/>
+      <c r="I121" s="10">
+        <v>46039</v>
+      </c>
+      <c r="J121" s="10">
+        <v>46039</v>
+      </c>
       <c r="K121" s="11" t="s">
         <v>28</v>
       </c>
@@ -8373,37 +8363,39 @@
         <v>0</v>
       </c>
       <c r="N121" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="O121" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="P121" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q121" s="11" t="s">
         <v>398</v>
-      </c>
-      <c r="O121" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="P121" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q121" s="11" t="s">
-        <v>399</v>
       </c>
       <c r="R121" s="11"/>
       <c r="S121" s="11"/>
-      <c r="T121" s="11"/>
+      <c r="T121" s="15" t="s">
+        <v>72</v>
+      </c>
       <c r="U121" s="11"/>
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="B122" s="5">
+        <v>46094.58194446759</v>
+      </c>
+      <c r="C122" s="5">
+        <v>46134.63920685185</v>
+      </c>
+      <c r="D122" s="5">
+        <v>46134.66324178241</v>
+      </c>
+      <c r="E122" s="6" t="s">
         <v>400</v>
-      </c>
-      <c r="B122" s="5">
-        <v>46093.557975625</v>
-      </c>
-      <c r="C122" s="5">
-        <v>46134.64221024305</v>
-      </c>
-      <c r="D122" s="5">
-        <v>46134.66266402778</v>
-      </c>
-      <c r="E122" s="6" t="s">
-        <v>401</v>
       </c>
       <c r="F122" s="6" t="s">
         <v>143</v>
@@ -8426,7 +8418,7 @@
         <v>0</v>
       </c>
       <c r="N122" s="6" t="s">
-        <v>28</v>
+        <v>392</v>
       </c>
       <c r="O122" s="6" t="s">
         <v>28</v>
@@ -8435,7 +8427,7 @@
         <v>28</v>
       </c>
       <c r="Q122" s="6" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="R122" s="6"/>
       <c r="S122" s="6"/>
@@ -8444,19 +8436,19 @@
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A123" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="B123" s="10">
+        <v>46094.58215357639</v>
+      </c>
+      <c r="C123" s="10">
+        <v>46134.63922920139</v>
+      </c>
+      <c r="D123" s="10">
+        <v>46134.66306040509</v>
+      </c>
+      <c r="E123" s="11" t="s">
         <v>403</v>
-      </c>
-      <c r="B123" s="10">
-        <v>46093.55797712963</v>
-      </c>
-      <c r="C123" s="10">
-        <v>46134.63987417824</v>
-      </c>
-      <c r="D123" s="10">
-        <v>46134.63988903935</v>
-      </c>
-      <c r="E123" s="11" t="s">
-        <v>398</v>
       </c>
       <c r="F123" s="11" t="s">
         <v>143</v>
@@ -8467,12 +8459,8 @@
       <c r="H123" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I123" s="10">
-        <v>46039</v>
-      </c>
-      <c r="J123" s="10">
-        <v>46039</v>
-      </c>
+      <c r="I123" s="11"/>
+      <c r="J123" s="11"/>
       <c r="K123" s="11" t="s">
         <v>28</v>
       </c>
@@ -8483,7 +8471,7 @@
         <v>0</v>
       </c>
       <c r="N123" s="11" t="s">
-        <v>28</v>
+        <v>392</v>
       </c>
       <c r="O123" s="11" t="s">
         <v>28</v>
@@ -8496,9 +8484,7 @@
       </c>
       <c r="R123" s="11"/>
       <c r="S123" s="11"/>
-      <c r="T123" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="T123" s="11"/>
       <c r="U123" s="11"/>
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
@@ -8506,13 +8492,13 @@
         <v>405</v>
       </c>
       <c r="B124" s="5">
-        <v>46094.58194446759</v>
+        <v>46094.5823130787</v>
       </c>
       <c r="C124" s="5">
-        <v>46134.63920685185</v>
+        <v>46134.63923450232</v>
       </c>
       <c r="D124" s="5">
-        <v>46134.66324178241</v>
+        <v>46134.66313976852</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>406</v>
@@ -8538,7 +8524,7 @@
         <v>0</v>
       </c>
       <c r="N124" s="6" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="O124" s="6" t="s">
         <v>28</v>
@@ -8559,13 +8545,13 @@
         <v>408</v>
       </c>
       <c r="B125" s="10">
-        <v>46094.58215357639</v>
+        <v>46094.582410393516</v>
       </c>
       <c r="C125" s="10">
-        <v>46134.63922920139</v>
+        <v>46134.63923954861</v>
       </c>
       <c r="D125" s="10">
-        <v>46134.66306040509</v>
+        <v>46134.662989178236</v>
       </c>
       <c r="E125" s="11" t="s">
         <v>409</v>
@@ -8591,7 +8577,7 @@
         <v>0</v>
       </c>
       <c r="N125" s="11" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="O125" s="11" t="s">
         <v>28</v>
@@ -8612,13 +8598,13 @@
         <v>411</v>
       </c>
       <c r="B126" s="5">
-        <v>46094.5823130787</v>
+        <v>46094.58253722222</v>
       </c>
       <c r="C126" s="5">
-        <v>46134.63923450232</v>
+        <v>46134.639245694445</v>
       </c>
       <c r="D126" s="5">
-        <v>46134.66313976852</v>
+        <v>46134.662925682875</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>412</v>
@@ -8644,7 +8630,7 @@
         <v>0</v>
       </c>
       <c r="N126" s="6" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="O126" s="6" t="s">
         <v>28</v>
@@ -8665,13 +8651,13 @@
         <v>414</v>
       </c>
       <c r="B127" s="10">
-        <v>46094.582410393516</v>
+        <v>46094.582797511575</v>
       </c>
       <c r="C127" s="10">
-        <v>46134.63923954861</v>
+        <v>46134.639255312504</v>
       </c>
       <c r="D127" s="10">
-        <v>46134.662989178236</v>
+        <v>46155.578320636574</v>
       </c>
       <c r="E127" s="11" t="s">
         <v>415</v>
@@ -8697,7 +8683,7 @@
         <v>0</v>
       </c>
       <c r="N127" s="11" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="O127" s="11" t="s">
         <v>28</v>
@@ -8718,13 +8704,13 @@
         <v>417</v>
       </c>
       <c r="B128" s="5">
-        <v>46094.58253722222</v>
+        <v>46094.58288509259</v>
       </c>
       <c r="C128" s="5">
-        <v>46134.639245694445</v>
+        <v>46134.63926054398</v>
       </c>
       <c r="D128" s="5">
-        <v>46134.662925682875</v>
+        <v>46134.662788738424</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>418</v>
@@ -8750,7 +8736,7 @@
         <v>0</v>
       </c>
       <c r="N128" s="6" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="O128" s="6" t="s">
         <v>28</v>
@@ -8771,13 +8757,13 @@
         <v>420</v>
       </c>
       <c r="B129" s="10">
-        <v>46094.582797511575</v>
+        <v>46094.58306329861</v>
       </c>
       <c r="C129" s="10">
-        <v>46134.639255312504</v>
+        <v>46134.639266087965</v>
       </c>
       <c r="D129" s="10">
-        <v>46155.578320636574</v>
+        <v>46134.66273581018</v>
       </c>
       <c r="E129" s="11" t="s">
         <v>421</v>
@@ -8803,7 +8789,7 @@
         <v>0</v>
       </c>
       <c r="N129" s="11" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="O129" s="11" t="s">
         <v>28</v>
@@ -8824,13 +8810,13 @@
         <v>423</v>
       </c>
       <c r="B130" s="5">
-        <v>46094.58288509259</v>
+        <v>46133.792176840274</v>
       </c>
       <c r="C130" s="5">
-        <v>46134.63926054398</v>
+        <v>46134.63605664352</v>
       </c>
       <c r="D130" s="5">
-        <v>46134.662788738424</v>
+        <v>46134.63619297453</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>424</v>
@@ -8845,18 +8831,20 @@
         <v>58</v>
       </c>
       <c r="I130" s="6"/>
-      <c r="J130" s="6"/>
+      <c r="J130" s="5">
+        <v>46112</v>
+      </c>
       <c r="K130" s="6" t="s">
         <v>28</v>
       </c>
       <c r="L130" s="6" t="s">
-        <v>28</v>
+        <v>425</v>
       </c>
       <c r="M130" s="6" t="s">
         <v>0</v>
       </c>
       <c r="N130" s="6" t="s">
-        <v>398</v>
+        <v>28</v>
       </c>
       <c r="O130" s="6" t="s">
         <v>28</v>
@@ -8865,38 +8853,38 @@
         <v>28</v>
       </c>
       <c r="Q130" s="6" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="R130" s="6"/>
-      <c r="S130" s="6"/>
-      <c r="T130" s="6"/>
+      <c r="S130" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T130" s="12" t="s">
+        <v>427</v>
+      </c>
       <c r="U130" s="6"/>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A131" s="9" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B131" s="10">
-        <v>46094.58306329861</v>
-      </c>
-      <c r="C131" s="10">
-        <v>46134.639266087965</v>
-      </c>
+        <v>46133.79263490741</v>
+      </c>
+      <c r="C131" s="11"/>
       <c r="D131" s="10">
-        <v>46134.66273581018</v>
+        <v>46133.79350961806</v>
       </c>
       <c r="E131" s="11" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F131" s="11" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G131" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H131" s="11" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H131" s="11"/>
       <c r="I131" s="11"/>
       <c r="J131" s="11"/>
       <c r="K131" s="11" t="s">
@@ -8906,10 +8894,10 @@
         <v>28</v>
       </c>
       <c r="M131" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N131" s="11" t="s">
-        <v>398</v>
+        <v>424</v>
       </c>
       <c r="O131" s="11" t="s">
         <v>28</v>
@@ -8918,7 +8906,7 @@
         <v>28</v>
       </c>
       <c r="Q131" s="11" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="R131" s="11"/>
       <c r="S131" s="11"/>
@@ -8927,19 +8915,19 @@
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B132" s="5">
-        <v>46133.792176840274</v>
+        <v>46091.59394065972</v>
       </c>
       <c r="C132" s="5">
-        <v>46134.63605664352</v>
+        <v>46133.70594085648</v>
       </c>
       <c r="D132" s="5">
-        <v>46134.63619297453</v>
+        <v>46133.7059553125</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="F132" s="6" t="s">
         <v>143</v>
@@ -8952,13 +8940,13 @@
       </c>
       <c r="I132" s="6"/>
       <c r="J132" s="5">
-        <v>46112</v>
+        <v>46083</v>
       </c>
       <c r="K132" s="6" t="s">
         <v>28</v>
       </c>
       <c r="L132" s="6" t="s">
-        <v>431</v>
+        <v>28</v>
       </c>
       <c r="M132" s="6" t="s">
         <v>0</v>
@@ -8973,14 +8961,14 @@
         <v>28</v>
       </c>
       <c r="Q132" s="6" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="R132" s="6"/>
       <c r="S132" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="T132" s="12" t="s">
-        <v>433</v>
+      <c r="T132" s="16" t="s">
+        <v>115</v>
       </c>
       <c r="U132" s="6"/>
     </row>
@@ -8989,11 +8977,11 @@
         <v>434</v>
       </c>
       <c r="B133" s="10">
-        <v>46133.79263490741</v>
+        <v>46094.62533957176</v>
       </c>
       <c r="C133" s="11"/>
       <c r="D133" s="10">
-        <v>46133.79350961806</v>
+        <v>46133.70593778935</v>
       </c>
       <c r="E133" s="11" t="s">
         <v>435</v>
@@ -9017,7 +9005,7 @@
         <v>28</v>
       </c>
       <c r="N133" s="11" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="O133" s="11" t="s">
         <v>28</v>
@@ -9038,30 +9026,24 @@
         <v>437</v>
       </c>
       <c r="B134" s="5">
-        <v>46091.59394065972</v>
-      </c>
-      <c r="C134" s="5">
-        <v>46133.70594085648</v>
-      </c>
+        <v>46094.62542793981</v>
+      </c>
+      <c r="C134" s="6"/>
       <c r="D134" s="5">
-        <v>46133.7059553125</v>
+        <v>46133.70593837963</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>438</v>
       </c>
       <c r="F134" s="6" t="s">
-        <v>143</v>
+        <v>28</v>
       </c>
       <c r="G134" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H134" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H134" s="6"/>
       <c r="I134" s="6"/>
-      <c r="J134" s="5">
-        <v>46083</v>
-      </c>
+      <c r="J134" s="6"/>
       <c r="K134" s="6" t="s">
         <v>28</v>
       </c>
@@ -9069,10 +9051,10 @@
         <v>28</v>
       </c>
       <c r="M134" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N134" s="6" t="s">
-        <v>28</v>
+        <v>432</v>
       </c>
       <c r="O134" s="6" t="s">
         <v>28</v>
@@ -9084,12 +9066,8 @@
         <v>439</v>
       </c>
       <c r="R134" s="6"/>
-      <c r="S134" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T134" s="16" t="s">
-        <v>115</v>
-      </c>
+      <c r="S134" s="6"/>
+      <c r="T134" s="6"/>
       <c r="U134" s="6"/>
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.25">
@@ -9097,11 +9075,11 @@
         <v>440</v>
       </c>
       <c r="B135" s="10">
-        <v>46094.62533957176</v>
+        <v>46094.62613793982</v>
       </c>
       <c r="C135" s="11"/>
       <c r="D135" s="10">
-        <v>46133.70593778935</v>
+        <v>46133.70593877315</v>
       </c>
       <c r="E135" s="11" t="s">
         <v>441</v>
@@ -9125,7 +9103,7 @@
         <v>28</v>
       </c>
       <c r="N135" s="11" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="O135" s="11" t="s">
         <v>28</v>
@@ -9146,11 +9124,11 @@
         <v>443</v>
       </c>
       <c r="B136" s="5">
-        <v>46094.62542793981</v>
+        <v>46094.626408703705</v>
       </c>
       <c r="C136" s="6"/>
       <c r="D136" s="5">
-        <v>46133.70593837963</v>
+        <v>46133.705939189815</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>444</v>
@@ -9174,7 +9152,7 @@
         <v>28</v>
       </c>
       <c r="N136" s="6" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="O136" s="6" t="s">
         <v>28</v>
@@ -9195,11 +9173,11 @@
         <v>446</v>
       </c>
       <c r="B137" s="10">
-        <v>46094.62613793982</v>
+        <v>46094.62648922454</v>
       </c>
       <c r="C137" s="11"/>
       <c r="D137" s="10">
-        <v>46133.70593877315</v>
+        <v>46133.705939618056</v>
       </c>
       <c r="E137" s="11" t="s">
         <v>447</v>
@@ -9223,7 +9201,7 @@
         <v>28</v>
       </c>
       <c r="N137" s="11" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="O137" s="11" t="s">
         <v>28</v>
@@ -9244,11 +9222,11 @@
         <v>449</v>
       </c>
       <c r="B138" s="5">
-        <v>46094.626408703705</v>
+        <v>46094.62660908565</v>
       </c>
       <c r="C138" s="6"/>
       <c r="D138" s="5">
-        <v>46133.705939189815</v>
+        <v>46133.7059399537</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>450</v>
@@ -9272,7 +9250,7 @@
         <v>28</v>
       </c>
       <c r="N138" s="6" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="O138" s="6" t="s">
         <v>28</v>
@@ -9293,11 +9271,11 @@
         <v>452</v>
       </c>
       <c r="B139" s="10">
-        <v>46094.62648922454</v>
+        <v>46094.626713460646</v>
       </c>
       <c r="C139" s="11"/>
       <c r="D139" s="10">
-        <v>46133.705939618056</v>
+        <v>46133.705940300926</v>
       </c>
       <c r="E139" s="11" t="s">
         <v>453</v>
@@ -9321,7 +9299,7 @@
         <v>28</v>
       </c>
       <c r="N139" s="11" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="O139" s="11" t="s">
         <v>28</v>
@@ -9342,11 +9320,11 @@
         <v>455</v>
       </c>
       <c r="B140" s="5">
-        <v>46094.62660908565</v>
+        <v>46094.62680802083</v>
       </c>
       <c r="C140" s="6"/>
       <c r="D140" s="5">
-        <v>46133.7059399537</v>
+        <v>46133.70594064815</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>456</v>
@@ -9370,7 +9348,7 @@
         <v>28</v>
       </c>
       <c r="N140" s="6" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="O140" s="6" t="s">
         <v>28</v>
@@ -9391,22 +9369,26 @@
         <v>458</v>
       </c>
       <c r="B141" s="10">
-        <v>46094.626713460646</v>
-      </c>
-      <c r="C141" s="11"/>
+        <v>46093.55797592593</v>
+      </c>
+      <c r="C141" s="10">
+        <v>46127.87503005787</v>
+      </c>
       <c r="D141" s="10">
-        <v>46133.705940300926</v>
+        <v>46134.66330939815</v>
       </c>
       <c r="E141" s="11" t="s">
         <v>459</v>
       </c>
       <c r="F141" s="11" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G141" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H141" s="11"/>
+        <v>57</v>
+      </c>
+      <c r="H141" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="I141" s="11"/>
       <c r="J141" s="11"/>
       <c r="K141" s="11" t="s">
@@ -9416,10 +9398,10 @@
         <v>28</v>
       </c>
       <c r="M141" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N141" s="11" t="s">
-        <v>438</v>
+        <v>28</v>
       </c>
       <c r="O141" s="11" t="s">
         <v>28</v>
@@ -9440,22 +9422,26 @@
         <v>461</v>
       </c>
       <c r="B142" s="5">
-        <v>46094.62680802083</v>
-      </c>
-      <c r="C142" s="6"/>
+        <v>46094.63474699074</v>
+      </c>
+      <c r="C142" s="5">
+        <v>46127.875013819445</v>
+      </c>
       <c r="D142" s="5">
-        <v>46133.70594064815</v>
+        <v>46134.66345291666</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>462</v>
       </c>
       <c r="F142" s="6" t="s">
-        <v>28</v>
+        <v>143</v>
       </c>
       <c r="G142" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H142" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="H142" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="I142" s="6"/>
       <c r="J142" s="6"/>
       <c r="K142" s="6" t="s">
@@ -9465,10 +9451,10 @@
         <v>28</v>
       </c>
       <c r="M142" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N142" s="6" t="s">
-        <v>438</v>
+        <v>459</v>
       </c>
       <c r="O142" s="6" t="s">
         <v>28</v>
@@ -9489,13 +9475,13 @@
         <v>464</v>
       </c>
       <c r="B143" s="10">
-        <v>46093.55797592593</v>
+        <v>46093.557976111115</v>
       </c>
       <c r="C143" s="10">
-        <v>46127.87503005787</v>
+        <v>46111.836577766204</v>
       </c>
       <c r="D143" s="10">
-        <v>46134.66330939815</v>
+        <v>46111.836592141204</v>
       </c>
       <c r="E143" s="11" t="s">
         <v>465</v>
@@ -9509,8 +9495,12 @@
       <c r="H143" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I143" s="11"/>
-      <c r="J143" s="11"/>
+      <c r="I143" s="10">
+        <v>46003</v>
+      </c>
+      <c r="J143" s="10">
+        <v>46003</v>
+      </c>
       <c r="K143" s="11" t="s">
         <v>28</v>
       </c>
@@ -9533,8 +9523,12 @@
         <v>466</v>
       </c>
       <c r="R143" s="11"/>
-      <c r="S143" s="11"/>
-      <c r="T143" s="11"/>
+      <c r="S143" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T143" s="17" t="s">
+        <v>128</v>
+      </c>
       <c r="U143" s="11"/>
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.25">
@@ -9542,13 +9536,13 @@
         <v>467</v>
       </c>
       <c r="B144" s="5">
-        <v>46094.63474699074</v>
+        <v>46094.57571935185</v>
       </c>
       <c r="C144" s="5">
-        <v>46127.875013819445</v>
+        <v>46111.83654524306</v>
       </c>
       <c r="D144" s="5">
-        <v>46134.66345291666</v>
+        <v>46111.83656112268</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>468</v>
@@ -9557,11 +9551,9 @@
         <v>143</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H144" s="6" t="s">
-        <v>58</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H144" s="6"/>
       <c r="I144" s="6"/>
       <c r="J144" s="6"/>
       <c r="K144" s="6" t="s">
@@ -9595,13 +9587,13 @@
         <v>470</v>
       </c>
       <c r="B145" s="10">
-        <v>46093.557976111115</v>
+        <v>46094.57601390046</v>
       </c>
       <c r="C145" s="10">
-        <v>46111.836577766204</v>
+        <v>46111.8365590162</v>
       </c>
       <c r="D145" s="10">
-        <v>46111.836592141204</v>
+        <v>46111.83657758102</v>
       </c>
       <c r="E145" s="11" t="s">
         <v>471</v>
@@ -9610,17 +9602,11 @@
         <v>143</v>
       </c>
       <c r="G145" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H145" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="I145" s="10">
-        <v>46003</v>
-      </c>
-      <c r="J145" s="10">
-        <v>46003</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H145" s="11"/>
+      <c r="I145" s="11"/>
+      <c r="J145" s="11"/>
       <c r="K145" s="11" t="s">
         <v>28</v>
       </c>
@@ -9631,7 +9617,7 @@
         <v>0</v>
       </c>
       <c r="N145" s="11" t="s">
-        <v>28</v>
+        <v>465</v>
       </c>
       <c r="O145" s="11" t="s">
         <v>28</v>
@@ -9643,12 +9629,8 @@
         <v>472</v>
       </c>
       <c r="R145" s="11"/>
-      <c r="S145" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T145" s="17" t="s">
-        <v>128</v>
-      </c>
+      <c r="S145" s="11"/>
+      <c r="T145" s="11"/>
       <c r="U145" s="11"/>
     </row>
     <row r="146" spans="1:21" x14ac:dyDescent="0.25">
@@ -9656,13 +9638,13 @@
         <v>473</v>
       </c>
       <c r="B146" s="5">
-        <v>46094.57571935185</v>
+        <v>46094.57620418981</v>
       </c>
       <c r="C146" s="5">
-        <v>46111.83654524306</v>
+        <v>46111.83657327546</v>
       </c>
       <c r="D146" s="5">
-        <v>46111.83656112268</v>
+        <v>46111.83659253472</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>474</v>
@@ -9686,7 +9668,7 @@
         <v>0</v>
       </c>
       <c r="N146" s="6" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="O146" s="6" t="s">
         <v>28</v>
@@ -9707,13 +9689,13 @@
         <v>476</v>
       </c>
       <c r="B147" s="10">
-        <v>46094.57601390046</v>
+        <v>46093.557975868054</v>
       </c>
       <c r="C147" s="10">
-        <v>46111.8365590162</v>
+        <v>46097.77705668981</v>
       </c>
       <c r="D147" s="10">
-        <v>46111.83657758102</v>
+        <v>46097.77707333333</v>
       </c>
       <c r="E147" s="11" t="s">
         <v>477</v>
@@ -9722,11 +9704,15 @@
         <v>143</v>
       </c>
       <c r="G147" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H147" s="11"/>
+        <v>40</v>
+      </c>
+      <c r="H147" s="11" t="s">
+        <v>41</v>
+      </c>
       <c r="I147" s="11"/>
-      <c r="J147" s="11"/>
+      <c r="J147" s="10">
+        <v>46031</v>
+      </c>
       <c r="K147" s="11" t="s">
         <v>28</v>
       </c>
@@ -9737,7 +9723,7 @@
         <v>0</v>
       </c>
       <c r="N147" s="11" t="s">
-        <v>471</v>
+        <v>28</v>
       </c>
       <c r="O147" s="11" t="s">
         <v>28</v>
@@ -9749,8 +9735,12 @@
         <v>478</v>
       </c>
       <c r="R147" s="11"/>
-      <c r="S147" s="11"/>
-      <c r="T147" s="11"/>
+      <c r="S147" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="T147" s="13" t="s">
+        <v>44</v>
+      </c>
       <c r="U147" s="11"/>
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.25">
@@ -9758,13 +9748,13 @@
         <v>479</v>
       </c>
       <c r="B148" s="5">
-        <v>46094.57620418981</v>
+        <v>46094.57453506945</v>
       </c>
       <c r="C148" s="5">
-        <v>46111.83657327546</v>
+        <v>46097.77703761574</v>
       </c>
       <c r="D148" s="5">
-        <v>46111.83659253472</v>
+        <v>46097.77705638889</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>480</v>
@@ -9788,7 +9778,7 @@
         <v>0</v>
       </c>
       <c r="N148" s="6" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="O148" s="6" t="s">
         <v>28</v>
@@ -9803,116 +9793,6 @@
       <c r="S148" s="6"/>
       <c r="T148" s="6"/>
       <c r="U148" s="6"/>
-    </row>
-    <row r="149" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A149" s="9" t="s">
-        <v>482</v>
-      </c>
-      <c r="B149" s="10">
-        <v>46093.557975868054</v>
-      </c>
-      <c r="C149" s="10">
-        <v>46097.77705668981</v>
-      </c>
-      <c r="D149" s="10">
-        <v>46097.77707333333</v>
-      </c>
-      <c r="E149" s="11" t="s">
-        <v>483</v>
-      </c>
-      <c r="F149" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="G149" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="H149" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="I149" s="11"/>
-      <c r="J149" s="10">
-        <v>46031</v>
-      </c>
-      <c r="K149" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="L149" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="M149" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="N149" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="O149" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="P149" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q149" s="11" t="s">
-        <v>484</v>
-      </c>
-      <c r="R149" s="11"/>
-      <c r="S149" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="T149" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="U149" s="11"/>
-    </row>
-    <row r="150" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A150" s="4" t="s">
-        <v>485</v>
-      </c>
-      <c r="B150" s="5">
-        <v>46094.57453506945</v>
-      </c>
-      <c r="C150" s="5">
-        <v>46097.77703761574</v>
-      </c>
-      <c r="D150" s="5">
-        <v>46097.77705638889</v>
-      </c>
-      <c r="E150" s="6" t="s">
-        <v>486</v>
-      </c>
-      <c r="F150" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="G150" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H150" s="6"/>
-      <c r="I150" s="6"/>
-      <c r="J150" s="6"/>
-      <c r="K150" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="L150" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M150" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="N150" s="6" t="s">
-        <v>483</v>
-      </c>
-      <c r="O150" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="P150" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q150" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="R150" s="6"/>
-      <c r="S150" s="6"/>
-      <c r="T150" s="6"/>
-      <c r="U150" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-08 16:07 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -2386,7 +2386,7 @@
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="5">
-        <v>46209.79300123843</v>
+        <v>46210.796130717594</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>45</v>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46209.79876372685</v>
+        <v>46210.80974820602</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>61</v>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46209.79847162037</v>
+        <v>46210.806753993056</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>67</v>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="C21" s="11"/>
       <c r="D21" s="10">
-        <v>46209.79905563657</v>
+        <v>46210.80365065973</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>89</v>
@@ -3167,7 +3167,7 @@
       </c>
       <c r="C23" s="11"/>
       <c r="D23" s="10">
-        <v>46209.79549576389</v>
+        <v>46210.798552395834</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>95</v>
@@ -3322,7 +3322,7 @@
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="5">
-        <v>46209.79656415509</v>
+        <v>46210.80012583333</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>104</v>
@@ -3428,7 +3428,7 @@
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46209.80187782407</v>
+        <v>46210.81134996528</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>110</v>
@@ -4874,7 +4874,7 @@
         <v>46209.92160893518</v>
       </c>
       <c r="D56" s="5">
-        <v>46209.92162813657</v>
+        <v>46210.78237596065</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>198</v>
@@ -4927,9 +4927,11 @@
       <c r="B57" s="10">
         <v>46188.630276365744</v>
       </c>
-      <c r="C57" s="11"/>
+      <c r="C57" s="10">
+        <v>46210.76125015046</v>
+      </c>
       <c r="D57" s="10">
-        <v>46209.92191615741</v>
+        <v>46210.761251979166</v>
       </c>
       <c r="E57" s="11" t="s">
         <v>201</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-09 13:48 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -216,6 +216,421 @@
     <t>TABL3-231</t>
   </si>
   <si>
+    <t>1214150417415449</t>
+  </si>
+  <si>
+    <t>50001529 - MINERA ROBLE</t>
+  </si>
+  <si>
+    <t>TABL3-232</t>
+  </si>
+  <si>
+    <t>1214150417415454</t>
+  </si>
+  <si>
+    <t>OT 4272-Rodete ZVN 1-9-86/2</t>
+  </si>
+  <si>
+    <t>TABL3-233</t>
+  </si>
+  <si>
+    <t>1213628910075654</t>
+  </si>
+  <si>
+    <t>50001493-GESVIAL</t>
+  </si>
+  <si>
+    <t>TABL3-47</t>
+  </si>
+  <si>
+    <t>Chile</t>
+  </si>
+  <si>
+    <t>1213655817740691</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4192 - TRANSPORTES </t>
+  </si>
+  <si>
+    <t>TABL3-196</t>
+  </si>
+  <si>
+    <t>1213628910075658</t>
+  </si>
+  <si>
+    <t>50001511-AURA INGENIERIA</t>
+  </si>
+  <si>
+    <t>TABL3-34</t>
+  </si>
+  <si>
+    <t>1213655817740708</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4236 -REPARACION ZVN 1-16-110/4 NS: 2751-01-2019 </t>
+  </si>
+  <si>
+    <t>TABL3-200</t>
+  </si>
+  <si>
+    <t>1213655817740710</t>
+  </si>
+  <si>
+    <t>OT 4237 - REPARACION ZVN 1-16-110/4 NS: 2751-02-2019</t>
+  </si>
+  <si>
+    <t>TABL3-201</t>
+  </si>
+  <si>
+    <t>1213628910075657</t>
+  </si>
+  <si>
+    <t>50001510-MINERA TIZAPA</t>
+  </si>
+  <si>
+    <t>TABL3-33</t>
+  </si>
+  <si>
+    <t>1213655817740704</t>
+  </si>
+  <si>
+    <t>OT 4235 - SET DE ÁLABES DE REPUESTO PARA VENTILADOR ZVN 1-24</t>
+  </si>
+  <si>
+    <t>TABL3-199</t>
+  </si>
+  <si>
+    <t>1213628910075663</t>
+  </si>
+  <si>
+    <t>50001521-CODELCO</t>
+  </si>
+  <si>
+    <t>TABL3-39</t>
+  </si>
+  <si>
+    <t>1213655817740745</t>
+  </si>
+  <si>
+    <t>OT 4250 - SET DE ALABES S/ PLANO 3806.01</t>
+  </si>
+  <si>
+    <t>TABL3-214</t>
+  </si>
+  <si>
+    <t>1213628910075662</t>
+  </si>
+  <si>
+    <t>50001519-AVO 1</t>
+  </si>
+  <si>
+    <t>Carlos Pérez</t>
+  </si>
+  <si>
+    <t>cperez@zitron.com</t>
+  </si>
+  <si>
+    <t>TABL3-38</t>
+  </si>
+  <si>
+    <t>1213655817740728</t>
+  </si>
+  <si>
+    <t>OT 4267 - ANALISIS Y MEJORAS VENTILACION CANTONES 1, 7 Y 8</t>
+  </si>
+  <si>
+    <t>TABL3-208</t>
+  </si>
+  <si>
+    <t>1213628909802199</t>
+  </si>
+  <si>
+    <t>50001353-ZITRON BRASIL</t>
+  </si>
+  <si>
+    <t>TABL3-58</t>
+  </si>
+  <si>
+    <t>brasil</t>
+  </si>
+  <si>
+    <t>1213655817740365</t>
+  </si>
+  <si>
+    <t>OT 3855-TABLERO PLC</t>
+  </si>
+  <si>
+    <t>TABL3-59</t>
+  </si>
+  <si>
+    <t>1213655817740367</t>
+  </si>
+  <si>
+    <t>OT 3856-TABLERO PLC + 2x DAMPER</t>
+  </si>
+  <si>
+    <t>TABL3-60</t>
+  </si>
+  <si>
+    <t>1213655817740369</t>
+  </si>
+  <si>
+    <t>OT 3857-TABLERO CCM 1x3.7 KW</t>
+  </si>
+  <si>
+    <t>TABL3-61</t>
+  </si>
+  <si>
+    <t>1213655817740371</t>
+  </si>
+  <si>
+    <t>OT 3858- TABLERO CCM 2X 15 KW</t>
+  </si>
+  <si>
+    <t>TABL3-62</t>
+  </si>
+  <si>
+    <t>1213628909802200</t>
+  </si>
+  <si>
+    <t>50001362-ZITRON BRASIL</t>
+  </si>
+  <si>
+    <t>TABL3-49</t>
+  </si>
+  <si>
+    <t>1213655817740379</t>
+  </si>
+  <si>
+    <t>OT 3886- CCM 2SSx15KW</t>
+  </si>
+  <si>
+    <t>TABL3-63</t>
+  </si>
+  <si>
+    <t>1213655817740381</t>
+  </si>
+  <si>
+    <t>OT 3887 -  CCM 2SSx18,5KW</t>
+  </si>
+  <si>
+    <t>TABL3-64</t>
+  </si>
+  <si>
+    <t>1213655817740383</t>
+  </si>
+  <si>
+    <t>OT 3888 - CCM 2SSx30KW</t>
+  </si>
+  <si>
+    <t>TABL3-65</t>
+  </si>
+  <si>
+    <t>1213655817740385</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 3889 -TABLERO PLC </t>
+  </si>
+  <si>
+    <t>TABL3-66</t>
+  </si>
+  <si>
+    <t>1213655817740387</t>
+  </si>
+  <si>
+    <t>OT 3890 - TABLERO PLC + DAMPER</t>
+  </si>
+  <si>
+    <t>TABL3-67</t>
+  </si>
+  <si>
+    <t>1213628910075661</t>
+  </si>
+  <si>
+    <t>50001517-ZITRON BRASIL</t>
+  </si>
+  <si>
+    <t>TABL3-37</t>
+  </si>
+  <si>
+    <t>1213655817740735</t>
+  </si>
+  <si>
+    <t>OT 4249 - RODETE S/PLANO 1991.10.30.D48</t>
+  </si>
+  <si>
+    <t>TABL3-209</t>
+  </si>
+  <si>
+    <t>1213655817740739</t>
+  </si>
+  <si>
+    <t>OT 4257 - TOBERAS AERODINAMICA Ø1100MM</t>
+  </si>
+  <si>
+    <t>TABL3-211</t>
+  </si>
+  <si>
+    <t>1213655817740741</t>
+  </si>
+  <si>
+    <t>OT 4258 - SENSOR VIBRACIONES IFM VKV021</t>
+  </si>
+  <si>
+    <t>TABL3-212</t>
+  </si>
+  <si>
+    <t>1213655817740743</t>
+  </si>
+  <si>
+    <t>OT 4259 - TACO ACELEROMETRO S/PLANO ZCHPC.CPA.40.40.M8</t>
+  </si>
+  <si>
+    <t>TABL3-213</t>
+  </si>
+  <si>
+    <t>1213628910075664</t>
+  </si>
+  <si>
+    <t>50001522-ZITRON BRASIL</t>
+  </si>
+  <si>
+    <t>TABL3-40</t>
+  </si>
+  <si>
+    <t>1213655817740750</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4252 -JUNTAS FLEXIBLES PARA VENTILADOR ZVN 1-24-800/6 </t>
+  </si>
+  <si>
+    <t>TABL3-215</t>
+  </si>
+  <si>
+    <t>1213628910075656</t>
+  </si>
+  <si>
+    <t>50001505-MINERA JUANICIPIO SA DE CV</t>
+  </si>
+  <si>
+    <t>TABL3-32</t>
+  </si>
+  <si>
+    <t>1213655817740698</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4224 - PIÑON MOTOREDUCTOR DAMPER  </t>
+  </si>
+  <si>
+    <t>TABL3-197</t>
+  </si>
+  <si>
+    <t>1213655817740700</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4225 -CREMALLERA DAMPER </t>
+  </si>
+  <si>
+    <t>TABL3-198</t>
+  </si>
+  <si>
+    <t>1213628909802210</t>
+  </si>
+  <si>
+    <t>50001455-GESVIAL</t>
+  </si>
+  <si>
+    <t>Producción</t>
+  </si>
+  <si>
+    <t>TABL3-30</t>
+  </si>
+  <si>
+    <t>1213655817740648</t>
+  </si>
+  <si>
+    <t>OT 4170 - CODOS Y BIFURCACIONES</t>
+  </si>
+  <si>
+    <t>TABL3-183</t>
+  </si>
+  <si>
+    <t>1215727726395453</t>
+  </si>
+  <si>
+    <t>50001561 - GESVIAL</t>
+  </si>
+  <si>
+    <t>TABL3-275</t>
+  </si>
+  <si>
+    <t>1215727726395457</t>
+  </si>
+  <si>
+    <t>OT 4352 - Reparacion ZVN 1-14-110/4</t>
+  </si>
+  <si>
+    <t>TABL3-276</t>
+  </si>
+  <si>
+    <t>1215727726395459</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4353 - Reparacion VDF Danfoss 110 KW </t>
+  </si>
+  <si>
+    <t>TABL3-277</t>
+  </si>
+  <si>
+    <t>1215727332551570</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50001564 - CONTINENTAL GOLD </t>
+  </si>
+  <si>
+    <t>TABL3-280</t>
+  </si>
+  <si>
+    <t>1215727332551573</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4358 - RODETES VENTILADOR GEL 9 </t>
+  </si>
+  <si>
+    <t>TABL3-281</t>
+  </si>
+  <si>
+    <t>1215052134888365</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50001560
+</t>
+  </si>
+  <si>
+    <t>TABL3-272</t>
+  </si>
+  <si>
+    <t>Nicaragua</t>
+  </si>
+  <si>
+    <t>1215052134888368</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4345 -BORNA REF: 3009118 UKH 50 MM2 50 GR </t>
+  </si>
+  <si>
+    <t>TABL3-273</t>
+  </si>
+  <si>
+    <t>1215052134888370</t>
+  </si>
+  <si>
+    <t>OT 4346 - RELE 1SVR508020R0000 ABB CT-MFC.12, 1C/O</t>
+  </si>
+  <si>
+    <t>TABL3-274</t>
+  </si>
+  <si>
     <t>1214150417415474</t>
   </si>
   <si>
@@ -226,9 +641,6 @@
     <t>TABL3-240</t>
   </si>
   <si>
-    <t>Chile</t>
-  </si>
-  <si>
     <t>1214150417415479</t>
   </si>
   <si>
@@ -263,418 +675,6 @@
   </si>
   <si>
     <t>TABL3-244</t>
-  </si>
-  <si>
-    <t>1214150417415449</t>
-  </si>
-  <si>
-    <t>50001529 - MINERA ROBLE</t>
-  </si>
-  <si>
-    <t>TABL3-232</t>
-  </si>
-  <si>
-    <t>1214150417415454</t>
-  </si>
-  <si>
-    <t>OT 4272-Rodete ZVN 1-9-86/2</t>
-  </si>
-  <si>
-    <t>TABL3-233</t>
-  </si>
-  <si>
-    <t>1213628910075654</t>
-  </si>
-  <si>
-    <t>50001493-GESVIAL</t>
-  </si>
-  <si>
-    <t>TABL3-47</t>
-  </si>
-  <si>
-    <t>1213655817740691</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4192 - TRANSPORTES </t>
-  </si>
-  <si>
-    <t>TABL3-196</t>
-  </si>
-  <si>
-    <t>1213628910075658</t>
-  </si>
-  <si>
-    <t>50001511-AURA INGENIERIA</t>
-  </si>
-  <si>
-    <t>TABL3-34</t>
-  </si>
-  <si>
-    <t>1213655817740708</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4236 -REPARACION ZVN 1-16-110/4 NS: 2751-01-2019 </t>
-  </si>
-  <si>
-    <t>TABL3-200</t>
-  </si>
-  <si>
-    <t>1213655817740710</t>
-  </si>
-  <si>
-    <t>OT 4237 - REPARACION ZVN 1-16-110/4 NS: 2751-02-2019</t>
-  </si>
-  <si>
-    <t>TABL3-201</t>
-  </si>
-  <si>
-    <t>1213628910075657</t>
-  </si>
-  <si>
-    <t>50001510-MINERA TIZAPA</t>
-  </si>
-  <si>
-    <t>TABL3-33</t>
-  </si>
-  <si>
-    <t>1213655817740704</t>
-  </si>
-  <si>
-    <t>OT 4235 - SET DE ÁLABES DE REPUESTO PARA VENTILADOR ZVN 1-24</t>
-  </si>
-  <si>
-    <t>TABL3-199</t>
-  </si>
-  <si>
-    <t>1213628910075663</t>
-  </si>
-  <si>
-    <t>50001521-CODELCO</t>
-  </si>
-  <si>
-    <t>TABL3-39</t>
-  </si>
-  <si>
-    <t>1213655817740745</t>
-  </si>
-  <si>
-    <t>OT 4250 - SET DE ALABES S/ PLANO 3806.01</t>
-  </si>
-  <si>
-    <t>TABL3-214</t>
-  </si>
-  <si>
-    <t>1213628910075662</t>
-  </si>
-  <si>
-    <t>50001519-AVO 1</t>
-  </si>
-  <si>
-    <t>Carlos Pérez</t>
-  </si>
-  <si>
-    <t>cperez@zitron.com</t>
-  </si>
-  <si>
-    <t>TABL3-38</t>
-  </si>
-  <si>
-    <t>1213655817740728</t>
-  </si>
-  <si>
-    <t>OT 4267 - ANALISIS Y MEJORAS VENTILACION CANTONES 1, 7 Y 8</t>
-  </si>
-  <si>
-    <t>TABL3-208</t>
-  </si>
-  <si>
-    <t>1213628909802199</t>
-  </si>
-  <si>
-    <t>50001353-ZITRON BRASIL</t>
-  </si>
-  <si>
-    <t>TABL3-58</t>
-  </si>
-  <si>
-    <t>brasil</t>
-  </si>
-  <si>
-    <t>1213655817740365</t>
-  </si>
-  <si>
-    <t>OT 3855-TABLERO PLC</t>
-  </si>
-  <si>
-    <t>TABL3-59</t>
-  </si>
-  <si>
-    <t>1213655817740367</t>
-  </si>
-  <si>
-    <t>OT 3856-TABLERO PLC + 2x DAMPER</t>
-  </si>
-  <si>
-    <t>TABL3-60</t>
-  </si>
-  <si>
-    <t>1213655817740369</t>
-  </si>
-  <si>
-    <t>OT 3857-TABLERO CCM 1x3.7 KW</t>
-  </si>
-  <si>
-    <t>TABL3-61</t>
-  </si>
-  <si>
-    <t>1213655817740371</t>
-  </si>
-  <si>
-    <t>OT 3858- TABLERO CCM 2X 15 KW</t>
-  </si>
-  <si>
-    <t>TABL3-62</t>
-  </si>
-  <si>
-    <t>1213628909802200</t>
-  </si>
-  <si>
-    <t>50001362-ZITRON BRASIL</t>
-  </si>
-  <si>
-    <t>TABL3-49</t>
-  </si>
-  <si>
-    <t>1213655817740379</t>
-  </si>
-  <si>
-    <t>OT 3886- CCM 2SSx15KW</t>
-  </si>
-  <si>
-    <t>TABL3-63</t>
-  </si>
-  <si>
-    <t>1213655817740381</t>
-  </si>
-  <si>
-    <t>OT 3887 -  CCM 2SSx18,5KW</t>
-  </si>
-  <si>
-    <t>TABL3-64</t>
-  </si>
-  <si>
-    <t>1213655817740383</t>
-  </si>
-  <si>
-    <t>OT 3888 - CCM 2SSx30KW</t>
-  </si>
-  <si>
-    <t>TABL3-65</t>
-  </si>
-  <si>
-    <t>1213655817740385</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 3889 -TABLERO PLC </t>
-  </si>
-  <si>
-    <t>TABL3-66</t>
-  </si>
-  <si>
-    <t>1213655817740387</t>
-  </si>
-  <si>
-    <t>OT 3890 - TABLERO PLC + DAMPER</t>
-  </si>
-  <si>
-    <t>TABL3-67</t>
-  </si>
-  <si>
-    <t>1213628910075661</t>
-  </si>
-  <si>
-    <t>50001517-ZITRON BRASIL</t>
-  </si>
-  <si>
-    <t>TABL3-37</t>
-  </si>
-  <si>
-    <t>1213655817740735</t>
-  </si>
-  <si>
-    <t>OT 4249 - RODETE S/PLANO 1991.10.30.D48</t>
-  </si>
-  <si>
-    <t>TABL3-209</t>
-  </si>
-  <si>
-    <t>1213655817740739</t>
-  </si>
-  <si>
-    <t>OT 4257 - TOBERAS AERODINAMICA Ø1100MM</t>
-  </si>
-  <si>
-    <t>TABL3-211</t>
-  </si>
-  <si>
-    <t>1213655817740741</t>
-  </si>
-  <si>
-    <t>OT 4258 - SENSOR VIBRACIONES IFM VKV021</t>
-  </si>
-  <si>
-    <t>TABL3-212</t>
-  </si>
-  <si>
-    <t>1213655817740743</t>
-  </si>
-  <si>
-    <t>OT 4259 - TACO ACELEROMETRO S/PLANO ZCHPC.CPA.40.40.M8</t>
-  </si>
-  <si>
-    <t>TABL3-213</t>
-  </si>
-  <si>
-    <t>1213628910075664</t>
-  </si>
-  <si>
-    <t>50001522-ZITRON BRASIL</t>
-  </si>
-  <si>
-    <t>TABL3-40</t>
-  </si>
-  <si>
-    <t>1213655817740750</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4252 -JUNTAS FLEXIBLES PARA VENTILADOR ZVN 1-24-800/6 </t>
-  </si>
-  <si>
-    <t>TABL3-215</t>
-  </si>
-  <si>
-    <t>1213628910075656</t>
-  </si>
-  <si>
-    <t>50001505-MINERA JUANICIPIO SA DE CV</t>
-  </si>
-  <si>
-    <t>TABL3-32</t>
-  </si>
-  <si>
-    <t>1213655817740698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4224 - PIÑON MOTOREDUCTOR DAMPER  </t>
-  </si>
-  <si>
-    <t>TABL3-197</t>
-  </si>
-  <si>
-    <t>1213655817740700</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4225 -CREMALLERA DAMPER </t>
-  </si>
-  <si>
-    <t>TABL3-198</t>
-  </si>
-  <si>
-    <t>1213628909802210</t>
-  </si>
-  <si>
-    <t>50001455-GESVIAL</t>
-  </si>
-  <si>
-    <t>Producción</t>
-  </si>
-  <si>
-    <t>TABL3-30</t>
-  </si>
-  <si>
-    <t>1213655817740648</t>
-  </si>
-  <si>
-    <t>OT 4170 - CODOS Y BIFURCACIONES</t>
-  </si>
-  <si>
-    <t>TABL3-183</t>
-  </si>
-  <si>
-    <t>1215727726395453</t>
-  </si>
-  <si>
-    <t>50001561 - GESVIAL</t>
-  </si>
-  <si>
-    <t>TABL3-275</t>
-  </si>
-  <si>
-    <t>1215727726395457</t>
-  </si>
-  <si>
-    <t>OT 4352 - Reparacion ZVN 1-14-110/4</t>
-  </si>
-  <si>
-    <t>TABL3-276</t>
-  </si>
-  <si>
-    <t>1215727726395459</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4353 - Reparacion VDF Danfoss 110 KW </t>
-  </si>
-  <si>
-    <t>TABL3-277</t>
-  </si>
-  <si>
-    <t>1215727332551570</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50001564 - CONTINENTAL GOLD </t>
-  </si>
-  <si>
-    <t>TABL3-280</t>
-  </si>
-  <si>
-    <t>1215727332551573</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4358 - RODETES VENTILADOR GEL 9 </t>
-  </si>
-  <si>
-    <t>TABL3-281</t>
-  </si>
-  <si>
-    <t>1215052134888365</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50001560
-</t>
-  </si>
-  <si>
-    <t>TABL3-272</t>
-  </si>
-  <si>
-    <t>Nicaragua</t>
-  </si>
-  <si>
-    <t>1215052134888368</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4345 -BORNA REF: 3009118 UKH 50 MM2 50 GR </t>
-  </si>
-  <si>
-    <t>TABL3-273</t>
-  </si>
-  <si>
-    <t>1215052134888370</t>
-  </si>
-  <si>
-    <t>OT 4346 - RELE 1SVR508020R0000 ABB CT-MFC.12, 1C/O</t>
-  </si>
-  <si>
-    <t>TABL3-274</t>
   </si>
   <si>
     <t>1214787972061588</t>
@@ -2800,11 +2800,11 @@
         <v>66</v>
       </c>
       <c r="B14" s="5">
-        <v>46133.80470612268</v>
+        <v>46133.79901350694</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46210.806753993056</v>
+        <v>46209.798431145835</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>67</v>
@@ -2820,7 +2820,7 @@
       </c>
       <c r="I14" s="6"/>
       <c r="J14" s="5">
-        <v>46161</v>
+        <v>46120</v>
       </c>
       <c r="K14" s="6" t="s">
         <v>28</v>
@@ -2847,24 +2847,24 @@
       <c r="S14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="T14" s="14" t="s">
-        <v>69</v>
+      <c r="T14" s="13" t="s">
+        <v>56</v>
       </c>
       <c r="U14" s="6"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B15" s="10">
-        <v>46133.80545771991</v>
+        <v>46133.79961443287</v>
       </c>
       <c r="C15" s="11"/>
       <c r="D15" s="10">
-        <v>46133.80564510416</v>
+        <v>46133.79989851852</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F15" s="11" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>28</v>
       </c>
       <c r="Q15" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="R15" s="11"/>
       <c r="S15" s="11"/>
@@ -2903,51 +2903,59 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B16" s="5">
-        <v>46133.80570512731</v>
+        <v>46093.557977812496</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="5">
-        <v>46133.80583366899</v>
+        <v>46210.80365065973</v>
       </c>
       <c r="E16" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="I16" s="6"/>
+      <c r="J16" s="5">
+        <v>46039</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="O16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q16" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="F16" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="L16" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="N16" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="O16" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="P16" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q16" s="6" t="s">
+      <c r="R16" s="6"/>
+      <c r="S16" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T16" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="R16" s="6"/>
-      <c r="S16" s="6"/>
-      <c r="T16" s="6"/>
       <c r="U16" s="6"/>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
@@ -2955,11 +2963,11 @@
         <v>76</v>
       </c>
       <c r="B17" s="10">
-        <v>46133.8058850463</v>
+        <v>46094.64358574074</v>
       </c>
       <c r="C17" s="11"/>
       <c r="D17" s="10">
-        <v>46133.80636234954</v>
+        <v>46094.643782430554</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>77</v>
@@ -2983,7 +2991,7 @@
         <v>28</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="O17" s="11" t="s">
         <v>28</v>
@@ -3004,24 +3012,28 @@
         <v>79</v>
       </c>
       <c r="B18" s="5">
-        <v>46133.80664880787</v>
+        <v>46093.55797666666</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46133.80681135417</v>
+        <v>46210.798552395834</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>80</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H18" s="6"/>
+        <v>46</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>47</v>
+      </c>
       <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
+      <c r="J18" s="5">
+        <v>46083</v>
+      </c>
       <c r="K18" s="6" t="s">
         <v>28</v>
       </c>
@@ -3029,10 +3041,10 @@
         <v>28</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>28</v>
@@ -3044,8 +3056,12 @@
         <v>81</v>
       </c>
       <c r="R18" s="6"/>
-      <c r="S18" s="6"/>
-      <c r="T18" s="6"/>
+      <c r="S18" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T18" s="14" t="s">
+        <v>75</v>
+      </c>
       <c r="U18" s="6"/>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
@@ -3053,28 +3069,24 @@
         <v>82</v>
       </c>
       <c r="B19" s="10">
-        <v>46133.79901350694</v>
+        <v>46094.64611630787</v>
       </c>
       <c r="C19" s="11"/>
       <c r="D19" s="10">
-        <v>46209.798431145835</v>
+        <v>46094.64631732639</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>83</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="H19" s="11" t="s">
-        <v>47</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H19" s="11"/>
       <c r="I19" s="11"/>
-      <c r="J19" s="10">
-        <v>46120</v>
-      </c>
+      <c r="J19" s="11"/>
       <c r="K19" s="11" t="s">
         <v>28</v>
       </c>
@@ -3082,10 +3094,10 @@
         <v>28</v>
       </c>
       <c r="M19" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="O19" s="11" t="s">
         <v>28</v>
@@ -3097,12 +3109,8 @@
         <v>84</v>
       </c>
       <c r="R19" s="11"/>
-      <c r="S19" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T19" s="13" t="s">
-        <v>56</v>
-      </c>
+      <c r="S19" s="11"/>
+      <c r="T19" s="11"/>
       <c r="U19" s="11"/>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
@@ -3110,11 +3118,11 @@
         <v>85</v>
       </c>
       <c r="B20" s="5">
-        <v>46133.79961443287</v>
+        <v>46094.64632454861</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="5">
-        <v>46133.79989851852</v>
+        <v>46094.64655788195</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>86</v>
@@ -3138,7 +3146,7 @@
         <v>28</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="O20" s="6" t="s">
         <v>28</v>
@@ -3159,11 +3167,11 @@
         <v>88</v>
       </c>
       <c r="B21" s="10">
-        <v>46093.557977812496</v>
+        <v>46093.55797637731</v>
       </c>
       <c r="C21" s="11"/>
       <c r="D21" s="10">
-        <v>46210.80365065973</v>
+        <v>46210.80012583333</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>89</v>
@@ -3179,7 +3187,7 @@
       </c>
       <c r="I21" s="11"/>
       <c r="J21" s="10">
-        <v>46039</v>
+        <v>46080</v>
       </c>
       <c r="K21" s="11" t="s">
         <v>28</v>
@@ -3206,8 +3214,8 @@
       <c r="S21" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="T21" s="14" t="s">
-        <v>69</v>
+      <c r="T21" s="13" t="s">
+        <v>56</v>
       </c>
       <c r="U21" s="11"/>
     </row>
@@ -3216,11 +3224,11 @@
         <v>91</v>
       </c>
       <c r="B22" s="5">
-        <v>46094.64358574074</v>
+        <v>46094.645434618054</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46094.643782430554</v>
+        <v>46094.645602916666</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>92</v>
@@ -3265,11 +3273,11 @@
         <v>94</v>
       </c>
       <c r="B23" s="10">
-        <v>46093.55797666666</v>
+        <v>46093.55797821759</v>
       </c>
       <c r="C23" s="11"/>
       <c r="D23" s="10">
-        <v>46210.798552395834</v>
+        <v>46210.81134996528</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>95</v>
@@ -3285,7 +3293,7 @@
       </c>
       <c r="I23" s="11"/>
       <c r="J23" s="10">
-        <v>46083</v>
+        <v>46092</v>
       </c>
       <c r="K23" s="11" t="s">
         <v>28</v>
@@ -3313,7 +3321,7 @@
         <v>30</v>
       </c>
       <c r="T23" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U23" s="11"/>
     </row>
@@ -3322,11 +3330,11 @@
         <v>97</v>
       </c>
       <c r="B24" s="5">
-        <v>46094.64611630787</v>
+        <v>46094.65140127315</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="5">
-        <v>46094.64631732639</v>
+        <v>46094.65150827546</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>98</v>
@@ -3371,24 +3379,28 @@
         <v>100</v>
       </c>
       <c r="B25" s="10">
-        <v>46094.64632454861</v>
+        <v>46093.55797792824</v>
       </c>
       <c r="C25" s="11"/>
       <c r="D25" s="10">
-        <v>46094.64655788195</v>
+        <v>46134.689549421295</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>101</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H25" s="11"/>
+        <v>102</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>103</v>
+      </c>
       <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
+      <c r="J25" s="10">
+        <v>46097</v>
+      </c>
       <c r="K25" s="11" t="s">
         <v>28</v>
       </c>
@@ -3396,10 +3408,10 @@
         <v>28</v>
       </c>
       <c r="M25" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N25" s="11" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="O25" s="11" t="s">
         <v>28</v>
@@ -3408,40 +3420,40 @@
         <v>28</v>
       </c>
       <c r="Q25" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="R25" s="11"/>
-      <c r="S25" s="11"/>
-      <c r="T25" s="11"/>
+      <c r="S25" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T25" s="14" t="s">
+        <v>75</v>
+      </c>
       <c r="U25" s="11"/>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B26" s="5">
-        <v>46093.55797637731</v>
+        <v>46094.64988140046</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="5">
-        <v>46210.80012583333</v>
+        <v>46094.64998811342</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>47</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H26" s="6"/>
       <c r="I26" s="6"/>
-      <c r="J26" s="5">
-        <v>46080</v>
-      </c>
+      <c r="J26" s="6"/>
       <c r="K26" s="6" t="s">
         <v>28</v>
       </c>
@@ -3449,10 +3461,10 @@
         <v>28</v>
       </c>
       <c r="M26" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>28</v>
+        <v>101</v>
       </c>
       <c r="O26" s="6" t="s">
         <v>28</v>
@@ -3461,40 +3473,42 @@
         <v>28</v>
       </c>
       <c r="Q26" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="R26" s="6"/>
-      <c r="S26" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T26" s="13" t="s">
-        <v>56</v>
-      </c>
+      <c r="S26" s="6"/>
+      <c r="T26" s="6"/>
       <c r="U26" s="6"/>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B27" s="10">
-        <v>46094.645434618054</v>
+        <v>46093.55797513889</v>
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="10">
-        <v>46094.645602916666</v>
+        <v>46098.62589137732</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
+        <v>102</v>
+      </c>
+      <c r="H27" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I27" s="10">
+        <v>46041</v>
+      </c>
+      <c r="J27" s="10">
+        <v>46041</v>
+      </c>
       <c r="K27" s="11" t="s">
         <v>28</v>
       </c>
@@ -3502,10 +3516,10 @@
         <v>28</v>
       </c>
       <c r="M27" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N27" s="11" t="s">
-        <v>104</v>
+        <v>28</v>
       </c>
       <c r="O27" s="11" t="s">
         <v>28</v>
@@ -3514,40 +3528,40 @@
         <v>28</v>
       </c>
       <c r="Q27" s="11" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="R27" s="11"/>
-      <c r="S27" s="11"/>
-      <c r="T27" s="11"/>
+      <c r="S27" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T27" s="13" t="s">
+        <v>111</v>
+      </c>
       <c r="U27" s="11"/>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B28" s="5">
-        <v>46093.55797821759</v>
+        <v>46094.566601597224</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46210.81134996528</v>
+        <v>46094.56736538194</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>47</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H28" s="6"/>
       <c r="I28" s="6"/>
-      <c r="J28" s="5">
-        <v>46092</v>
-      </c>
+      <c r="J28" s="6"/>
       <c r="K28" s="6" t="s">
         <v>28</v>
       </c>
@@ -3555,10 +3569,10 @@
         <v>28</v>
       </c>
       <c r="M28" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>28</v>
+        <v>109</v>
       </c>
       <c r="O28" s="6" t="s">
         <v>28</v>
@@ -3567,30 +3581,26 @@
         <v>28</v>
       </c>
       <c r="Q28" s="6" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="R28" s="6"/>
-      <c r="S28" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T28" s="14" t="s">
-        <v>69</v>
-      </c>
+      <c r="S28" s="6"/>
+      <c r="T28" s="6"/>
       <c r="U28" s="6"/>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B29" s="10">
-        <v>46094.65140127315</v>
+        <v>46094.566937951386</v>
       </c>
       <c r="C29" s="11"/>
       <c r="D29" s="10">
-        <v>46094.65150827546</v>
+        <v>46094.56773407407</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F29" s="11" t="s">
         <v>28</v>
@@ -3611,7 +3621,7 @@
         <v>28</v>
       </c>
       <c r="N29" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O29" s="11" t="s">
         <v>28</v>
@@ -3620,7 +3630,7 @@
         <v>28</v>
       </c>
       <c r="Q29" s="11" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="R29" s="11"/>
       <c r="S29" s="11"/>
@@ -3629,31 +3639,27 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B30" s="5">
-        <v>46093.55797792824</v>
+        <v>46094.56748170139</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46134.689549421295</v>
+        <v>46094.56795886574</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>118</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H30" s="6"/>
       <c r="I30" s="6"/>
-      <c r="J30" s="5">
-        <v>46097</v>
-      </c>
+      <c r="J30" s="6"/>
       <c r="K30" s="6" t="s">
         <v>28</v>
       </c>
@@ -3661,10 +3667,10 @@
         <v>28</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>28</v>
+        <v>109</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>28</v>
@@ -3673,30 +3679,26 @@
         <v>28</v>
       </c>
       <c r="Q30" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="R30" s="6"/>
-      <c r="S30" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T30" s="14" t="s">
-        <v>69</v>
-      </c>
+      <c r="S30" s="6"/>
+      <c r="T30" s="6"/>
       <c r="U30" s="6"/>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B31" s="10">
-        <v>46094.64988140046</v>
+        <v>46094.56796667824</v>
       </c>
       <c r="C31" s="11"/>
       <c r="D31" s="10">
-        <v>46094.64998811342</v>
+        <v>46094.56820407408</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F31" s="11" t="s">
         <v>28</v>
@@ -3717,7 +3719,7 @@
         <v>28</v>
       </c>
       <c r="N31" s="11" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="O31" s="11" t="s">
         <v>28</v>
@@ -3726,7 +3728,7 @@
         <v>28</v>
       </c>
       <c r="Q31" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="R31" s="11"/>
       <c r="S31" s="11"/>
@@ -3735,26 +3737,26 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B32" s="5">
-        <v>46093.55797513889</v>
+        <v>46093.557975625</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="5">
-        <v>46098.62589137732</v>
+        <v>46112.84178105324</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>54</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="I32" s="5">
         <v>46041</v>
@@ -3781,14 +3783,14 @@
         <v>28</v>
       </c>
       <c r="Q32" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="R32" s="6"/>
       <c r="S32" s="7" t="s">
         <v>30</v>
       </c>
       <c r="T32" s="13" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="U32" s="6"/>
     </row>
@@ -3797,11 +3799,11 @@
         <v>127</v>
       </c>
       <c r="B33" s="10">
-        <v>46094.566601597224</v>
+        <v>46094.57064802083</v>
       </c>
       <c r="C33" s="11"/>
       <c r="D33" s="10">
-        <v>46094.56736538194</v>
+        <v>46094.59020585648</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>128</v>
@@ -3825,7 +3827,7 @@
         <v>28</v>
       </c>
       <c r="N33" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O33" s="11" t="s">
         <v>28</v>
@@ -3846,11 +3848,11 @@
         <v>130</v>
       </c>
       <c r="B34" s="5">
-        <v>46094.566937951386</v>
+        <v>46094.57343428241</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="5">
-        <v>46094.56773407407</v>
+        <v>46094.59023394676</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>131</v>
@@ -3874,7 +3876,7 @@
         <v>28</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>28</v>
@@ -3895,11 +3897,11 @@
         <v>133</v>
       </c>
       <c r="B35" s="10">
-        <v>46094.56748170139</v>
+        <v>46094.573594710644</v>
       </c>
       <c r="C35" s="11"/>
       <c r="D35" s="10">
-        <v>46094.56795886574</v>
+        <v>46094.59026199074</v>
       </c>
       <c r="E35" s="11" t="s">
         <v>134</v>
@@ -3923,7 +3925,7 @@
         <v>28</v>
       </c>
       <c r="N35" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O35" s="11" t="s">
         <v>28</v>
@@ -3944,11 +3946,11 @@
         <v>136</v>
       </c>
       <c r="B36" s="5">
-        <v>46094.56796667824</v>
+        <v>46094.57373981482</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46094.56820407408</v>
+        <v>46094.59030239584</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>137</v>
@@ -3972,7 +3974,7 @@
         <v>28</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O36" s="6" t="s">
         <v>28</v>
@@ -3993,30 +3995,24 @@
         <v>139</v>
       </c>
       <c r="B37" s="10">
-        <v>46093.557975625</v>
+        <v>46094.573880254626</v>
       </c>
       <c r="C37" s="11"/>
       <c r="D37" s="10">
-        <v>46112.84178105324</v>
+        <v>46094.59033287037</v>
       </c>
       <c r="E37" s="11" t="s">
         <v>140</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="H37" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="I37" s="10">
-        <v>46041</v>
-      </c>
-      <c r="J37" s="10">
-        <v>46041</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+      <c r="J37" s="11"/>
       <c r="K37" s="11" t="s">
         <v>28</v>
       </c>
@@ -4024,10 +4020,10 @@
         <v>28</v>
       </c>
       <c r="M37" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N37" s="11" t="s">
-        <v>28</v>
+        <v>125</v>
       </c>
       <c r="O37" s="11" t="s">
         <v>28</v>
@@ -4039,12 +4035,8 @@
         <v>141</v>
       </c>
       <c r="R37" s="11"/>
-      <c r="S37" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T37" s="13" t="s">
-        <v>126</v>
-      </c>
+      <c r="S37" s="11"/>
+      <c r="T37" s="11"/>
       <c r="U37" s="11"/>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
@@ -4052,24 +4044,28 @@
         <v>142</v>
       </c>
       <c r="B38" s="5">
-        <v>46094.57064802083</v>
+        <v>46093.55797761574</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46094.59020585648</v>
+        <v>46099.63241893519</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>143</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H38" s="6"/>
+        <v>102</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>103</v>
+      </c>
       <c r="I38" s="6"/>
-      <c r="J38" s="6"/>
+      <c r="J38" s="5">
+        <v>46092</v>
+      </c>
       <c r="K38" s="6" t="s">
         <v>28</v>
       </c>
@@ -4077,10 +4073,10 @@
         <v>28</v>
       </c>
       <c r="M38" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>140</v>
+        <v>28</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>28</v>
@@ -4092,8 +4088,12 @@
         <v>144</v>
       </c>
       <c r="R38" s="6"/>
-      <c r="S38" s="6"/>
-      <c r="T38" s="6"/>
+      <c r="S38" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T38" s="13" t="s">
+        <v>111</v>
+      </c>
       <c r="U38" s="6"/>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
@@ -4101,17 +4101,17 @@
         <v>145</v>
       </c>
       <c r="B39" s="10">
-        <v>46094.57343428241</v>
+        <v>46094.65047047454</v>
       </c>
       <c r="C39" s="11"/>
       <c r="D39" s="10">
-        <v>46094.59023394676</v>
+        <v>46111.83610230324</v>
       </c>
       <c r="E39" s="11" t="s">
         <v>146</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G39" s="11" t="s">
         <v>28</v>
@@ -4126,10 +4126,10 @@
         <v>28</v>
       </c>
       <c r="M39" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N39" s="11" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="O39" s="11" t="s">
         <v>28</v>
@@ -4150,11 +4150,11 @@
         <v>148</v>
       </c>
       <c r="B40" s="5">
-        <v>46094.573594710644</v>
+        <v>46094.65072855324</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46094.59026199074</v>
+        <v>46094.65083585648</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>149</v>
@@ -4178,7 +4178,7 @@
         <v>28</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>28</v>
@@ -4199,11 +4199,11 @@
         <v>151</v>
       </c>
       <c r="B41" s="10">
-        <v>46094.57373981482</v>
+        <v>46094.650843634256</v>
       </c>
       <c r="C41" s="11"/>
       <c r="D41" s="10">
-        <v>46094.59030239584</v>
+        <v>46094.65119138889</v>
       </c>
       <c r="E41" s="11" t="s">
         <v>152</v>
@@ -4227,7 +4227,7 @@
         <v>28</v>
       </c>
       <c r="N41" s="11" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="O41" s="11" t="s">
         <v>28</v>
@@ -4248,11 +4248,11 @@
         <v>154</v>
       </c>
       <c r="B42" s="5">
-        <v>46094.573880254626</v>
+        <v>46094.65095365741</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46094.59033287037</v>
+        <v>46094.65121894676</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>155</v>
@@ -4276,7 +4276,7 @@
         <v>28</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>28</v>
@@ -4297,11 +4297,11 @@
         <v>157</v>
       </c>
       <c r="B43" s="10">
-        <v>46093.55797761574</v>
+        <v>46093.55797850694</v>
       </c>
       <c r="C43" s="11"/>
       <c r="D43" s="10">
-        <v>46099.63241893519</v>
+        <v>46099.62486652778</v>
       </c>
       <c r="E43" s="11" t="s">
         <v>158</v>
@@ -4310,10 +4310,10 @@
         <v>54</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="H43" s="11" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="I43" s="11"/>
       <c r="J43" s="10">
@@ -4345,7 +4345,7 @@
         <v>30</v>
       </c>
       <c r="T43" s="13" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="U43" s="11"/>
     </row>
@@ -4354,17 +4354,17 @@
         <v>160</v>
       </c>
       <c r="B44" s="5">
-        <v>46094.65047047454</v>
+        <v>46094.65201979167</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46111.83610230324</v>
+        <v>46094.652139756945</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>161</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G44" s="6" t="s">
         <v>28</v>
@@ -4379,7 +4379,7 @@
         <v>28</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N44" s="6" t="s">
         <v>158</v>
@@ -4403,24 +4403,30 @@
         <v>163</v>
       </c>
       <c r="B45" s="10">
-        <v>46094.65072855324</v>
-      </c>
-      <c r="C45" s="11"/>
+        <v>46093.55797605324</v>
+      </c>
+      <c r="C45" s="10">
+        <v>46140.73067185185</v>
+      </c>
       <c r="D45" s="10">
-        <v>46094.65083585648</v>
+        <v>46140.730673252314</v>
       </c>
       <c r="E45" s="11" t="s">
         <v>164</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H45" s="11"/>
+        <v>46</v>
+      </c>
+      <c r="H45" s="11" t="s">
+        <v>47</v>
+      </c>
       <c r="I45" s="11"/>
-      <c r="J45" s="11"/>
+      <c r="J45" s="10">
+        <v>46059</v>
+      </c>
       <c r="K45" s="11" t="s">
         <v>28</v>
       </c>
@@ -4428,10 +4434,10 @@
         <v>28</v>
       </c>
       <c r="M45" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N45" s="11" t="s">
-        <v>158</v>
+        <v>28</v>
       </c>
       <c r="O45" s="11" t="s">
         <v>28</v>
@@ -4443,8 +4449,12 @@
         <v>165</v>
       </c>
       <c r="R45" s="11"/>
-      <c r="S45" s="11"/>
-      <c r="T45" s="11"/>
+      <c r="S45" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T45" s="13" t="s">
+        <v>56</v>
+      </c>
       <c r="U45" s="11"/>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
@@ -4452,11 +4462,11 @@
         <v>166</v>
       </c>
       <c r="B46" s="5">
-        <v>46094.650843634256</v>
+        <v>46094.644745763886</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46094.65119138889</v>
+        <v>46094.644892048615</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>167</v>
@@ -4480,7 +4490,7 @@
         <v>28</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>28</v>
@@ -4501,11 +4511,11 @@
         <v>169</v>
       </c>
       <c r="B47" s="10">
-        <v>46094.65095365741</v>
+        <v>46094.64489846065</v>
       </c>
       <c r="C47" s="11"/>
       <c r="D47" s="10">
-        <v>46094.65121894676</v>
+        <v>46094.64504228009</v>
       </c>
       <c r="E47" s="11" t="s">
         <v>170</v>
@@ -4529,7 +4539,7 @@
         <v>28</v>
       </c>
       <c r="N47" s="11" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="O47" s="11" t="s">
         <v>28</v>
@@ -4550,27 +4560,27 @@
         <v>172</v>
       </c>
       <c r="B48" s="5">
-        <v>46093.55797850694</v>
+        <v>46093.557975648146</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46099.62486652778</v>
+        <v>46209.809115578704</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>173</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>54</v>
+        <v>174</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>117</v>
+        <v>46</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>118</v>
+        <v>47</v>
       </c>
       <c r="I48" s="6"/>
       <c r="J48" s="5">
-        <v>46092</v>
+        <v>46031</v>
       </c>
       <c r="K48" s="6" t="s">
         <v>28</v>
@@ -4591,30 +4601,26 @@
         <v>28</v>
       </c>
       <c r="Q48" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="R48" s="6"/>
-      <c r="S48" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T48" s="13" t="s">
-        <v>126</v>
-      </c>
+      <c r="S48" s="6"/>
+      <c r="T48" s="6"/>
       <c r="U48" s="6"/>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B49" s="10">
-        <v>46094.65201979167</v>
+        <v>46094.63446598379</v>
       </c>
       <c r="C49" s="11"/>
       <c r="D49" s="10">
-        <v>46094.652139756945</v>
+        <v>46094.63463712963</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F49" s="11" t="s">
         <v>28</v>
@@ -4644,7 +4650,7 @@
         <v>28</v>
       </c>
       <c r="Q49" s="11" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="R49" s="11"/>
       <c r="S49" s="11"/>
@@ -4653,22 +4659,20 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B50" s="5">
-        <v>46093.55797605324</v>
-      </c>
-      <c r="C50" s="5">
-        <v>46140.73067185185</v>
-      </c>
+        <v>46188.62962413194</v>
+      </c>
+      <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46140.730673252314</v>
+        <v>46210.660290995365</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>54</v>
+        <v>174</v>
       </c>
       <c r="G50" s="6" t="s">
         <v>46</v>
@@ -4677,9 +4681,7 @@
         <v>47</v>
       </c>
       <c r="I50" s="6"/>
-      <c r="J50" s="5">
-        <v>46059</v>
-      </c>
+      <c r="J50" s="6"/>
       <c r="K50" s="6" t="s">
         <v>28</v>
       </c>
@@ -4699,40 +4701,46 @@
         <v>28</v>
       </c>
       <c r="Q50" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="R50" s="6"/>
-      <c r="S50" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T50" s="13" t="s">
-        <v>56</v>
+      <c r="S50" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="T50" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="U50" s="6"/>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B51" s="10">
-        <v>46094.644745763886</v>
-      </c>
-      <c r="C51" s="11"/>
+        <v>46188.63002254629</v>
+      </c>
+      <c r="C51" s="10">
+        <v>46209.92160893518</v>
+      </c>
       <c r="D51" s="10">
-        <v>46094.644892048615</v>
+        <v>46210.78237596065</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G51" s="11" t="s">
         <v>28</v>
       </c>
       <c r="H51" s="11"/>
-      <c r="I51" s="11"/>
-      <c r="J51" s="11"/>
+      <c r="I51" s="10">
+        <v>46195</v>
+      </c>
+      <c r="J51" s="10">
+        <v>46195</v>
+      </c>
       <c r="K51" s="11" t="s">
         <v>28</v>
       </c>
@@ -4740,10 +4748,10 @@
         <v>28</v>
       </c>
       <c r="M51" s="11" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N51" s="11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="O51" s="11" t="s">
         <v>28</v>
@@ -4752,36 +4760,42 @@
         <v>28</v>
       </c>
       <c r="Q51" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="R51" s="11"/>
-      <c r="S51" s="11"/>
+      <c r="S51" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="T51" s="11"/>
       <c r="U51" s="11"/>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B52" s="5">
-        <v>46094.64489846065</v>
-      </c>
-      <c r="C52" s="6"/>
+        <v>46188.630276365744</v>
+      </c>
+      <c r="C52" s="5">
+        <v>46210.76125015046</v>
+      </c>
       <c r="D52" s="5">
-        <v>46094.64504228009</v>
+        <v>46210.761251979166</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G52" s="6" t="s">
         <v>28</v>
       </c>
       <c r="H52" s="6"/>
       <c r="I52" s="6"/>
-      <c r="J52" s="6"/>
+      <c r="J52" s="5">
+        <v>46195</v>
+      </c>
       <c r="K52" s="6" t="s">
         <v>28</v>
       </c>
@@ -4789,10 +4803,10 @@
         <v>28</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>28</v>
@@ -4801,7 +4815,7 @@
         <v>28</v>
       </c>
       <c r="Q52" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="R52" s="6"/>
       <c r="S52" s="6"/>
@@ -4810,31 +4824,29 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B53" s="10">
-        <v>46093.557975648146</v>
+        <v>46188.632178113425</v>
       </c>
       <c r="C53" s="11"/>
       <c r="D53" s="10">
-        <v>46209.809115578704</v>
+        <v>46209.63852795139</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="G53" s="11" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="H53" s="11" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="I53" s="11"/>
-      <c r="J53" s="10">
-        <v>46031</v>
-      </c>
+      <c r="J53" s="11"/>
       <c r="K53" s="11" t="s">
         <v>28</v>
       </c>
@@ -4857,8 +4869,12 @@
         <v>190</v>
       </c>
       <c r="R53" s="11"/>
-      <c r="S53" s="11"/>
-      <c r="T53" s="11"/>
+      <c r="S53" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="T53" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="U53" s="11"/>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -4866,11 +4882,11 @@
         <v>191</v>
       </c>
       <c r="B54" s="5">
-        <v>46094.63446598379</v>
+        <v>46188.632380717594</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46094.63463712963</v>
+        <v>46188.63256951389</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>192</v>
@@ -4894,7 +4910,7 @@
         <v>28</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>28</v>
@@ -4915,26 +4931,30 @@
         <v>194</v>
       </c>
       <c r="B55" s="10">
-        <v>46188.62962413194</v>
+        <v>46164.69760407407</v>
       </c>
       <c r="C55" s="11"/>
       <c r="D55" s="10">
-        <v>46210.660290995365</v>
+        <v>46209.64180571759</v>
       </c>
       <c r="E55" s="11" t="s">
         <v>195</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>46</v>
+        <v>102</v>
       </c>
       <c r="H55" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="I55" s="11"/>
-      <c r="J55" s="11"/>
+        <v>103</v>
+      </c>
+      <c r="I55" s="10">
+        <v>46203</v>
+      </c>
+      <c r="J55" s="10">
+        <v>46203</v>
+      </c>
       <c r="K55" s="11" t="s">
         <v>28</v>
       </c>
@@ -4957,43 +4977,37 @@
         <v>196</v>
       </c>
       <c r="R55" s="11"/>
-      <c r="S55" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T55" s="14" t="s">
-        <v>69</v>
+      <c r="S55" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T55" s="15" t="s">
+        <v>197</v>
       </c>
       <c r="U55" s="11"/>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B56" s="5">
-        <v>46188.63002254629</v>
-      </c>
-      <c r="C56" s="5">
-        <v>46209.92160893518</v>
-      </c>
+        <v>46164.69785174768</v>
+      </c>
+      <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46210.78237596065</v>
+        <v>46164.69809590278</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G56" s="6" t="s">
         <v>28</v>
       </c>
       <c r="H56" s="6"/>
-      <c r="I56" s="5">
-        <v>46195</v>
-      </c>
-      <c r="J56" s="5">
-        <v>46195</v>
-      </c>
+      <c r="I56" s="6"/>
+      <c r="J56" s="6"/>
       <c r="K56" s="6" t="s">
         <v>28</v>
       </c>
@@ -5001,7 +5015,7 @@
         <v>28</v>
       </c>
       <c r="M56" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N56" s="6" t="s">
         <v>195</v>
@@ -5013,42 +5027,36 @@
         <v>28</v>
       </c>
       <c r="Q56" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="R56" s="6"/>
-      <c r="S56" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="S56" s="6"/>
       <c r="T56" s="6"/>
       <c r="U56" s="6"/>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B57" s="10">
-        <v>46188.630276365744</v>
-      </c>
-      <c r="C57" s="10">
-        <v>46210.76125015046</v>
-      </c>
+        <v>46164.69792900463</v>
+      </c>
+      <c r="C57" s="11"/>
       <c r="D57" s="10">
-        <v>46210.761251979166</v>
+        <v>46164.698260185185</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G57" s="11" t="s">
         <v>28</v>
       </c>
       <c r="H57" s="11"/>
       <c r="I57" s="11"/>
-      <c r="J57" s="10">
-        <v>46195</v>
-      </c>
+      <c r="J57" s="11"/>
       <c r="K57" s="11" t="s">
         <v>28</v>
       </c>
@@ -5056,7 +5064,7 @@
         <v>28</v>
       </c>
       <c r="M57" s="11" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N57" s="11" t="s">
         <v>195</v>
@@ -5068,7 +5076,7 @@
         <v>28</v>
       </c>
       <c r="Q57" s="11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="R57" s="11"/>
       <c r="S57" s="11"/>
@@ -5077,29 +5085,31 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B58" s="5">
-        <v>46188.632178113425</v>
+        <v>46133.80470612268</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46209.63852795139</v>
+        <v>46212.571661180555</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="I58" s="6"/>
-      <c r="J58" s="6"/>
+      <c r="J58" s="5">
+        <v>46161</v>
+      </c>
       <c r="K58" s="6" t="s">
         <v>28</v>
       </c>
@@ -5119,30 +5129,30 @@
         <v>28</v>
       </c>
       <c r="Q58" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="R58" s="6"/>
-      <c r="S58" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T58" s="8" t="s">
-        <v>31</v>
+      <c r="S58" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T58" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="U58" s="6"/>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B59" s="10">
-        <v>46188.632380717594</v>
+        <v>46133.80545771991</v>
       </c>
       <c r="C59" s="11"/>
       <c r="D59" s="10">
-        <v>46188.63256951389</v>
+        <v>46133.80564510416</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F59" s="11" t="s">
         <v>28</v>
@@ -5163,7 +5173,7 @@
         <v>28</v>
       </c>
       <c r="N59" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="O59" s="11" t="s">
         <v>28</v>
@@ -5172,7 +5182,7 @@
         <v>28</v>
       </c>
       <c r="Q59" s="11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="R59" s="11"/>
       <c r="S59" s="11"/>
@@ -5181,33 +5191,27 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B60" s="5">
-        <v>46164.69760407407</v>
+        <v>46133.80570512731</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46209.64180571759</v>
+        <v>46133.80583366899</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>189</v>
+        <v>28</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="I60" s="5">
-        <v>46203</v>
-      </c>
-      <c r="J60" s="5">
-        <v>46203</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H60" s="6"/>
+      <c r="I60" s="6"/>
+      <c r="J60" s="6"/>
       <c r="K60" s="6" t="s">
         <v>28</v>
       </c>
@@ -5215,10 +5219,10 @@
         <v>28</v>
       </c>
       <c r="M60" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>28</v>
+        <v>205</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>28</v>
@@ -5227,15 +5231,11 @@
         <v>28</v>
       </c>
       <c r="Q60" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="R60" s="6"/>
-      <c r="S60" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T60" s="15" t="s">
-        <v>212</v>
-      </c>
+      <c r="S60" s="6"/>
+      <c r="T60" s="6"/>
       <c r="U60" s="6"/>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -5243,11 +5243,11 @@
         <v>213</v>
       </c>
       <c r="B61" s="10">
-        <v>46164.69785174768</v>
+        <v>46133.8058850463</v>
       </c>
       <c r="C61" s="11"/>
       <c r="D61" s="10">
-        <v>46164.69809590278</v>
+        <v>46133.80636234954</v>
       </c>
       <c r="E61" s="11" t="s">
         <v>214</v>
@@ -5271,7 +5271,7 @@
         <v>28</v>
       </c>
       <c r="N61" s="11" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="O61" s="11" t="s">
         <v>28</v>
@@ -5292,11 +5292,11 @@
         <v>216</v>
       </c>
       <c r="B62" s="5">
-        <v>46164.69792900463</v>
+        <v>46133.80664880787</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46164.698260185185</v>
+        <v>46133.80681135417</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>217</v>
@@ -5320,7 +5320,7 @@
         <v>28</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>28</v>
@@ -5351,7 +5351,7 @@
         <v>220</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="G63" s="11" t="s">
         <v>46</v>
@@ -5518,7 +5518,7 @@
         <v>229</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="G66" s="6" t="s">
         <v>46</v>
@@ -5764,7 +5764,7 @@
         <v>243</v>
       </c>
       <c r="T70" s="13" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="U70" s="6"/>
     </row>
@@ -6039,7 +6039,7 @@
         <v>30</v>
       </c>
       <c r="T75" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U75" s="11"/>
     </row>
@@ -6253,7 +6253,7 @@
         <v>30</v>
       </c>
       <c r="T79" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U79" s="11"/>
     </row>
@@ -6567,7 +6567,7 @@
         <v>30</v>
       </c>
       <c r="T85" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U85" s="11"/>
     </row>
@@ -6675,7 +6675,7 @@
         <v>40</v>
       </c>
       <c r="T87" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U87" s="11"/>
     </row>
@@ -6783,7 +6783,7 @@
         <v>243</v>
       </c>
       <c r="T89" s="15" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="U89" s="11"/>
     </row>
@@ -6997,7 +6997,7 @@
         <v>30</v>
       </c>
       <c r="T93" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U93" s="11"/>
     </row>
@@ -7376,7 +7376,7 @@
         <v>30</v>
       </c>
       <c r="T100" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U100" s="6"/>
     </row>
@@ -7435,7 +7435,7 @@
         <v>243</v>
       </c>
       <c r="T101" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U101" s="11"/>
     </row>
@@ -7659,7 +7659,7 @@
         <v>30</v>
       </c>
       <c r="T105" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U105" s="11"/>
     </row>
@@ -7718,7 +7718,7 @@
         <v>30</v>
       </c>
       <c r="T106" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U106" s="6"/>
     </row>
@@ -7924,7 +7924,7 @@
         <v>30</v>
       </c>
       <c r="T110" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U110" s="6"/>
     </row>
@@ -8164,10 +8164,10 @@
         <v>34</v>
       </c>
       <c r="G115" s="11" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="H115" s="11" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="I115" s="11"/>
       <c r="J115" s="10">
@@ -8199,7 +8199,7 @@
         <v>40</v>
       </c>
       <c r="T115" s="15" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="U115" s="11"/>
     </row>
@@ -8274,10 +8274,10 @@
         <v>34</v>
       </c>
       <c r="G117" s="11" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="H117" s="11" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="I117" s="11"/>
       <c r="J117" s="10">
@@ -8309,7 +8309,7 @@
         <v>30</v>
       </c>
       <c r="T117" s="15" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="U117" s="11"/>
     </row>
@@ -8439,10 +8439,10 @@
         <v>34</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="H120" s="6" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="I120" s="6"/>
       <c r="J120" s="5">
@@ -8474,7 +8474,7 @@
         <v>30</v>
       </c>
       <c r="T120" s="15" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="U120" s="6"/>
     </row>
@@ -8639,7 +8639,7 @@
       <c r="R123" s="11"/>
       <c r="S123" s="11"/>
       <c r="T123" s="14" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="U123" s="11"/>
     </row>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-20 15:37 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1924" uniqueCount="523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1924" uniqueCount="525">
   <si>
     <t>Tablero Servicios y mantención</t>
   </si>
@@ -1576,6 +1576,23 @@
     <t>50001574 - CORPORACION NACIONAL DEL COBRE DE CHILE</t>
   </si>
   <si>
+    <t xml:space="preserve">Buenas,
+Para el pedido 1574, se debe suministrar 20 unidades de Finales de Carrera y 60 unidades de Interlock para Escotilla para Codelco Andina:
+    Propuestas a la OT- 4372:
+        Final de Carrera Schneider
+        Modelo: ZCMD21L5
+        20 unidades
+    Propuestas a la OT- 4373:
+        Interlock para escotilla de inspección Schneider
+        Modelo: XCSZ05+2NA
+        60 unidades
+ecarico@zitron.com, tu apoyo con la OC.
+    Fecha de entrega: 31-07-2026
+    Material se debe entregar en bodegas Lampa.
+Quedo atenta.
+Saludos,</t>
+  </si>
+  <si>
     <t>TABL3-291</t>
   </si>
   <si>
@@ -1601,6 +1618,19 @@
   </si>
   <si>
     <t>50001575 - CORPORACION NACIONAL DEL COBRE DE CHILE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buenas,
+Para el pedido 1575, se debe suministrar 15 unidades de Sensor Anti-bombeo para Codelco Andina:
+    Reservar a la OT- 4374:
+        Sensor de Bombeo PREMASGARD DS-205F
+        15 unidades
+        Código: 300711
+nespinoza@zitron.com, apóyame con la reserva de los sensores.
+    Fecha de entrega: Inmediata.
+    Material se debe entregar en bodegas Lampa.
+Quedo atenta.
+Saludos,</t>
   </si>
   <si>
     <t>TABL3-294</t>
@@ -10363,7 +10393,7 @@
       </c>
       <c r="C157" s="9"/>
       <c r="D157" s="8">
-        <v>46211.8087634375</v>
+        <v>46220.58485814815</v>
       </c>
       <c r="E157" s="9" t="s">
         <v>509</v>
@@ -10381,7 +10411,7 @@
         <v>28</v>
       </c>
       <c r="L157" s="9" t="s">
-        <v>28</v>
+        <v>510</v>
       </c>
       <c r="M157" s="9" t="s">
         <v>0</v>
@@ -10396,7 +10426,7 @@
         <v>28</v>
       </c>
       <c r="Q157" s="9" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="R157" s="9"/>
       <c r="S157" s="9"/>
@@ -10405,7 +10435,7 @@
     </row>
     <row r="158" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A158" s="4" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B158" s="5">
         <v>46211.80798403935</v>
@@ -10415,7 +10445,7 @@
         <v>46211.808294560185</v>
       </c>
       <c r="E158" s="6" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F158" s="6" t="s">
         <v>28</v>
@@ -10445,7 +10475,7 @@
         <v>28</v>
       </c>
       <c r="Q158" s="6" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="R158" s="6"/>
       <c r="S158" s="6"/>
@@ -10454,7 +10484,7 @@
     </row>
     <row r="159" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A159" s="7" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B159" s="8">
         <v>46211.80830369213</v>
@@ -10464,7 +10494,7 @@
         <v>46211.80867633102</v>
       </c>
       <c r="E159" s="9" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -10494,7 +10524,7 @@
         <v>28</v>
       </c>
       <c r="Q159" s="9" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="R159" s="9"/>
       <c r="S159" s="9"/>
@@ -10503,17 +10533,17 @@
     </row>
     <row r="160" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A160" s="4" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B160" s="5">
         <v>46211.810599143515</v>
       </c>
       <c r="C160" s="6"/>
       <c r="D160" s="5">
-        <v>46211.81092942129</v>
+        <v>46220.58463327546</v>
       </c>
       <c r="E160" s="6" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F160" s="6" t="s">
         <v>491</v>
@@ -10528,7 +10558,7 @@
         <v>28</v>
       </c>
       <c r="L160" s="6" t="s">
-        <v>28</v>
+        <v>520</v>
       </c>
       <c r="M160" s="6" t="s">
         <v>0</v>
@@ -10543,7 +10573,7 @@
         <v>28</v>
       </c>
       <c r="Q160" s="6" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="R160" s="6"/>
       <c r="S160" s="6"/>
@@ -10552,7 +10582,7 @@
     </row>
     <row r="161" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A161" s="7" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B161" s="8">
         <v>46211.810926921295</v>
@@ -10562,7 +10592,7 @@
         <v>46211.81116517361</v>
       </c>
       <c r="E161" s="9" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -10583,7 +10613,7 @@
         <v>28</v>
       </c>
       <c r="N161" s="9" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="O161" s="9" t="s">
         <v>28</v>
@@ -10592,7 +10622,7 @@
         <v>28</v>
       </c>
       <c r="Q161" s="9" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="R161" s="9"/>
       <c r="S161" s="9"/>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-22 14:03 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1924" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1925" uniqueCount="524">
   <si>
     <t>Tablero Servicios y mantención</t>
   </si>
@@ -1614,35 +1614,22 @@
     <t>TABL3-293</t>
   </si>
   <si>
-    <t>1216403382440842</t>
+    <t>1216730497556421</t>
   </si>
   <si>
     <t>50001575 - CORPORACION NACIONAL DEL COBRE DE CHILE</t>
   </si>
   <si>
-    <t xml:space="preserve">Buenas,
-Para el pedido 1575, se debe suministrar 15 unidades de Sensor Anti-bombeo para Codelco Andina:
-    Reservar a la OT- 4374:
-        Sensor de Bombeo PREMASGARD DS-205F
-        15 unidades
-        Código: 300711
-nespinoza@zitron.com, apóyame con la reserva de los sensores.
-    Fecha de entrega: Inmediata.
-    Material se debe entregar en bodegas Lampa.
-Quedo atenta.
-Saludos,</t>
-  </si>
-  <si>
-    <t>TABL3-294</t>
-  </si>
-  <si>
-    <t>1216403382440845</t>
-  </si>
-  <si>
-    <t>ot 4374  - SENSOR DE BOMBEO PREMASGARD S+S DS205</t>
-  </si>
-  <si>
-    <t>TABL3-295</t>
+    <t>TABL3-298</t>
+  </si>
+  <si>
+    <t>1216730497556424</t>
+  </si>
+  <si>
+    <t>OT  4374- SENSOR DE BOMBEO PREMASGARD S+S DS205</t>
+  </si>
+  <si>
+    <t>TABL3-299</t>
   </si>
 </sst>
 </file>
@@ -10536,11 +10523,11 @@
         <v>518</v>
       </c>
       <c r="B160" s="5">
-        <v>46211.810599143515</v>
+        <v>46224.686933460645</v>
       </c>
       <c r="C160" s="6"/>
       <c r="D160" s="5">
-        <v>46220.58463327546</v>
+        <v>46224.68809549768</v>
       </c>
       <c r="E160" s="6" t="s">
         <v>519</v>
@@ -10549,16 +10536,18 @@
         <v>491</v>
       </c>
       <c r="G160" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H160" s="6"/>
+        <v>26</v>
+      </c>
+      <c r="H160" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="I160" s="6"/>
       <c r="J160" s="6"/>
       <c r="K160" s="6" t="s">
         <v>28</v>
       </c>
       <c r="L160" s="6" t="s">
-        <v>520</v>
+        <v>28</v>
       </c>
       <c r="M160" s="6" t="s">
         <v>0</v>
@@ -10573,7 +10562,7 @@
         <v>28</v>
       </c>
       <c r="Q160" s="6" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="R160" s="6"/>
       <c r="S160" s="6"/>
@@ -10582,17 +10571,17 @@
     </row>
     <row r="161" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A161" s="7" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B161" s="8">
-        <v>46211.810926921295</v>
+        <v>46224.68809222222</v>
       </c>
       <c r="C161" s="9"/>
       <c r="D161" s="8">
-        <v>46211.81116517361</v>
+        <v>46224.68857803241</v>
       </c>
       <c r="E161" s="9" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10611,7 @@
         <v>28</v>
       </c>
       <c r="Q161" s="9" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="R161" s="9"/>
       <c r="S161" s="9"/>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-23 16:30 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1925" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1949" uniqueCount="530">
   <si>
     <t>Tablero Servicios y mantención</t>
   </si>
@@ -1532,6 +1532,25 @@
   </si>
   <si>
     <t>TABL3-286</t>
+  </si>
+  <si>
+    <t>1216769310026821</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50001581 -"ZITRON PERU
+(CHUNGAR)"</t>
+  </si>
+  <si>
+    <t>TABL3-300</t>
+  </si>
+  <si>
+    <t>1216769310026824</t>
+  </si>
+  <si>
+    <t>ot 4380 - SENSOR DE VIBRACIONES + ANTIBOMBEO</t>
+  </si>
+  <si>
+    <t>TABL3-301</t>
   </si>
   <si>
     <t>1216403382440825</t>
@@ -2183,7 +2202,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U161"/>
+  <dimension ref="A1:U163"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10.4" customWidth="1"/>
@@ -5085,7 +5104,7 @@
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46209.64557245371</v>
+        <v>46225.84111758102</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>204</v>
@@ -10180,11 +10199,11 @@
         <v>496</v>
       </c>
       <c r="B153" s="8">
-        <v>46211.80559402778</v>
+        <v>46225.85971481481</v>
       </c>
       <c r="C153" s="9"/>
       <c r="D153" s="8">
-        <v>46211.80646408565</v>
+        <v>46226.172708935184</v>
       </c>
       <c r="E153" s="9" t="s">
         <v>497</v>
@@ -10193,11 +10212,17 @@
         <v>491</v>
       </c>
       <c r="G153" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H153" s="9"/>
-      <c r="I153" s="9"/>
-      <c r="J153" s="9"/>
+        <v>165</v>
+      </c>
+      <c r="H153" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="I153" s="8">
+        <v>46225</v>
+      </c>
+      <c r="J153" s="8">
+        <v>46225</v>
+      </c>
       <c r="K153" s="9" t="s">
         <v>28</v>
       </c>
@@ -10220,7 +10245,9 @@
         <v>498</v>
       </c>
       <c r="R153" s="9"/>
-      <c r="S153" s="9"/>
+      <c r="S153" s="10" t="s">
+        <v>33</v>
+      </c>
       <c r="T153" s="9"/>
       <c r="U153" s="9"/>
     </row>
@@ -10229,11 +10256,11 @@
         <v>499</v>
       </c>
       <c r="B154" s="5">
-        <v>46211.80578127315</v>
+        <v>46225.85993190973</v>
       </c>
       <c r="C154" s="6"/>
       <c r="D154" s="5">
-        <v>46211.806155949074</v>
+        <v>46225.86004826389</v>
       </c>
       <c r="E154" s="6" t="s">
         <v>500</v>
@@ -10278,11 +10305,11 @@
         <v>502</v>
       </c>
       <c r="B155" s="8">
-        <v>46211.80647546296</v>
+        <v>46211.80559402778</v>
       </c>
       <c r="C155" s="9"/>
       <c r="D155" s="8">
-        <v>46211.80707378472</v>
+        <v>46211.80646408565</v>
       </c>
       <c r="E155" s="9" t="s">
         <v>503</v>
@@ -10327,11 +10354,11 @@
         <v>505</v>
       </c>
       <c r="B156" s="5">
-        <v>46211.806657256944</v>
+        <v>46211.80578127315</v>
       </c>
       <c r="C156" s="6"/>
       <c r="D156" s="5">
-        <v>46211.80699726852</v>
+        <v>46211.806155949074</v>
       </c>
       <c r="E156" s="6" t="s">
         <v>506</v>
@@ -10376,11 +10403,11 @@
         <v>508</v>
       </c>
       <c r="B157" s="8">
-        <v>46211.80751076389</v>
+        <v>46211.80647546296</v>
       </c>
       <c r="C157" s="9"/>
       <c r="D157" s="8">
-        <v>46220.58485814815</v>
+        <v>46211.80707378472</v>
       </c>
       <c r="E157" s="9" t="s">
         <v>509</v>
@@ -10398,7 +10425,7 @@
         <v>28</v>
       </c>
       <c r="L157" s="9" t="s">
-        <v>510</v>
+        <v>28</v>
       </c>
       <c r="M157" s="9" t="s">
         <v>0</v>
@@ -10413,7 +10440,7 @@
         <v>28</v>
       </c>
       <c r="Q157" s="9" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="R157" s="9"/>
       <c r="S157" s="9"/>
@@ -10422,17 +10449,17 @@
     </row>
     <row r="158" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A158" s="4" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B158" s="5">
-        <v>46211.80798403935</v>
+        <v>46211.806657256944</v>
       </c>
       <c r="C158" s="6"/>
       <c r="D158" s="5">
-        <v>46211.808294560185</v>
+        <v>46211.80699726852</v>
       </c>
       <c r="E158" s="6" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F158" s="6" t="s">
         <v>28</v>
@@ -10462,7 +10489,7 @@
         <v>28</v>
       </c>
       <c r="Q158" s="6" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="R158" s="6"/>
       <c r="S158" s="6"/>
@@ -10471,20 +10498,20 @@
     </row>
     <row r="159" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A159" s="7" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B159" s="8">
-        <v>46211.80830369213</v>
+        <v>46211.80751076389</v>
       </c>
       <c r="C159" s="9"/>
       <c r="D159" s="8">
-        <v>46211.80867633102</v>
+        <v>46220.58485814815</v>
       </c>
       <c r="E159" s="9" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="F159" s="9" t="s">
-        <v>28</v>
+        <v>491</v>
       </c>
       <c r="G159" s="9" t="s">
         <v>28</v>
@@ -10496,13 +10523,13 @@
         <v>28</v>
       </c>
       <c r="L159" s="9" t="s">
-        <v>28</v>
+        <v>516</v>
       </c>
       <c r="M159" s="9" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="N159" s="9" t="s">
-        <v>509</v>
+        <v>28</v>
       </c>
       <c r="O159" s="9" t="s">
         <v>28</v>
@@ -10523,24 +10550,22 @@
         <v>518</v>
       </c>
       <c r="B160" s="5">
-        <v>46224.686933460645</v>
+        <v>46211.80798403935</v>
       </c>
       <c r="C160" s="6"/>
       <c r="D160" s="5">
-        <v>46224.68809549768</v>
+        <v>46211.808294560185</v>
       </c>
       <c r="E160" s="6" t="s">
         <v>519</v>
       </c>
       <c r="F160" s="6" t="s">
-        <v>491</v>
+        <v>28</v>
       </c>
       <c r="G160" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H160" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="H160" s="6"/>
       <c r="I160" s="6"/>
       <c r="J160" s="6"/>
       <c r="K160" s="6" t="s">
@@ -10550,10 +10575,10 @@
         <v>28</v>
       </c>
       <c r="M160" s="6" t="s">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N160" s="6" t="s">
-        <v>28</v>
+        <v>515</v>
       </c>
       <c r="O160" s="6" t="s">
         <v>28</v>
@@ -10574,11 +10599,11 @@
         <v>521</v>
       </c>
       <c r="B161" s="8">
-        <v>46224.68809222222</v>
+        <v>46211.80830369213</v>
       </c>
       <c r="C161" s="9"/>
       <c r="D161" s="8">
-        <v>46224.68857803241</v>
+        <v>46211.80867633102</v>
       </c>
       <c r="E161" s="9" t="s">
         <v>522</v>
@@ -10602,7 +10627,7 @@
         <v>28</v>
       </c>
       <c r="N161" s="9" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="O161" s="9" t="s">
         <v>28</v>
@@ -10617,6 +10642,106 @@
       <c r="S161" s="9"/>
       <c r="T161" s="9"/>
       <c r="U161" s="9"/>
+    </row>
+    <row r="162" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A162" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B162" s="5">
+        <v>46224.686933460645</v>
+      </c>
+      <c r="C162" s="6"/>
+      <c r="D162" s="5">
+        <v>46224.68809549768</v>
+      </c>
+      <c r="E162" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="F162" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="G162" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H162" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I162" s="6"/>
+      <c r="J162" s="6"/>
+      <c r="K162" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L162" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M162" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N162" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="O162" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P162" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q162" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="R162" s="6"/>
+      <c r="S162" s="6"/>
+      <c r="T162" s="6"/>
+      <c r="U162" s="6"/>
+    </row>
+    <row r="163" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A163" s="7" t="s">
+        <v>527</v>
+      </c>
+      <c r="B163" s="8">
+        <v>46224.68809222222</v>
+      </c>
+      <c r="C163" s="9"/>
+      <c r="D163" s="8">
+        <v>46224.68857803241</v>
+      </c>
+      <c r="E163" s="9" t="s">
+        <v>528</v>
+      </c>
+      <c r="F163" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="G163" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H163" s="9"/>
+      <c r="I163" s="9"/>
+      <c r="J163" s="9"/>
+      <c r="K163" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="L163" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="M163" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="N163" s="9" t="s">
+        <v>525</v>
+      </c>
+      <c r="O163" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="P163" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q163" s="9" t="s">
+        <v>529</v>
+      </c>
+      <c r="R163" s="9"/>
+      <c r="S163" s="9"/>
+      <c r="T163" s="9"/>
+      <c r="U163" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualizacion automatica 2026-09-11 17:09 UTC
</commit_message>
<xml_diff>
--- a/data/servicios/Servicios y Mantencion.xlsx
+++ b/data/servicios/Servicios y Mantencion.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2331" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2317" uniqueCount="614">
   <si>
     <t>Tablero Servicios y mantención</t>
   </si>
@@ -11636,7 +11636,7 @@
       </c>
       <c r="C176" s="6"/>
       <c r="D176" s="5">
-        <v>46276.16991603009</v>
+        <v>46245.57038168982</v>
       </c>
       <c r="E176" s="6" t="s">
         <v>562</v>
@@ -11676,9 +11676,7 @@
         <v>563</v>
       </c>
       <c r="R176" s="6"/>
-      <c r="S176" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S176" s="6"/>
       <c r="T176" s="6"/>
       <c r="U176" s="6"/>
     </row>
@@ -11691,7 +11689,7 @@
       </c>
       <c r="C177" s="11"/>
       <c r="D177" s="10">
-        <v>46269.17778488426</v>
+        <v>46245.57032159722</v>
       </c>
       <c r="E177" s="11" t="s">
         <v>565</v>
@@ -11731,9 +11729,7 @@
         <v>566</v>
       </c>
       <c r="R177" s="11"/>
-      <c r="S177" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S177" s="11"/>
       <c r="T177" s="11"/>
       <c r="U177" s="11"/>
     </row>
@@ -11746,7 +11742,7 @@
       </c>
       <c r="C178" s="6"/>
       <c r="D178" s="5">
-        <v>46269.17778503472</v>
+        <v>46245.570321747684</v>
       </c>
       <c r="E178" s="6" t="s">
         <v>565</v>
@@ -11786,9 +11782,7 @@
         <v>568</v>
       </c>
       <c r="R178" s="6"/>
-      <c r="S178" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S178" s="6"/>
       <c r="T178" s="6"/>
       <c r="U178" s="6"/>
     </row>
@@ -11801,7 +11795,7 @@
       </c>
       <c r="C179" s="11"/>
       <c r="D179" s="10">
-        <v>46269.177784907406</v>
+        <v>46245.57032184028</v>
       </c>
       <c r="E179" s="11" t="s">
         <v>565</v>
@@ -11841,9 +11835,7 @@
         <v>570</v>
       </c>
       <c r="R179" s="11"/>
-      <c r="S179" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S179" s="11"/>
       <c r="T179" s="11"/>
       <c r="U179" s="11"/>
     </row>
@@ -11856,7 +11848,7 @@
       </c>
       <c r="C180" s="6"/>
       <c r="D180" s="5">
-        <v>46269.17778489583</v>
+        <v>46245.57032194444</v>
       </c>
       <c r="E180" s="6" t="s">
         <v>572</v>
@@ -11896,9 +11888,7 @@
         <v>573</v>
       </c>
       <c r="R180" s="6"/>
-      <c r="S180" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S180" s="6"/>
       <c r="T180" s="6"/>
       <c r="U180" s="6"/>
     </row>
@@ -11911,7 +11901,7 @@
       </c>
       <c r="C181" s="11"/>
       <c r="D181" s="10">
-        <v>46269.177790138885</v>
+        <v>46245.570322025465</v>
       </c>
       <c r="E181" s="11" t="s">
         <v>572</v>
@@ -11951,9 +11941,7 @@
         <v>575</v>
       </c>
       <c r="R181" s="11"/>
-      <c r="S181" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S181" s="11"/>
       <c r="T181" s="11"/>
       <c r="U181" s="11"/>
     </row>
@@ -11966,7 +11954,7 @@
       </c>
       <c r="C182" s="6"/>
       <c r="D182" s="5">
-        <v>46269.17778440972</v>
+        <v>46245.57032210648</v>
       </c>
       <c r="E182" s="6" t="s">
         <v>572</v>
@@ -12006,9 +11994,7 @@
         <v>577</v>
       </c>
       <c r="R182" s="6"/>
-      <c r="S182" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S182" s="6"/>
       <c r="T182" s="6"/>
       <c r="U182" s="6"/>
     </row>
@@ -12021,7 +12007,7 @@
       </c>
       <c r="C183" s="11"/>
       <c r="D183" s="10">
-        <v>46269.177784733794</v>
+        <v>46245.5703221875</v>
       </c>
       <c r="E183" s="11" t="s">
         <v>572</v>
@@ -12061,9 +12047,7 @@
         <v>579</v>
       </c>
       <c r="R183" s="11"/>
-      <c r="S183" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S183" s="11"/>
       <c r="T183" s="11"/>
       <c r="U183" s="11"/>
     </row>
@@ -12076,7 +12060,7 @@
       </c>
       <c r="C184" s="6"/>
       <c r="D184" s="5">
-        <v>46269.177784837964</v>
+        <v>46245.57032229166</v>
       </c>
       <c r="E184" s="6" t="s">
         <v>572</v>
@@ -12116,9 +12100,7 @@
         <v>581</v>
       </c>
       <c r="R184" s="6"/>
-      <c r="S184" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S184" s="6"/>
       <c r="T184" s="6"/>
       <c r="U184" s="6"/>
     </row>
@@ -12131,7 +12113,7 @@
       </c>
       <c r="C185" s="11"/>
       <c r="D185" s="10">
-        <v>46269.17778493055</v>
+        <v>46245.57032237269</v>
       </c>
       <c r="E185" s="11" t="s">
         <v>572</v>
@@ -12171,9 +12153,7 @@
         <v>583</v>
       </c>
       <c r="R185" s="11"/>
-      <c r="S185" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S185" s="11"/>
       <c r="T185" s="11"/>
       <c r="U185" s="11"/>
     </row>
@@ -12186,7 +12166,7 @@
       </c>
       <c r="C186" s="6"/>
       <c r="D186" s="5">
-        <v>46269.17778439815</v>
+        <v>46245.57032246528</v>
       </c>
       <c r="E186" s="6" t="s">
         <v>572</v>
@@ -12226,9 +12206,7 @@
         <v>585</v>
       </c>
       <c r="R186" s="6"/>
-      <c r="S186" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S186" s="6"/>
       <c r="T186" s="6"/>
       <c r="U186" s="6"/>
     </row>
@@ -12241,7 +12219,7 @@
       </c>
       <c r="C187" s="11"/>
       <c r="D187" s="10">
-        <v>46269.17778489583</v>
+        <v>46245.570322534724</v>
       </c>
       <c r="E187" s="11" t="s">
         <v>572</v>
@@ -12281,9 +12259,7 @@
         <v>587</v>
       </c>
       <c r="R187" s="11"/>
-      <c r="S187" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S187" s="11"/>
       <c r="T187" s="11"/>
       <c r="U187" s="11"/>
     </row>
@@ -12296,7 +12272,7 @@
       </c>
       <c r="C188" s="6"/>
       <c r="D188" s="5">
-        <v>46269.17778454861</v>
+        <v>46245.57032261574</v>
       </c>
       <c r="E188" s="6" t="s">
         <v>572</v>
@@ -12336,9 +12312,7 @@
         <v>589</v>
       </c>
       <c r="R188" s="6"/>
-      <c r="S188" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S188" s="6"/>
       <c r="T188" s="6"/>
       <c r="U188" s="6"/>
     </row>
@@ -12351,7 +12325,7 @@
       </c>
       <c r="C189" s="11"/>
       <c r="D189" s="10">
-        <v>46269.177784837964</v>
+        <v>46245.57032271991</v>
       </c>
       <c r="E189" s="11" t="s">
         <v>572</v>
@@ -12391,9 +12365,7 @@
         <v>591</v>
       </c>
       <c r="R189" s="11"/>
-      <c r="S189" s="16" t="s">
-        <v>265</v>
-      </c>
+      <c r="S189" s="11"/>
       <c r="T189" s="11"/>
       <c r="U189" s="11"/>
     </row>

</xml_diff>